<commit_message>
📰 Daily news update: 2026-05-03
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Germany says U.S. troop withdrawal 'anticipated', Spain and Italy could be next</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Germany says U.S. troop withdrawal 'anticipated', </t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/02/nx-s1-5808891/europe-allies-germany-troop-withdrawal-us</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-04
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1653,1094 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>政治, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260504 19:00</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道五四青年节、假日文旅、返程保障、大国工匠及国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDE8Pkm2I6Uc6H58zuw9ovj260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>[视频]自信自强 昂扬向上 以实干担当书写无悔青春——习近平总书记给中国青年五四奖章暨新时代青年先锋奖获奖者代表的回信在广大青年中引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>习近平回信勉励青年，引发热烈反响，激励青年投身强国建设。</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDE36SPoZPf2k3dezn63sue260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>[视频]各地开展“青年大学习 建功‘十五五’”主题团日活动</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>各地开展“青年大学习”主题团日活动，展现青年活力与担当。</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEcwlWDwqJdKpMV6vTL5Ua260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Former New York City mayor Rudy Giuliani in critical condition in hospital</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>前纽约市长、特朗普盟友朱利安尼病情危重住院。</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c7941rgy4lyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Modi's BJP conquers Bengal, one of India's toughest political frontiers</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>莫迪所在印人党征服西孟加拉邦，或改变该邦及全国政治格局。</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8pdvp5x5ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>New alliances shakes up Nigerian political landscape</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>尼日利亚政坛重组，上次大选第三、四名的候选人转投新政党。</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0q20xzwppdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Reform pledges to open migrant detention centres in Green-voting areas</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>改革党承诺在绿党票仓设立移民拘留中心，遭绿党谴责。</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c362e9p385yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Chris Mason: Elections this week set to show how politics is changing</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>分析称本周选举将暴露工党的广泛弱点，显示政治变迁。</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c202wg747qpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Trump says the U.S. will 'guide' stranded ships from the Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>特朗普称美国将引导霍尔木兹海峡被困船只。</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/03/nx-s1-5809536/trump-strait-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>经济, 科技, 文体</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>一季度电商增长、广交会活动多、数字峰会闭幕、汤姆斯杯卫冕等快讯。</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEB9RvYaBV0E7666y9UbEc260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>What an empty car park tells us about the UK's debt problem</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>从空停车场看英国债务问题：BBC采访了英格兰最贫困社区之一。</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy816xdp226o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>[视频]【大国工匠】梁凌宇：为电网铸造“AI底座”</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>大国工匠梁凌宇打造首个电力AI大模型，支撑新型电力系统。</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEEvreM4XxUXyvzVtt6UHG260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Ukrainian drone hits upmarket Moscow high-rise ahead of Victory Day celebrations</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>乌克兰无人机袭击莫斯科高档住宅楼，俄胜利日阅兵前夕局势紧张。</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy234llx3vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2 U.S. service members missing after military exercises in Morocco</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>两名美军在摩洛哥参加多国演习后失踪。</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/04/g-s1-119963/2-us-service-members-missing-in-morocco</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>[视频]假日活动丰富多彩 文旅市场持续火热</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>五一假期文旅市场火热，各地推出丰富活动吸引游客。</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEIVKYZU1tWpe8BH3KgWpW260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>[视频]交通部门全力做好返程出行服务保障</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>返程客流高峰，交通部门加开列车、监控路况保障出行。</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEZ9GcVUIQ5n4wRCTb3nem260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[视频]活力中国</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>春夏之交，中国各地农事繁忙，展现现代农业蓬勃生机。</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEy5v18MKL4IvEPy4RxLLG260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>[视频]多国人士敦促日本正视东京审判 彻底反省历史罪责</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>多国人士敦促日本正视东京审判，彻底反省历史罪责，维护国际秩序。</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEWHtcrpwE5jBb5JT9zlnN260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>[视频]日本人士呼吁守护和平宪法</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>日本人士呼吁守护和平宪法，反对高市政权修宪和扩军政策。</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEv5tFfDAVjr6OHqO8bPST260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称现阶段谈判不涉及核问题 美称将在霍尔木兹海峡开始疏导行动</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>伊朗称谈判不涉核问题，美将在霍尔木兹海峡疏导船只，双方对峙加剧。</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEchigdrbLJs9BgAKN4AA2260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Antisemitism 'allowed to come into the open' says Bondi victim's daughter</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>邦迪袭击案受害者女儿称反犹太主义已“公开化”，首次在皇家委员会作证。</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1m2rk209mzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>North Korean side to make rare trip to South Korea</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>朝鲜男足代表团本月将罕见访问韩国，参加比赛。</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cx216122kv1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Nigeria plans to repatriate nationals willing to leave South Africa after attacks</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>尼日利亚计划从南非接回愿回国的国民，因当地发生反移民暴力抗议。</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78q6e98878o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Israeli attacks kill dozens within days in Lebanon despite ceasefire</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>尽管有停火协议，以色列几天内在黎巴嫩南部空袭致77人死亡。</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy523z7x0g5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>国际, 政治, 经济</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>UK joining Ukraine loan scheme would be good for EU ties, Starmer says</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>英首相表示，加入欧盟对乌780亿英镑贷款计划有利于英欧关系。</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1420e1p1l0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>What we know about Trump's 'Project Freedom' aimed to help stranded ships through Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>特朗普的“自由计划”旨在引导被困船只通过霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g437depzpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Trump says U.S. will 'guide' stranded ships through the Strait. And, key Senate races to watch</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>特朗普称美国将引导霍尔木兹海峡被困船只；参议院关键席位待关注。</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/04/g-s1-119970/up-first-newsletter-strait-of-hormuz-iran-lousiana-congressional-maps-senate-democrats-claim-sharks-rudy-giuliani</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>[视频]【你要为谁点个赞】点赞奋斗者 每一份付出都有光</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>五一劳动节，街头采访为劳动者点赞，致敬每一份付出。</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/04/VIDEIK69MHWb8WzonyNW0MAZ260504.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Three dead in suspected virus outbreak on Atlantic cruise ship</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>大西洋邮轮疑似病毒爆发，三名乘客死亡，原因尚待确认。</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy0294829ndo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>BBC uncovers the scammers exploiting dogs to elicit donations from animal lovers</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>BBC揭露乌干达骗子利用狗骗取动物爱好者捐款，中饱私囊。</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g9l74wvd7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Princess Eugenie expecting third child this summer</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>尤金妮公主宣布今夏将迎来第三个孩子，查尔斯国王闻讯欣喜。</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp246d9k1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Peter Kay bomb hoax accused removed from court</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>喜剧演员皮特·凯遭遇炸弹恶作剧，伯明翰体育馆被紧急疏散。</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp3pzgdgx53o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Rescuers help Timmy, a stranded whale, return home</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>救援人员不顾警告，用驳船将搁浅座头鲸“蒂米”送回北海。</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/04/nx-s1-5807511/rescuers-help-timmy-a-stranded-whale-return-home</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Met Gala 2026: How to watch, the price of tickets and this year's theme</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2026年Met Gala公布主题、票价及观看方式，碧昂丝将担任联合主席。</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdrm7gp5er3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-05
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3541,6 +3541,966 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>政治, 民生, 经济</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260505 19:00</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道习近平对烟花厂爆炸作指示、重大工程、春耕、大宗商品、五一消费等。</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEWUEAuJ5qBfFf7MbXch3e260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[视频]习近平对湖南长沙浏阳市一烟花厂爆炸事故作出重要指示强调 抓好重点行业领域风险隐患排查整治 加强公共安全管理 确保人民群众生命财产安全 李强作出批示</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>习近平对湖南浏阳烟花厂爆炸事故作出重要指示，要求排查隐患、确保安全。</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEYJnXJGFqKKCc5qSxHnCL260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Romanian PM ousted in no-confidence vote</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>罗马尼亚总理在不信任投票中被罢免，其联盟最大党与极右翼联手倒戈。</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgkpjz2638ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Hate crime prosecutions to be fast-tracked after antisemitic attacks</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>英格兰和威尔士检察长指示对仇恨犯罪起诉从速处理，以应对反犹袭击。</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz72eye5zzeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SCOTUS temporarily restores mifepristone access. And, Indiana, Ohio vote in primaries</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>美国最高法院暂时恢复堕胎药米非司酮使用；印第安纳州初选考验特朗普影响力。</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/05/g-s1-120151/up-first-newsletter-iran-us-strait-of-hormuz-ohio-indiana-primaries-medication-abortion</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>[视频]【实干笃行创伟业 团结奋斗新征程】重大工程扎实推进 夯实经济发展根基</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>五一期间“十五五”重大工程和各地重点工程加速推进，夯实经济发展根基。</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEEr1VdhqGiNSy5zyXghfU260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】各地加大科技支撑 夯实粮食生产基础</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>各地加大科技支撑，推广良种和新技术，夯实粮食生产基础。</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDE2N8ibYYkO6DHse3TonJu260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>[视频]大宗商品市场运行稳定向好</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>4月大宗商品价格指数环比上涨1.7%，市场运行稳定向好。</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEoYHQERmHHgVAwXQx1z6Z260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>[视频]“五一”假期消费活力持续释放</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>五一假期消费活力释放，商圈客流增长，服务消费和以旧换新需求旺盛。</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEY7wTXCM9jWj6rHWf5Uqb260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>[视频]第139届广交会今天闭幕</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>第139届广交会闭幕，境外采购商超31万，参展企业结构优化，高科技产品成焦点。</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEXyKNv8rww8HzjjE0225u260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>[视频]美称将推进对欧盟汽车加征关税计划 欧方称美方有政治目的将予以反制</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>美国将推进对欧盟汽车加征关税计划，欧盟称有政治目的将反制，德国汽车行业受重创。</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEwhtb6JrWaG3rnFHKgJpv260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>科技, 经济, 文体</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>数据设施覆盖15行业；华龙一号机组进入带核调试；五一档票房超7.37亿；吴宜泽夺斯诺克世锦赛冠军。</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDElDpn6JwEjOJ9me2lMjWG260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Russian attacks kill at least 20 ahead of rival ceasefires proposed by Kyiv and Moscow</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>俄袭击致至少20死，乌方提议5月6日停火，俄方为胜利日游行宣布暂停。</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1e2zjz22p9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Bowen: Strait of Hormuz standoff raises risk of sliding back into all-out war</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>霍尔木兹海峡对峙升级，美伊持续施压危及脆弱海湾停火，有全面战争风险。</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgrpnq00j5vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>国际, 经济, 社会</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>[视频]“五一”入境游升温 外国游客感受多彩中国</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>五一入境游升温，外国游客深入小城体验非遗和科技，消费增长显著。</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEj1j1s1kRrrwXY7yLom9K260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>[视频]中国代表：国际社会应高度警惕日本涉核消极动向</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>中国代表在联合国警告日本涉核消极动向，并对美英澳核潜艇合作表达严重关切。</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDE6EeNHukhKaczkh4VWjO1260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>[视频]美称在霍尔木兹海峡击沉6艘伊朗小型船只 伊称美“疏导”行动将酿僵局</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>美军在霍尔木兹海峡击沉6艘伊朗小船，伊朗称造成平民死亡，阿联酋遭无人机袭击。</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDE3mFSl2MxMbItaIkeppRx260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>中国向黎交付援助；俄乌宣布本周停火；欧洲政治共同体聚焦自主；华盛顿发生枪击事件。</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEQEMoA6hJ9T26ASqclBHV260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Hantavirus may have spread between passengers on cruise ship, WHO says</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>世界卫生组织称汉坦病毒可能在邮轮上人传人，已确认两例，三人死亡。</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2p186gyp2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Palestine Action activists guilty of criminal damage</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>四名巴勒斯坦行动活动者因闯入布里斯托尔附近工厂被判刑事破坏罪。</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2p99rxr5po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Canadian prime minister says Europe will anchor world order</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>加拿大总理马克·卡尼称欧洲将替代美国成为未来世界秩序核心。</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/05/nx-s1-5810533/canadian-prime-minister-says-europe-will-anchor-world-order</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>U.S. says the Iran ceasefire holds despite attacks in Strait of Hormuz and against UAE</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>美国称伊朗停火协议有效，仅两艘商船通过霍尔木兹海峡新航线。</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/05/nx-s1-5811770/iran-war-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>[视频]“五一”假期 全社会跨区域人员流动量预计超15亿人次</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>五一假期全社会跨区域人员流动量预计超15亿人次，创历史新高。</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEL6kuYyrOAQd8VQmtfjkC260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>[视频]【劳动者之歌】马晓晨：像石子一样 扎根戈壁盐滩</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>90后博士马晓晨扎根青海戈壁盐滩，创新技术寻找国家紧缺矿产资源。</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDEenQ0ra9pAcI46ZfYieua260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>[视频]二十四节气·立夏</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>立夏至，万物生长，农事繁忙，各地有喝七家茶、吃立夏饭等风俗。</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/05/VIDERwhHGP6SWjGKIQnOq5wo260505.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>社会, 经济</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Nine coal miners die in gas explosion in Colombia</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>哥伦比亚煤矿瓦斯爆炸致9名矿工死亡，该地2023年曾发生致命事故。</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdxpe02y05go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Two killed and many injured after car driven into crowd in German city of Leipzig</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>德国莱比锡汽车冲入人群致2死多伤，一33岁德国公民被拘留。</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ckgpzgxgz58o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Woman, 35, died in explosion after ex-partner 'forced entry' into her home</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>35岁女子因前伴侣强行闯入家中爆炸身亡，警方按凶杀案处理。</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21q55gz12o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>An explosion at a fireworks plant in China kills at least 26 people, state media says</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>中国一烟花厂发生爆炸，至少26人死亡，救援已基本完成。</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/05/g-s1-120137/explosion-fireworks-plant-china</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Cruise ship waiting for help after 3 people died in a suspected hantavirus outbreak</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>一艘游轮因疑似汉坦病毒爆发致3人死亡，在大西洋佛得角外海等待救援。</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/05/g-s1-120130/cruise-ship-hantavirus-outbreak</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-06
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4501,6 +4501,902 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见孟加拉国外交部长</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>王沪宁在京会见孟加拉国外交部长，双方就深化中孟关系达成共识。</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDE4u9DPCiIJky5MNLROo6H260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】奋力谱写中国式现代化广西篇章 浙江高质量发展建设共同富裕示范区</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>广西和浙江分别发布“十五五”规划纲要，聚焦高质量发展和共同富裕。</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEANcXFzt7lHWssOA8kv6N260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Trump's hopes for an Iran peace deal come with caveats</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>特朗普对伊朗和平协议持谨慎态度，称有进展但需警惕。</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzp74rvj5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Democrats gain midterm edge, NPR poll shows. And, U.S. pauses 'Project Freedom'</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>民调显示民主党在中期选举中势头领先。特朗普称因伊朗协议进展暂停“自由计划”。</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/06/g-s1-120384/up-first-newsletter-economy-democrats-poll-advantage-indiana-primary-project-freedom-paused</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>经济, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260506 19:00</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>五一假期消费市场活力迸发，机器人出口开门红，各地推动好房子建设。</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEQy8Im6CGN6Tuojujmyjt260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】“五一”假期消费市场活力迸发</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>五一假期消费活力迸发，新场景新业态涌现，超大规模市场优势释放。</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEQVjedku2OJmSEl2b4J88260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】草原上的新产业</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>内蒙古乌兰察布因低温吸引AI企业落户，算力中心快速增长，绿电直连保障用电。</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEgDCVXMjP7VaUdfnRMUkG260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>五一假期银联网联交易额7.85万亿元，城市公园接待超2.12亿人次，食品及免税购物数据公布。</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDECZyGqyaF1KzkjatUxY4P260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>[视频]欧盟敦促美国遵守已有贸易协议</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>欧盟敦促美国遵守已签贸易协议，批评关税威胁破坏稳定，将启用应对工具。</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEezdSB4XC7C0AYVemEnog260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>经济, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>People urged not to cancel flights over fuel shortage fears</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>中东冲突致油价飙升，全球5月航班削减1.3万架次。</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cyv24v3mpdmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Up to 150 former WHSmith high street stores to close</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>WHSmith百货150家店将关闭，易主后更名TGJones。</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypzvqzqd7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国机器人出口实现开门红</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>一季度我国机器人出口113.2亿元，清洁机器人出口占68.5%成主力。</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEjOzbhq12kK61xpDKdJZF260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>[视频]我国生态环境监测体系持续向数字化智能化转型</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>我国生态环境监测网络将扩容至5万余个点位，向数字化智能化转型。</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEa6rMhB2wQjUhjMpUFtyS260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Massive Alaska megatsunami was second largest ever recorded</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>新研究称冰川融化致气候变暖，增大了巨型海啸风险。</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1m253033m4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Russia ignores Ukraine's unilateral ceasefire and attacks kindergarten</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>俄无视乌单方停火，袭击幼儿园，乌方决定进一步行动。</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpdpxdd5n6yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>军事, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Skeletons in their clothing: Recovering bodies from the rubble in Gaza</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>加沙冲突中最致命袭击之一，一年半后幸存者仍在废墟中寻找亲人遗骸。</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/06/nx-s1-5811930/gaza-recovering-bodies</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>U.S. stages largest-ever annual military drills in the Philippines</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>美国在菲律宾举行史上最大规模军演，展示新战术威慑中国，中方也在附近演习。</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/06/nx-s1-5810616/u-s-stages-largest-ever-annual-military-drills-in-the-philippines</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>[视频]“五一”假期全社会跨区域人员流动量创历史同期新高</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>五一假期全社会跨区域人员流动量达15.17亿人次，创历史新高。</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEdNaAtziQFJs1dvCn8D48260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>[视频]各地加快推动“好房子”建设</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>各地加快制定地方标准，推动安全、舒适、绿色、智慧的“好房子”建设。</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEtMuhq6mbnlPqUy7N1Xq3260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>What is hantavirus and how does it spread? Key questions after outbreak</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>汉坦病毒疫情暴发，安第斯病毒株可人际传播引担忧。</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8r8j1l6j0go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>[视频]日本和平团体举行集会 抗议日本政府一系列危险动向</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>日本和平团体在东京集会，抗议政府危险动向，要求维护和平宪法。</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEQ7xgJX69RnnxY4PAI0ZY260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称美极限施压不会成功 美宣布暂停“自由计划”行动</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>伊朗拒绝对话强迫，启动霍尔木兹海峡新管理机制；美暂停自由计划行动。</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDETfet1jplVrQx1eqNDUgD260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>黎以停火后冲突仍频，中东能源危机重创欧盟，古巴外长驳斥美方言论。</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/06/VIDEqARCfFE4pF9GSDA73vrE260506.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Oil prices drop and stock markets rise after reports of deal to end Iran war</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>报道称美伊接近达成协议，油价下跌，股市上涨。</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g8zejyyr3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Iran is reviewing a U.S. proposal as Trump threatens renewed bombing if it doesn't agree</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>伊朗正评估美国提案，特朗普威胁若不同意将重启轰炸。伊朗将通过巴基斯坦转达回应。</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/06/nx-s1-5813497/iran-war-strait-hormuz-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Ted Turner, media mogul who revolutionised TV news by launching CNN, dies at 87</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>CNN创始人、媒体大亨特德·特纳去世，享年87岁，曾开创24小时新闻时代。</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1k2jnx8gmlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>German police raid neo-Nazi criminal youth groups</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>德国警方在12州突袭搜查新纳粹青年犯罪团伙。</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgkpmy6l2deo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Greetings from a sea village in Indonesia, where Indigenous fishing gets help from mangroves</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>印尼海上村庄，原住民靠红树林辅助传统捕鱼。</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/06/g-s1-119852/indonesia-mangrove-conservation-fishing-sulawesi-bajau</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-07
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5397,6 +5397,902 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260507 21:00</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道新型能源体系、领导人会见、五一出行、天舟九号等多项国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEUecn865Ag3UAKa7rUkrh260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>[视频]李强会见乌兹别克斯坦总理</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>李强会见乌兹别克斯坦总理，双方愿深化贸易投资、能源资源等合作，推动中乌命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEvUyAlguQlUYzHZqBP0Eq260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>[视频]李强会见美国国会参议员代表团</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>李强会见美国会参议员，强调加强对话、管控分歧，重申台湾问题是中美关系第一条不可逾越的红线。</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEPEDhmXsjllmkwPhrbotw260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见美国国会参议员代表团</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>赵乐际会见美国会参议员，希望美方恪守一个中国原则，推动中美立法机构交流，稳定中美关系。</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEbzpXGPUSA6NGGUwozXvM260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>[视频]魏凤和案、李尚福案一审宣判</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>魏凤和、李尚福因受贿等罪被军事法院判处死刑，缓期二年执行，终身监禁不得减刑假释。</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEbQenhjLeLrBNmgcPwZYD260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>UK immigration officer among two men guilty of working for Chinese intelligence</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>英国一名移民官员因利用数据库追踪香港异见人士被判为华间谍。</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0m2wjlkzplo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Rubio visits Vatican amid escalating tensions between Trump and Pope Leo</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>鲁比奥访问梵蒂冈，试图缓解特朗普与教皇间的紧张关系。</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/07/g-s1-120813/rubio-visits-vatican-amid-escalating-tensions-between-trump-and-pope-leo</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>China gives suspended death sentences to 2 ex-defense ministers</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>中国前国防部长被判处死刑缓期执行，系反腐运动最新案例。</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/07/g-s1-120688/china-gives-suspended-death-sentences-to-2-former-defense-ministers-accused-of-bribery</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】新型能源体系加快建设 筑牢能源安全根基</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>我国加快推进新型能源体系建设，清洁能源装机增长迅速，能源自给率稳定在80%以上。</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEourQxV3z0WexTWDRngpx260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】奋力谱写中国式现代化甘肃篇章 推动吉林全面振兴取得新突破</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>甘肃、吉林发布“十五五”规划，聚焦产业升级、新能源、科技创新等，推动区域全面振兴。</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEZG3KwtaRL4g9y3RSy1yW260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>经济, 社会, 文体</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>[视频]“五一”假期国内出游3.25亿人次</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>五一假期国内出游3.25亿人次，同比增长3.6%，文旅消费升级，入境游客达243万人次。</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEXJqbAUhpQYwLdggwJoSO260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国智能消费设备制造增长明显</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>一季度我国智能消费设备制造增长明显，智能手机产量同比增6.9%，集成电路产量增24.3%。</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEjywkOHJp7FBMHBrh2egt260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Dirty nickel: The cost of mining in Indonesia</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>印尼镍矿开采带来就业，但引发环境和健康担忧。</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/07/g-s1-118218/indonesia-nickel-mineral-mining</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>[视频]天舟九号货运飞船顺利撤离空间站并受控再入大气层</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>天舟九号货运飞船撤离空间站并受控再入大气层，残骸落入预定安全海域。</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEIu5dlBadtvAmdCGkERxS260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Rosenberg: Russia's Victory Day parade with no tanks a sign Ukraine war not going to plan</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>俄罗斯胜利日阅兵多年首次无坦克，显示乌克兰战事不顺。</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2gj2jlr8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】办好为民实事 推动学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>四川宜宾、福建厦门深入学习教育，聚焦老旧小区改造、教育医疗等民生实事，提升治理效能。</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEehvXctEs5Iw5VOAVpfVT260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>民生, 经济, 政治</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>国家防总部署南方强降雨防范；4月末外汇储备34105亿美元；五一高速充电量增52.8%；发明专利有效量达631.8万件。</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEUMB44XTiIFFrsPVUHP9B260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>[视频]美总统称对美伊达成协议表示乐观 伊朗称美国必须赔偿伊朗损失</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>特朗普对美伊达成协议表示乐观，伊朗要求美国赔偿损失，以色列称准备对伊军事行动。</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEVJTKjUwKRc1kwuH57VTa260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>[视频]俄外交部呼吁各国准备好及时从基辅撤离人员 乌称乌单方面停火后俄袭击未停</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>俄方敦促驻基辅人员撤离，乌称单方面停火后俄袭击未停，双方相互指责。</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDE73Z8OAsKJRy0khOKhefn260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>以军空袭贝鲁特南郊致2死；美议员要求披露以色列核武详情；法国通过简化文物归还草案。</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/07/VIDEvMTuU6LRaioxsHjhJIpF260507.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Hantavirus outbreak on cruise ship not start of pandemic, UN health agency says</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>世卫组织称邮轮汉坦病毒爆发不构成新大流行，因其传播方式与新冠不同。</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cnvpzgn26edo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Three women linked to Islamic State arrested in Australia on return from Syria</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>三名涉嫌支持伊斯兰国的女性从叙利亚返回澳大利亚后被捕。</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czj2emlv2kjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Fears of renewed Gaza war as Hamas disarmament talks stall</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>加沙停火谈判陷入僵局，以色列被指准备恢复战斗致战争风险上升。</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd6p5l3n2q3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Iran reviews U.S. proposal. And, Rubio to meet Pope Leo after Trump's criticism</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>伊朗审议美国提案终止战争，鲁比奥将见教皇。</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/07/g-s1-120673/up-first-newsletter-iran-trump-oil-production-pope-leo-marco-rubio-prediction-markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>About 40 passengers previously left ship hit by hantavirus at island of St. Helena</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>约40名乘客因汉坦病毒在圣赫勒拿岛离船。</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/07/nx-s1-5814632/passengers-left-ship-hantavirus-st-helena</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>US judge releases Jeffrey Epstein's purported suicide note</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>美国法官公布爱泼斯坦疑似自杀遗书，其前狱友称发现该字条。</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd7pd0rqwreo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>David Attenborough says he is 'overwhelmed' by 100th birthday messages</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>大卫·爱登堡在百岁生日前夕感谢粉丝祝福，称“非常感动”。</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp3pww9g0p5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Police say man arrested over 'intimidating behaviour' near Andrew's home</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>一男子因在安德鲁王子寓所附近实施恐吓行为被警方逮捕。</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c072z2gm5lxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-08
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F183"/>
+  <dimension ref="A1:F210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6293,6 +6293,870 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260508 19:00</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>塔吉克斯坦总统将访华；粤港澳大湾区发展；行政复议法条例修订；天舟十号即将发射等要闻。</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDECLp0nkVofw5YOQBdZC4G260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 塔吉克斯坦总统将对华进行国事访问</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>应习近平邀请，塔吉克斯坦总统拉赫蒙将于5月11日至14日对华进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEnp2540SNtrH9w6h2FABM260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>[视频]李强签署国务院令 公布修订后的《中华人民共和国行政复议法实施条例》</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>李强签署国务院令，公布修订后的《行政复议法实施条例》，自7月1日起施行。</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEdrRZUuzP2yyhE3dhd3i9260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>多部门部署三下乡活动；完善儿童用药保障；科技型中小企业贷款增长；发布人工智能终端分级标准。</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEnipXAwW79jjYVaqwjftH260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Henry Zeffman: Election results leave Starmer vulnerable</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>选举结果使英国首相斯塔默处境脆弱，分析人士评论。</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/clyp1qgxke7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>What latest election results show us in maps and charts</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>最新选举结果以地图图表展示各党派在英国胜败情况。</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0ljrp76ywxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Reform election gains show historic shift in British politics, says Farage</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>法拉奇称改革党选举进展彰显英国政治历史性转变。</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0r255xlr59o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Election results so far - and what's still to come</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>初步计票显示改革党在地方选举中蚕食工党与保守党席位。</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgz155y9exo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】粤港澳大湾区加快打造高质量发展动力源</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>粤港澳大湾区加快打造高质量发展动力源，推进科技创新与新质生产力培育。</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEKQ40grZWnfvNVZLFC1iu260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>[视频]我国营商环境持续改善</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>我国营商环境持续改善，五项“一件事”改革完成，市场准入壁垒得到清理。</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDE4aGosQiEBVWjcvErHwSH260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>[视频]培育消费新场景新业态 激发消费新动能</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>各地培育消费新场景新业态，首店首发密集落地，激发消费市场新活力。</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEqO0d9GJRlRfCrXmKfrAV260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】新技术新装备助力农业生产</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>各地采用新技术新装备，提升播种与收割效率，为丰产丰收打基础。</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDErhtMmyJIZXZLTLtcfU7Q260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥在调研基础研究时强调 深入贯彻落实加强基础研究座谈会精神 全面提升基础研究水平和原始创新能力</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>丁薛祥调研基础研究，强调发挥举国体制优势，全面提升原始创新能力。</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEzWmpgcXYM1J32g0ccwkb260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>[视频]天舟十号船箭组合体转运至发射区 将于近日择机发射</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>天舟十号船箭组合体转运至文昌发射区，将于近日择机发射。</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEur5WDeTkHoX0Sai0f9Ks260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>International cyber attack disrupts swathe of universities and schools</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>全球多地学校遭网络攻击，黑客入侵学术软件Canvas系统。</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce3pq0136eqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>U.S. intercepts Iranian attacks on 3 ships. And, what to know about hantavirus</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>美国拦截伊朗对三艘军舰的攻击，同时关注汉坦病毒疫情。</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/08/g-s1-121064/up-first-newsletter-iran-us-tennessee-congressional-maps-hantavirus-tariffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>The U.S. fires on 2 Iranian tankers trying to evade its blockade in Gulf of Oman</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>美军在阿曼湾开火击中两艘试图突破封锁的伊朗油轮，脆弱的停火协议再遭重创。</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/08/g-s1-121061/iran-war-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Military drills on the edge: U.S. and allies test capabilities near Asia's flash points</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>美国及其盟友在菲律宾测试无人机船和远程导弹等新战术，增强对华威慑。</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/08/g-s1-120681/drills-us-allies-test-capabilities-asia-flash-points</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>[视频]日本民众举行集会抗议高市政权推动扩军修宪等危险动向</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>日本民众集会反对扩军修宪；俄方警告日本再军事化威胁地区安全。</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEqdJMXeIqclC6LkgwoMkL260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>[视频]美国和伊朗在霍尔木兹海峡区域再度交火 伊媒称目前局势恢复正常</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>美伊在霍尔木兹海峡交火，双方均称遭袭并回击，但无意升级局势。</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDEaUy9pHUIhTXVWMAtHlrS260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>俄宣布胜利日停火但指责乌方违反；粮农组织警告中东紧张影响粮食；美关税政策被判违法。</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/08/VIDE4cSjcT4g0eO1PlPuY7BD260508.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Iran accuses US of 'reckless military adventure'</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>伊朗外长指责美国在有外交解决方案时采取鲁莽军事行动。</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c99lpn9ze8ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Russia and Ukraine accuse each other of breaching Victory Day ceasefire</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>俄乌互指违反胜利日停火协议，各自报告遭受数百次无人机攻击。</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c202zn5gg0lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Worldwide race to trace passengers from hantavirus-hit cruise ship</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>多国追踪汉坦病毒爆发邮轮乘客，联合国证实至少五例病例。</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp1505p84o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Colombia's rogue hippos could find refuge in India</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>哥伦比亚计划扑杀河马遭印富豪反对，提议转移至保护区。</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/08/nx-s1-5814169/cocaine-hippos-colombia-india</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>White House calls Mark Hamill 'sick' after actor's Trump grave post</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>《星球大战》演员因发侮辱特朗普AI图道歉删帖，白宫批其病态。</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g723pkgllo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>社会, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Spain readies for evacuations as a hantavirus-hit cruise ship heads for Canary Islands</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>西班牙准备安置一艘驶往加那利群岛的游轮上140余名感染汉坦病毒的乘客和船员。</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/08/g-s1-121055/spain-readies-for-evacuations</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-09
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:F242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7157,6 +7157,1030 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260509 19:00</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道种业振兴、外贸增长、造船领跑、天舟十号合练等多项重要新闻。</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEPTr4753lNDBEfcVBAH9z260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】加快推进种业振兴 提升种源安全保障能力</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>我国深入实施种业振兴行动，提升种源安全保障，实现“中国粮”主要用“中国种”。</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEpgKSDXMejGHiHUzxYu40260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，部署经济工作、基础研究及风险化解，强调稳中向好。</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDE9DKu589hmyRC3CRWUtry260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】奋力开创中国式现代化福建实践新局面 谱写社会主义现代化新疆新篇章</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>福建、新疆发布“十五五”规划，聚焦高质量发展、两岸融合和现代化建设。</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDESobBUnFfUrDxhLadzosq260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>[视频]俄罗斯纪念卫国战争胜利81周年</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>俄罗斯在莫斯科红场举行阅兵式，纪念卫国战争胜利81周年，普京出席并发表讲话。</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEQuafGaWYN36bSbJsY2Al260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Putin denounces Nato at scaled back Victory Day parade</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>普京在缩水的胜利日阅兵式上谴责北约，并为其在乌克兰的军事行动辩护。</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c626xjq0q0vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>'I will serve not rule over Hungary,' says new PM</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>匈牙利新总理表示将服务而非统治国家，其政党终结了欧尔班16年执政。</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce3pqvvzgnko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Australia's right-wing One Nation party scores historic parliamentary win</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>澳大利亚右翼单一民族党在补选中首次赢得众议院席位。</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2e4z4npro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>PM turns to old Labour hands after election losses but some MPs left baffled</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默选举失利后重用老工党成员，部分议员困惑。</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2k2vyw88n8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Labour MPs have put Starmer on notice after election battering. Can he turn it around?</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>工党议员对斯塔默施压要求改革，首相面临扭转局面的压力。</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21e79qqlgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Lib Dems offer alternative to extremes of Reform and Greens, Davey says</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>自由民主党领袖称该党在工党和保守党支持率下滑中获益。</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2029ljyq25o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>We welcome scrutiny, Reform UK says after major election gains</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>改革党在大选获重大进展后表示欢迎 scrutiny，不视选民为理所当然。</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz62d2482x1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>[视频]前4个月我国外贸继续保持两位数增长</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>前4个月我国外贸总值16.23万亿元，同比增长14.9%，绿色产品出口强劲。</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEy4Jvyi5Djk8tfMczmxW4260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国服务出口同比增长11.2% “含新量”不断提升</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>一季度服务出口同比增长11.2%，知识密集型及旅行服务增长最快。</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEznogSO16p9aaA6K4DCFT260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>[视频]一季度中国造船领跑全球 新接订单量增长近三倍</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>一季度中国造船三大指标领跑全球，新接订单量同比增长195.2%。</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEdgZNqdYcPDr7Hak0HwX2260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>经济, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>APEC贸易部长会议将在苏州举办；中央环保督察全部进驻；4月仓储指数扩张；中央下达458亿元支持学前教育。</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEWKkumab8Yo10zhgtF6Gn260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>[视频]天舟十号货运飞船发射任务完成全区合练</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>天舟十号货运飞船发射任务完成全区合练，各系统准备就绪，空间站已调相变轨。</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEyYze2vFdr0kJnqTtq0ur260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>International cyber attack disrupts swathe of universities and schools</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>国际网络攻击入侵学术软件Canvas，全球数千所院校受影响。</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce3pq0136eqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Rosenberg: Scaled-back Victory Parade in Moscow's Red Square</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>莫斯科红场胜利日阅兵规模缩减，场面较往年冷清。</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/ckgp541p5ndo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>HMS Dragon heads to Middle East for potential Strait of Hormuz mission</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>英国“龙”号驱逐舰将赴中东，待地区战事结束后加入护航任务。</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g42j15p7qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Moscow marks Victory Day with a Red Square parade under tight security</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>莫斯科红场胜利日阅兵加强安保，美斡旋三日停火缓解乌滋扰担忧。</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/09/nx-s1-5816876/russia-victory-day</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Britons on virus-hit cruise ship to isolate at hospital after being flown to UK</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>英国“MV Hondius”号邮轮因疫情停靠加那利群岛，乘客将隔离于医院。</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2029r42w8wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Warm weekend forecast before Arctic air brings cold spell next week</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>本周末短暂回暖，下周北极寒流来袭，气温将大幅下降。</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/c152v24kg5wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>[视频]美称可能恢复“自由计划”行动 伊称将回击任何侵略</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>美称可能恢复霍尔木兹海峡“自由计划”行动，伊朗回击美方武力并警告将全力反击侵略。</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEt7bddqLRhHRlYowxTLBi260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>全球粮价连续三个月上涨；德国对美出口大幅下滑；英国工党在地方选举中失利。</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEzLwlNV6k5tSW0DO2RP68260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Iran accuses US of 'reckless military adventure'</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>伊朗指责美国在出现外交解决途径时仍发动攻击，称其“鲁莽军事冒险”。</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c99lpn9ze8ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>An expert on Iranian politics reviews the status of negotiations to end the war on Iran</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>伊朗政治专家分析特朗普政府就结束对伊战争谈判的进展。</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/09/nx-s1-5814972/an-expert-on-iranian-politics-review-the-status-of-negotiations-to-end-the-war-on-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Trump says Russia and Ukraine have agreed to his request for a 3-day ceasefire</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>特朗普称俄乌同意三天停火及换俘，双方官员确认协议。</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/09/nx-s1-5816478/trump-russia-ukraine-ceasefire</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>[视频]国务院成立湖南长沙浏阳市华盛烟花制造燃放有限公司“5·4”特别重大爆炸事故调查组</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>湖南浏阳烟花厂发生特别重大爆炸事故，国务院成立调查组，已致37人死亡。</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/09/VIDEWwim9yhwmXZPcPAaX3GJ260509.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Anger and resignation in Tenerife as hantavirus ship approaches</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>西班牙特内里费岛民众对即将抵达的疑似携带汉坦病毒的船只感到愤怒与无奈。</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y0gkg038yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Man critically injured after car hits pedestrians in Nottinghamshire town</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>英国诺丁汉郡一男子驾车撞伤5名行人，疑似事发前发生争执。</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgrpgp91rwwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Revisiting Guy Goma's iconic accidental BBC interview 20 years ago this week</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>回顾20年前盖伊·戈马误入BBC直播采访的经典意外瞬间。</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/09/nx-s1-5814110/revisiting-guy-gomas-iconic-accidental-bbc-interview-20-years-ago-this-week</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-10
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F242"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8181,6 +8181,1126 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260510 19:00</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>我国推进新型基建、经济向好，多领域发展，国际关注美伊及俄二战立场。</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEj6sgBGGhWkZPKBi6knhW260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】以学促干 将学习教育成效落到实处</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>贵州贵阳与山西长治以学促干，解决民生问题，提升政务效率。</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEzKwxc6mgu6NPrMJEtzBO260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Australia's right-wing One Nation party scores historic parliamentary win</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>澳大利亚右翼单一民族党在补选中首次赢得众议院席位。</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2e4z4npro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Labour MP challenges ministers to move against Starmer</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>工党议员威胁挑战首相斯塔默，部长力挺其继续领导。</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c362573l4gdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Tories are still biggest party on the right, claims Cleverly</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>保守党自称仍是右翼最大党，称改革党为“个人崇拜”。</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c7v9778r9q9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Can Starmer survive as PM? Seven scenarios for what might happen next</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>斯塔默面临党内逼宫，誓言坚守首相职位，分析多种可能走向。</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr7pz99l370o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Plaid Cymru's Rhun ap Iorwerth willing to 'take the fight' to Keir Starmer</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>威尔士党领袖称愿“向斯塔默开火”，必要时批评英国政府。</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62rnglzv2eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Sarwar says he will 'absolutely' stay on as Labour leader</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>苏格兰工党领袖虽选举失利，仍表态“绝对”留任。</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypgg10p83o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Keir Starmer's party lost big in U.K. local elections. Here's what comes next.</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>英国工党在地方选举中惨败，斯塔默拒绝辞职。</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/10/nx-s1-5817491/uk-elections-keir-starmer-resign-reform-green</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>[视频]多项先行指标显示我国经济稳步向好态势</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>多项先行指标显示4月我国经济稳步向好，投资结构优化，消费增长。</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDE75KHi92fFX03EkmYZaeB260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>[视频]2025年度秋粮收购顺利收官</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>2025年度秋粮收购超3.38亿吨，智能技术保障粮食安全。</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEszdiR9oMgKaeJmuPiIx0260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】我国加快推进新型基础设施建设</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>我国加快推进新型基础设施建设，算力网络四通八达，为高质量发展筑牢底座。</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEAWT1N6XdQR3dgt0mpr0h260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>[视频]“全球深渊探索计划”完成太平洋穿越科考航次</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>中国牵头“全球深渊探索计划”完成太平洋科考，发现8000米深海底生命绿洲及新物种。</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEaxSqbSyA7Z59fWgjHCO0260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>[视频]全面扩围 我国加快建设一刻钟便民生活圈</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>我国一刻钟便民生活圈全面扩围，服务1.68亿居民，养老托育设施优化。</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEGmNOwfeYlffOePSncHQA260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>[视频]各地全面推进国家免疫规划HPV疫苗接种服务</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>国家免疫规划HPV疫苗免费接种有序推进，已接种275万剂次。</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEAojRaejfM6KvzEWm2nwl260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>我国开展人力资源市场整顿、职教活动周启动，并启动人工智能伦理审查计划与人形机器人运动会。</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEho6ROz6sK27k6dR4VCJS260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Lidl says customers can turn points into pastries. But shoppers want the old app back</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Lidl推出积分换糕点活动，但顾客怀念旧版应用程序。</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ceqprgz18wro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>[视频]美军称继续对伊朗海上封锁 伊朗称侵犯伊朗船只将引发猛烈打击</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>美军对伊朗海上封锁，伊朗警告将猛烈打击侵犯船只；英法派舰艇赴中东护航。</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDELfRg3IYy50MuoyO8pgJe260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>[视频]俄总统表示坚决制止篡改二战历史图谋</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>普京称坚决制止篡改二战历史、美化纳粹的图谋，强调纽伦堡审判定罪不变。</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDE4PxBScJj1YuyT2aFQpJz260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>俄乌互指破坏停火；以军在黎南部行动；美媒称以色列在伊拉克设秘密哨所。</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEgO7addCRht9TessiaJ0m260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Countries airlift nationals evacuated from from virus-hit cruise ship</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>多国从暴发疫情的MV Hondius游轮上撤离本国公民，已有3人死亡。</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn7pzmg8zeno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Army parachutes onto remote island to help Briton with suspected hantavirus</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>军方跳伞至偏远岛屿，帮助一名疑似感染汉坦病毒的英国人。</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzv77ldpdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Iran sends response to US proposals to end war</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>伊朗已回应美国提出的结束战争建议，但未透露具体细节。</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypgz9e5pmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Putin says he thinks Ukraine conflict 'coming to an end'</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>普京称乌克兰冲突“接近尾声”，谴责西方支持泽连斯基。</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn8p4j2jzwwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Israel deports two activists detained on board Gaza flotilla</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>以色列驱逐两名乘坐加沙援助船队被扣押的活动人士。</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzdpxv2d7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Cape Verde: Tiny nation, massive World Cup dream</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>西非岛国佛得角的世界杯晋级之路，正改变球场内外的梦想。</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/10/nx-s1-5796264/cape-verde-tiny-nation-massive-world-cup-dream</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Iran ceasefire tested as cargo ship catches fire after being hit off Qatar's coast</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>一艘货船在卡塔尔海岸附近被不明弹丸击中起火，伊朗停火协议受考验。</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/10/nx-s1-5817437/iran-cargo-ship-hit-off-qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>国际, 社会, 文体</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Protests and boycotts rock prestigious Venice Biennale</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>第61届威尼斯双年展在地缘政治冲突中开幕，遭抗议和抵制。</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/09/nx-s1-5817005/protests-and-boycotts-rock-prestigious-venice-biennale</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>[视频]依托美好生态 夏日文旅持续升温</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>各地依托生态优势打造文旅新场景，夏日文旅持续升温。</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEcFiF6pYyq7baHC86KNDD260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】珠算乾坤 指尖上的华夏智慧</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>珠算承载千年智慧，源于商周，盛于元明，被列入非遗美育大会展示。</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/10/VIDEerck3L4ENRIxVynNJLPQ260510.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Bread dresses and gowns inspired by cathedrals at Nigeria fashion spectacle</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>尼日利亚时尚盛宴展示面包礼服和教堂灵感礼服。</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g0d3d5zn4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Suspected boat explosion injures 11 in Miami</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>迈阿密一码头疑似船只爆炸致11人受伤，官方正调查。</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c7076k4e31do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Buddhist monk arrested over alleged rape of teen in Sri Lanka</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>斯里兰卡一名资深佛教僧侣因涉嫌强奸少女被捕。</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy42kp0x92jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Our relationship with food is messed up - let's sort it out, says Stanley Tucci</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>演员斯坦利·图齐新季节目探索意大利饮食文化深层内涵。</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c98r1k1j844o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>体育, 民生</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>How could extreme weather affect World Cup 2026?</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>气象专家分析极端天气可能如何影响2026年世界杯。</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/ce9p8m9xz13o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-11
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F277"/>
+  <dimension ref="A1:F306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9301,6 +9301,934 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260511 19:00</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>美总统将访华；长三角一体化新突破；天舟十号成功发射；CPI温和回升。</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDET5JCLv3K8ofp0eyRlgW1260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 美国总统将对中国进行国事访问</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>应习近平邀请，美国总统特朗普将于5月13日至15日访华。</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEB3BXuyVHiFMDnyxD1ylC260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见出席第三届海峡两岸中华文化峰会两岸文化界人士代表</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>王沪宁会见两岸文化界人士，强调中华文化是两岸同胞的根与魂，反对台独。</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDERfDVcT5grjqog8eJbUSw260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>政治, 科技, 文体</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>发布多项政策：促进AI与能源融合、严惩非法占地、核电项目开工、世乒赛夺冠。</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEU5sE6YPUtEIK3qie7Jnd260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Analysis: Has Starmer done enough to save his premiership?</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>分析：英国首相斯塔默能否稳住民调？演说是否足以避免领导危机？</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3r2pr95yq0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Watch: Macron interrupts speaker to tell audience to be quiet</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>法国总统马克龙在肯尼亚演讲时打断发言，要求台下观众安静。</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/czx2wd20evyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】长三角一体化发展不断取得新突破</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>长三角一体化取得新突破，低空飞行、工业机器人、算力网提速，引领示范作用增强。</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEqWWGD5hHdaNUjYU7G0EK260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>[视频]4月居民消费价格指数温和回升 工业生产者出厂价格指数涨幅扩大</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>4月CPI同比上涨1.2%，PPI同比上涨2.8%，工业生产者价格涨幅扩大。</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDELkwxJlYum9JiQfyfalBP260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国中小企业经济运行势头良好</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>一季度中小企业利润增16%，专精特新企业表现亮眼，出口指数连续24个月扩张。</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEZTMwhVqytwC9FxfgVfKj260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>[视频]4月新能源汽车产销量及出口量均实现稳定增长</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>4月我国新能源汽车产销量及出口量均稳定增长，销量占比达53.2%。</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDErbQUTHVzAZHiuAzreo6l260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>[视频]海洋经济良好开局 向海图强释放新动能</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>一季度海洋经济开局良好，新兴产业加快成长，立体赋能成新亮点。</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEPU18sjnPEcJGZ1mDB8iw260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>经济, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Elon Musk and Tim Cook among CEOs expected to accompany Trump on China trip</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>马斯克和库克等17位美企CEO预计随特朗普访华，将会晤中方领导人。</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yx757w048o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>[视频]韩正出席2026世界数字教育大会开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>韩正出席世界数字教育大会，强调数字教育需以人为本、普惠公平、智能向善。</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEQ9yCniN8QBTPSzUyF4Ui260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>[视频]天舟十号货运飞船发射任务取得圆满成功</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>天舟十号货运飞船发射成功，与空间站完成交会对接，上行物资约6.2吨。</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEjsICkvsZaUF7LPVg0ORO260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】田野里的智慧农机</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>全国夏收在即，超1700万台智慧农机将投入使用，提升作业效率。</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDExnAEs9Djbgzk1gOnXxLE260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Remains of a U.S. soldier who went missing in Morocco have been recovered</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>在摩洛哥军演中失踪的美军士兵遗体在大西洋被发现，另一人仍在搜寻。</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/11/g-s1-121363/remains-of-missing-us-soldier</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】小麦进入灌浆期 各地科学防控干热风</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>小麦进入灌浆期，各地多措并举科学防控干热风，护航夏粮丰收。</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDECztTumT31cIZNQ98m8vz260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>US passengers being monitored for hantavirus as officials say public risk 'very low'</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>美国亚特兰大两人正接受汉坦病毒监测，另有16人在国家隔离中心，官方称公众风险极低。</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2e9e1g0wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>British passengers from hantavirus-hit cruise ship isolating in hospital</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>来自汉坦病毒疫区邮轮的英国乘客已隔离入院，无人出现症状，将观察72小时。</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g83vddnz0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>[视频]伊媒称伊朗最新回应要求美国尽快解除海上封锁 美称伊方回应不可接受</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>伊朗要求美国尽快解除海上封锁，美方称其回应不可接受。</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEbns7yTv4NSSoJYLL47MB260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>俄日关系陷入冰河期；以军袭击黎南部；全球石油供应减少约10亿桶。</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/11/VIDEoyJC9zZvotfiXG9ygdAL260511.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>US and French nationals test positive for hantavirus after leaving ship</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>一名美国人和一名法国人离船后检测出汉坦病毒阳性。</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjep78l5835o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Trump says Iran ceasefire is on 'massive life support'</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>特朗普批评伊朗停火提议，称持续一个月的停火协议“难以置信地脆弱”。</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgznxn18zgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Trump rejects Iran's ceasefire proposal response. And, Congress to tackle ICE funding</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>特朗普拒绝伊朗的停火提议，称其完全不可接受；国会共和党推动移民执法资金。</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/11/g-s1-121375/up-first-newsletter-trump-iran-congress-ice-cbp-hantavirus</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Trump heads to China amid ongoing war with Iran</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>尽管与伊朗交战，特朗普仍将按计划访问中国。</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/11/nx-s1-5816150/trump-heads-to-china-amid-ongoing-war-with-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Nobel laureate Narges Mohammadi transferred to a Tehran hospital, her foundation says</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>诺贝尔和平奖得主纳尔吉斯·穆罕默迪在狱中晕倒后，被转至德黑兰医院。</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/11/g-s1-121365/nobel-laureate-mohammadi-transferred-to-a-tehran-hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>国际, 科技</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>AI on the agenda as Trump heads to China</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>人工智能将成为特朗普与中国领导人会晤的议题。</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/11/nx-s1-5812681/ai-on-the-agenda-as-trump-heads-to-china</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Portrait looted by Nazis found in home of Dutch SS leader's descendants</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>一幅被纳粹掠夺的肖像画在荷兰党卫军领袖后代家中被发现。</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgmpj0p9k08o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Pupils hopeless and crying after 'poorly worded' Higher Maths exam</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>超1.1万人请愿要求重审高级数学考试，学生称考题表述不清、无法应对。</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21j20l9wlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-12
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F306"/>
+  <dimension ref="A1:F336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10229,6 +10229,966 @@
         </is>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260512 21:00</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>习近平会见塔吉克斯坦总统等多国政要；未来产业布局提速；农村供水保障提升。</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEsAbPAUFSpzUyG3RYBi0C260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎塔吉克斯坦总统访华</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>习近平为塔吉克斯坦总统拉赫蒙访华举行欢迎仪式。</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDETvRL2OSxRI5llz8kQ9Mg260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>[视频]习近平同塔吉克斯坦总统会谈</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>习近平与塔吉克斯坦总统会谈，强调深化战略对接与共建一带一路。</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEiANynxKjFw4tb8iQOVBA260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见文莱王储</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>习近平会见文莱王储，建议加强战略、发展、文明与全球治理合作。</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDE3nQODqXJp3yyziynbLlu260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见联合国教科文组织总干事</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>习近平会见联合国教科文组织总干事，愿深化人工智能、数字教育等合作。</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEboAm50lR1GNEdLBiNyAF260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>[视频]李强会见塔吉克斯坦总统</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>李强会见塔吉克斯坦总统，强调深化贸易投资与基础设施合作。</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEEegdJNQKZahzcvB3ZNEa260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>[视频]李强致电祝贺毛焦尔就任匈牙利总理</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>李强致电祝贺毛焦尔就任匈牙利总理，愿推动中匈关系发展。</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEBnXl6rNWjqdksB0s4u6U260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见塔吉克斯坦总统</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>赵乐际会见塔吉克斯坦总统，强调深化战略互信与立法机构交流。</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEATOIXZbhk7SsbMg6I9zS260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>[视频]韩正同文莱王储举行会谈</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>国家副主席韩正同文莱王储比拉会谈，庆祝建交35周年，推动命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDE1JpspfOCGMx1yrrgwCYn260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>[视频]国际社会高度关注中美元首会晤 期待两国合作为世界注入更多稳定性</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>国际社会高度关注中美元首会晤，期待两国合作为世界注入更多稳定性。</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDESQEIGjjeTrtIYvZVVIwV260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Zelensky's ex-chief of staff in court as Ukraine corruption probe escalates</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>乌克兰前总统办公室主任因洗钱案被列为嫌疑人。</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g48kj40lwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>The potential challengers to Keir Starmer</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>英工党多人被提名为首相潜在挑战者，包括伯纳姆等。</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3e2n7xn14xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Read all the ministers' resignation letters in full</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>多名英国部长因反对斯塔默领导而辞职，含菲利普斯。</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cglpz89265jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>All the Labour MPs who have come out against Starmer, and the ones who want him to stay</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>工党议员公开反对首相斯塔默的人数持续增加。</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgepqxj30pqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Watch: Reporters shout questions at ministers leaving No 10</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>部长们离开内阁会议时遭记者追问首相前途。</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/cn8p175l7v2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>'Crisis in Great Britain!' How global media is reporting Starmer's fight for survival</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默因选举惨败面临生存危机，引发全球媒体关注。</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crkp67pdy81o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Israel's government is expected to collapse over ultra-Orthodox military draft</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>以色列极右翼正统犹太政党要求解散议会，内塔尼亚胡政府面临垮台风险。</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/12/g-s1-121631/israel-military-ultra-orthodox-netanyahu-coalition</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Trump heads to China for state visit. And, how the war in Iran has affected inflation</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>特朗普访华会晤习近平，同时伊朗战争对美国通胀的影响备受关注。</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/12/g-s1-121602/up-first-newsletter-trump-china-xi-jinping-inflation-mifepristone-cameron-hamilton</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>[视频]今年以来我国未来产业布局提速</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>我国加速布局未来产业，太空算力、人形机器人等前沿技术取得突破，新赛道培育提速。</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEqwL0c62uEDbdRk5Z991x260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>US inflation jumps to 3.8% as energy costs surge from Iran war</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>受伊朗战争影响，美国通胀率升至3.8%，创2023年5月以来新高。</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c202pgxx89lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>伊朗呼吁美国接受其方案；以军袭击黎南部致多人死亡；德乌将联合研发无人机。</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEiTEZEb91n7r17YCtSUE4260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Kuwait says Iran attacked an island where China is helping to build a port</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>科威特指控伊朗袭击中国援建港口岛屿，美方透露以色列曾向阿联酋部署“铁穹”。</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/12/nx-s1-5819174/israel-sent-iron-dome-uae</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Israel to hold military tribunal for Palestinians accused in 2023 Hamas-led attacks</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>以色列计划设立军事法庭，审判数百名涉嫌参与2023年10月7日袭击的巴勒斯坦人。</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/12/nx-s1-5818455/israel-to-hold-military-tribunal-for-palestinians-accused-in-2023-hamas-led-attacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>[视频]我国农村供水保障水平显著提升</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>我国农村供水保障水平显著提升，自来水普及率已达96%，提前完成规划目标。</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEUYDaAG1jwvfgqRgGDTMT260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>No sign of larger hantavirus outbreak, says UN health agency</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>世卫组织称尚无迹象表明汉坦病毒更大规模爆发，但情况可能变化。</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cqjpqynj1nlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Trump says Iran ceasefire is on 'massive life support'</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>特朗普称伊朗停火协议“极度脆弱”，批评伊方反提议。</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgznxn18zgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Lebanon says two paramedics among 10 killed in Israeli strikes</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>黎巴嫩称以色列空袭致10人死亡，包括两名医护人员。</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21j3xl72zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>As Trump goes to China, what do Americans say about tariffs, Iran and world standing?</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>民调显示多数美国人视中国为经济威胁，而非主要军事对手。</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/12/nx-s1-5817601/trump-xi-china-tariffs-poll</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>[视频]各地各部门开展防灾减灾科普教育活动</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>第18个全国防灾减灾日，各地开展科普教育活动，提升群众防灾避险能力。</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEQ5AqGcNJw9KYYPjcuYlF260512.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>社会, 科技, 经济</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>护士总数达606万；世界数字教育大会发布成果；规范短视频内容标注；前4月食品贸易增长6.5%。</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/12/VIDEeHLQpZ5aCZi4nBDBJOm6260512.shtml</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-13
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F336"/>
+  <dimension ref="A1:F367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11189,6 +11189,998 @@
         </is>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260513 19:00</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>推进国际科技创新中心建设；中美举行经贸磋商；一季度新设经营主体509.8万户；外资加速布局中国服务业。</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEI0JMTE8TfxTTrAHyYt6z260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】奋力谱写中国式现代化建设四川新篇章 接续奋斗 开创云南发展新局面</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>四川和云南发布“十五五”规划，聚焦新质生产力、绿色发展和区域经济增长极建设。</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEO8VvjLT08uCnNcwMahfs260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>[视频]中美在韩国举行经贸磋商</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>中美在韩国举行经贸磋商，就解决彼此关切的经贸问题进行了坦诚、建设性交流。</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEVzBms5SdGZgqaexE1dMY260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Chris Mason: Starmer hopes to save his job with promise of change - and warnings of chaos</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>斯塔默承诺变革并警告混乱，试图保住首相职位。</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c392djn3zzdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Watch: What next after the King's Speech?</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>BBC首席政治记者解读国王演讲后政府下一步计划。</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/crepv72x5xqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Farage faces standards probe into £5m gift from crypto billionaire</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>改革英国党领袖法拉奇因接受加密富豪55万英镑捐赠面临调查。</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0l26g01703o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Gunfire breaks out in Philippine Senate as police try to arrest senator</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>菲律宾警方在参议院逮捕一名国际刑警通缉参议员时发生枪战。</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/13/g-s1-121827/gunfire-breaks-out-in-philippine-senate-as-police-try-to-arrest-senator</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Trump expected to talk Iran and trade during summit in China</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>特朗普访华将与中方讨论伊朗战争、贸易政策和台湾问题。</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/13/nx-s1-5819712/trump-expected-to-talk-iran-and-trade-during-summit-in-china</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>[视频]一季度全国新设经营主体509.8万户</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>一季度全国新设经营主体509.8万户，高技术制造业和服务业增长显著。</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEJ1iXI33cGTavBASyJweW260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>[视频]外资加速布局中国服务业</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>外资加速布局中国服务业，一季度新设外企同比增长11%，高技术服务业实际使用外资翻番。</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEdzPJ494hFbPm839RJGYS260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国水电清洁能源基地建设全面提速</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>我国水电清洁能源基地建设全面提速，金沙江、雅砻江等流域多个重大项目推进。</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEkGE68lmFHB1HJeqCfRgX260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>[视频]前4个月全国铁路完成固定资产投资2008亿元</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>前4个月全国铁路完成固定资产投资2008亿元，同比增长3.2%，多项重点工程取得进展。</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDE3LiiocahJzsD5CLgzKwp260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>[视频]2025年我国新发现大中型矿产地200处</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>2025年我国非油气地质勘查投入252.50亿元，同比增长10%，新发现大中型矿产地200处。</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEmdu9X4DrEI1bBlwe8lge260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>[视频]多元化文旅场景赋能入境游提质扩容</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>多元文旅场景和便利化政策吸引海外游客，带动入境游提质扩容，消费服务国际化。</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEKW2peWVFDlJHyTN9rzqV260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>药品注册审结创新高；林草种苗质量提升；义新欧班列出口增长；四川发现千亿方页岩气田。</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEzgGpLGmIhUaQGsylXcDz260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Chinese economist talks about the competing interest of China and the U.S.</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>中国经济学家分析中美经济利益竞争格局。</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/13/nx-s1-5818679/chinese-economist-talks-about-the-competing-interest-of-china-and-the-u-s</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】推进国际科技创新中心建设 打造世界级科技创新策源地</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>习近平总书记强调科技创新是关键变量，我国高水平推进三大国际科技创新中心建设。</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEoNtKHK1zANjurrlRmmga260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>军事, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>War in Iran costs $29 billion so far. And, students are finally improving in math</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>美国防部称伊朗战争已耗资290亿美元；学生数学成绩提升。</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/13/g-s1-121812/up-first-newsletter-war-iran-marty-makary-student-education-scorecard-trump-pardons</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>[视频]全国春灌已全面展开</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>全国春灌全面展开，水源充足，智慧灌溉系统助力精细化灌溉，推进灌区改造。</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEcfRgnRfx6pSGi81rTEoU260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>[视频]国际社会期待中美元首会晤引领中美关系平稳前行 惠及世界</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>国际人士期待中美元首会晤引领关系平稳前行，促进世界和平与繁荣。</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEhjd3svST0t1KIQ1gRj9v260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>[视频]日本民众集会抗议高市政权“扩军”修宪等危险动向</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>日本民众集会抗议高市政权修宪扩武等危险动向。</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEU90PVVlZevpzK35oCBrp260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>黎以冲突升级；英工党内部要求首相辞职；日本国债收益率升至近30年新高。</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEMOWXFzguMIE6fOXvQq0Z260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Trade, Iran and Taiwan on the agenda as Trump arrives in China for high-stakes talks with Xi</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>特朗普访华与习近平会晤，议程涉及贸易、伊朗和台湾问题。</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1w28qw1e0xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Woman isolating on British island in South Pacific after hantavirus contact</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>接触汉坦病毒后，一名女性在英属皮特凯恩群岛隔离，无患病迹象。</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21p7k70reo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>What to know as Trump visits Xi in China</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>特朗普抵达北京访华，系2017年后首次有美国领导人访问。</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cyv2n7l1z14o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>国新办举行“新征程上的奋斗者”记者见面会，5位教师代表分享育人实践。</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/13/VIDEscxYGR8zbxd5OvlrcCQ2260513.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Court overturns Alex Murdaugh's murder convictions and orders new trial</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>法院推翻亚历克斯·默多夫谋杀罪判决，下令重新审判。</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cedpvnq7wn1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Dozens of dogs rescued and suspect arrested in Uganda after BBC investigation</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>BBC调查曝光诈骗后，乌干达警方救出数十只狗并逮捕嫌疑人。</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1j2n008k5lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Met Police prepares armoured vehicles and 4,000 officers for dual London protests</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>伦敦将同时举行两场抗议活动，警方部署装甲车和4000警力。</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c172n5e0prko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Bodies of three young women pulled from sea off Brighton</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>布莱顿海域发现三名年轻女性遗体，海滩已重新开放。</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0e29n94ze4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Greetings from Seville, where springtime means caracoles</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>塞维利亚春季食蜗季来临，小蜗牛是当地特色小吃。</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/13/g-s1-121409/seville-spain-snails-caracoles</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-14
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F367"/>
+  <dimension ref="A1:F396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12181,6 +12181,934 @@
         </is>
       </c>
     </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260514 21:00</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>习近平举行仪式欢迎特朗普访华并会谈，中美元首达成建设性战略稳定关系新定位。央行数据等多个经济利好发布。</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEr0Mtz3C4E5WIYDH68D9f260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎美国总统访华</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂举行仪式欢迎特朗普国事访问，鸣礼炮21响并检阅仪仗队。</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDESVsLjIP48le8m8a4TqmM260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>[视频]习近平同美国总统会谈</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>习近平与特朗普会谈，提出构建“中美建设性战略稳定关系”新定位，强调合作共赢。</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEr7cLOoSjQpqQH46fcmNV260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>政治, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>[视频]习近平同美国总统参观天坛</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>习近平同特朗普参观天坛，介绍中华文化理念，强调民为邦本与人民友好。</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEaLUR5SClib8MiJiUpUOa260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>[视频]习近平为美国总统举行欢迎宴会</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>习近平为特朗普举行欢迎宴会，指出中美合则两利，应成为伙伴而非对手。</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEBZ5bZW5kLR23X0xoywAG260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>[视频]李强会见美国工商界代表</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>李强会见随特朗普访华的美国工商界代表，鼓励美企深耕中国市场促合作。</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDE3mMxtWEcozuyuOmO97tn260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Key excerpts from Streeting's resignation letter as he quits as health secretary</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>英国卫生大臣斯特里廷辞职，此前被指准备挑战首相斯塔默领导地位。</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c626wvqy1yzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>At a glance: Starmer fights to stay on as prime minister</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默因选举惨败面临党内反叛，艰难维持首相职位。</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8jv1mzzkjgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>As Trump meets with Xi, security expert says China now faces the U.S. as a peer</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>前国安官员称，特朗普高额对华关税引发冲突，中国取胜，中美现为平等对手。</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/14/nx-s1-5821644/as-trump-meets-with-xi-security-expert-says-china-now-faces-the-u-s-as-a-peer</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>政治, 国际, 社会</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>A Philippine senator wanted by the International Criminal Court flees from Senate</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>菲律宾参议员被国际刑事法院通缉，从参议院逃走，警方怀疑是假逃亡。</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/14/g-s1-122021/philippines-senator-escape-wanted-icc</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Trump tries to make deals in China. And, Senate confirms Kevin Warsh as Fed leader</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>特朗普访华寻求与习近平达成协议，参议院确认凯文·沃什任美联储主席。</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/14/g-s1-122014/up-first-newsletter-china-taiwan-trump-law-firms-kevin-warsh-denise-powell-nebraska</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Cordial Trump-Xi meeting is a 'good sign,' says longtime U.S. diplomat</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>美外交官称特朗普与习近平会晤友好，是“好兆头”，但双方优先事项不同。</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/14/nx-s1-5822225/richard-haass-trump-xi-meeting-china-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>China's leader warns Trump that differences over Taiwan could lead to a clash</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>中国领导人在峰会上警告特朗普，台湾问题是中美冲突的关键点。</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/14/nx-s1-5822168/trump-xi-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>[视频]4月末我国社会融资规模存量同比增长7.8%</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>4月末我国社会融资规模存量457万亿元，同比增长7.8%，M2增长8.6%，信贷结构优化。</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEloiMjmROD9R7T4tLKILA260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>[视频]4月份我国电商物流运行稳中有升</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>4月电商物流指数110.6点稳中有升，总业务量同比增约20%，农村业务量增约25%。</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEkM4YQg39Zz37cEOQcFWx260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>[视频]一季度工程机械产品出口保持快速增长</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>一季度我国工程机械产品出口额160.66亿美元，同比增长24.3%，保持快速增长。</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDELsgP4t6NjXYh2uYekh5H260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Cuba considers $100m US aid offer as energy crisis worsens</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>古巴能源危机加剧，考虑接受美国1亿美元援助，但不确定形式。</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd7pyrj0vx7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>UK economy sees surprising growth - these six charts explain what is going on</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>英国经济出人意料增长，图表显示其韧性超预期，不受伊朗战争影响。</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyprjddgj3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Giant new dinosaur identified from fossils in Thailand</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>泰国发现新巨型恐龙“那伽泰坦”，为东南亚最大恐龙，重如九头象。</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21pk5g20ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>'Floating armoury' ship reportedly seized by Iran</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>伊朗军方在阿曼湾扣押一艘据称为“浮动军火库”的船只。</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx219xwxg9no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>军事, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Ukraine rescuers pull dead from rubble of Kyiv flats after massive Russian strikes</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>俄大规模袭击基辅致至少12死，含两名儿童，救援人员搜寻废墟。</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq5p8yygq94o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>[视频]夏粮旺季收购即将启动 预计收购小麦1亿吨左右</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>2026年夏粮旺季收购即将启动，预计收购小麦约1亿吨，国家继续实施最低收购价政策。</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEhR2DsaaGeCHne2lP7OOK260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>2025年城市再生水利用量突破220亿立方米；1-4月期货成交额增42.75%；医保飞检启动。</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEhhLCyY0DtFFRQYFhu0cK260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>[视频]国际社会高度关注中美元首会谈</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>国际社会高度关注中美元首会谈，多国人士称会谈发出积极正面信号。</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEOclaPTwhsPRbZAznwqGX260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>[视频]以军袭击黎南部多地 以称在所有战区创造“新的安全现实”</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>以军空袭黎南部多地，称创造“新安全现实”；黎方统计伤亡数字高企。</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEED2mJa76NOXQDAGwJmt5260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>欧佩克下调石油需求预期；欧盟一季度进口俄液化天然气创新高；日本破产企业数连续5月增加。</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEsBAxlO6ulCkbnP3TeEvt260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Flattery and fanfare as Trump welcomed to China - but thorny issues remain</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>特朗普访华获隆重欢迎，中美领导人会谈展现友好，但棘手问题仍存。</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdxpypg9dgeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>国新办举行快递从业者中外记者见面会，分享快递进村、科技赋能等基层实践。</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/14/VIDEMIZ7Ws85z2DibdAXUhzW260514.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Former imam sentenced to life for sexual assaults</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>前伊玛目阿卜杜勒·哈利姆·汗因九年性侵七名穆斯林受害者被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdrpk4end65o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-15
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F396"/>
+  <dimension ref="A1:F423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13109,6 +13109,870 @@
         </is>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260515 21:00</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>新闻联播报道中美元首会晤、国务院会议、贵州调研及国内经济民生等多条要闻。</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEAs0XdoNVdkpFCA93Htz8260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>[视频]习近平同美国总统在中南海小范围会晤</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>习近平与特朗普在中南海小范围会晤，确定建设性战略稳定关系，达成多项共识。</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEnhwt6ckJE6JKTjut85eu260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，审议通过城市更新和农业农村现代化“十五五”规划。</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDE8XZKPRcy5r9MLiEuCcTg260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际在贵州调研</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>赵乐际在贵州调研，强调人大要围绕“十五五”规划推进立法与监督工作。</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEN1XhSyA3hrOZYw9qwMeG260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>What does Makerfield think of by-election and can Burnham win?</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>工党议员辞职后，伯纳姆表示将参选梅克菲尔德选区补选。</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cyv26e7yd89o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>SCOTUS upholds abortion pill telehealth access. And, Trump returns from China visit</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>美最高法院维持堕胎药远程获取，特朗普结束访华并宣布多项贸易协议。</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/15/g-s1-122218/up-first-newsletter-mifepristone-trump-china-keir-starmer-new-york-salmon-river-students</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】江苏奋力在推进中国式现代化中走在前做示范 奋力谱写中国式现代化安徽篇章</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>江苏和安徽发布“十五五”规划，聚焦高质量发展、科技创新与产业升级。</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEafhgQHg4o0Z022IorlLc260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>[视频]一季度我国数字产业收入同比增长12.9%</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>一季度我国数字产业收入9.5万亿元，同比增12.9%，利润增长23.6%。</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEQf8iihx0kMmefF7RQKnM260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>军事, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Death toll in attack on Kyiv apartment building now stands at 24</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>俄导弹袭击基辅公寓楼致24死，含3名儿童。</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/15/nx-s1-5823388/death-toll-in-attack-on-kyiv-apartment-building-now-stands-at-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】西南麦区迎来大面积收获</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>西南麦区冬小麦大面积收获，各地推广小型农机和智能无人机提升效率。</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEyQeH1idCHZGBtz2VySiA260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>[视频]1至4月全国铁路发送旅客15.55亿人次</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>1至4月全国铁路发送旅客15.55亿人次，同比增长6.8%。</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEKoRVIBWumeAJxRHEtV8e260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>[视频]多国人士表示中美元首会谈为两国关系提供战略指引 为全球注入稳定性</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>多国人士表示中美元首会谈为两国关系提供战略指引，为全球注入稳定性。</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEkLJ8YMGQlq6xjpghQ9IX260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>[视频]国际媒体高度关注中美元首会谈</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>国际媒体高度关注中美元首会谈，认为中美加强合作具有重大全球性意义。</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDE8sa6x3LVJvDpRp1b8OJ9260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>以黎第三轮会谈分歧明显；也门达成人员释放协议；印度恶劣天气致超百人死亡；夏威夷火山喷发。</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEJH17B0PiF5ddS2aI5ovE260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Trump warns Taiwan against declaring independence, hours after summit with China's Xi</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>特朗普在与习近平会晤数小时后警告台湾不要宣布“独立”。</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8p61v7l68o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Trump and Xi conclude 'very successful' talks but no deals confirmed</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>特朗普和习近平结束“非常成功”的会谈，但未确认任何贸易突破。</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypj01189lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Prisoner swap goes ahead as Kyiv mourns 24 killed in Russian strike on flats</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>乌克兰进行战俘交换，基辅哀悼24名死于俄军袭击公寓楼的遇难者。</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y049w8nqwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>New York Times defends journalist after Israel threatens to sue</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>以色列总理因记者报道性侵指控威胁起诉《纽约时报》。</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9wedpk155jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Key takeaways from Trump's China trip</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>特朗普结束对中国的旋风访问，返回美国。</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/15/nx-s1-5822512/trump-china-xi-summit-takeaways</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>China economist shares takeaways from the Trump-Xi summit</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>中国经济学家金刻羽分享特朗普与习近平峰会成果。</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/15/nx-s1-5822445/china-economist-shares-takeaways-from-the-trump-xi-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>How the relationship between the U.S. and China has changed under Trump</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>中国学者达巍谈特朗普时期美中关系变化。</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/15/nx-s1-5819194/how-the-relationship-between-the-u-s-and-china-has-changed-under-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行中外记者见面会，5位残疾人代表讲述奋斗故事，展现自强精神。</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEcKuKqmE4e6e3Se53YteM260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>社会, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>发布2026年“最美家庭”；新修订《药品管理法实施条例》施行；力箭系列火箭完成百星发射；中央财政两年投入10亿元支持校园足球。</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/15/VIDEDxLJWbHOg2Mp8XDtGSkU260515.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>AI vigilante trap snares alleged paedophile ex-teacher in France</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>法国一位前教师被AI钓捕，冒充14岁女孩的网络侦探使其自首。</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1m2xg7x0m3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Teenager's family 'heartbroken' by meningitis death</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>一名六年级学生因脑膜炎去世，家人心碎致哀。</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy42jn311y1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Judge declares another mistrial in Harvey Weinstein New York rape charge</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>哈维·韦恩斯坦在纽约强奸案中第三次审判无效。</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c152lexw1vxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Five Italians die during cave scuba dive in Maldives</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>五名意大利人在马尔代夫洞穴潜水时遇难，其中四人是大学团队。</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62e0p7rd2ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-16
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F423"/>
+  <dimension ref="A1:F453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13973,6 +13973,966 @@
         </is>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>政治, 经济, 军事</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260516 19:00</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>《求是》发表习近平重要文章；俄总统将访华；神舟二十三号待发射；普惠型小微企业贷款余额增长9.9%。</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEzxXEzMNNjN4cmPaib5In260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>[视频]《求是》杂志发表习近平总书记重要文章《做强做优做大实体经济》</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>《求是》发表习近平重要文章，强调做强做优做大实体经济，推进新型工业化。</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEyEZn6kwsDRKfeFoXxfZR260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 俄罗斯总统将对华进行国事访问</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>应习近平邀请，俄罗斯总统普京将于5月19日至20日对华进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEaOWZBLK8jEGVMQK7iEvR260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>US planning to charge ex-Cuban leader Raúl Castro</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>美国计划起诉古巴前领导人劳尔·卡斯特罗，涉1996年击落飞机案。</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1w2gnd9xp2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Trump warns Taiwan against declaring independence, hours after summit with China's Xi</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>特朗普警告台湾勿宣布独立，称希望两岸降温紧张局势。</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8p61v7l68o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>The race to replace Starmer is on - but he still faces a momentous choice</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>工党内部竞争激烈，英首相仍面临重大抉择。</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx213m1d82lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>[视频]【凝心聚力 真抓实干 奋力实现“十五五”良好开局】青海立足资源禀赋 推进绿色算电协同发展 宁夏持续加力 筑牢西北地区重要生态安全屏障</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>青海推进绿色算电协同发展，宁夏筑牢生态安全屏障，助力“十五五”绿色发展。</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDENZsBoIFrPpjU2qakyNlg260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>[视频]一季度末普惠型小微企业贷款余额同比增长9.9%</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>一季度末普惠型小微企业贷款余额38.8万亿元，同比增长9.9%，政策支持小微企业。</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEvqXuE8dLYNPlsA4XMzQl260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】我国夏油作物收获进入高峰</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>我国夏油作物收获进入高峰，冬油菜长势良好，中央财政专项支持油菜生产。</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEt9oXZ5ZvsDKpx7OJ8CgY260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>[视频]我国工业资源循环利用提速升级</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>我国工业资源循环利用提速，退役列车回收率超98%，再生资源回收总额达1.39万亿元。</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEnnTIUs0cAiVxn9BqLQN1260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>[视频]以旧换新 持续激发消费活力</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>各地以旧换新政策扩围，多措并举激发消费活力，智能家居成新热点。</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDE9cPItSCzQ7Cjln6L4yZj260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>平陆运河主体工程完成；城市体检全面开展；第二艘国产大型邮轮试航。</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEqP75BXD501TK7uQz9VJR260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>经济, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>美经济学家预测二季度通胀飙升；刚果（金）埃博拉致死80人；泰国火车与巴士相撞致8死；欧洲成全球变暖最快大陆。</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEH9FfEk999dF6vAowh2xw260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号船箭组合体转运至发射区 计划近日择机发射</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>神舟二十三号船箭组合体转运至发射区，计划近日择机发射。</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEhgDuRyCoByeFtc0zqoyF260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>[视频]我国储能产业发展势头强劲</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>我国储能产业强劲发展，抽水蓄能及新型储能装机快速增长，技术不断突破。</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDE0pyDtiflnctcbMHCc7LD260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Senior IS leader killed in joint operation, US and Nigeria say</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>美尼联合行动击毙IS高级头目阿布-比拉尔·米努基。</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy72p2kpd03o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>The war in Ukraine is at a standstill as societal fatigue grows in Russia</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>乌克兰战事陷入僵局，俄罗斯社会战争疲劳加剧。</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5822468/the-war-in-ukraine-is-at-a-standstill-as-societal-fatigue-grows-in-russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>[视频]南水北调已累计向北方调水880亿立方米</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>南水北调已累计向北方调水880亿立方米，受益人口1.95亿，生态补水效果显著。</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDE27J2EcR7bRpeMDdgSttZ260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>[视频]我国将全面推行家庭病床服务</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>我国将全面推行家庭病床服务，行动不便患者可在家享受专业康复护理。</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDENROpPtV2eBIxne7jY2GR260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>[视频]黎以停火延长45天 以军持续袭击黎南部</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>黎以停火延长45天，以军仍持续袭击黎南部，致多人伤亡。</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDEbZdg6TnsMBKYxYCyUWkV260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称为外交谈判争取机会 以色列称正准备重启对伊朗军事行动</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>伊朗称争取外交机会，以色列准备重启军事行动，油价显著上涨。</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDE143ql7mzxHgYne419Te8260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Timmy the humpback whale found dead off Danish coast</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>曾获救援的座头鲸蒂米在丹麦海岸被发现死亡。</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/g-s1-122490/timmy-humpback-whale-dead-stranded-rescue-denmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>The townspeople of Vilseck, Germany, worry that Trump may pull out 5,000 U.S. troops</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>德国小镇居民担忧特朗普可能撤走5000名驻军。</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5815881/trump-germany-withdrawal-nato-us-troops-vilseck</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Trump says Islamic State group leader was killed in a joint U.S.-Nigerian mission</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>特朗普宣布美尼联合行动击毙ISIS二号头目。</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/g-s1-122461/islamic-state-leader-killed</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>[视频]大范围降雨持续 各地全力做好强降雨防范应对工作</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>大范围强降雨持续，多地抢险应对，国家防总启动防汛四级应急响应。</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/16/VIDExPbvk7znl5HKV2DdNIDA260516.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Rescue diver dies during search for bodies of Italians who drowned in Maldives caves</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>马尔代夫救援潜水员在搜寻意大利溺水者遗体时丧生。</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1w2gv1gdnjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Toddlers among more than 50 schoolchildren kidnapped in Nigeria</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>尼日利亚50多名学童被绑架，包括幼儿，尚无组织认领。</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c202vrxlwqgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Tens of thousands join rival marches in London</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>伦敦两场对立游行数万人参与，逮捕31人。</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3d2ryyz0jzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Tonight's the Eurovision final. Here's what you can expect</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>欧洲歌唱大赛决赛今晚在维也纳举行，亮点前瞻。</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1d2qe73ly7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>The Eurovision Song Contest reaches its grand final with pop and protests</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>欧洲歌唱大赛决赛举行，安保森严，以色列参赛引争议。</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5824325/eurovision-final-vienna</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-17
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F453"/>
+  <dimension ref="A1:F483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14933,6 +14933,966 @@
         </is>
       </c>
     </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260517 19:00</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>习近平指示推动哲学社会科学高质量发展，中俄博览会开幕，各地推进数字赋能与产业升级。</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDErA75q2Ns7YFd24uDeVUT260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>[视频]习近平就推动哲学社会科学高质量发展作出重要指示强调 加快构建中国哲学社会科学自主知识体系 更好回答中国之问世界之问人民之问时代之问</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>习近平强调加快构建中国哲学社会科学自主知识体系，回答中国之问、世界之问等。</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDE9hcoitZFwTf6IdobwRjh260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：更好回答中国之问世界之问人民之问时代之问</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>央视快评：更好回答中国之问、世界之问、人民之问、时代之问。</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEz2599sRZibHyzEwZaYHu260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统分别向第十届中俄博览会致贺信</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>习近平与普京向第十届中俄博览会致贺信，强调深化全方位务实合作。</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEVqu9fkgchEMLqOVTU8uf260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>[视频]社科界学习贯彻习近平文化思想座谈会在京举行</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>社科界在京座谈，学习贯彻习近平文化思想，加快构建中国哲学社会科学自主知识体系。</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEbmqNM1Z507LUvp5oILM7260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Personal decision for Starmer on whether to fight leadership contest, minister says</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>英文化大臣称是否参加党魁竞选是斯塔默的个人决定，不排除其可能性。</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypg60k25ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>The UK is churning through leaders. Is the country becoming harder to govern?</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>英国领导人更迭频繁，民众对政治阶层不满加剧，国家治理难度上升。</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cqjpe7q0j1xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>[视频]我国县域消费市场供应持续改善</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>我国县域商业体系持续完善，消费供给优化，县乡消费活力释放，占比持续提高。</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEDZe5YZPz9E9CEnQQaa4R260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>[视频]工业遗产焕新 活化利用释放新活力</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>多地工业遗产改造为文旅地标、创业园区，九成以上实现活化利用。</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEKoxRzcTHDzqbnXwLTCy8260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>[视频]【凝心聚力 真抓实干 奋力实现“十五五”良好开局】湖南：深化人工智能产业赋能和场景应用 河北：数字赋能 推动传统产业转型升级</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>湖南、河北深化人工智能赋能，推动传统产业数字化转型，打造智能经济新形态。</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDENU5Pchf0pkymkfC2HrO5260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>科技, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>国内联播快讯：算力调度、高原病规范、流动儿童服务、澳车北上等。</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDERoN23SAfD3EnG34kuWLr260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Large-scale Ukrainian drone attack kills three in Moscow region, says Russia</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>乌克兰大规模无人机袭击莫斯科地区致三人死亡，俄方称乌方回应其攻击。</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5ye480kxpmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>UAE reports drone strike near Abu Dhabi nuclear power plant</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>阿联酋报告阿布扎比核电站附近遭无人机袭击，正调查来源。</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy27pkj1l1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Ukraine conducts large-scale drone strikes on Russia, killing 4 and wounding 12 others</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>乌克兰大规模无人机袭击俄罗斯，致4死12伤，包括莫斯科附近3人。</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/17/nx-s1-5824987/ukrainian-drone-strikes-on-russia-kill-4-moscow</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>[视频]我国残疾人社会保障和关爱服务水平不断提升</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>全国助残日，我国残疾人社会保障和关爱服务水平不断提升，就业人数达891.5万。</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDE0ik4zEeKsoEhYiIH7ZcA260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>[视频]一批水利重点工程有序推进</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>淮河、山东、新疆等地一批国家重大水利工程有序推进，保障防洪、供水与发电。</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDELyejwfKURpK4Uia3WxMs260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>[视频]多地强降雨持续 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>中东部多地持续强降雨，各部门积极抢险救援，清理积水。</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDESqcbBFyrPIinaw2IIQLe260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称已制定管理霍尔木兹海峡指定航道的专业机制</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>伊朗称已制定管理霍尔木兹海峡航道机制，俄伊核电站建设恢复。</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEPtBpcQ15qfoqnLUsF84I260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>国际, 科技, 文体</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>中企承建哈萨克斯坦轻轨通车；非洲埃博拉疫情升级；朝鲜女足抵韩。</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDE8cEFgsz3PBurG6d0pgyf260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>WHO declares Ebola outbreak in DR Congo an international emergency</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>世卫组织宣布刚果（金）埃博拉疫情为国际紧急事件，但未达大流行标准。</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2l2p0wwzzdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>How worrying is the Ebola outbreak in DR Congo?</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>刚果（金）埃博拉疫情被宣布为卫生紧急事件，近250例疑似病例。</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9q311nj5r3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>The foreign fighters who helped topple Assad — and why China worries about them</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>数千维吾尔人成为推翻叙利亚阿萨德政权的主力，受访讲述逃离中国原因。</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/17/g-s1-113270/uyghurs-china-syria-war-fighters-rebels-bashar-al-assad</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Iranian man barely survives bombing, but wants war to go on</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>伊朗男子在美以轰炸中幸存，却仍希望战争继续以摧毁现政权。</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5820984/iranian-man-barely-survives-bombing-but-wants-war-to-go-on</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>[视频]【暖心一瞬】危急时刻施援手 见义勇为显担当</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>江苏、广州热心群众危急时刻挺身救人，彰显见义勇为精神。</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEOqTNWTWoNt5gc5yqeE9y260517.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Man drives car into pedestrians in Italy, injuring eight</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>意大利一男子驾车冲撞行人致八人受伤，路人将其制服。</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cyv28pd4n22o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Forty-three arrests after £4.5m police operation to keep rival London protests apart</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>伦敦警方耗资450万英镑维持对立抗议秩序，逮捕43人避免严重冲突。</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ckgpznn202po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Life on the edge: why Indonesians living near volcanoes won't leave</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>印尼爪哇岛数千居民不愿撤离默拉皮火山，尽管面临持续风险。</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5818295/life-on-the-edge-why-indonesians-living-near-volcanoes-wont-leave</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>'Look Mum, one point': How the UK keeps getting Eurovision wrong</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>BBC需反思2027年欧洲电视网参赛策略，此前连续四年表现不佳。</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy72e81dp28o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Bulgarian banger 'Bangaranga' bags country its 1st Eurovision win</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>保加利亚歌曲《Bangaranga》赢得第70届欧洲电视网大赛冠军，爆冷击败24国。</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/16/nx-s1-5824393/eurovision-winner-dara-bangaranga-bulgaria-vienna-austria</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>文化</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】青铜铸文明 礼乐传古今</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>通过青铜文物展现中华礼乐文明，实证中华文明延绵不绝与多元一体。</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/17/VIDEtQvrMbWtojiKlCODaTvZ260517.shtml</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-18
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F483"/>
+  <dimension ref="A1:F513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15893,6 +15893,966 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260518 21:00</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>新闻联播报道生态文明建设、领导人活动、国内经济、国际局势等多条要闻。</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEHsvE6OHU4yZhJUDSa8fY260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】奋力谱写新时代生态文明建设新篇章</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>习近平强调以更高站位推进生态文明建设，我国降碳减污成效显著。</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEeMupriTJy5mWsYc5uYJX260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际同格鲁吉亚议长会谈</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>赵乐际同格鲁吉亚议长会谈，推动战略伙伴关系深化。</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEELmYpSgvUtM40oQPfnDz260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见格鲁吉亚议长</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>王沪宁会见格鲁吉亚议长，强调深化互尊互信合作。</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEmng0Tbtfci3gKlbxXtuy260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>[视频]中共中央办公厅印发《中国共产党发展党员工作细则》</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>中共中央办公厅印发《中国共产党发展党员工作细则》。</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEv1CRSiqmQAJasuF0tYjn260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Burnham pledges not to 're-run' Brexit arguments</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>伯纳姆承诺不再重提脱欧争论，不提议英国重返欧盟。</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21en4807wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>政治, 国际, 社会</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Sen. Bill Cassidy loses primary. And, WHO declares Ebola outbreak a global emergency</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>投票定罪特朗普的参议员初选失利；世卫宣布埃博拉疫情为全球紧急事件。</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/18/g-s1-122577/up-first-newsletter-bill-cassidy-trump-ebola-elon-musk-openai-sam-altman-idaho-airshow-collision</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>North Korea is relieved its nuclear weapons have prevented a fate like Iran's</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>目睹伊朗领导人被杀后，金正恩认为拥核决定正确。</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/18/nx-s1-5820631/trump-north-korea-nuclear</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>[视频]李强在北京调研</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>李强在北京调研，强调推动AI与先进制造业融合，加快智能机器人发展。</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEoRuINXFJcZ2PuOwfHK5i260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>[视频]韩正出席2026年全球贸易投资促进峰会开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>韩正出席全球贸易投资促进峰会，提出四点合作建议。</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEs8J7JBmSH4xEmMwqbQyH260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>[视频]前4个月国民经济保持稳中有进发展态势</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>前4个月国民经济稳中有进，工业增长5.6%，消费扩大，就业稳定。</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEx3gaxC4AkvMPGw6z9ZPr260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>[视频]加力优化离境退税 打造国际化消费环境</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>六部门优化离境退税政策，扩大入境消费，推动即买即退异地互认。</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEZh9nGxu46Baxy8juh6Qc260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>经济, 社会, 科技</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>一线城市房价环比上涨，稳岗扩容方案发布，千帆星座第九批卫星成功发射。</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEJKKydHa4XuOvCb7j45Cz260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Prince William selling 20% of duchy property for housing and nature projects</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>康沃尔公爵领地出售部分地产，筹资用于住房和自然项目。</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8pg8ryjkzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥在调研算力网建设时强调 加快构建全国一体化算力网 赋能经济社会高质量发展</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>丁薛祥调研算力网建设，强调加快构建全国一体化算力网。</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEwX4uPghLxboMMYxTmrhW260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Jury tosses Elon Musk's lawsuit against OpenAI and its boss Sam Altman</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>陪审团驳回马斯克诉OpenAI及奥尔特曼的“窃取慈善”案。</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cewpyv79pw1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Ukraine launches large-scale drone strikes on Russia</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>和平谈判停滞，乌克兰发动大规模无人机袭击俄罗斯。</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/18/nx-s1-5824988/ukraine-launches-large-scale-drone-strikes-on-russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>U.S. and Israel prepare for potential return to full-scale war with Iran</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>美以准备与伊朗可能重返全面战争，局势风险升高。</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/18/nx-s1-5825574/u-s-and-iran-signal-readiness-to-fight-again-as-weekend-tensions-mount</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>[视频]强降雨持续 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>多地强降雨持续，国家防总启动应急响应，支援湖北贵州等地防汛救灾。</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEsCQXcMCOPaCpYIANN56U260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Four killed in protests during Kenyan strikes over high fuel prices</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>肯尼亚罢工抗议油价高涨，致四人死亡，交通瘫痪。</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2p0n44drvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>[视频]伊朗总统称美以试图通过煽动使地区关系分裂</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>伊朗总统指责美以煽动区域分裂，美伊核谈判僵持，美以讨论重启军事行动。</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEy3n2E1a7JsvKq3Tke1rY260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>以色列计划在原联合国机构建国防设施，美国空军基地两机相撞无人伤亡。</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDE3MdHUzAfuMFF5KgKBUgT260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>At least 100 deaths reported in Ebola outbreak in DR Congo as six Americans exposed</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>刚果（金）埃博拉疫情致至少100人死亡，6名美国人接触后1人出现症状。</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq6pz60p996o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>What is Ebola and why is stopping this outbreak so difficult?</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>刚果（金）埃博拉疫情涉及罕见毒株，冲突地区防控困难。</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz72p75zg4qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Death toll from Israeli strikes on Lebanon passes 3,000, officials say</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>以色列对黎巴嫩袭击致超3000人死亡，冲突升级。</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cqjpglyjwjeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Bodies of missing Italian divers found in Maldives</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>马尔代夫失踪的五名意大利潜水员遗体全部找到。</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c332mngz25vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>[视频]各地举办丰富多彩的国际博物馆日活动</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>国际博物馆日各地举办活动，全国博物馆超15.6亿人次接待，免费开放率逾91%。</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/18/VIDEKtOpsAF1CwIOM9M4WdAD260518.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Two men arrested over stunt at enclosure of famous monkey Punch</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>两名美国人因翻入围栏闯入网红猴子展区被捕。</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr5pz4jvlp5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Married at First Sight UK brides tell BBC they were raped by on-screen husbands</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>英国真人秀女嘉宾指控被节目中的丈夫强奸，主办方提前知情。</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8pz1k4r2lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Pop star Shakira is acquitted in a Spanish tax fraud case</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>哥伦比亚巨星夏奇拉在西班牙逃税案中被判无罪。</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/18/g-s1-122563/pop-star-shakira-is-acquitted-in-a-spanish-tax-fraud-case</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-19
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F513"/>
+  <dimension ref="A1:F543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16853,6 +16853,966 @@
         </is>
       </c>
     </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260519 19:00</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>新闻联播报道长江经济带、国务院条例、政协协商会、中俄会晤、网络文明大会等多项要闻。</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEYIhNt8SvBF46DbIOcL9F260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】共绘长江经济带高质量发展新画卷</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>长江经济带坚持生态优先，十年修复成效显著，森林覆盖率超46%，水质保持II类。</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDErYtsPvTxTADh8shVbeLk260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>[视频]李强签署国务院令 公布修订后的《行政法规制定程序条例》</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>李强签署国务院令，公布修订后的《行政法规制定程序条例》，自2026年7月1日起施行。</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEc5QOf5wGyjxZDwwukzck260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>政治, 科技, 社会</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>[视频]全国政协召开“一体推进教育科技人才发展”专题协商会 王沪宁出席并讲话</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>全国政协召开专题协商会，聚焦一体推进教育科技人才发展，王沪宁出席并讲话。</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEP13PllhTf1b3iISG7y0Z260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>[视频]中央宣传部等部门部署开展2026年“强国复兴有我”群众性主题宣传教育活动</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>21部门联合部署2026年“强国复兴有我”主题宣传教育活动，庆祝建党105周年等。</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEZAtwJa1uGCDbyihnq1KS260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>[视频]4月份我国制造业新动能引领持续增强</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>4月制造业新动能增强，装备制造和高技术制造业增长显著，出口交货值同比增长10.6%。</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEJ6sWCouQp1q1tf9limhE260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>[视频]多措并举助力民营经济高质量发展</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>市场监管总局完成民营经济配套制度清单38项，审查政策措施7.3万件，查办不正当竞争案1.46万件。</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEqMZGCWZOj02qrsccQnxs260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>经济, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>4月外汇市场稳健；20亿元支持15城打造国际化消费环境；中国旅游日推出惠民措施；应急通信平台启动全国应用。</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEk8KqVT4NCkrO5aseZAiP260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>HS2 could cost up to £102.7bn and trains will be slower than first planned</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>HS2高铁项目成本或达1027亿英镑，列车速度将低于原计划。</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c794xw7p2dqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>[视频]南方强降雨持续 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>南方多地强降雨持续，湖北、湖南、贵州积极应对，转移群众、抢险救灾。</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEq0wHNm91LZtBLtkMipxG260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥会见俄罗斯第一副总理</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>丁薛祥会见俄罗斯第一副总理，强调深化中俄投资合作，推动重点项目取得更多成果。</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEfkX5YJtIkSYofyEHM8ZR260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>[视频]俄罗斯各界期待元首外交引领中俄关系开启新篇章</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>俄各界期待元首外交引领中俄关系开启新篇章，国际人士盼为世界注入稳定性。</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDE5np4BS6KWXEljKNORLrh260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>[视频]世界卫生大会连续第10年拒绝涉台提案</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>世卫大会连续第10年拒绝涉台提案，中国代表强调一个中国原则。</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEGNM0uBD8RvB3u5FJjvp9260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称已回应美谈判意见 美称推迟其打击计划</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>伊朗称已回应美谈判意见，美总统称应多方请求推迟对伊军事打击。</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEKfU5MUv5qg0Pr1SDMQ3p260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>国际, 经济, 社会</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>中企承建阿联酋大型民航机库项目启动；格陵兰重申不卖岛；刚果（金）埃博拉疫情已致131人死亡。</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDEq7Ivb4bkRaerv35xTUOL260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>'Ebola has tortured us': Fear grips eastern DR Congo as deadly virus spreads</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>刚果（金）埃博拉疫情扩散致131人死亡，卫生部长承认应对迟缓。</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzj0pqpyyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Ebola outbreak may be spreading faster than first thought, WHO doctor warns</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>世卫组织医生警告，埃博拉疫情在非洲中部扩散速度或超预期。</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ceqp11gn1l8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Key people smuggler arrested after BBC uncovered identity</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>BBC曝光身份后，一名涉嫌走私数千移民的人口贩子被捕。</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yejzmvy56o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Israel's trying to expel a whole Palestinian district in East Jerusalem, activists say</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>活动人士称，以色列自与伊朗开战以来，加速在东耶路撒冷驱逐巴勒斯坦人。</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/19/nx-s1-5823861/israel-palestinians-east-jerusalem</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>One Palestinian man's life of survival</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>加沙一位90岁巴勒斯坦老人回忆流离失所与战争，称一生从未感到安全。</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/19/nx-s1-5825865/one-palestinian-mans-life-of-survival</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Putin visits China to reaffirm Russia ties, as Xi also seeks stable U.S. relations</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>普京访华巩固俄中关系，同时习近平寻求稳定美中关系。</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/19/g-s1-122775/putin-visits-china</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>[视频]2026年中国网络文明大会在南宁举行</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>2026年中国网络文明大会在南宁举行，主题为“文明网络空间 昂扬奋进力量”。</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/19/VIDERIglIlCsWtfKzyP29mZD260519.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Father-of-eight killed in San Diego mosque shooting hailed as hero</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>圣地亚哥清真寺枪击案中，保安阿明·阿卜杜拉因英勇行为被赞为英雄。</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp3gkrwg9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Victim or enabler? Epstein girlfriend who could face questions despite plea deal</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>爱泼斯坦女友纳迪亚·马辛科可能面临美国立法者质询。</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz92j3n3jvvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Surrey Police investigating child sex abuse allegations after Epstein files release</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>萨里警方调查爱泼斯坦文件涉及的儿童性虐待指控，无人被捕。</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0k2d2pl6x0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Channel 4 contacted by police after Married at First Sight UK rape claims</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>BBC调查曝《英国结婚即离婚》节目拍摄期间两女子遭强奸，警方介入。</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62xv7n4xwdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>California mosque shooting leaves 5 dead. And, judge dismisses Trump's IRS lawsuit</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>加州清真寺枪击案致5死，被调查为仇恨犯罪；特朗普放弃起诉国税局。</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/19/g-s1-122806/up-first-newsletter-islamic-center-san-diego-primary-elections-trump-irs-elon-musk-openai</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>BBC confirms new Strictly Come Dancing hosts</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>BBC确认《舞动奇迹》新主持人阵容，取代去年离任的泰丝和克劳迪娅。</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgep5ez80rzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>The French Open courts are clay, a tricky surface for some. Here's how the pros do it</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>法网红土场地难打，职业选手分享保持状态技巧。</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/19/nx-s1-5822888/french-open-clay-hailey-baptiste</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>体育</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Southampton expelled from Championship play-offs for spying on Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>南安普顿因承认在英冠赛季中监视三支球队，被逐出季后赛。</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cwy2pnpqjl7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-20
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F543"/>
+  <dimension ref="A1:F569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17813,6 +17813,838 @@
         </is>
       </c>
     </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260520 19:00</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>习近平欢迎普京访华并会谈；李强签署矿产资源法实施条例；神舟二十三号演练。</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEwtcCKjErR5iOXfwr5QXU260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎俄罗斯总统访华</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂举行仪式，欢迎俄罗斯总统普京对中国进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEE9t8SuJM1FTNSmMtVGbk260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统会谈</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>习近平同普京会谈，同意《中俄睦邻友好合作条约》继续延期。</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEJfeyvnOY5D6qT2QJM3yB260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统共同会见记者</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>习近平与普京会谈后共同会见记者，强调中俄关系高水平发展。</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDE8lbx8F8aVCUdOyAWpfE4260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>政治, 文体</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统共同出席“中俄教育年”开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>习近平与普京共同出席“中俄教育年”开幕式并致辞。</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEL42auGiM34MBIbZDyWom260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 塞尔维亚总统将对中国进行国事访问</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>应习近平邀请，塞尔维亚总统武契奇将于5月24日至28日访华。</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEuZSJK6w4FWcwqyQrci14260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>[视频]李强会见俄罗斯总统</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>李强会见俄罗斯总统普京，表示愿深化多领域合作。</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEHmuWAVkbrKyrtsoMRwWW260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Takeaways from Tuesday's primaries. And, victims of mosque shooting revealed</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>特朗普支持的候选人击败众议员马西；加州清真寺枪击案遇难者身份已确认。</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/20/g-s1-122996/up-first-newsletter-primary-elections-iran-war-mosque-shooting-victims-minnesota-prediction-markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Former Spanish Prime Minister Zapatero is under investigation</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>西班牙法院调查前首相萨帕特罗，涉政府航空救助案中的权力滥用。</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/20/nx-s1-5828248/former-spanish-pm-zapatero-investigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>[视频]李强签署国务院令 公布《中华人民共和国矿产资源法实施条例》</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>李强签署国务院令，公布《矿产资源法实施条例》，2026年6月15日施行。</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEpcXCOHUtC379kWgy5GJ9260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>[视频]服务业经济平稳增长 发展潜力持续释放</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>我国服务业平稳增长，高技术服务业投资增10.5%，服务零售额增5.6%。</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEjYErelfNVplzTjx0by1p260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>4月用电量增6%；网售食品新规实施；最高检开展长江水污染专项监督。</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEX2WJdEzoNi1VoIuzpnL9260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Fuel duty freeze extended until the end of the year</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>英国燃油税削减政策延期至年底，维持5便士降幅。</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3021md6jq6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号载人飞行任务各系统进行发射场区演练</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>神舟二十三号近日择机发射，今日进行全系统合练，流程精准无误。</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEMweWnfd2Nhnf90xg2kZc260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Russian jets 'dangerously' intercept RAF spy plane over Black Sea</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>俄战机在黑海危险拦截英军间谍飞机，英国防部证实。</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq8p40e2zx1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>国新办举行记者见面会，五位生态环境代表分享环保工作实践。</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/20/VIDEzLP6P2ZjxrDCOBNiygY2260520.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>US charges Cuba's Raúl Castro with murder over 1996 downing of two planes</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>美国指控古巴劳尔·卡斯特罗等人涉嫌1996年击落两架飞机致谋杀。</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3r219yxl5eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Rosenberg: Putin enjoys Xi's Chinese welcome but heads home without pipeline deal</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>普京访华受热情接待，但未达成管道协议，显示中俄合作有边界。</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8r8me3nlllo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Far-right Israeli minister condemned for taunting handcuffed Gaza flotilla activists</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>以色列极右翼部长嘲弄被拘留的加沙船队活动人士，遭法意等国谴责。</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp32weyn8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Ebola vaccine could take nine months as death toll rises further, WHO warns</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>世卫警告埃博拉疫苗研发需九个月，当前死亡139例，病例达600。</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2g197dp8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Murder or accident? Mystery of Mango tycoon's hiking death after son's arrest</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>芒果帝国创始人死亡疑云，其子否认谋杀指控。</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2g09yvgmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>The U.S. threatens to revoke the Palestinian U.N. ambassador's visa</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>美国威胁撤销巴勒斯坦驻联合国大使签证。</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/20/nx-s1-5828826/us-palestinians-un</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>U.S. grand jury indicts Raul Castro, ex-Cuban president</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>美国大陪审团起诉古巴前领导人劳尔·卡斯特罗，涉谋杀等罪名。</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/20/g-s1-122383/us-cuba-raul-castro-indictment</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Women who died in sea off Brighton were sisters</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>布莱顿海域溺亡女性为三姐妹，父亲悲痛悼念。</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62dn5r4elqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>London bus driver dies after assault on bridge</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>伦敦公交司机在桥上遇袭身亡，嫌疑人被捕。</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypnj4dnk5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Greetings from Bali, where a kecak dance shows the triumph of good over evil</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>巴厘岛凯卡克舞表演《罗摩衍那》故事，展示正义战胜邪恶。</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/20/g-s1-122603/bali-indonesia-kecak-dance-ramayana</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-21
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F569"/>
+  <dimension ref="A1:F601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18645,6 +18645,1030 @@
         </is>
       </c>
     </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>政治, 经济, 文化</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260521 19:00</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>今日新闻联播报道中俄元首会晤、文化强国论坛开幕、财政收入向好等要闻。</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEqt0hnbBgn7TOaWSGTnUs260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统茶叙</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>习近平同俄罗斯总统普京茶叙，就推进中俄战略协作达成重要共识。</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEtfkvutItYEXPciW5TQzT260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>[视频]习近平同俄罗斯总统共同参观“传承中俄世代友好 树立大国关系典范”图片展</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>习近平同普京共同参观中俄世代友好图片展，忆及友好交往瞬间。</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEyer1Af9D9t5RV288txSO260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>[视频]习近平同巴基斯坦总统就中巴建交75周年互致贺电 李强同巴基斯坦总理互致贺电</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>习近平同巴基斯坦总统就建交75周年互致贺电，强调深化中巴命运共同体。</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEb1xSbYwCHJHCUqedi1uw260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，研究推进全国统一大市场建设和应急体系规划。</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDE9PV2XVXFt8gze175MFd4260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>[视频]纠治涉企执法突出问题 持续优化营商环境</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>全国纠治涉企执法突出问题，查纠案件6.6万多件，挽回经济损失307亿元，行政检查总量下降34%。</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEYtt4nRdvabrH8Ul2nNzY260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Late Queen was 'very keen' for Andrew to be given trade envoy role</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>文件显示，英女王伊丽莎白希望儿子安德鲁担任贸易特使。</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2pjg397l2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>UK migration drops to 171,000 - almost half 2024's figure</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>英国移民人数降至17.1万，首相称兑现边境管控承诺。</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp1ekd584o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Palestinians drop bid for a senior U.N. role after U.S. pressure</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>巴勒斯坦在美国压力下放弃争取联合国高级职位。</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/21/g-s1-123450/us-palestinians-united-nations-general-assembly</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>GOP races to fund immigration enforcement. And, U.S. indicts former Cuban president</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>共和党推进720亿移民执法法案，美国起诉古巴前总统。</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/21/g-s1-123307/up-first-newsletter-congress-ice-border-patrol-funding-iran-war-raul-castro</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Netanyahu scolds Israeli security minister for videos taunting flotilla activists</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>内塔尼亚胡谴责安全部长发布视频嘲弄被扣活动人士。</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/21/nx-s1-5829616/israeli-security-minister-flotilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>[视频]我国财政收入巩固向好态势</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>前四月全国一般公共预算收入8.34万亿，同比增长3.5%，支出进度为近5年最快。</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEiQJOrYry0XbupKdklPu9260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>[视频]前四个月国家铁路发送货物13.1亿吨</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>今年1至4月，国家铁路发送货物13.1亿吨，同比增长0.9%，铁水联运和中欧中亚班列增长显著。</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEOJHPzWpOux9CyXuVc9BJ260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Cheaper theme park tickets and children's meals as VAT to be cut for some attractions this summer</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>英国财相宣布今夏部分景点增值税降低，包括更便宜主题公园门票和儿童餐。</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd7pzr88de1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>After the sirens: Lebanon's first responders swing between duty and grief</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>黎巴嫩战争致近3000人死亡，停火后仍有近400人遇难。</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/sections/the-picture-show/2026/05/21/nx-s1-5821157/lebanons-first-responders-balance-duty-and-grief</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>[视频]南方地区降雨持续 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>南方多地持续强降雨，江西、广东、广西等地受灾，国家发改委安排资金支持灾后应急恢复。</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEOsO0aWusiwDO1Qs3KPYz260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>国际, 社会, 文体</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>第十届中俄博览会闭幕；文化企业30强发布；广西地震启动四级应急响应；长三角一体化清单发布。</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEGqQCTce9X90sG6B6M9TJ260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>[视频]俄罗斯各界人士表示俄中元首会谈对两国关系实现更高质量发展意义重大</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>俄罗斯各界人士表示，俄中元首会谈对两国关系高质量发展及构建公正全球治理体系意义重大。</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDE0nCAC4wXGgGQnUpbs4nA260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>[视频]伊称继续推进谈判同时坚决维护国家利益 美称签署协议前不会有制裁减免</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>伊朗称继续谈判维护国家利益，美称签署协议前不减免制裁，美在阿曼湾扣押伊朗油轮。</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEHEmqZpWoCpe6RppQT9cJ260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>以军空袭黎南部致19死，多国谴责以粗暴对待援助船队；联合国报告称地缘紧张考验经济韧性。</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDE2p3Zi5jMWt2Fx2sC9zlj260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Iran steps up claim to control Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>伊朗发布地图，主张对霍尔木兹海峡超2.2万平方公里水域拥有“武装部队监督权”。</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq5py64gvwzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Gaza flotilla activists deported from Israel as backlash over treatment grows</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>以色列极右翼部长羞辱加沙救援船活动家的视频引发广泛谴责。</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9d3v2d6p1eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Russia and China condemn US over indictment of former Cuban leader</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>俄中谴责美国指控古巴前领导人劳尔·卡斯特罗谋杀，施压古巴政权。</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clype0x7pkgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】危急时刻 党员冲锋在前</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>湖南常德强降雨致村庄成孤岛，党员干部冲锋在前，转移124名群众至安全区域。</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDE0Qa4jACfxbkn5CJVUphq260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>[视频]二十四节气·小满</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>小满节气到来，夏收作物籽粒渐满，三候与农事活动展现生活热忱。</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEU3Inmoogb4HyCxq6OHDt260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Pair arrested after boys abandoned by road in Portugal</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>两名男孩被发现遗弃在葡萄牙路边，携带食物和水，一名司机发现后报警。</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9wex9v57ndo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Air France and Airbus found guilty of manslaughter over 2009 plane crash</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>法航和空客因2009年空难致228人死亡被法国法院裁定过失杀人罪成立。</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czd2qmdvmq6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Toilets and changing rooms must be used on basis of biological sex, guidance confirms</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>英国指南确认厕所和更衣室必须按生物性别使用，基于去年最高法院裁决。</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0e2rj3zj02o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>As floods get worse, Britain tries a new solution: beavers</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>英国重新引入海狸，利用其筑坝技术缓解洪水。</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/21/nx-s1-5738979/beavers-britain-climate-change-flooding</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Foden and Palmer to miss out on World Cup squad</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>福登和帕尔默将无缘世界杯阵容，但伊万·托尼入选。</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c78ke277pmdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>文化, 社会</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>[视频]2026文化强国建设高峰论坛在深圳开幕</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>2026文化强国建设高峰论坛在深圳开幕，聚焦文脉传承与数智化赋能。</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEbM0qk27rCdgV96ihkrtl260521.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>文化, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>[视频]第二十二届中国（深圳）国际文化产业博览交易会开幕</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>第二十二届深圳文博会开幕，展出超12万件文化精品，首次设APEC展区。</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/21/VIDEFhmrw5howUH4l0A6m1Cc260521.shtml</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-22
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F601"/>
+  <dimension ref="A1:F631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19669,6 +19669,966 @@
         </is>
       </c>
     </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>政治, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260522 21:00</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>新闻联播今晚报道：美丽中国建设、赵乐际出访、国务院推常住地基本公共服务等多项内容。</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDESH60j321H6iN0rXEww2N260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>[视频]《习近平的文化情缘》《习主席的来信》在塞尔维亚启播</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>总台制作专题节目《习近平的文化情缘》《习主席的来信》在塞尔维亚启播。</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEtvhDzSUcxUS3sBwGayg6260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际将访问哈萨克斯坦、俄罗斯并在俄出席中俄议会合作委员会第十一次会议</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>赵乐际将于5月25日至30日访问哈萨克斯坦、俄罗斯，并出席中俄议会合作会议。</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDE0qAvdjqJWfOUooCKMER7260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】助力发展 务实为民 推动学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>义乌和天津武清开展树立正确政绩观学习教育，深查实改优化企业服务。</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEliMEh1UqUAHelcdjinRg260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Rubio tries to reassure Nato allies over US troop deployments</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>特朗普表示将向波兰增派美军，其官员此前取消类似部署。</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cedpz9669deo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Trump is putting pressure on Cuba - why and to what end?</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>美国对古巴施压，警告和平协议无望；古巴称美国借口军事干预。</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yrkl96xwvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>'Stupid on stilts' - Trump's investigation compensation fund draws ire of Republicans</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>特朗普18亿美元赔偿基金引发共和党强烈不满。</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21d41p6dzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Tulsi Gabbard to resign as US director of national intelligence</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>美国国家情报总监因丈夫患病辞职。</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgj2gkv1x1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Rubio doubtful of diplomacy with Cuba as Trump raises new threat of military action</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>特朗普与鲁比奥对古巴再提军事威胁。</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/22/nx-s1-5830999/rubio-diplomacy-cuba-trump-military-action</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>[视频]我国将抓紧出台“六张网”相关规划和实施方案</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>我国将出台水网、新型电网等“六张网”规划，明确投资重点和年度安排。</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEhhBhpciPfLCPilrJSyqz260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>[视频]第四届链博会将于6月22日至26日在北京举行</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>第四届链博会将于6月22日至26日在北京举行，设置六链一展区，首次设立人工智能专区。</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEQXh5VZh8KXbphRgOmaKu260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>[视频]2025年全国核发绿证超过29亿个</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>2025年全国核发绿证超29亿个，绿证交易规模创历史新高，企业是消费主力。</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDExn9BmzWxtPhwn9C251mW260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号载人飞船发射任务组织全区合练</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>神舟二十三号发射任务组织全区合练，各系统准备就绪，航天员在轨待命。</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEakbMlIl3tUosOYlbF21r260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>UK scientists developing Ebola vaccine that could be ready for trials in months</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>英国科学家研发针对罕见埃博拉病毒疫苗，数月内或可试验。</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy82gkr7xzlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Trump says he's sending 5,000 more troops to Poland</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>特朗普宣布向波兰增派5000名美军，引发欧洲困惑。</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/22/g-s1-123596/trump-sending-5-000-troops-to-poland</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《关于推行常住地提供基本公共服务的实施意见》</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>国务院发文推行常住地提供基本公共服务，涵盖教育、社保、住房等多领域。</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEH9pIc3IRZN8xSFEXp9e8260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】主产区应对降雨天气 确保夏粮颗粒归仓</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>主产区应对降雨天气，采取无人机作业、备收割机等举措，确保夏粮颗粒归仓。</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDExoWHNqk9icC6hschmOsk260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>国际生物多样性日等活动举行，发布生态补偿方案、办学底线要求，并安排资金支持广西灾后恢复。</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDELsrFc2vE5phcBXEoFpcw260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>UK sees hottest day of year as bank holiday travellers face queues</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>英国迎今年最热一天，多地交通拥堵影响银行假期出行。</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpqpygjwywjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称正讨论谈判文本 美再度威胁伊朗交出浓缩铀</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>伊朗与美国讨论谈判文本，美方要求伊朗交出浓缩铀；国际能源署警告石油市场或面临高风险。</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEGlvm17pJrVqXaB1fIHsx260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>[视频]以军袭击巴勒斯坦加沙地带多地</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>以军袭击加沙多地致人死亡，多方要求制裁以色列国家安全部长本-格维尔。</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEwa97EW1V7s1nPafFJxW1260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>俄白举行首次联合核力量演习；美国对北约失望；格陵兰岛民众抗议美国新领事馆开馆。</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEmG6gp1KNmRZQN3uCFNRz260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Russia's Putin vows retaliation after accusing Ukraine of hitting student dormitory</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>俄罗斯指控乌克兰袭击学生宿舍并誓言报复，乌克兰称打击了俄精英无人机部队。</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y74lwx395o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Ebola risk raised to 'very high' in DR Congo</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>世卫组织将刚果（金）埃博拉风险升至“非常高”，全球风险仍低。</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr7p30m1dn1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>The aftermath of Trump-Xi summit: comparing U.S. and China announcements</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>特朗普与习近平峰会后的美中声明存在“微小差异”。</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/22/g-s1-123647/comparing-u-s-and-china-announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Italy's prime minister wants Israel to apologize for treatment of flotilla activists</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>意大利总理要求以色列就处理船队行动道歉。</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/22/nx-s1-5830108/italys-prime-minister-wants-israel-to-apologize-for-treatment-of-flotilla-activists</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>UN gravely concerned by an Afghan Taliban law that has provisions on child marriage</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>联合国对阿富汗塔利班涉及童婚的新法表担忧。</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/22/nx-s1-5831001/un-concerned-afghan-taliban-law-child-marriage</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】美丽中国 万物共生</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>我国加快构建国家公园体系，藏羚羊等珍稀物种种群增长，生物多样性保护成效显著。</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/22/VIDEfmpigFsjVolk08y4zvkK260522.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Bodies of Italian divers did not have optimal equipment, says rescuer</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>救援人员称，4名意大利潜水员尸体被发现时未配备最佳装备。</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0l2j723nrxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Attorney general to review teen boys' rape sentences</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>司法部长将审查三名青少年因强奸两名女孩未被判监禁的判决。</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2x7wxjego?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-23
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F631"/>
+  <dimension ref="A1:F658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20629,6 +20629,870 @@
         </is>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260523 19:00</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道习近平对山西煤矿事故指示、十五五规划、神舟二十三号、外资增长、邮寄业务、油气供应、北斗产值等要闻。</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEDgpPxpOIiYAMogYJo6t3260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>[视频]习近平对山西长治市沁源县一煤矿瓦斯爆炸事故作出重要指示强调 全力救治伤员 科学组织搜救 坚决防范遏制重特大事故发生 李强作出批示</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>习近平就山西煤矿瓦斯爆炸事故作指示，要求全力救治伤员、科学搜救、防范重特大事故，李强作出批示。</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEAUIXx66V9InB7JeqvjkW260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】上海以“五个聚力”推进“十五五”高质量发展 黑龙江在全面振兴中开创高质量发展新局面</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>上海以“五个聚力”推进十五五高质量发展；黑龙江在全面振兴中开创高质量发展新局面。</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEWWHCZUl5P2nQdK5PMShQ260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>[视频]前4个月我国高技术产业实际使用外资同比增长20.3%</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>前4月我国高技术产业实际使用外资同比增长20.3%，占全国外资40.4%。</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEV2aY0XCV7JJfp2Db2X6A260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>[视频]前4个月我国邮政行业寄递业务量达701.6亿件</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>前4月我国邮政行业寄递业务量达701.6亿件，同比增长4.1%。</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEgMed9HTZUyiUpuoebykq260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>[视频]织密“全国一张网” 我国油气供应能力持续提升</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>我国油气供应能力持续提升，“全国一张网”不断织密，在建管网超9000公里。</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEfW8owM5BFQGYZBYYioT8260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】省级经开区“瘦身”记</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>辽宁撤并21个省级经开区，避免产业同质化竞争，集中优势资源促高质量发展。</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEUqv97tiBAgWU2Ilu3EVL260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>八部门整治非法跨境证券期货；发布AI伦理安全指引；4月民航旅客量超6100万；西部陆海新通道进出口创新高。</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEBSl0TeRv3jbhBE0walGf260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号载人飞船发射窗口确定 航天员乘组亮相</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>神舟二十三号发射窗口确定，航天员乘组亮相，含首位港澳女性载荷专家，将开展1年期在轨试验。</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEwlCAFBz11OAcy170plbB260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>[视频]2025年我国北斗时空产业产值超1.3万亿元</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>2025年我国北斗时空产业产值超1.3万亿元，应用场景拓展至通信、交通等领域。</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDE8JKmW59QxAOeMGVZ8TBi260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>SpaceX launches massive Starship V3 rocket on test flight</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>SpaceX发射史上最大最强星舰V3火箭，进行测试飞行。</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62d65y16nno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>'Shameful' more spent on benefits than jobs for young people, says Milburn</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>米尔本称福利支出多于青年就业投入是“可耻的”，呼吁改革。</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crrpx4p1z71o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Hottest day of year so far as temperatures soar on bank holiday weekend</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>英国银行假日气温飙升，为今年最热一天，多地发布健康警报。</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/crmp8dlyz3ko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称谈判重点是结束战争 暂不涉及核问题</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>伊朗称谈判重点为结束战争，暂不讨论核问题；美方考虑军事打击，伊方已制定新方案应对。</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEaR4A4Vt9JRHyrEUzuvgM260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>[视频]以军继续袭击巴勒斯坦加沙地带多地</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>以军袭击加沙多地致伤亡；西方多国敦促以色列停止扩大定居点，称其严重违反国际法。</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDE3ywH8w4t3pyV6T1ufong260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>俄称乌无人机袭击学校致伤亡，乌否认；古巴抗议美国起诉革命领袖；美国家情报总监辞职。</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEpf2nlGUwwQdYDXUTat9e260523.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Putin vows retaliation after accusing Ukraine of hitting student dormitory</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>普京指控乌克兰袭击学生宿舍并誓言报复；乌方称打击的是俄军事单位。</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y74lwx395o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>French mum and partner held until trial after sons abandoned by road in Portugal</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>法国母亲和伴侣因在葡萄牙路边遗弃儿子，被拘留候审。</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq5p75l7n17o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Rubio meets Modi during India visit with energy high on agenda</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>美国国务卿鲁比奥访印，议程聚焦向印度销售能源以弥补伊朗战争缺口。</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c87qrwyyrn2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>France suspends extra EU border checks at Dover after hours-long queues</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>法国暂停多佛尔额外欧盟边境检查，此前旅客排长队。</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp3p2ver9k6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>U.S. passengers flying from Ebola-affected countries rerouted</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>美国对埃博拉疫情国家实施旅行限制，乘客需飞往三个指定机场。</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5831963/u-s-passengers-flying-from-ebola-affected-countries-rerouted</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>NATO allies confused by Trump's unexpected move to deploy 5,000 U.S. troops to Poland</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>特朗普突然决定向波兰部署5000美军，北约盟友表示困惑。</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5831245/nato-allies-confused-by-trumps-unexpected-move-to-deploy-5-000-u-s-troops-to-poland</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Chile's MAGA-inspired border control</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>智利总统模仿特朗普政策，在北部边境挖沟遏制移民，被批效果甚微。</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5806607/chile-maga-inspired-border-control</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Trump administration to force foreigners in the U.S. to apply for a green card abroad</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>特朗普政府突然改变政策，要求美国境内外国人离境申请绿卡。</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5832399/trump-administration-green-card-abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>At least 82 killed in Chinese coal mine explosion</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>中国山西煤矿爆炸致82人死亡，为16年来最严重矿难。</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y0ve18qlko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Coal mine gas explosion in China kills 90 people, state media say</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>中国山西一煤矿发生瓦斯爆炸，至少90人死亡，247人在岗。</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5832405/coal-mine-gas-explosion-china</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>生态, 社会</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>[视频]长江口十年来生态保护成效显著</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>长江口十年生态保护成效显著，湿地保护率68%，鸟类超360种，江豚种群回升。</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/23/VIDEndUxoTeCIBVwBhZbZz4n260523.shtml</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-24
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F658"/>
+  <dimension ref="A1:F684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21493,6 +21493,838 @@
         </is>
       </c>
     </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260524 19:00</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>西藏和平解放75周年成果显著；神舟二十三号发射在即；全球超九成超大型油轮订单涌向中国；强降雨来袭各地应对。</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEwnt9vC0R2V9gqz0FFwX7260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】努力建设社会主义现代化新西藏</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>西藏和平解放75周年，社会主义现代化新西藏建设取得历史性成就，林芝嘎拉村依托生态旅游致富。</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEs6qXybAo6GRWJSu3gJwT260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>最高检发布长江经济带白皮书；我国研究制定算力网技术标准；F406涡扇发动机首飞成功；首届中学生人形机器人足球赛决出冠军。</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEdIym43qEMAOQXRt0rp6B260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Turkish riot police storm opposition offices after leaders ousted</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>土耳其防暴警察闯入反对党总部，此前该党誓言违抗法院罢免其领导人的裁决。</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c87qwrqre83o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>[视频]全球超九成超大型油轮订单涌向中国</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>中国造船业超大型油轮订单占全球92%，交付快且技术先进，建造周期排至2030年。</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEo8zV8o6ja2jC7Kcu6THs260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>'Six eggs used to be £1' - why everyday essentials cost so much more now</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>2022年6枚鸡蛋仅1英镑，如今为何暴涨？调查背后涨价原因。</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd6pw4zg5p9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号飞船发射准备就绪</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>神舟二十三号载人飞船今日23时08分发射，飞船在多方面升级，预留国际合作接口。</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEWd4JkXS9QjrYPN4NTyHG260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>[视频]俄称使用“榛树”导弹等对乌发动大规模打击 乌称打击俄黑海沿岸石油码头</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>俄使用高超音速导弹大规模打击乌克兰，乌打击俄黑海沿岸石油码头等目标。</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEyzaObBOB7VYVHXSf671b260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Large-scale Russian attack on Ukraine leaves four dead and dozens injured</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>俄罗斯大规模袭击乌克兰，使用高超音速导弹，造成4人死亡、数十人受伤。</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyp6831yp5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Blast targeting train kills at least 20 in Pakistan</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>巴基斯坦一列运载军人的列车遭武装分子袭击，爆炸致至少20人死亡。</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2pkd58xldo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Russia pounds Kyiv in powerful drone and missile attack</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>俄军动用可携核弹头高超音速导弹袭击基辅，致2死77伤。</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/24/nx-s1-5833050/russia-uses-hypersonic-oreshnik-missile-in-mass-attack-on-kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】暖民心 惠民生 推动学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>山东青岛和吉林吉林市开展学习教育，立查立改，解决基层医疗和老旧小区改造等民生问题。</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEgFeqdOBVyEzvt9bSx7X4260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>[视频]强降雨来袭 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>强降雨影响黄淮江淮等地，重庆永川出现特大暴雨致人失联，各地正全力防汛救灾。</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEFfPapAtwWdAs1tVzsDXG260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>[视频]【新闻特写】黄龙镇的麦收48小时</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>湖北襄阳黄龙镇抢抓雨停间隙，调动农机连夜抢收小麦，多方协同保障夏粮收获。</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDE6GN1UmtspVFBws2LhmiF260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>[视频]美称美伊协议基本谈成 伊称双方正努力敲定谅解备忘录</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>特朗普称美伊协议基本谈成，伊朗正努力敲定备忘录，涉及开放霍尔木兹海峡、解除制裁等。</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEDlZwRZEuZxoJkONcMgpV260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>国际, 社会, 文体</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>以轰炸加沙致5死，法国制裁以官员；刚果（金）埃博拉疫情恶化；伊朗队世界杯驻地改至墨西哥。</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDEvoS1lIezOWYPw5aYDq5e260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Suspect killed after opening fire on Secret Service near White House</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>一名嫌疑人靠近白宫附近检查站开枪，被特勤局击毙，一名路人受伤。</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjwp82ye4y3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>What both sides have said about a U.S.-Iran deal</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>特朗普称美伊接近达成结束战争协议，但未提供细节，伊方立场不明。</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/24/nx-s1-5832613/what-both-sides-have-said-about-a-u-s-iran-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>What we know about the status of a U.S.-Iran deal</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>专家解读美伊潜在协议现状，分析双方谈判进展与障碍。</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/24/nx-s1-5833058/what-we-know-about-the-status-of-a-u-s-iran-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Romanian director Cristian Mungiu's 'Fjord' wins top prize at Cannes</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>罗马尼亚导演蒙吉凭新作《峡湾》获戛纳金棕榈奖。</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/nx-s1-5832564/palme-dor-cannes-film-festival</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Trump touts Iran breakthrough but details remain unclear</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>特朗普宣称伊朗协议突破，但细节模糊且未获伊朗官方确认。</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/23/g-s1-124145/trump-iran-deal-strait-of-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>BBC at the site of China's worst mining disaster in more than a decade</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>中国刘什宇煤矿发生瓦斯爆炸，至少82人死亡，为十多年来最严重矿难。</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c809m33yjz7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Keir Starmer says rape of two girls by boys spared custody 'appalling'</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>英国首相称两男孩强奸少女却免于拘留“令人震惊”，已紧急审查量刑。</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c332ljdkd81o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Why did I put myself through the pain of going to court, rape victim tells BBC</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>强奸案受害者向BBC倾诉：法官判施暴男孩免刑，如同“一记重拳”。</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/ce9pmyz7jrxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】一叶连古今 一茶和天下</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>中国茶文化源远流长，抹茶申遗成功后创新传承，茶文旅融合推动非遗活态发展。</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/24/VIDECE0plJFt6pIlhCQmICKl260524.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>It's like the Olympics, except steroids are allowed</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>首届“增强运动会”在拉斯维加斯开幕，允许使用兴奋剂引争议。</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cedpz1zqp8po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-25
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F684"/>
+  <dimension ref="A1:F713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22325,6 +22325,934 @@
         </is>
       </c>
     </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260525 21:00</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>习近平欢迎塞尔维亚总统访华并会谈，会见巴总理；《习近平谈治国理政》第五卷多文版发行；神舟二十三号发射成功。</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDERRr0sdSAvMiBtMFFODlF260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎塞尔维亚总统访华</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂为塞尔维亚总统武契奇举行欢迎仪式，鸣礼炮21响。</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEhvcOp9B4W5A9Y5olEDbq260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>[视频]习近平同塞尔维亚总统会谈</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>习近平同塞尔维亚总统武契奇会谈，强调深化中塞命运共同体建设，加强多领域合作。</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEMrM0LyShhI3ck9Xdn3aN260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见巴基斯坦总理</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>习近平会见巴基斯坦总理夏巴兹，强调加快构建中巴命运共同体，深化全方位合作。</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDECsTPFKOSFXRgXXi5gX4g260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>[视频]《习近平谈治国理政》第五卷法俄阿等文版及中文繁体版出版发行</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>《习近平谈治国理政》第五卷8个文版出版发行，收录总书记2022至2024年重要著作。</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEZeIQmFSxL2lvnzNUncEa260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>[视频]李强会见塞尔维亚总统</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>李强会见塞尔维亚总统武契奇，强调深化贸易、投资、人文合作，推进匈塞铁路等重点项目。</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEW2K5I1JZ0cBn47SbD8rK260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>[视频]李强举行仪式欢迎巴基斯坦总理访华</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>李强在人民大会堂为巴基斯坦总理夏巴兹举行欢迎仪式，检阅仪仗队。</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEw3jOTamNhR5xIFWJTkFj260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>[视频]李强同巴基斯坦总理会谈</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>李强同巴基斯坦总理夏巴兹会谈，推动中巴经济走廊建设及多领域合作。</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEXbpafpT7Mxbf2VLA2vgi260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁主持召开全国政协主席会议</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>王沪宁主持召开全国政协主席会议，强调学习贯彻习近平经济、科技、防灾减灾等重要指示精神，引导委员建言献策。</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEie1L6UBenVV3DlYSKzdI260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>[视频]全国人大常委会启动海南自由贸易港法、旅游法执法检查</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>全国人大常委会启动海南自由贸易港法和旅游法执法检查，重点检查贸易、投资、旅游权益等8方面内容。</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEEmzWJNbwxKjs9XAHOjgc260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Former SNP chief executive Peter Murrell in custody after admitting £400,000 embezzlement</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>苏格兰前首席大臣丈夫穆雷尔承认侵占40万英镑，被还押候审。</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g4q7yl3kno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>The questions raised by the Murrell embezzlement controversy</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>苏格兰民族党前首席执行官穆雷尔侵占案引发诸多疑问。</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c74dd82w943o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>经济, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>文博会闭幕；五部门出台超龄劳动者权益保障暂行规定；美称伊核协议未谈妥，伊朗回应谈判底线。</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEluibLkfaX3Nxe3wJMtiJ260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号载人飞船发射取得圆满成功 两个乘组航天员会师太空</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>神舟二十三号载人飞船发射成功，与神舟二十一号乘组太空会师，为第8次会师，首迎香港航天员。</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEMqyaXrR8WN9dsTBpOSFE260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Russia threatens more Kyiv strikes and tells foreign nationals to leave</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>俄罗斯威胁对基辅发动更多袭击，要求外国人离开乌克兰。</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1e22n55zn4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Hottest May day on record in UK as temperatures pass 34C</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>英国五月气温突破34摄氏度，创下历史最高记录。</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8xwwpkrgj1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见塞尔维亚总统</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>王沪宁在京会见塞尔维亚总统武契奇，双方表示将深化中塞命运共同体建设，坚定相互支持，加强战略对接。</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDENI7bkduFhskB8gzHDXIS260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>[视频]蔡奇会见塞尔维亚前进党代表团</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>蔡奇会见塞尔维亚前进党代表团，表示愿加强党际交往，共同落实两国元首共识，推动中塞命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDEyaUEOBjb10Z5DXz9iIdf260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Deal with US not imminent, Iran says</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>伊朗称与美国的协议并非即将达成，此前美方曾暗示协议可能于周一达成。</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cglpp2yk336o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Oil prices slide on hopes of US-Iran peace deal</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>特朗普称美伊和平协议将包括重开霍尔木兹海峡，油价应声下跌。</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c809m7g29r7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Trump says U.S. and Iran nearing a peace deal. And, Pope Leo weighs in on AI's rise</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>特朗普称美伊接近达成和平协议；教皇方济各就人工智能崛起发表首道通谕。</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/25/g-s1-124191/up-first-newsletter-iran-war-trump-ebola-california-chemical-tank-pope-leo-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Trump says more countries should normalize ties with Israel in any Iran deal</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>特朗普要求更多国家与以色列关系正常化作为伊朗协议条件，伊朗代表团赴多哈谈判。</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/25/nx-s1-5833690/u-s-iran-negotiations-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Venezuela's government faces calls for elections after failed release of prisoners</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>委内瑞拉释放政治犯承诺未兑现，反对派要求选举并呼吁自由。</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/25/nx-s1-5831506/venezuelas-government-faces-calls-for-elections-after-failed-release-of-prisoners</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>[视频]各地各部门积极应对持续强降雨</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>多地持续强降雨，江西、湖北等地积极排涝抢险，安全转移群众，水库动态泄洪。中央气象台预警持续。</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/25/VIDE5F6boeQj7TsVhtN8krXd260525.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>White House gunman had previous run-ins with Secret Service, court documents show</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>白宫枪击案嫌犯此前曾与特勤局发生冲突，并自称耶稣基督。</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1l22pg12mpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Three killed in Uganda after crashing into elephant</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>乌干达发生汽车撞象事故，致3人死亡，4人受伤。</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyppgvd3qzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Woman dies after being shot outside Sheffield bar</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>一名30岁女子在谢菲尔德酒吧外遭枪击身亡，三人被拘。</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2022lwyex1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>In Beirut, refugee girls and women learn more than self-defense in martial arts class</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>贝鲁特难民营中，女性通过武术课程学习自卫并寻求赋权。</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/25/g-s1-120826/lebanon-women-martial-arts</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>'My body carried me,' Elizabeth Smart says. Now she's celebrating it</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>14岁遭绑架的伊丽莎白·斯玛特通过健美重塑身体认知，克服羞耻感。</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/25/nx-s1-5832603/elizabeth-smart-bodybuilding-trauma-exercise</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-26
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F713"/>
+  <dimension ref="A1:F741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23253,6 +23253,902 @@
         </is>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260526 19:00</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>习近平为塞尔维亚总统授勋；卫塞节开幕；中巴建交75周年；辽宁青海发布十五五规划；提升公共服务水平；消费市场平稳运行；跨国公司峰会定于6月举行；各地抢收夏粮；南方强降雨持续。</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDETLLlN0XAWYpnFbo25Qud260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>[视频]习近平为塞尔维亚总统举行“友谊勋章”颁授仪式</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>习近平为塞尔维亚总统武契奇颁发“友谊勋章”，表彰其推动中塞友好关系。</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDENpaRHc5JRDvxuTUiYHv7260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>政治, 国际, 社会</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>[视频]第21届联合国卫塞节在中国无锡开幕 王沪宁致信祝贺</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>第21届联合国卫塞节在无锡开幕，王沪宁致贺信，强调佛教交流与全球倡议。</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEQX0Q41v8RtE4Z1CxlhhM260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>[视频]韩正同巴基斯坦总理共同出席庆祝中巴建交75周年招待会</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>韩正与巴总理出席中巴建交75周年招待会，强调深化全天候战略合作伙伴关系。</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEdXcX4MIB4cXDZXLpyZpT260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】推动新时代辽宁全面振兴取得新突破 奋力谱写中国式现代化青海篇章</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>辽宁、青海发布“十五五”规划，聚焦产业升级、科技创新和民生福祉。</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEawbXtjEkny5OPiIVSumI260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>[视频]前四个月消费市场平稳运行 向新向优发展</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>前4月消费市场平稳运行，以旧换新带动绿色智能产品销售，乡村消费增长快于城镇。</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEq2CJskGuBV2W51zoUv1d260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>[视频]第七届跨国公司领导人青岛峰会将于6月15日至17日举行</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>第七届跨国公司领导人青岛峰会将于6月15日至17日举行，主题为“携手‘十五五’向新向未来”。</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEmga88cc9qGWbIA4wdS5s260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>'Bullying' and 'overbearing' behaviour behind abrupt BP chairman removal</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>英国石油公司前董事长因霸凌和专横行为被突然解职，公司拒评具体原因。</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjrppppwvwlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Eleven killed in Lebanon village as Israel intensifies strikes</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>以色列加强空袭黎巴嫩，声称打击100处真主党目标，总理誓言摧毁该组织。</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx211rgngp0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>[视频]我国加力提升未落户常住人口基本公共服务水平</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>我国出台实施意见，提升未落户常住人口在教育、住房、社保等方面的基本公共服务。</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEQYexSPogMCPC6JbyOYiq260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>[视频]各地全力抢收抢烘 护航夏粮颗粒归仓</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>中东部强降雨影响麦收，主产区全力抢收抢烘，保障夏粮颗粒归仓。</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEYKeBtf4NGxkhIL80C4mg260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>[视频]主雨带南压 南方仍有大范围强降雨</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>主雨带南压，南方多地仍有强降雨，需警惕次生灾害。</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEIsqqCEgXrGQ65mk7t55X260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>民生, 国际, 科技</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>两部门预拨1.6亿元救灾；部署“六一”活动；中国-中东欧地方会议开幕；公布“人工智能+”能源场景清单。</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEkCBKd0uxVJpBezsV9w6M260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>An exceptionally early heat wave shatters records and brings deaths in Europe</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>欧洲遭遇异常早热浪，伦敦气温达95华氏度，极端天气频发致人死亡。</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/g-s1-124360/europe-heat-wave-deaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>[视频]伊朗南部港口传出爆炸声 美称打击伊导弹发射阵地等目标</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>美称打击伊朗导弹阵地，伊方击落美军无人机并驱离战机，伊美紧张局势持续。</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEN0Hnnoa864PhbKwGZKGj260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>[视频]以总理称将对黎真主党进行决定性打击 黎总统要求以色列全面撤军</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>以总理称将对黎真主党决定性打击，黎总统要求以方全面撤军。</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEwHh7bXHJG4IZMYcwuuln260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>俄称系统打击乌首都军事目标；加沙停火后超900人死亡；刚果(金)埃博拉疫情严峻。</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/26/VIDEHy5VrnfKytMTxXo7KiZV260526.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Iran condemns US strikes as 'gross violation' of ceasefire</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>伊朗谴责美国在谈判期间发动打击，称其严重违反停火。</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g44yl7q70o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Russia threatens more Kyiv strikes and tells foreign nationals to leave</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>俄罗斯威胁对基辅发动更多打击，并敦促外国公民离开。</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1e22n55zn4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Almost 1,000 migrants cross Channel over bank holiday</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>英国银行假日期间，近千名移民乘小船穿越英吉利海峡抵达英国。</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy422k3z83vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Prospects fade for imminent end to Iran war as attacks restart</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>以色列将加强打击黎巴嫩真主党，美国袭击伊朗船只，战争谈判前景黯淡。</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/nx-s1-5834840/iran-lebanon-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>U.S. strikes Iran. And, immigration courts use new tactic to speed up deportations</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>美国对伊朗发动新攻击，同时司法部在移民法庭加速遣返程序。</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/g-s1-124277/up-first-newsletter-iran-war-russia-ukraine-immigration-courts-trump-health</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Ecuadorian survivors of suspected drone strike seek answers and restitution</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>厄瓜多尔渔民疑似遭无人机袭击，寻求赔偿，被移交萨尔瓦多未受指控。</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/nx-s1-5828756/ecuadorian-survivors-of-suspected-drone-strike-seek-answers-and-restitution</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Four killed as school minibus collides with train in Belgium</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>比利时一辆校车与火车相撞，造成两名学生、一名护工和司机共四人死亡。</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c70vvd17rg7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Why temperature records are being not only broken but smashed</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>热穹顶与气候变化叠加，导致西欧极端高温频现，温度纪录屡被大幅打破。</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62rrj66p3eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>UK's hottest May day record broken for second day in a row</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>英国连续第二天打破五月高温纪录，伦敦邱园气温达35.1摄氏度。</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypp7ljvpvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Sentences of boys spared custody over rape referred to Court of Appeal</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>英国两名男孩因强奸女孩未被判监禁，首相将案件提交上诉法院重审。</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y779yeq0eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Why the French Open is named after Roland Garros, who didn't play tennis</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>法网以一战飞行员罗兰·加洛斯命名，他非网球选手，因革新空战而闻名。</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/nx-s1-5834922/roland-garros-french-open-namesake</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-27
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F741"/>
+  <dimension ref="A1:F770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24149,6 +24149,934 @@
         </is>
       </c>
     </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>政治, 经济, 军事</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260527 19:00</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道传统产业升级、高层调研、外交访问、军队管理、法治建设等综合新闻。</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEIVdT84KqZ0qbTqVbsYJv260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际对哈萨克斯坦进行正式友好访问</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>赵乐际访问哈萨克斯坦，深化中哈永久全面战略伙伴关系，推进共建“一带一路”。</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDElUazcn5inORO54JFdxY9260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】合力开创法治中国建设新局面</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>国新办介绍“十五五”法治建设规划，强调全面依法治国，护航发展。</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEiuA2L1mlAK1XbkPRJVXa260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行记者见面会，四位移民管理代表分享坚守国门、服务开放的奋斗故事。</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDE8hE7O2uSnHhVC0ArMqGQ260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>[视频]日本民众集会反对设立“国家情报会议”</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>日本国会通过“国家情报会议”法案，民众集会反对，批评政府加速战争准备。</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEmH6CZhFUz8hrKEmJGJMv260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Burnham accuses Blair of ignoring inequality as he hits back at ex-PM</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>工党市长回击前首相布莱尔，指责其忽视不平等。</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ckgp4llnn12o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>政治, 军事, 国际</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Trump gathers Cabinet as he looks to seal deal to end war</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>特朗普召集内阁会议，寻求敲定结束与伊朗战争的协议，但已招致强烈批评。</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/27/nx-s1-5836202/trump-cabinet-meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】传统产业的“蝶变”跃迁</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>习近平总书记强调以科技创新推动传统产业转型升级，实现高质量发展。</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDE8ANG6tSTpha8G8WFK54G260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>[视频]李强在浙江舟山宁波调研</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>李强在浙江调研，强调完善大宗商品储备体系，提升产业链供应链韧性。</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEFfjLu4xHl6uTkuXOjZsJ260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>[视频]前4个月规模以上工业企业利润总额同比增长18.2%</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>1-4月全国规模以上工业企业利润同比增长18.2%，高技术制造业增长44.8%。</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEdCelE8e7dBNQIkHDTyKb260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>前4月我国对外投资增3.9%；发电装机容量增14.2%；水利部发布河流泥沙公报；成功发射通信技术试验卫星。</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDErZJ9td8FB2F945DdUVzm260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>[视频]中央军委印发《关于加强军队高级干部教育管理监督的若干措施》</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>中央军委印发措施，加强军队高级干部教育管理监督，推进全面从严治党治军。</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEgc4oJLt8wZpFKcM4YKS5260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】促发展惠民生 推动学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>新疆阿克苏和江苏苏州通过学习教育，聚焦民生需求，解决群众和企业实际问题。</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDExzZaRQNZCZmSfcWoLELR260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Resident doctors in England to strike for 16th time over pay</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>英国住院医生因薪资问题宣布6月15日起罢工四天。</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8xw2vvlxeko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>[视频]联合国安理会“维护联合国宪章宗旨和原则，加强以联合国为核心的国际体系”高级别会议举行</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>联合国安理会围绕维护宪章举行高级别会议，中方呼吁团结维护联合国，推动构建人类命运共同体。</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEG3YfUxjUqusspgJhNltm260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>[视频]伊朗强烈谴责美国破坏停火 美称双方仍在就协议进行磋商</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>伊朗谴责美国破坏停火，美伊仍在磋商协议；美称霍尔木兹海峡须保持开放。</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEOeFwDKPWtHrsX83aDrUz260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>国际, 军事, 民生</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>以军向黎巴嫩纵深行动，造成31死；欧洲多国遭遇破纪录高温，交通受阻。</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/27/VIDEpOX8S0YmM6Ga99Eb2CGi260527.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Ebola-hit DR Congo faces 'catastrophic collision' of disease and conflict, WHO warns</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>世卫组织警告：埃博拉疫情与冲突在刚果（金）形成“灾难性碰撞”。</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdxpdex062yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Israel orders evacuation of Lebanese city as conflict with Hezbollah escalates</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>以色列下令撤离黎巴嫩城市提尔，称将强力打击真主党。</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj3pgrpmlklo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Five people found alive after week trapped in flooded Laos cave</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>老挝洪水洞穴被困一周，五人生还，仍有两人失踪。</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crkpvxrxgp6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Israeli strike in Gaza City kills new head of Hamas's military wing</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>以色列空袭加沙，哈马斯新军事首领及家人身亡。</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjwppj1yn7go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Almost 500,000 Russian soldiers killed in Ukraine war, GCHQ says</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>GCHQ称近50万俄军在乌克兰战争中死亡。</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g44gprnnvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Greetings from Cape Verde, where the sounds of samba, jazz and morna fill the air</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>西非岛国佛得角音乐融入日常生活，四月举办两场音乐节，获评2028年非洲文化之都。</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/27/g-s1-124325/cape-verde-music-morna-african-capital-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Palestinians use recycling as Israel's restrictions trigger a trash crisis</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>以色列限制导致西岸垃圾危机，两名巴勒斯坦企业家尝试通过回收改变现状。</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/27/g-s1-121673/israel-palestinians-trash-west-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>An exceptionally early heat wave shatters records and brings deaths in Europe</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>欧洲遭遇异常早热浪，伦敦连续两日35℃破纪录，专家称极端天气更频繁。</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/g-s1-124360/europe-heat-wave-deaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Woman caught after 30 years on the run is jailed for armed robberies</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>逃亡30年的女劫匪在柏林被捕，被判入狱。</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21dr3lekpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Family of mum, 30, shot dead outside Sheffield bar pay tribute to 'beautiful soul'</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>30岁女子在谢菲尔德酒吧外遭枪杀，家人称其“美丽灵魂”。</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0q2yle5e0yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Safety warning after nine water-related deaths during heatwave</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>热浪期间九人因水上活动死亡，慈善机构呼吁谨慎。</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8plymvm47o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Why the French Open is named after Roland Garros, who didn't play tennis</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>法网以飞行员罗兰·加洛斯命名，他革新了空战技术，1928年球场以他名字纪念。</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/26/nx-s1-5834922/roland-garros-french-open-namesake</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-28
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F770"/>
+  <dimension ref="A1:F802"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25077,6 +25077,1030 @@
         </is>
       </c>
     </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>政治, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260528 19:00</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>今日新闻联播报道中奥、中苏建交贺电，中美青年复信，城市更新规划，及多领域进展。</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEZSkNfIITCzj5FM1NfG8s260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>[视频]习近平同奥地利总统就中奥建交55周年互致贺电</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>习近平与奥地利总统互致贺电，庆祝中奥建交55周年，强调深化友好战略伙伴关系。</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEjpw0NlD99F8bx5zHoCBA260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>[视频]习近平同苏里南总统就中苏建交50周年互致贺电</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>习近平与苏里南总统互致贺电，庆祝中苏建交50周年，共启战略合作伙伴关系新篇章。</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDE1hJmdG6DCEsTh9qbL1Lv260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>[视频]习近平复信参加“共航蔚蓝：中美青年友谊行”活动的两国学生</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>习近平复信中美学生，肯定“5年5万”倡议成果，鼓励青年成为友谊使者。</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEZ2091V6ek890rAbOyMOo260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见英国跨党派议员代表团</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>王沪宁会见英国跨党派议员代表团，强调加强政党交往与互利合作。</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEtGF9QEPGBfJzZNJnTwoI260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>In Colombia, a flashy lawyer touts his tough-on-crime approach in presidential race</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>哥伦比亚总统大选中，一名高调刑事律师以强硬打击犯罪为竞选口号，展示财富与音乐视频。</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/nx-s1-5830412/in-colombia-a-flashy-lawyer-touts-his-tough-on-crime-approach-in-presidential-race</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>[视频]前4个月全国网上商品和服务零售额增长6.6%</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>前4月全国网上零售额同比增长6.6%，旅游餐饮业网上销售实现两位数增长。</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEwpI0o5qDFdgalyPk1BVr260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>[视频]前4个月我国交通运输经济运行平稳</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>1-4月我国货运量、港口吞吐量及跨区域人员流动量均实现同比增长。</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEENokpdx9TV0z8YWb4thU260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>[视频]各地一批重大工程扎实推进</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>平陆运河主体工程完成，渝万高铁、崇启大桥等重大工程扎实推进。</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEohxHnPzziPS35vKqDSZP260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>国新办举行记者见面会，5位民营企业家分享奋斗历程与担当。</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEWc0AR35Rea1GkFT12OHv260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十一号、神舟二十三号航天员乘组进行在轨交接 东风着陆场完成最后一次全系统综合演练</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>神舟二十一号与二十三号乘组完成在轨交接，东风着陆场准备就绪迎接返回。</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDE62R4hX8EGCLl1o12F9j6260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>[视频]截至4月底我国5G基站总数超500万个</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>截至4月底我国5G基站总数超500万个，移动互联网流量同比增长18.5%。</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEQ8S96aYEEoeTfnwSmLYS260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《城市更新“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>国务院印发《城市更新“十五五”规划》，部署6方面重点任务及14项工程。</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEVCvDkGjISBkTo1O6hi87260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>[视频]中央组织部从代中央管理党费中划拨7200万元用于支持安徽、广西等6省区市抗灾救灾工作</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>中央组织部划拨7200万元党费，支持安徽、广西等6省区市抗灾救灾。</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEmgXEk2jh4IN259cMhdtu260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国大规模小麦机收全面展开</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>全国大规模小麦机收全面展开，主产区河南、安徽进入集中收获期。</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEKCc0CaORdGNHkFOx0xUK260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>'I've applied for more than 400 roles' - how young people are facing the job shortage</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>BBC报道称年轻人面临就业短缺，有求职者已申请超400个职位仍难找到工作。</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czx2qll4rlyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Prostate cancer screening only for "a few thousand" high risk men</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>英国顾问建议仅对携带高危基因且有癌症家族史的少数男性开展前列腺癌筛查。</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn0pvxe5jgzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Australian woman charged over travel to Syria to join Islamic State</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>一名澳大利亚女性因前往叙利亚加入伊斯兰国被起诉，此前她已从黎巴嫩返回澳洲八个月。</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/g-s1-124669/australian-woman-charged-over-travel-to-syria-to-join-islamic-state</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>国际, 政治, 科技</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>U.S. strikes Iran again. And, DOJ charges Google staffer over Polymarket trades</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>美国再次对伊朗发动打击，同时司法部指控谷歌员工利用内幕信息进行Polymarket交易。</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/g-s1-124621/up-first-newsletter-iran-lebanon-israel-us-war-ebola-congo-food-insecurity-google-polymarket</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>More than 500 people have died in Bangladesh measles outbreak</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>孟加拉国麻疹疫情已致超500人死亡，多为儿童，当局正紧急为更多儿童接种疫苗。</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/nx-s1-5836674/more-than-500-people-have-died-in-bangladesh-measles-outbreak</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>[视频]国务院成立山西长治山西通洲集团留神峪煤业有限公司“5·22”特别重大瓦斯爆炸事故调查组</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>国务院成立山西长治瓦斯爆炸事故调查组，启动调查工作。</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDElZgWCUuNmZkUC4uha1tf260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>社会, 科技, 经济</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>全国安全生产月启动、智能产业博览会开幕、人工智能及海洋生物医药政策发布。</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEac4M6CrNCrN799kkw3mK260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Two more boys die in latest heatwave water deaths</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>英国热浪致两名男孩溺水身亡，一具遗体在肯特郡池塘找到，另一人在牛津泰晤士河遇难。</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn0p7j3lwepo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Orthodox Jewish women in Israel may now take a rabbinic exam, like men</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>以色列东正教犹太女性获准参加拉比考试，但通过后仍不能成为拉比。</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/g-s1-124466/israel-orthodox-jewish-women-exam-religion</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>[视频]伊朗南部港口传出爆炸声 美媒称美军在伊朗实施空袭</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>[视频]伊朗南部港口传出爆炸声 美媒称美军在伊朗实施空袭</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDEyZ1c8HVFfJ46Vy31pDGy260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/28/VIDENNMdgRqWe7ZGhpZnB9Cn260528.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Gaza City hospitals say several killed in strike, as Israel targets Hamas leaders</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gaza City hospitals say several killed in strike, </t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn9p40en4ngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Are US and Iran close to peace or sliding back to war?</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are US and Iran close to peace or sliding back to </t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cze29764067o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Iran says it targeted American base after fresh US strikes</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Iran says it targeted American base after fresh US</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c98r2qy5809o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Israel hits Lebanese capital in 'targeted strike'</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Israel hits Lebanese capital in 'targeted strike'</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgqpjwdv7xeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Villas, cars and cash: Italy seizes dead Mafia mobster's millions</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Villas, cars and cash: Italy seizes dead Mafia mob</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ceqpd4gqgveo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>未分类</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Opportunities shrinking for too many young people, says major report on 'lost generation'</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Opportunities shrinking for too many young people,</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy026x9jpd0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-29
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F802"/>
+  <dimension ref="A1:F829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26101,6 +26101,870 @@
         </is>
       </c>
     </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260529 19:00</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>老挝领导人将访华；服务业高质量发展；神舟飞船返航；前四月物流增长等综合新闻。</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEun3qOWrQ5euwT2ML31NF260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 老挝人革党中央总书记、国家主席通伦将访华</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>老挝人革党中央总书记、国家主席通伦将于6月2日至6日对中国进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEWgMFvIsmrfTsU32gbi2k260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】广东奋力在推进中国式现代化建设中走在前列 在中国式现代化进程中展现贵州新风采</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>广东和贵州发布“十五五”规划，重点聚焦高质量发展、粤港澳大湾区建设及科技创新。</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEhQWMv2UpLGzijnzc1n7W260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Former US attorney general Pam Bondi testifies in congressional Epstein probe</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>前美司法部长邦迪就爱泼斯坦案在国会作证。</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czj2ldllgwgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Trump holding meeting to make 'final determination' on Iran deal</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>特朗普将与顾问开会，就伊朗协议做最终决定。</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0r2d40r91qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】扩能提质 开创服务业高质量发展新局面</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>服务业成国民经济第一大产业，一季度增加值占GDP比重61.7%，强调高质量发展。</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEEB1i5v5qA1JXJd0UJCKs260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>[视频]今年前四个月我国物流需求保持韧性增长</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>1-4月全国物流总额121.7万亿元同比增长5.5%，高端制造业物流需求增长超10%。</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEAP9tvTzcMdVA70cXFjat260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>[视频]第10届中国—南亚博览会将于6月11日至16日在昆明举行</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>第10届中国—南亚博览会将于6月11日在昆明举行，首次设立服务贸易馆。</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDElrPZhcs7jaUlrc0UPKDZ260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十二号载人飞船撤离空间站组合体 神舟二十一号航天员乘组踏上回家之旅</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>神舟二十二号飞船与空间站分离，航天员张陆等三人踏上返回地球之旅。</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEa6ijGrrmaRBxa6vi91kj260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>[视频]2025年中央企业基础研究投入首破千亿元</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>2025年央企基础研究投入首破千亿元，达1024亿元，将成为基础研究重要生力军。</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEfUNmAQPg6zCRHgOAJiq9260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>科技, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>联播快讯：发布最美科技工作者、电力交易电量增长、农发行1500亿助夏粮收购、幼儿园集中用餐新规发布。</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEuT0NBY5ZyDdoOeHXWDUO260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Exploding rocket casts doubts over Nasa's Moon plans</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>蓝色起源火箭爆炸，给NASA登月计划蒙上阴影。</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2q0g07kgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>[视频]俄外交部表示日本允许美在日部署中导系统威胁亚太稳定安全</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>俄外交部称日本允许美部署中导系统威胁亚太安全，谴责日本“再军事化”。</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEqzfY3LH2vGLaYnJMsbwu260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Nato condemns Russian 'recklessness' after drone hits Romanian residential block</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>北约谴责俄罗斯“鲁莽”，因其无人机击中罗马尼亚居民楼致两人受伤。</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c93x4nxlkjeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Asia defense summit opens amid doubts over U.S. priorities</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>亚洲防务峰会开幕，聚焦美国优先政策及中东、乌克兰局势。</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/29/g-s1-124788/asia-defense-summit-opens-amid-doubts-over-u-s-priorities</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Russian drone launched against Ukraine crashes in Romania, injuring 2</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>俄罗斯无人机袭击乌克兰时坠入罗马尼亚公寓楼，致两人受伤。</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/29/g-s1-124773/russian-drone-romania</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>[视频]2025年全国城市声环境质量总体良好</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>2025年全国城市声环境良好，昼间达标率93.3%，已建成3272个宁静小区。</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDE5ML3UAKoghSfsal7dz8k260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】700公里抢收路背后的夏收保障网</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>“00后”农机手跨省700公里抢收夏粮，多部门提供绿色通道与后勤保障。</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEJ4rwURlE22uS3hg0qknn260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>[视频]“全球治理之友小组”会议呼吁维护联合国权威 完善全球治理</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>60余国代表在联合国呼吁维护联合国权威，改革完善全球治理体系。</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDEtiLqjHVb7b6BfpTveKoU260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>美伊被曝就备忘录达成一致遭伊朗否认；以称将扩大对加沙控制范围至70%，中东战事拖累增长。</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/29/VIDETxMy8UbkYrjr7oUDzkCG260529.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Israel, Lebanon officials to meet. And, judge won't block Trump's mail-in voting order</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>以色列与黎巴嫩官员将会面；法官未阻止特朗普邮寄投票令。</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/29/g-s1-124776/up-first-newsletter-israel-lebanon-iran-war-e-jean-carroll-trump-cbs-60-minutes-voting</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>WHO chief lands in Congo to address rare Ebola outbreak amid distrust and insecurity</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>世卫组织总干事抵达刚果（金），应对罕见埃博拉疫情。</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/29/nx-s1-5838635/who-chief-visits-congo-ebola-outbreak</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>'Poison seller' who sold toxic chemicals online to people across world admits aiding suicides</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>加拿大男子肯尼斯·劳承认通过网络出售毒药帮助自杀，面临多项指控。</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c70vg7glglyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Eight students arrested in Kenya after suspected deadly school arson attack</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>肯尼亚一学校宿舍遭纵火，致16名学生死亡，8名学生被捕。</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx21r3138m9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Child among three dead in tower block fall</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>伦敦象堡公寓楼三人坠亡，包括一名儿童。</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1k21077k7lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>'Controversial' North Korean invasion setting for next Call of Duty game</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>《使命召唤》新作以争议性的朝鲜入侵为背景，强调军事真实性。</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9q391y5088o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Arsenal's glory weekend beckons, and soccer fans all over the world are watching</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>阿森纳足球俱乐部举行胜利巡游，全球球迷关注能否再夺一冠。</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/28/nx-s1-5836382/arsenal-premier-league-champions-league-soccer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-30
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F829"/>
+  <dimension ref="A1:F863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26965,6 +26965,1094 @@
         </is>
       </c>
     </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260530 19:00</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>习近平与埃及总统互致建交贺电；神舟二十一号返回成功；科技工作者日多场活动；湖南党员先锋队抢险。</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEdSWNPa3SftEVmyYtELaA260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>[视频]习近平同埃及总统就中埃建交70周年互致贺电 李强同埃及总理互致贺电</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>习近平同埃及总统塞西互致贺电，庆祝中埃建交70周年，强调构建命运共同体。</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEx54CNFGRi2okdoq2AQxl260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>[视频]湖北省委主要负责同志职务调整</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>中共中央决定：关志鸥任湖北省委书记，王忠林不再担任，另有任用。</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEHzxrU2IQrQbXozK2LKr4260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Spain's Sánchez digs in after eight years as PM as wave of scandals threatens survival</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>西班牙首相桑切斯因腐败调查面临执政危机。</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1w21gn340xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Ex-US attorney general defends Epstein files handling in congressional probe</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>美前司法部长就爱泼斯坦文件处理出席国会听证。</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czj2ldllgwgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Palace was handed Andrew's controversial envoy emails six years ago</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>白金汉宫六年前已收到安德鲁王子争议邮件。</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy02j5pl98no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>U.S. Embassy in India launches Trump-themed rickshaws to mark America's 250th birthday</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>美国驻印度使馆推出特朗普主题三轮车庆祝美国250岁生日。</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/30/nx-s1-5833149/u-s-embassy-in-india-launches-trump-themed-rickshaws-to-mark-americas-250th-birthday</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Myanmar's Min Aung Hlaing takes first foreign tour as leader, with visit to India</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>缅甸领导人敏昂莱就任后首次外访印度，旨在巩固地区政治地位，同时继续残酷内战。</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/30/nx-s1-5838637/myanmar-hlaing-india-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>经济, 文体</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Tickets for festivals are getting more expensive - we compared them</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>英国多个音乐节票价大幅上涨，包括雷丁、格拉斯顿伯里等。</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj9pgmw3yz2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】矢志创新勇攀高峰 加快建设科技强国</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>全国科技工作者日强调科技创新，广大科技工作者矢志创新，加快建设科技强国。</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEhaN2Pcj6KnOZCj1kzOxf260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十一号飞行乘组返回任务圆满成功</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>神舟二十一号乘组返回任务圆满成功，三名航天员平安抵京，在轨驻留210天创纪录。</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEsliE9Etqr47Q4Ky6tlU9260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>[视频]全国科技工作者日 多场活动弘扬科学家精神</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>全国科技工作者日举办表彰、展览及科普活动，弘扬科学家精神。</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEdK6hcgu7iBTFDq2XJI2j260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>US, UK and Australia to develop underwater drone technology</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>美英澳在AUKUS框架下联合研发水下无人机技术。</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y8wjvd1ypo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Millions of breast cancer patients could safely avoid chemotherapy, study suggests</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>新DNA测试或帮助数百万乳腺癌患者避免不必要的化疗。</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2325j0xk1vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>[视频]俄总统称俄乌冲突临近收尾 乌称前线战事激烈</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>普京称俄乌冲突临近收尾；乌方称战事激烈。罗马尼亚指俄无人机坠毁，俄方否认。</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDExnUXdPf6cBh0atLh78tW260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>军事, 科技</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Ukraine using AI drones to strike vital convoys supplying Russian troops</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>乌克兰使用AI无人机攻击俄军补给车队。</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdjp0n7rn41o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>[视频]李强对安全生产工作作出重要批示强调 坚决贯彻落实习近平总书记关于安全生产的重要指示精神 切实维护人民群众生命财产安全和社会大局稳定</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>李强对安全生产作批示，要求坚决遏制重特大事故，加强防汛救灾和重点行业监管。</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEvVN9qUjG8kouX9BJydLE260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】党员先锋队抢通群众出行路</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>武警党员先锋队在湖南暴雨中抢通道路，连续奋战打通13个村庄出行路。</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEhE8b6dyUIH8DFTZRjaHd260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>全国“三下乡”活动在甘肃举行；前四月软件业收入增长10.9%；七部门印发文旅与工业融合发展通知；财政部在港发行60亿元绿色债券。</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDETvKV9hsxhCdbOiXAooQz260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Arrive three hours before flight home, airline boss tells UK holidaymakers</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>维兹航空CEO建议英国游客提前三小时到机场，带充电宝和水。</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8xw2kjlrlxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>How one borough is bucking the UK's youth unemployment trend</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>英国一地区通过早期干预成功降低青少年失业率。</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd6p9yyg64vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>[视频]日本民众集会反对高市政府危险动向</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>日本民众在东京集会，反对高市早苗政府扩军、修宪等危险动向。</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEqfj7cKDpr1NlQANGdVYb260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>伊朗与阿曼讨论霍尔木兹海峡问题；欧亚经济联盟四国敦促亚美尼亚决定去留；日本外汇干预规模创新高。</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDE9e0xtzu67tzn9Qz0WZZo260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>No deal announced after Trump meeting to make 'final determination' on Iran</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>特朗普与顾问会面，拟就伊朗问题做出“最终决定”。</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0r2d40r91qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>US not 'turning back' on Asia allies, but expects them to boost defence, says Hegseth</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>美防长称不会背弃亚洲盟友，但希望盟友加强国防。</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5ye34k7yejo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Four more men freed from flooded Laos cave after 10 days</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>老挝洪水洞穴中4名被困者获救，仍有2人失踪。</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4pn4ex0ymo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Carcass of Timmy the humpback whale brought to shore in Denmark</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>名为“蒂米”的座头鲸尸体在丹麦海岸被冲上岸。</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/30/nx-s1-5839921/timmy-humpback-whale-autopsy</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>[视频]【暖心一瞬】合力救援 托起生命希望</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>江西赣州和江苏盐城发生合力救援事件，群众挺身而出挽救落水者和车祸伤者。</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/30/VIDEDAO5FpjR63jPdygnYl6K260530.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Ghana's parliament passes anti-LGBTQ+ bill</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>加纳议会通过反同性恋法案，同性行为将面临监禁。</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yedendprko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>'Gifts' from a lover and 'botched' cocaine raids: Police inquiry grips South Africa</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>南非调查委员会听证会涉及毒品突袭和贿赂指控。</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce9p5e1jg72o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Girl, 15, dies after swimming at beach</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>15岁女孩在海滩游泳时不幸溺水身亡。</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62rjmgmk55o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Colombia's untapped wonder: The Mavecure Mountains</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>哥伦比亚马维库雷山脉从亚马逊丛林中崛起，曾是冲突禁区，现吸引冒险者探索稀有野生动物与圣地。</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/30/nx-s1-5787938/colombias-untapped-wonder-the-mavecure-mountains</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>'Men written by women': How ice hockey romances like Off Campus became TV's hottest new genre</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>冰球题材浪漫小说改编剧集在亚马逊获热播。</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypz87rqy1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Liverpool sack head coach Arne Slot year after Premier League title win</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>利物浦解雇主教练斯洛特，伊劳拉为主要继任者。</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cglp7kelrljo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-05-31
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F863"/>
+  <dimension ref="A1:F892"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28053,6 +28053,934 @@
         </is>
       </c>
     </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260531 19:00</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>习近平回信勉励红领巾讲解员；《习近平法治文选》英文版出版；赵乐际访俄；制造业稳定运行；AI拉动外贸增长。</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEWsdAMINqwQHlctnySuIV260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>[视频]习近平回信勉励中共一大纪念馆、南湖革命纪念馆少先队红领巾讲解员 传承红色基因增长知识本领 在新征程上跑好历史接力赛 祝全国小朋友们“六一”国际儿童节快乐</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>习近平回信勉励中共一大纪念馆、南湖革命纪念馆红领巾讲解员，传承红色基因，祝全国儿童节日快乐。</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDE2mreeoryDrR0coJ9VoKQ260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：做党和人民的红孩子，在新征程上跑好历史接力赛</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>央视快评：做党和人民的红孩子，在新征程上跑好历史接力赛。</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEYRmNUcmXtomkXntOLY3R260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>[视频]《习近平法治文选》第一卷英文版出版发行</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>《习近平法治文选》第一卷英文版出版发行，面向海内外推广习近平法治思想。</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEXzODZabx83fnwRo0RBvh260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际对俄罗斯进行正式友好访问 并出席中俄议会合作委员会第十一次会议</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>赵乐际访俄并出席中俄议会合作委员会会议，推动两国关系高质量发展。</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEwuJaifESBnR4hvCBFs2o260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Colombia votes in presidential election that could redefine relations with US</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>哥伦比亚总统大选投票，或重新定义与美国的关系。</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2027g423glo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Sturgeon tells BBC: I'm serving a sentence for crime I didn't commit</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>苏格兰前首席大臣斯特金辩称未犯罪，谈及SNP丑闻落泪。</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c2027k1ev3zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Watch: Key moments from Nicola Sturgeon's interview with Laura Kuenssberg</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>斯特金首次受访，回应丈夫挪用SNP公款案。</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c70vl59vd9vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Streeting suggests NI cut and North Sea drilling</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>斯特里廷暗示削减北爱尔兰事务经费并推进北海钻探，与斯塔默政府切割。</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy42z03r18xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Nicola Sturgeon speaks to the BBC</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>前苏格兰首席大臣斯特金接受BBC独家专访。</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sounds/play/p0np7qln?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】活力迸发 民营经济走向更加广阔的舞台</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>政策密集落地，民营企业创新动能增强，在高质量发展中发挥重要作用。</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEhWuG1ch1Xn2YW7yqM8sD260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>[视频]制造业稳定运行 新动能加速扩张</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>5月制造业采购经理指数为50%，高技术制造业和装备制造业加速扩张。</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEQ3VfMczEEKs7lmmWEWYZ260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>[视频]人工智能相关产品拉动外贸增长</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>人工智能相关产品和服务加快出口，前4月集成电路出口额同比增长78.3%。</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEzQSBoaGs7TS7AEPn75fF260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称对霍尔木兹海峡航运实施全面管理 美军称击中一艘试图驶往伊朗港口的货船</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>伊朗宣布全面管控霍尔木兹海峡航运，击落美军无人机；美方击中驶往伊朗货船。</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEHiUb9tSQV6cezaKb4gEo260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Israel seizes castle in Lebanon as it expands ground offensive</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>以色列在黎巴嫩夺取博福特城堡，扩大地面攻势。</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdep04kzz5wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Israel seizes medieval castle as it expands major offensive in southern Lebanon</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>以色列占领黎巴嫩12世纪城堡，或在黎南部扩大长期军事存在。</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/05/31/g-s1-125056/israel-seizes-medieval-beaufort-castle-southern-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>[视频]绿化带美出新颜值 公园城市尽显新风貌</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>绿化带美化升级，展现公园城市新风貌。</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDE9W9bVd6r9S4UBpO0J6bO260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>6月起实施102项国家标准；儿童用药批准数量创新高；启动未成年人救助保护机构专项行动。</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDE6LjEQRcBgBomC4H7oVOp260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Cuba’s blackouts leave high-rise residents with constant uncertainty</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>古巴断电致高层居民生活陷入持续不确定。</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c809nj57drxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Why renaming my health condition could help other women</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>全球超1.7亿女性患多囊卵巢综合征，罗谢尔呼吁改名以消除污名化。</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd9p50j3ljko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>黎总理谴责以色列在黎南部实施焦土政策；世卫呼吁支持埃博拉疫区；日本乙烯工厂开工率创新低。</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDEgD528OMTeAlLn48FXTHP260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Hundreds arrested and dozens of police injured after Champions League riots in France</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>法国欧冠骚乱后，近800人被捕，219人受伤含57名警察。</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0r2ejg1w9xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Japan defence minister denies militarism and criticises China's 'huge arsenal'</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>日本防相否认军国主义，批评中国拥有庞大武器库。</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8p4ejy8ppo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Ebola spread in DR Congo 'deeply alarming', MSF warns</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>无国界医生警告刚果（金）埃博拉疫情传播令人深感忧虑。</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c99ldxykz4zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>South Africa made to look like fools after World Cup visa issues, says minister</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>南非部长批评世界杯签证问题让国家蒙羞。</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c86dxvql3qno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>[视频]【新闻特写】跨越26年的绿色约定</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>殷玉珍与美国人赛·考斯基因治沙捐助结缘，26年后重续绿色约定。</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/05/31/VIDECkoRSJQOc8cTst749l0X260531.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Laos cave survivors help with plan to find last two missing men</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>老挝洞穴救援：五人已获救，继续搜寻最后两名失踪者。</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8094jdpzv3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>社会, 军事</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Nigerian retired general abducted with his wife in the north-west</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>尼日利亚退休将军与妻子在西北部被绑架。</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz02zgkgn08o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Jeremy Clarkson's choir wins Britain's Got Talent</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>杰里米·克拉克森的农民合唱团赢得英国达人秀冠军。</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g9j4282qdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-01
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F892"/>
+  <dimension ref="A1:F918"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28981,6 +28981,838 @@
         </is>
       </c>
     </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260601 19:00</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道习近平总书记重要文章、韩正会见巴西外长、少先队员数据、儿童友好建设、制造业转型等综合新闻。</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEcoJC2O09w7SfavgBv5FM260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>[视频]《求是》杂志发表习近平总书记重要文章《前瞻布局和发展未来产业》</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>《求是》杂志发表习近平总书记文章，强调前瞻布局和发展未来产业，加强科技创新与统筹谋划。</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEVfdberd1ogtuBx9rpYFO260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】传承红色基因增长知识本领 在新征程上跑好历史接力赛</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>习近平总书记给少先队讲解员回信，勉励传承红色基因，在新征程上跑好历史接力赛。</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEpoN9utmwQiMplWUfQ0gD260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见巴西外长</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>国家副主席韩正会见巴西外长，强调推进中巴命运共同体建设，深化高水平战略协作。</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEJRhOI0SkYJ4Y0lhTZE6L260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】谱写中原大地推进中国式现代化新篇章 重庆打造新时代西部大开发重要战略支点</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>河南与重庆发布“十五五”规划纲要，聚焦创新驱动、乡村振兴与西部大开发战略支点建设。</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEWPpxMdIVeoaaqYegZN8L260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Hungarian PM threatens to oust Orbán-era president</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>匈牙利总统拒绝总理要求，引发宪法冲突。</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3w2vdd6jj3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Chris Mason: Decision to appoint Mandelson continues to inflict damage</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>斯塔默任命曼德尔森使节职务持续招致批评。</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzr6pn0nko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>[视频]今年以来我国制造业高端化智能化转型加速</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>今年1至4月制造业销售收入同比增长6.9%，高技术制造业与人工智能产业增长显著。</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDE3xVtCO4PAIJvHEDCjGOj260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】科技赋能夏收夏种 助力粮食稳产丰收</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>各地推广智慧农机助力夏收夏种，安徽推广新型收割机降低损失率，新疆用AI机器人套种玉米实现增产增收。</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDECIw2OgsFAMEI9EIpkGkq260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>AI giant Anthropic says it plans to list on US stock market</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>AI公司Anthropic计划今年在美国股市上市。</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0k203kzp10o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>[视频]美称打击霍尔木兹海峡附近伊朗军事目标 伊称打击美空军基地以回应侵略</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>美打击霍尔木兹海峡附近伊朗目标，伊回击美军基地，双方就核问题协议谈判立场强硬。</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEZGHdUT1riATjl5yvtO16260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>U.S. strikes Iranian military sites. And, Trump's $1.8 billion fund faces scrutiny</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>美国空袭伊朗军事基地，特朗普基金遭审查。</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/01/g-s1-125147/up-first-newsletter-iran-us-anti-weaponization-fund-graham-platner-newsmakers</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>[视频]我国推进儿童友好建设城乡全覆盖</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>我国将推动儿童友好建设从城市向农村延伸，实现城乡全域覆盖。</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEMpslZcmDupKX8mSBJTPI260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>[视频]我国全面进入汛期</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>我国全面进入汛期，南方主汛期到来，部分河流可能超警，水利部门加强预报和调度确保度汛安全。</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEiQ9inafjcLdRRZy3XRtF260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>医保目录调整启动，最高检发布未检白皮书，《供水条例》和网络餐饮新规今起施行。</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEeISZSBklhSMrKuRLVxtq260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>民生, 军事</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>After Russian missile strike, owners of Ukrainian coffee shop pledge to rebuild</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>基辅咖啡店遭俄导弹袭击后，店主迅速恢复营业并计划重建。</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/01/nx-s1-5838859/after-russian-missile-strike-owners-of-ukrainian-coffee-shop-pledge-to-rebuild</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>以升级在黎军事行动遭多方批评；扎波罗热核电站遭袭，国际原子能机构呼吁停止；卢卡申科警告后果严重。</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEuJEdrBX3idJgGrScIzEb260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Iran warns Israeli attacks in Lebanon threaten ceasefire with US</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>伊朗警告以色列在黎巴嫩的袭击可能危及与美国达成的停火协议。</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c202rxp1z15o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Bowen: Trump needs this war to end but Iran is not backing down</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>分析称特朗普需结束战争，但伊朗不妥协，白宫面临民意和盟友压力，正推动协议。</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cedp3lee059o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>国际, 科技</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Three Ebola vaccines in development amid growing outbreak fears</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>埃博拉疫情担忧加剧，三家机构正研发新疫苗。</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn8pw93929wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Confirmed Ebola cases in Congo reach 282 as survivors describe their recoveries</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>刚果埃博拉确诊病例达282例，无批准药或疫苗。</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/01/g-s1-125143/ebola-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>国际, 政治, 经济</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Funds for Trump's Board of Peace aren't in World Bank account. So where are they?</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>特朗普加沙和平基金未存入世行账户，去向不明。</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/01/nx-s1-5837603/funds-for-trumps-board-of-peace-arent-in-world-bank-account-so-where-are-they</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>[视频]全国共有少先队员1.12亿名</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>全国少工委发布数据，截至2025年底全国共有少先队员1.12亿名。</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDEbVutoJONhpu8eKapQpeI260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>[视频]全国人大常委会启动职业教育法执法检查</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>全国人大常委会启动职业教育法执法检查，6月至9月赴7省实地检查，重点检查产教融合等7方面内容。</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/01/VIDER4Ru8NXCfoyP5KWyOQ3g260601.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Weapons-obsessed killer jailed for student's murder</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>痴迷武器的凶手因谋杀大学生被判入狱。</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1d2w411rgro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Violent clashes give way to peaceful PSG parade after Champions League win</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>巴黎圣日耳曼欧冠胜利游行由暴力转为和平庆祝，数百人被拘。</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/01/nx-s1-5842841/peaceful-psg-parade</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-02
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F918"/>
+  <dimension ref="A1:F945"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29813,6 +29813,870 @@
         </is>
       </c>
     </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260602 19:00</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平社区治理理念、中老纪录片启播、国务院农业农村规划等多项国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEN2kbyXpowVQvD7GDyjl5260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁与欧美同学会（中国留学人员联谊会）第九届理事会会长会成员座谈</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>王沪宁与欧美同学会座谈，强调弘扬留学报国传统，服务中国式现代化建设。</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDExAYmxsSGewGcby48XUcd260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】开天辟地 中国共产党成立</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>庆祝建党105周年，新闻联播推出《伟大征程》，首集回顾中共一大召开及初心使命。</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEpguCNNVGkdrzXeax3ozX260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Murrell used fake invoices to cover up £400,000 spending spree</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>前苏格兰民族党首席执行官因伪造发票挪用公款面临监禁。</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgmp0pxyze8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Five questions left unanswered by the Mandelson files</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>曼德尔森任美大使相关第二批文件公布，留下五个未解问题。</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4p9pv13kdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>EU strikes migration deal for more deportations and detention centers abroad</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>欧盟推进移民政策改革，计划加强驱逐并建设海外拘留中心。</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/nx-s1-5844100/eu-migration-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《加快农业农村现代化“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>国务院印发农业农村现代化“十五五”规划，聚焦农业强国和乡村振兴。</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEL5Qogct5jsF1elq8hh7d260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>[视频]产业焕新 带动就业提质扩容</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>制造业数字化智能化改造催生大量新兴岗位，带动就业质量提升，并将扩大培训。</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEVpTe9V1LRNUQdnfgwteb260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>[视频]助力三夏抢收 设备更新政策发力显效</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>国家推进设备更新，补贴粮食烘干等农机，助力夏粮抢收和配套产业发展。</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEqFp8Zi9XluzDLAHu3EDJ260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Canada formally requests renewal of North American free trade pact</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>加拿大正式请求续签北美自由贸易协定。</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn9prr3w9nlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>经济, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Global conflicts push Sri Lanka's economy to the brink</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>全球冲突使斯里兰卡经济濒临崩溃，民众称已无缓冲余地。</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/nx-s1-5823430/global-conflicts-push-sri-lankas-economy-to-the-brink</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>军事, 民生</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Ultra-Orthodox protesters block roads and trains across Israel over military draft</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>以色列数万 ultra-Orthodox 抗议强制兵役，封锁道路与火车，并纵火烧车。</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/nx-s1-5844080/ultra-orthodox-protests-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>What to know about U.S. military strikes on alleged drug boats</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>美国打击涉嫌贩毒船只，已致超200人死亡，行动合法性遭质疑。</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/g-s1-125314/us-military-strikes-on-alleged-drug-boats</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Russian attack on Ukraine kills at least 16 and traps others in damaged buildings</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>俄军向乌克兰发射数百架无人机与导弹，致至少16名平民死亡，多人被困。</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/nx-s1-5844071/russian-attack-ukraine</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】让社区成为居民最放心最安心的港湾</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>习近平总书记强调社区治理现代化，各地推进便民服务、智慧赋能，提升居民幸福感。</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEH6rEEfLVAuCbXuib240x260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>[视频]《习近平的文化情缘》等纪录片在老挝启播</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>《习近平的文化情缘》等纪录片在老挝启播，老挝国家主席致贺信，庆祝中老建交65周年。</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEz3Y71CKiDpMOInx0Gt90260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见英国外交大臣</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>韩正会见英国外交大臣，双方同意发展中英全面战略伙伴关系，加强多领域合作。</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEJLoaaQrk1UUyulsCjb9c260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>[视频]韩正将赴俄罗斯出席第二十九届圣彼得堡国际经济论坛并访问白俄罗斯</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>韩正将赴俄出席圣彼得堡论坛并访问白俄罗斯，促进国际合作。</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEv94e1A7FUqyRwSTA2xF7260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>[视频]黎政府称黎真主党同意相关停火方案 以称将继续在黎南部开展行动</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>黎真主党同意停火方案，以称继续行动；伊朗暗示管控曼德海峡，美伊谈判推进。</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEUp0VVwfS8CMDufAJjubx260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>俄大规模打击乌目标；美英士兵在伊训练身亡；台风袭日；美火箭发射平台受损。</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDE6ikmQanau5qq5amUvElS260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Ukraine rescuers pull dead from rubble after Russian strikes kill 22 people</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>俄导弹袭击乌克兰致22人死亡，包括一名8岁男孩，救援人员从废墟中搜寻。</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5y8nq8ljqwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Israel strikes southern Lebanon but partial truce with Hezbollah appears to hold</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>以色列继续打击黎巴嫩南部，但未袭击贝鲁特，美国宣布的停火协议暂时维持。</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c936zvne0l6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>British couple lose Iran jail sentence appeal, family says</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>英国夫妇环球摩托车旅行时被捕，上诉失败。</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjrpwxe82ypo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Two people shot dead amid Kenya protests against US Ebola quarantine centre plan</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>肯尼亚抗议美国埃博拉隔离中心计划，两人被枪杀。</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgz7zny3pzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>社会, 民生, 政治</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>多项快讯：启动探访国家公园、下达育儿补贴、出台非化石能源核算办法、护航高考。</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDE0NaWm5SzmodAxoEUFwWi260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>[视频]美丽中国行</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>展现中国国家公园生态美景，讲述人与自然和谐共生故事。</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/02/VIDEnOiPU5gCnGcdu2qnU6Dc260602.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Police bodycam shows officers handcuffing stabbed student as he lay dying</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>警方执法记录仪显示，遇刺学生临终被戴上手铐。</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c172kkwpd9xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-03
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F945"/>
+  <dimension ref="A1:F972"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30677,6 +30677,870 @@
         </is>
       </c>
     </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>[视频]树立和践行正确政绩观学习教育中央指导组工作座谈会暨继续派出中央指导组培训会议召开</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>正确政绩观学习教育中央指导组座谈会召开，部署指导督导工作。</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEQXFWsXC4bU1SHI1PM19k260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>政治, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>国内联播快讯：市长对话在京举行；多部门促科研助理岗位就业；社区卫生体系将健全；网络餐饮抽检良好。</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEDOlDWUnUbzZBI4SKZD2I260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>PM accuses Farage of exploiting Nowak case and denies 'two-tier policing' claim</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>英首相指责法拉奇利用诺瓦克案，否认存在“双重标准”警务。</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgz23p8117o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>EU strikes migration deal for more deportations and detention centers abroad</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>欧盟达成移民协议，旨在加速遣返并建立海外拘留中心，被批类似特朗普政策。</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/02/nx-s1-5844100/eu-migration-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>经济, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260603 19:00</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>西部陆海新通道加速对外开放；物流业景气指数回升；外资加码硬科技；麦收推进。</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEojsgGEibjPsOWHRkLbD9260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】通江达海 西部陆海新通道跑出高水平对外开放“加速度”</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>西部陆海新通道骨干工程平陆运河全线通水，将形成便捷水运大通道。</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDE8C4zfWzt5yPle16fhogq260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】北京锚定城市战略定位推进“十五五”高质量发展 山西坚定有序推进转型发展 奋力谱写中国式现代化西藏新篇章</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>北京、山西、西藏发布“十五五”规划，聚焦高质量发展目标。</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEKN73WHvDltQx8devOIUP260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>[视频]5月份中国物流业景气指数重回扩张区间</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>5月中国物流业景气指数50.3%，重回扩张区间，需求回升。</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEgWrc73vngS0FAt9KT3Ou260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>[视频]长线外资看好中国 持续加码硬科技</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>多家国际机构看好中国，外资持续流入A股，加码硬科技领域。</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEnQmSxBxX3dGH3OvBzvMO260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Shell pumped oil through Nigeria pipeline for years despite pollution evidence, documents show</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>文件显示壳牌曾多年在尼日利亚管道漏油，公司称文件忽略复杂背景。</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdrp8v7407ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称打击美军基地等目标 美称空袭伊朗格什姆岛</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>伊朗称打击美军基地，美方否认并称空袭伊朗目标，双方信息交换暂停。</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEjbWsrrGoNQFjBlE7ySqf260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>One killed and dozens injured in Iranian drone strikes on Kuwait airport</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>伊朗无人机袭击科威特机场致1死数十伤，称报复美军此前打击。</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yx135yg53o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Ukrainian drones hit St Petersburg as Putin's flagship economic forum opens</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>乌克兰无人机袭击圣彼得堡油库，普京经济论坛即将开幕。</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0e2vqd3j1vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Three die in Royal Navy helicopter crash during training exercise</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>英国皇家海军直升机训练时坠毁致3死，王室及首相致哀。</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce3pdv1gl41o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Iran and the U.S. trade strikes in the Persian Gulf, further testing the ceasefire</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>伊朗与美国在波斯湾交火，科威特机场遭伊朗无人机袭击后关闭，脆弱停火受考验。</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/03/g-s1-125566/iran-war-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Scenes from the aftermath of Russia's latest massive attack on Kyiv</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>俄罗斯对基辅发动大规模导弹和无人机袭击，造成乌克兰平民伤亡。</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/sections/the-picture-show/2026/06/02/nx-s1-5844159/ukraine-kyiv-russia-drone-missile-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥在云南调研</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>丁薛祥在云南调研基础教育，强调推进教育高质量发展。</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDErP6Zu2ei2erAuWHBTlor260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国麦收高效有序推进</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>全国麦收高效有序，已收获冬小麦1.4亿亩，进度过四成，主产区进入高峰。</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEWnKyQgkzcSt34hJlUOMe260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见下任联合国秘书长候选人</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>韩正会见下任联合国秘书长候选人，表示支持联合国发挥核心作用。</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEbn9MvDZ7qpDQFgYm0jKV260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>[视频]中老跨境游火热 水果“鲜”达餐桌</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>中老跨境游火热，前5月跨境旅客同比增超35%，两国货物通关效率提升35%。</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEfWwvaQ8vyTpLATLtJWde260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>以军袭击黎南部致12死；孟加拉国外长当选联大主席；丹麦新政府坚守格陵兰岛主权；刚果金埃博拉死亡60例。</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDElpRhqnmSCjFpYh1YrS8u260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Foreign nationals among at least 21 killed in Delhi fire</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>印度德里火灾致至少21人死亡，多为赴印就医南亚人。</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czd29327qzvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Eight killed after drone hits bus in Russian-occupied part of Ukraine</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>俄控乌克兰地区一架无人机击中巴士，致8人死亡。</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp3peyykxd5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Ukrainian drones strike a St. Petersburg oil terminal ahead of Putin visit</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>乌克兰无人机袭击圣彼得堡油库，时值普京出席经济论坛。</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/03/nx-s1-5844793/ukrainian-drones-hit-st-petersburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>[视频]美丽中国行</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>美丽中国行：中国国家公园守护万物栖息，展现人与自然和谐共生的壮美画卷。</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/03/VIDEqoRiuGdRYqjYZnUgU5pk260603.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>How a content creator tried to use a YouTube alibi to get away with murder</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>北爱尔兰一内容创作者用YouTube不在场证明谋杀怀孕伴侣，被判至少31年。</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c893zygkvy8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>社会, 经济</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Greetings from Porto, whose lanes are lined with colorful textiles</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>葡萄牙波尔图街头挂满彩色纺织品，许多纪念品店由孟加拉人经营。</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/03/g-s1-124469/porto-portugal-linens-textiles</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-04
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F972"/>
+  <dimension ref="A1:F999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31541,6 +31541,870 @@
         </is>
       </c>
     </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260604 19:00</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>新闻联播报道绿色发展、政绩观教育、自贸区开放、外资电信试点、高端钢材、3D打印、海水淡化、消费权益等。</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEB7PwD2aa5fLu0gc8EpIc260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】践行绿色发展 人与自然和谐共生</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>习近平总书记强调绿色发展，我国全面转型，浙江瑞安母亲河黑臭治理后重现碧水。</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEQ2Q42XNsihvYSlN5rBz8260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】坚持民生为大 推进学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>重庆渝中、广东梅州开展政绩观教育，解决群众出行和政务服务难题。</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEEBJ2kLgnCLWOB8YGnqv7260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Trump hits back at 'unpatriotic' vote after House rebukes him over Iran</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>特朗普抨击众议院“不爱国”投票，该决议旨在限制其对伊朗的军事行动，但仅具象征意义。</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn0pl0wvvz0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>政治, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Starmer accuses Musk of trying to whip up division over Henry Nowak murder</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默指责马斯克就少年谋杀案煽动分裂。</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1e2ww900zno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Peru election could add to string of right-wing victories in Latin America</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>秘鲁周日大选，极右翼候选人可能获胜，延续拉美保守化趋势。</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/04/nx-s1-5844281/peru-election-could-add-to-string-of-right-wing-victories-in-latin-america</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>[视频]我国自贸试验区持续提升对外开放水平</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>我国自贸试验区优化布局，前4月利用外资和外贸进出口增长超30%创新高。</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDE7XnoEBKXINmvYdYmACWb260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>[视频]166家外资企业获增值电信业务经营试点批复</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>166家外资企业获增值电信业务经营试点批复，覆盖全部10项业务。</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDE0EgGCEghNlIh1tA5zq98260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>[视频]我国高端钢材供给持续增强</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>我国高端钢材供给增强，研发蝉翼钢等特种钢，自给率近100%。</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDECCQ2BapRtDf5v3kEOpZ9260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>[视频]各地培育新场景新业态 激发消费活力</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>各地培育新场景新业态，天津、成都等地利用老建筑、老厂房激活消费，推动农文旅融合。</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEXXrsrckAtvnCvlGkZ5mB260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>经济, 科技, 国际</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>1-4月电子信息制造业增长14%；端午火车票发售；北京发布文旅科技应用场景；广州直飞阿斯塔纳航线开通。</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDE2ogamFH4dMIGOpgHWhMd260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>经济, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Russia's economic forum opens against backdrop of Ukrainian strikes</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>俄罗斯经济论坛在乌克兰无人机袭击与经济不确定性下开幕。</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/04/nx-s1-5844903/russias-economic-forum-opens-against-backdrop-of-ukrainian-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>[视频]我国3D打印产业进入快速发展新阶段</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>我国3D打印产业快速发展，前4月产量增长50.9%，出口量增长100.3%。</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDE6UcYbMjA5ifFSNlxoy8J260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>[视频]海水淡化能力显著提升 有力保障沿海地区用水需求</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>我国海水淡化能力提升，突破核心技术，保障沿海用水，惠及偏远海岛。</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEARl1wi7PbZ3YH70wq4gg260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称在阿曼湾打击一艘美军舰 美军予以否认</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>伊朗称在阿曼湾打击美军舰，美军否认；特朗普表示希望分开处理以黎冲突与美伊谈判；美众院通过限制对伊朗动武决议。</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEyV0oVPfncbBQrnMwT7kH260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>军事, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Israeli strikes kill 11 people in Gaza City, medics say</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>以色列空袭加沙城多处住宅，致11人死亡，含妇女儿童。</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cg5prr9gr1ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>军事, 社会</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Royal Navy crew killed in helicopter crash named</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>英国皇家海军直升机训练时坠毁，遇难机组人员身份公布。</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cg4p69gzd4po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>[视频]《中国消费者权益保护状况年度报告（2025）》发布</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>中消协发布年度报告，2025年受理投诉201.6万件，挽回经济损失9.3亿元，相关法规标准进一步完善。</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDEV9VlEnHRTll8beqfXYJZ260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】信息流背后的精准麦收</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>受苗情和天气影响，麦收调度采用精准气象和AI大模型，确保信息准确，保障跨区机收。</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDETYla6epN6tyVx0qRUtFC260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>以黎同意有条件停火，真主党未回应；吉尔吉斯斯坦首次当选安理会非常任理事国；俄乌互相拦截无人机。</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/04/VIDENb9JDi6g1vIZHWMwG0dj260604.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Hezbollah rejects renewed ceasefire agreed by Israel and Lebanon</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>以色列与黎巴嫩同意停火，黎巴嫩真主党拒绝接受该协议。</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c052343r812o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>'Crazy' phone call between Trump and Netanyahu complicates Iran talks</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>特朗普与内塔尼亚胡的“疯狂”通话使伊朗谈判复杂化。</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgz21pq3g6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Israel and Lebanon reach an agreement, but ceasefire stalls</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>以色列与黎巴嫩达成协议，但停火推进受阻，一名维和人员遇难。</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/04/g-s1-125942/israel-lebanon-ceasefire</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Plans for a Trump family-linked resort spark protests in Albania</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>库什纳关联的阿尔巴尼亚海岸开发项目遭环保人士与批评者反对。</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/04/g-s1-125926/albania-protests-trump-family-linked-resort</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Missing Sherpa guide found on Mount Everest after 'miracle' self-rescue</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>失踪六天的夏尔巴向导在珠峰奇迹般自救爬回大本营。</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgz2yjl4y3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Man shot with crossbow on university campus</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>英国吉尔福德大学学生村内一男子遭十字弓射击。</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4p4yllq1lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Video of a dying teen handcuffed by police sparks outrage and riots across Britain</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>英国警方手铐濒死少年视频引发全国愤怒与抗议浪潮。</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/03/nx-s1-5844898/british-student-nowak-handcuffed-police-video-farage</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-05
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F999"/>
+  <dimension ref="A1:F1040"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32405,6 +32405,1318 @@
         </is>
       </c>
     </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>政治, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260605 21:00</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>习近平迎老挝元首；将对朝鲜国事访问；李强主持国务院会；医保跨省共济等。</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEYgzKDmM12c3iPhXr0kP6260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎老挝人民革命党中央总书记、国家主席通伦访华</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂为老挝元首通伦访华举行欢迎仪式。</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEGxc9angi0s9cJALFOWyP260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>[视频]习近平同老挝人民革命党中央总书记、国家主席通伦举行会谈</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>习近平同老挝元首会谈，提四点看法推动中老命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEENTCvgVaQQlSGttPO4Xy260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>[视频]习近平将对朝鲜民主主义人民共和国进行国事访问</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>习近平将于6月8日至9日对朝鲜进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEVCVNgjQtGSF48I62iMBA260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>李强主持国务院会，通过就业优先规划及退役军人就业条例。</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDE09rptXGwerkZXjiAernW260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>[视频]李强会见老挝人民革命党中央总书记、国家主席通伦</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>李强会见老挝元首，愿加强战略对接与各领域合作。</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEIDjZHdqfWV7WVJdF1sCu260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见老挝人民革命党中央总书记、国家主席通伦</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>赵乐际会见老挝元首，望深化立法机构合作。</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDE7bS4mmJF8fo6HtIDD6ox260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>[视频]中央党校（国家行政学院）举行2026年春季学期第二批班次毕业典礼 蔡奇出席并为学员颁发毕业证书</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>中央党校春季班毕业，蔡奇出席，强调学习成果转化。</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDE4kfPctmIq8boiYBCVQW7260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>[视频]全国人大常委会启动无障碍环境建设法执法检查</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>全国人大常委会启动无障碍环境建设法执法检查，将赴多省实地检查法律实施情况。</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDErMurVgRunvECHDBcqn3u260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Xi Jinping to meet Kim Jong Un in rare visit to North Korea</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>习近平将罕见访问朝鲜，会晤金正恩。</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypym3q7p1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Two weeks out from crucial Makerfield by-election, here's how the contest is shaping up</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>梅克菲尔德补选倒计时两周，候选人辩论焦点突出。</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cg7p7nmj52jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>政治, 军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Putin says Russia will bolster air defenses in response to Ukrainian drone attacks</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>普京称俄罗斯将加强防空以应对乌克兰无人机袭击，该袭击已深入俄境内并影响其经济论坛。</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/05/g-s1-126268/russia-ukraine-war</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>经济, 科技, 社会</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>国内联播快讯：2026年将办超百场‘出口中国’活动；最高法发布环境资源审判报告等。</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEr67W1ixW6m79cNHk0b91260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Hospitality jobs boom as US prepares for World Cup</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>美国为世界杯做准备，酒店业就业连续三月增长超预期。</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdxpx4gel1yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>[视频]6G创新发展部省协同试点专项行动启动</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>工信部启动6G创新发展部省协同试点专项行动，计划到2029年为6G商用落地提供支撑。</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEkq7umCKGATI21JiFbHU8260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>科技, 民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>China's highest bridge brings tourists and internet access to remote communities</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>中国最高桥贯通高速公路，缩短偏远地区出行时间并带来互联网。</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/05/g-s1-126304/chinas-highest-bridge-brings-tourists-and-internet-access-to-remote-communities</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Ukraine strikes cargo ships and admits Romania drone blast</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>乌克兰称在亚速海和俄占区沿海袭击五艘非法货运船只。</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c707098wkzpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>[视频]今年职工基本医保个人账户实现跨省共济</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>国家医保局、财政部通知，今年内职工医保个人账户跨省共济将在全国所有省份全面开通。</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEZadUxliClNVsBngONyFV260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】各地麦收高效推进 助力夏粮颗粒归仓</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>各地加快冬小麦收获进度，河北、安徽、河南等主产区全力抢收，确保夏粮颗粒归仓。</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEclWj20OpLMzrl8NVhsPg260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>A-level maths exam marking to be watched closely by regulator after students say paper was 'unfair'</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>A-level数学考试被指不公，超2万人请愿要求审查评分。</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4g9gz9d2qzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>民生, 科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>South Africa rolls out game-changing HIV shot amid funding shortfalls</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>南非推出革命性HIV预防注射，但资金短缺和剂量有限影响效果。</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/05/nx-s1-5846846/south-africa-hiv-lenacapavir-aid</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>[视频]黎真主党称将继续抵抗以色列的占领 以指责黎真主党破坏稳定</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>黎真主党拒绝有条件停火，称将继续抵抗以色列占领；伊朗要求以色列从黎巴嫩被占领土撤军。</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDE53TmDi8xj05QwReBevJM260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>国际, 民生, 军事</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>世粮署称中东危机冲击全球粮食安全；普京表示愿和谈；古巴谴责美国制裁；美媒称“福特”号动态。</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEvNl49r8QJ7tzGGv24KfP260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Zelensky proposes face-to-face talks in open letter to Putin</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>泽连斯基公开致信普京，提议直接面对面会谈以结束战争。</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy2ypyp4x4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Ex-wife of Dubai ruler's nephew in custody, prosecutors say</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>迪拜酋长侄子前妻被拘留，自周二起失联。</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx2124zylxno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>US journalist pleads guilty to working as China's agent</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>美国记者承认多年来为中国政府担任代理人。</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crmpmxg1ym4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Two Romanians found guilty of stabbing Iranian opposition journalist</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>两名罗马尼亚人因刺伤伊朗反对派记者被判有罪。</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czx2xn2gq65o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>国际, 社会, 政治</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Protesters in Albania oppose plan for Trump family-linked resort</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚民众抗议特朗普家族关联度假村计划，担忧环境破坏。</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/05/nx-s1-5846829/protesters-in-albania-oppose-plan-for-trump-family-linked-resort</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>[视频]环境日：全民参与 共建美丽中国</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>环境日之际，全国多形式开展生态环保宣传实践活动，发布首批美丽中国建设打卡点及生态环境状况公报。</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEfnf0p2Hcz22jG5q5jRv0260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行记者见面会，五位广电行业代表分享服务人民群众的奋斗故事。</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDENh71RqNMpSK12znehXDe260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>[视频]二十四节气·芒种</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>芒种节气到来，反映农业物候现象，寓意忙碌与收获。</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/05/VIDEVx7ETpPrqi26xuma0kuq260605.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Fury in France after child murder suspect's criminal record released</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>法国儿童谋杀案嫌疑人曾有性侵记录，引发公众愤怒。</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1424v7mk8go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Nearly 50 people die of thirst in Sahara desert after lorry breaks down</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>撒哈拉沙漠中车辆故障导致近50人渴死，仅2人生还。</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62r2ldyejro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>US actor James Handy stabbed to death, with girlfriend's son arrested</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>美国81岁演员詹姆斯·汉迪被刺身亡，女友儿子被捕。</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czd2dj24jgdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Three jailed over heist of ancient golden helmet from Dutch museum</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>三人因从荷兰博物馆盗窃2500年历史金盔被判监禁47个月。</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy020317g1no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Rapist Paul Quinn sentenced to 24 years in case that saw Andrew Malkinson wrongly convicted</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>强奸犯保罗·奎因被判24年，安德鲁·马尔金森曾被误判服刑17年。</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c99l93md0gko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Andrew was sub-letting Royal Lodge cottages, watchdog reveals</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>监管机构披露安德鲁王子转租皇家小屋农舍。</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8p8dzvjy9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Teen rapists spared jail partly because of intellectual limitations, judge's full remarks show</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>法官称智力受限，两名少年强奸犯免于监禁引争议。</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3d2d55kvy1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Buffy and Ted Lasso star Anthony Head dies at 72</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>英国演员安东尼·海德去世，享年72岁，曾出演《巴菲》和《足球教练》。</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd0p0rz4n0mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>The deeply contentious debate around what it means to be English</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>关于英格兰身份的辩论日益激烈，话题变得更具争议性。</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3626n0lgj3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>社会, 法律</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Three admit violent disorder after Nowak protest</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>三名男子因在诺瓦克抗议中参与暴力骚乱认罪，将于下周一判刑。</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1m2mxv0pzmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-06
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1040"/>
+  <dimension ref="A1:F1072"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33717,6 +33717,1030 @@
         </is>
       </c>
     </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>[视频]【牢记初心使命 奋进复兴征程】红色沃土不断书写时代华章</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>纪念建党105周年，系列报道走进上海和嘉兴，展示红色沃土时代变迁与成就。</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEqF2FPzuYBH2UkM870eLO260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见俄罗斯总统</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>韩正会见普京，双方强调深化中俄关系，为世界和平发展贡献稳定性。</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDECH1WOikGEW4mRdO165rH260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>[视频]韩正出席第二十九届圣彼得堡国际经济论坛全会并致辞</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>韩正在圣彼得堡论坛致辞，提出践行全球治理倡议四点建议，倡导多边合作。</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEHBGlXQqiE7ArzoJEd730260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Armenia braces for election as Russia piles pressure on pro-West government</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>亚美尼亚面临大选，俄施压亲西方政府，现任总理支持率下降仍求连任。</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3626n1epd5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Giant banquets rile radical left in France</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>法国“巨型宴会”现象引发极左翼不满，成政治热点。</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78q215vyd7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>The Nowak murder has lit a match under British politics. This is how we got here</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>亨利·诺瓦克谋杀案引发英国警方应对争议及跨大西洋辩论。</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c39297vxmw2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Peru is set to elect its 10th president in a decade</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>秘鲁将选十年内第十任总统，极右翼与左翼候选人竞争激烈。</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/06/nx-s1-5847845/peru-election</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>[视频]我国服务贸易持续扩能提质</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>我国服务贸易规模增长，知识密集型出口增11.7%，传统旅行运输服务也提速。</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEncuGXLwF1zk6TXM9519d260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>[视频]财政金融“组合拳” 更大力度支持扩内需</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>设立千亿专项资金，运用贴息担保等工具，引导资金流向消费投资重点领域。</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEOJr26dGlRl4iSckbUe6S260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>国开行前四月发放4406亿基础设施贷款；国家防总启动防汛应急响应等。</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDE9j4CbsbnK4xaTKb3X9FE260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>[视频]我国海上风电加快向深远海发展</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>海上风电向深远海发展，攻克换流站等关键技术，装机容量持续扩大。</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEhGbmRjxasf9jcNOKTbuY260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>[视频]美军袭击伊朗部分沿海地区 伊朗称打击美海军第五舰队重要设施</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>伊朗称打击美军第五舰队，美军否认遭破坏，双方在波斯湾交火。</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEnZU1aonNJ9EuNrnP4w1d260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Ukrainian drones target St Petersburg in attack Russia calls 'unprecedented'</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>乌克兰无人机罕见袭击圣彼得堡，俄称史无前例，州长呼吁民众居家。</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cg7498kz808o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>US and Iran exchange strikes in Gulf in latest test of ceasefire</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>美国与伊朗在波斯湾互袭，美方称打击伊雷达和无人机，伊方反击。</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgzgyjk2weo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Lebanon says three soldiers killed in Israeli attack on car</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>黎巴嫩称三名士兵在以色列对车辆袭击中丧生，以军正在调查。</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj0g8jymg92o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Israeli airstrikes kill 9 including Lebanese army officers after ceasefire deal</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>以色列空袭致9死含黎巴嫩军官，违反停火协议。</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/06/nx-s1-5848595/israeli-airstrikes-kill-lebanese-army-officers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>U.S. military says it shot down Iranian drones launched toward Gulf allies</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>美军称击落伊朗飞向海湾盟友的无人机。</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/06/nx-s1-5848184/u-s-military-shot-down-iranian-drones</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>民生, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260606 19:00</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>本期内容包括麦收近六成、服务贸易提质、财政金融扩内需、海上风电发展及国际动态等。</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEkMEIhWWMUwUhfkKYBNLE260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国麦收近六成 夏播陆续展开</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>全国麦收近六成，黄淮海主产区进入高峰，夏播有序推进并推广智能农机。</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEEDoohVJtVV3QvSSyZZep260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】一张网夯实水安全坚实底座</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>我国推进“六网”建设，雷州半岛缺水问题因国家水网骨干工程迎转机。</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDE9VTulUtPPilBUI7DOS5n260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Canada bans Texas cattle over flesh-eating screwworm outbreak in US</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>加拿大因美国得州食肉蛆疫情，禁止进口得州牛。</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cevpv3r7jmpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>俄乌交换185名被俘人员；世贸组织称今年全球货物贸易保持韧性。</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/06/VIDEn0O6yojzpfhCygHPZTU8260606.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Iran says staff blocked from entering US after players given World Cup visas</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>伊朗称技术员工遭美拒签，此前美国为球员发世界杯签证。</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy8286nqz87o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Man dies after bitten by shark in Western Australia, police say</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>西澳一男子在矛鱼时遭鲨鱼袭击身亡。</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c74yl98kv37o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>King's nephew Peter Phillips weds NHS nurse with William and Kate among guests</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>英国国王侄子菲利普斯与护士结婚，威廉夫妇出席。</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj9gl0x7lj9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Four more admit violent disorder after Nowak protest</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>四人承认在诺瓦克抗议后实施暴力骚乱。</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c05yjg452geo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Singer Duffy to perform first live concert in 15 years after sex assault ordeal</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>歌手达菲时隔15年重返舞台，此前因性侵离开公众视野。</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8p8mzj4e8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Three British men admit killing restaurant owner in Canada after 'unpaid bill' row</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>三名英国男子在加拿大因账单纠纷杀害餐厅老板认罪。</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78y5w6d15no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Tributes to Buffy and Ted Lasso star Anthony Head after death aged 72</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>英国演员安东尼·海德去世，享年72岁，曾演《巴菲》《足球教练》。</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd0p0rz4n0mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Rumours and speculation as fans forecast date of Taylor Swift's wedding</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>全球粉丝猜测泰勒·斯威夫特与特拉维斯·凯尔斯的婚期。</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cqjpj80qz1ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>West Ham joint chairman David Sullivan steps down after 'serious' historical allegations</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>西汉姆联联席主席因历史性严重指控立即辞职。</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/clypyk2e7vyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Steven Spielberg makes surprise appearance at London pub quiz</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>斯皮尔伯格突现伦敦酒吧问答赛宣传新片。</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cd0m5e4301mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-07
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1072"/>
+  <dimension ref="A1:F1099"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34741,6 +34741,870 @@
         </is>
       </c>
     </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260607 19:00</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>新闻联播主要内容：三北工程、农村公路、船舶海工、革命历史、通信网、高考开考、国内快讯及国际新闻。</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEDXMLq9HcrbO78iCSvgE3260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】攻坚“三北” 筑牢北疆万里绿色屏障</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>三年来“三北”工程防沙治沙成效显著，林草覆盖率提升，应用新技术加速治理流动沙地。</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEWT9UwxEXgZpWz1drMsxY260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】星星之火 可以燎原</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>回顾土地革命时期，中国共产党开辟农村包围城市道路，创建红军和革命根据地。</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEGFBw0sMXlaKTKJCXbhF7260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Armenia votes as Russia piles pressure on pro-West government</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>亚美尼亚议会选举，亲西方总理帕希尼扬寻求连任。</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3626n1epd5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Hegseth attacks Europe over migration with beach 'invasion' D-Day speech</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>美防长在诺曼底演讲，借D-Day比喻抨击欧洲移民政策。</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c802e7jk458o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Delays to defence plan undermine UK credibility, MPs say</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>议员称国防投资计划延迟将损害英国信誉，计划于北约峰会前发布。</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0ky47v6d1no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>[视频]我国持续优化完善农村公路网络</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>我国持续优化农村公路网络，前4月投资821亿元，新改建1.6万公里，带动就业增收。</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEppotQGGNDNKq7JB4lULh260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>[视频]我国船舶海工装备产业加速提质升级</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>我国船舶海工装备产业加速升级，高端定制船舶和海工装备订单增长，全球份额稳居首位。</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEpWbZlkmgRBYRKX09QXaR260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>经济, 民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>5月末外汇储备升317亿美元；41条改革经验将推广；农业保险提供1.82万亿元保障；南方防汛应急响应启动。</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDED3mB4Y5OeCdKLBJu5dPp260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>经济, 军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Steve Rosenberg: Russia's economic forum overshadowed by drone attacks on St Petersburg</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>俄经济论坛被乌克兰无人机袭击圣彼得堡事件蒙上阴影。</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9q2gp52rgro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>M&amp;S launches new traineeship for 1,000 young people</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>玛莎百货启动新培训计划，面向1000名未就业未就学的年轻人。</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr7xr3dvxp9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>经济, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Russia's elite gather for Putin's pet project — an economic forum in St Petersburg</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>俄罗斯精英齐聚圣彼得堡经济论坛，在乌克兰战争持续之际展现乐观姿态。</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/07/nx-s1-5847010/russias-elite-gather-for-putins-pet-project-an-economic-forum-in-st-petersburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】天地织密通信网 赋能产业新发展</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>新一代通信网支撑低空经济等产业，通过升级基站实现空地实时互联，提升安全与效率。</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEKUPtRzVZneJD7oQI8hsK260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Zelensky criticises 'vile' Chornobyl drone strike ahead of London talks</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>乌称俄无人机袭击切尔诺贝利核废料存储设施，泽连斯基谴责。</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr7xr1g3nvvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>[视频]2026年全国统一高考今天开考</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>2026年全国高考开考，报名1290万人，设34.8万考场，严控高科技作弊，保障残障考生。</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEhY5TmztMLZXthW2AVJsH260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>[视频]伊朗谴责美国持续违反停火协议</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>伊朗谴责美军袭击其雷达设施，称美一再违反停火协议，地区紧张持续百天。</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDEAjMiSJz3bVQrCMW4ycrY260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>巴勒斯坦称以在约旦河西岸袭击升级；美称以间谍威胁级别升至最高；劳尔·卡斯特罗公开露面。</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/07/VIDE3Egi0D1kFD6MoXWqRAzP260607.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Iran's World Cup team lands in Mexico amid US visa row</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>伊朗世界杯球队因签证问题在美比赛需当日往返墨西哥。</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yz3zdp3jqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Hundreds of captives freed from Boko Haram mountain hideout</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>数百名被博科圣地绑架的妇女儿童获释，她们于3月在喀麦隆附近被劫持。</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8j0jn4xjgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Lammy says he told JD Vance his Nowak comments were 'wrong'</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>拉米称曾告知万斯，他将诺瓦克之死归咎于移民的说法是错误的。</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjwg387040wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Son calls for Iran prisoner exchange for British pair</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>被伊朗扣押的英国夫妇之子呼吁英国政府探讨换囚方案。</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ced414n2vyxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>国际, 民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>When U.S. foreign aid changed, AIDS workers in Africa felt it</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>美国对外援助变化，导致南非和莫桑比克艾滋病救治中断，危及生命。</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/07/nx-s1-5837324/usaid-aids-africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Huge crowds throng Madrid streets for Pope's open-air Mass</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>教皇在马德里露天弥撒吸引大批民众，乘坐教皇专车互动。</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4gyejvzx9eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Who is NHS nurse and newest royal Harriet Sperling?</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>NHS护士哈丽特·斯珀林与彼得·菲利普斯结婚，王室成员出席婚礼。</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1jylk8wxgno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Girl, 16, among five arrested over Nowak protests as three charged</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>南安普顿因诺瓦克遇刺引发骚乱，五名嫌疑人被捕含16岁女孩。</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c07ye0zx1dzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>社会, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>1 million people flood Madrid streets to see the pope's flower-carpeted procession</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>百万人涌上马德里街头，观看教皇鲜花地毯游行，这是15年来首次教皇访西班牙。</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/07/nx-s1-5849147/1-million-flood-madrid-streets-pope-procession</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Simone Biles reveals health scare after 'almost dying'</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>七届奥运冠军西蒙·拜尔斯透露曾遭遇健康危机，称“差点死去”。</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/olympics/articles/cjeg2pqx2ppo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-08
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1099"/>
+  <dimension ref="A1:F1124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35605,6 +35605,806 @@
         </is>
       </c>
     </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260608 19:00</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>习近平离京对朝鲜进行国事访问；丁薛祥出席三峡水运新通道开工；国务院印发应急体系规划等要闻。</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEO52tKHJTSDyMZlCuHDOt260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>[视频]习近平离京对朝鲜进行国事访问</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>习近平应金正恩邀请，乘专机离京对朝鲜进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDECC0jmvGvWVMlkxnawjpd260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>[视频]习近平抵达平壤开始对朝鲜进行国事访问</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>习近平抵达平壤，金正恩夫妇到机场迎接，开始对朝鲜国事访问。</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEhpj4Z4APgEqA8ttWGr1i260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>[视频]习近平出席金正恩举行的欢迎仪式</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>金正恩在平壤为习近平举行盛大欢迎仪式，检阅仪仗队和分列式。</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEERWuxUKOoThkpAYbMqIA260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>[视频]习近平同金正恩举行会谈</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>习近平同金正恩举行会谈，强调加强战略指引，深化中朝传统友谊。</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDE1PCryEXC67mzAWtN7Z4A260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>[视频]习近平在朝鲜媒体发表署名文章</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>习近平在朝鲜《劳动新闻》发表署名文章，续写中朝传统友谊新篇章。</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDENVElayHpBe7r8jdln6uu260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Xi and Kim express hopes for greater ties between China and North Korea</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>习近平与金正恩表达加强中朝关系的愿望，习近平访问平壤。</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/08/g-s1-126863/xi-and-kim-express-hopes-for-greater-ties-between-china-and-north-korea</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Chinese president visits North Korea for the first time in 7 years</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>中国国家主席习近平七年来首次访问朝鲜，旨在重申地区影响力。</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/08/nx-s1-5847691/chinese-president-visits-north-korea-for-the-first-time-in-7-years</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥出席三峡水运新通道工程开工仪式</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>丁薛祥在湖北宜昌宣布三峡水运新通道工程开工，提升长江通航能力。</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEsjsYU1Vb4nU4RfDlIfCG260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>科技, 政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>国家发布数据建设方案、网络测评规范及药物试验新规；伊朗和以色列互相发动新打击行动。</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEZjy75yyD6OG9XxATBUnA260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>New drug to stop 'Ozempic butt' muscle loss</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>新药旨在阻止减肥针导致的肌肉流失，专家称三分之一的减重来自肌肉。</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c62r285l46eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《现代化应急体系建设“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>国务院印发应急体系“十五五”规划，部署安全整治与防灾减灾重点任务。</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEO2kKXEnWkoCOF3AJJMNC260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>民生, 生态</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>[视频]我国海洋生态状况稳中向好</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>我国海洋生态状况总体稳中向好，珊瑚礁等生态系统优良，人工修复海域实现规模化自然排卵繁育。</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/08/VIDEYootUoAGwzFCeqWkC4IV260608.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Iran says it has halted attacks on Israel after first exchange of fire since truce</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>伊朗称停火后首次与以色列交火后停止攻击，双方互射导弹。</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj6ge150z5go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Iran releases footage of missiles launched at Israel</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>伊朗发布向以色列发射导弹视频，称是连续一周打击的开始。</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c2kyd52wje4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>At least 32 dead after major earthquake strikes southern Philippines</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>菲律宾南部发生7.8级地震，至少32人死亡，引发小海啸。</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyel78e6p5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Armenia's pro-West government wins election despite Russian pressure</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>亚美尼亚亲西方政府赢得选举，总理党获近50%选票。</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgel990n51o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>'A World Cup for them not us': Fans' anger at US travel bans and visa restrictions</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>全球球迷愤怒美国旅行禁令和签证限制，感觉被世界杯排除在外。</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx212p8r28eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Iran's strike on Israel suggests the regime's sense of resilience is growing</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>伊朗对以色列发动打击，显示其政权韧性增强，冒险危及和平谈判。</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cly72ryrd1jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Israel-Iran strikes threaten truce. And, Ebola is spreading at an unprecedented rate</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>以色列与伊朗交火威胁中东停火；刚果埃博拉疫情空前蔓延。</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/08/g-s1-126858/up-first-newsletter-iran-lebanon-israel-trump-meet-the-press-interview-congo-ebola</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>In speech to Spanish parliament, pope demands respect for the dignity of all people</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>教皇在西班牙议会发表讲话，要求尊重所有人的固有尊严。</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/08/nx-s1-5849821/spanish-parliament-pope-speech</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Ebola outbreak spreading at an unprecedented pace, Africa CDC says</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>非洲疾控中心警告，刚果（金）埃博拉疫情以前所未有的速度蔓延。</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/08/nx-s1-5849203/ebola-outbreak-spreading-at-an-unprecedented-pace-africa-cdc-says</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Billionaire West Ham co-owner accused of abusing his power and preying on women for sex</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>西汉姆联亿万富翁联合老板被指控滥用权力，以性关系换取新闻出镜。</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cj9p2lm7epeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Who is David Sullivan - football boss, 'king of porn' and alleged sexual predator?</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>前西汉姆联老板大卫·沙利文被指控性剥削，其曾自夸性征服史。</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8pk06wrx0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Rare footage captured of Great White shark in Mediterranean Sea</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>志愿者潜水员在地中海水域拍摄到濒危大白鲨的罕见影像。</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/cd6p6zqzj6do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-09
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1124"/>
+  <dimension ref="A1:F1164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36405,6 +36405,1286 @@
         </is>
       </c>
     </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>政治, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260609 21:00</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>习近平结束访朝回国，与多国领导人互动，国务院举行宪法宣誓仪式，前5月外贸同比增长。</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEtwZ9ud5Hpu0jBw43sgYa260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>[视频]习近平出席金正恩举行的欢迎宴会</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>习近平出席金正恩举行的欢迎宴会，双方强调深化中朝传统友谊与合作。</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEKTvaPwYa4HtIAD2aeTOv260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>政治, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>[视频]习近平和彭丽媛观看朝鲜专场文艺演出</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>习近平和彭丽媛观看朝鲜专场文艺演出，中朝友好歌曲引发全场共鸣。</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDE2n8Uh4OwnHuQhwsFLVAU260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>[视频]习近平和彭丽媛参谒中朝友谊塔</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>习近平参谒中朝友谊塔，缅怀志愿军烈士，强调传承抗美援朝精神。</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEJKN9ks5yycbG3jegN3qn260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>[视频]习近平参访朝鲜劳动党中央干部学校</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>习近平参访朝鲜劳动党中央干部学校，与金正恩共同种下友谊树。</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEGxMX2IUHwkM102RUs5W2260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>[视频]习近平夫妇出席金正恩夫妇举行的小范围午宴</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>习近平夫妇出席金正恩夫妇举行的小范围午宴，就深化中朝关系达成共识。</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDENnLmDK7lQdEgJfgyxgpP260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>[视频]习近平出席金正恩举行的欢送仪式</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>习近平结束访朝，金正恩到机场送行，平壤群众热情欢送。</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEbsnglfHmTVbjmMW0erbQ260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>[视频]习近平结束对朝鲜国事访问回到北京</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>习近平圆满结束对朝鲜国事访问后回到北京。</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEkhDbKMgRje1LKF76Ebw2260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>[视频]习近平向加拿大新任总督致贺电</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>习近平致电路易丝·阿伯，祝贺她就任加拿大第三十一任总督，强调推动中加关系发展。</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDESaq4X49TKqGnwU9O7e4Y260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>[视频]习近平同格鲁吉亚总统就中格建交34周年互致贺电并共同宣布将双边关系提升为全面战略伙伴关系</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>习近平同格鲁吉亚总统互致贺电，共同宣布将中格关系提升为全面战略伙伴关系。</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEW5gMig4z7JaLkW5WsGUm260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>[视频]国务院举行宪法宣誓仪式 李强总理监誓</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>国务院举行宪法宣誓仪式，李强总理监誓，强调政治过硬、法治思维和实干精神。</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDE9ziwOKi2DIIHuT6Sc55W260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁在新疆调研</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>王沪宁在新疆调研，强调社会稳定、民族团结和文化润疆，推动长治久安。</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDExqOV5w9BLlLpjU3Os5rI260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>[视频]韩正访问白俄罗斯</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>韩正访问白俄罗斯，会见总统和总理，推动中白全天候全面战略伙伴关系深化。</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEynqbpB9zgd1lWq5m1UYl260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Xi Jinping and Kim Jong Un vow stronger ties as North Korea visit wraps up</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>习近平结束对朝鲜的首次正式访问，承诺加强双边关系。</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ceqdnpzv45po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Scrap legal equality duty for public services, says Badenoch</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>保守党领袖巴德诺赫呼吁废除公共服务的法律平等义务。</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy5vyqykpx5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>4 states head to the polls. And, global conflicts are on the rise, new report says</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>四州今日举行初选，报告称全球冲突达二战后最高水平。</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/g-s1-126975/up-first-newsletter-iran-israel-lebanon-primaries-election-fraud-los-angeles-global-conflicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Pentagon labels tech giant Alibaba and car maker BYD as aiding Chinese military</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>五角大楼将阿里巴巴和比亚迪等中企列入涉军企业名单，禁止其获美防务合同。</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/g-s1-126961/pentagon-labels-alibaba-and-byd-as-aiding-chinese-military</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Federal judge strikes down Trump's $100,000 fee on new H-1B visas</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>联邦法官驳回特朗普政府对新H-1B签证收取10万美元费用的规定。</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/nx-s1-5851474/federal-judge-fee-h1b-visa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>[视频]前5个月我国货物贸易进出口同比增长15.3%</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>前5个月我国货物贸易进出口同比增长15.3%，机电产品出口增长显著。</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEzAEu80lkby0LvlxVHzn8260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Final piece of 'iconic' Denby Pottery signed</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>历史悠久的丹碧陶瓷因成本高涨签署托管协议。</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx2vljzw5ego?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>军事, 科技</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Sea drone rescues US army helicopter crew near Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>无人艇在霍尔木兹海峡附近救起坠落的阿帕奇直升机两名机组人员。</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy0l44ex5wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Trump says pilots are fine after U.S. helicopter crashes near Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>美军直升机在霍尔木兹海峡附近坠毁，特朗普称两名飞行员安全。</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/nx-s1-5851482/trump-pilots-us-helicopter-crash</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Hundreds of aftershocks jolt Philippines as officials say death toll could rise</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>菲律宾南部地震致数十人死亡，数百人受伤，余震不断。</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ckg50pypn2eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Sweden set to ban mobile phones in schools</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>瑞典将从秋季起禁止中小学生在学校使用手机。</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/g-s1-126967/sweden-set-to-ban-mobile-phones-in-schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>伊朗和以色列暂停袭击对方；美军直升机坠毁；联合国警告海洋生态恶化。</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDE7LLTYMbFtU3Go4RZHucV260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Israeli air strikes hit Lebanese city of Tyre despite Iranian warning to stop attacks</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>伊朗警告以色列停止攻击黎巴嫩真主党，否则可能恢复敌对行动。</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c36y16nkr5no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>300 migrants bound for UK kidnapped and threatened with kidney removal</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>约300名前往英国的伊拉克库尔德人被民兵绑架，勒索赎金。</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8xwxdgvx8lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>ICC suspends top prosecutor after investigating misconduct allegations</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>国际刑事法院暂停首席检察官职务，其否认不当行为指控。</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c77yx53015no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>国际, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Man reportedly shot at Kenya protest against US Ebola quarantine centre</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>肯尼亚抗议者反对美国埃博拉隔离中心，担心跨境感染。</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3wypjz3n57o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Conflicts around the globe hit highest levels since World War II, new report says</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>报告称全球冲突达二战后最高，非洲单边暴力达1994年以来之最。</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/nx-s1-5849221/conflicts-around-the-globe-hit-highest-levels-since-world-war-ii-new-report-says</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Global violence reaches record levels due to war and attacks on civilians</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>对平民的攻击使全球暴力达到创纪录水平，专家接受采访。</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/nx-s1-5847687/global-violence-reaches-record-levels-due-to-war-and-attacks-on-civilians</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Conflicts are on the rise globally, at the highest level since WWII, data shows</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>数据显示全球冲突激增，2025年约24.46万人死于冲突，为1994年以来最高。</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/09/nx-s1-5850355/data-highest-conflicts-iran-israel-ukraine-russia-world-war-ii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>[视频]第二届世界古典学大会在希腊雅典举办</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>第二届世界古典学大会在希腊雅典举办，聚焦古典文明对话与智慧传承。</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/09/VIDEYAFi70pibUee8nqsFn1G260609.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Man accused of killing mother-in-law with poison-laced satay</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>印尼男子因感觉被岳母侮辱，涉嫌用毒沙爹将其杀害。</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crkvd376jxno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Football regulator contacts West Ham over 'serious allegations' against Sullivan</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>足协联系西汉姆联调查对苏利文的严重性侵指控。</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c1ky7gndnlyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Man who murdered partner and blew up home jailed</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>男子谋杀伴侣并炸毁房屋，被判入狱。</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cddl4jq9d3do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Carer 'who couldn't go on' jailed for killing her mother</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>护工因杀害母亲被判刑，承认过失杀人。</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8re26zl7do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Man who grabbed woman's hair and asked for kiss sentenced in legal first</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>男子因抓女性头发并索吻被定罪，开创性骚扰判例。</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8rl45jmv7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Tickets for Iran fans revoked, says federation</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>伊朗足协称世界杯小组赛门票分配在赛前被撤销。</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c9q2vrdx0ewo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Ariana Grande and Ethan Slater split after three years</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>爱莉安娜·格兰德与伊桑·斯拉特相恋三年后分手。</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn0ve7952jqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-10
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1164"/>
+  <dimension ref="A1:F1193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37685,6 +37685,934 @@
         </is>
       </c>
     </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260610 21:00</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>《新闻联播》主要内容涵盖农业现代化、李希河南调研、长征纪念、物价指数、汽车出口、新型电网、全球媒体论坛及国内外重要新闻。</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDExxePYdc9ayHBIqu2GO4I260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>[视频]李希在河南调研</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>李希在河南调研，强调纪检监察工作服务“十五五”开局，强化政治监督保障粮食安全与生态保护。</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDE08nbDr7zsJvPOavEXgGx260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】长征：气壮山河的英雄史诗</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>纪念红军长征胜利90周年，回顾长征历程与遵义会议历史转折，弘扬伟大长征精神。</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEHA3rDjk2mFVSholNk7vJ260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>[视频]树立和践行正确政绩观学习教育继续派出的4个中央指导组完成进驻</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>党中央继续派出4个中央指导组完成进驻，推动树立和践行正确政绩观学习教育。</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDElgs2jXqOzavMDVR3tetj260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】提升农业综合生产能力 加快农业现代化步伐</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>习近平总书记强调农业现代化，“十五五”开局提升农业综合生产能力，推动“三夏”生产高质高效。</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEw3bugdCzESezUbtHPXW3260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>[视频]5月居民消费价格指数总体平稳 工业生产者出厂价格指数继续上涨</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>5月CPI同比上涨1.2%总体平稳，PPI同比上涨3.9%连续三个月上涨，有色金属及电子设备价格改善。</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEmi5S9IlP5GQwSrYt8k5x260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>[视频]5月汽车出口延续快速增长态势</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>5月汽车出口93万辆同比增长68.7%，新能源出口增长1.1倍，产业链优势明显。</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEsZhP6N2IEb5W32Jg6z96260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>[视频]“活力中国调研行”主题采访活动今天启动</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>中宣部启动“活力中国调研行”，多角度展现中国经济稳中向好态势。</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEGKtLAXs2fQ2L4PM8FygW260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>期货成交额增40%，水路客运量1.2亿人次，海洋经济指数发布，反诈宣传月启动。</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEFJCKAciDhNCitnOARrDI260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】新型电网筑牢能源大国绿色转型基石</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>新型电网建设应对风电光伏装机超火电的挑战，保障绿电接得住、送得出、用得好。</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEiwkyd0m5JKhHmBbC57jg260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>[视频]第五届全球媒体创新论坛在重庆举行</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>第五届全球媒体创新论坛在重庆举行，聚焦人工智能赋能媒体转型。</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEWlqyGVnXZwNTpGg237g6260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>国新办举行见面会，五位央企青年科技人才讲述科技报国故事。</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEWQimHR2A1veLT4R06B8I260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>[视频]美称打击伊朗防空系统等 伊朗称打击美军基地</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>美军打击伊朗防空系统，伊朗反击美军基地，双方交火升级。</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEYodQxEQb5ccj5aAs8MAF260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Israeli strikes in southern Lebanon kill 17, reports say</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>据报道，以色列对黎巴嫩南部的袭击造成17人死亡，其中9人死于泰尔德巴镇。</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpq3d44l907o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Ukraine says missiles hit military plant deep inside Russia</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>乌克兰称导弹击中俄境内军事工厂、炼油厂及黑海“影子舰队”油轮。</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yzm2nzgr2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Taiwan drills with U.S. rocket system, firing in China's direction</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>台湾与美军联合演习，向台湾海峡发射HIMARS火箭系统。</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/10/g-s1-127253/taiwan-drills-with-us-rocket-system-firing-in-chinas-direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>[视频]联合国“文明对话国际日”主题活动在日内瓦举行</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>联合国“文明对话国际日”活动在日内瓦举行，中方呼吁维护文明多样性。</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEVuttXMnWsUmUaqDcmMhQ260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>国际, 军事, 民生</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>以军空袭黎南部致8死；英法加挪制裁约旦河西岸袭击者；刚果（金）埃博拉病例增至598例。</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/10/VIDEFXNcpFLBG2DFrIcX1zsn260610.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Trump says US will hit Iran 'hard' again on Wednesday</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>特朗普称美国将在周三再次“猛烈”打击伊朗，警告伊朗为拖延谈判付出代价。</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce371kw2ex2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>U.S. and Iran exchange strikes. And, House passes ICE and Border Patrol funding</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>美国与伊朗互相袭击，众议院通过边境巡逻资金法案。</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/10/g-s1-127216/up-first-newsletter-iran-us-war-primary-results-ice-funding-bill-gates</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>China re‑centers North Korea ties as nuclear silence reshapes balance</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>中国对朝鲜核计划保持沉默，朝鲜强化核武地位。</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/10/g-s1-127013/xi-jinping-visits-pyongyang-china-north-korea-ties</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>China and North Korea renew ties, complicating U.S. response to Kim's nuclear program</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>中朝重申关系，美国应对核武装朝鲜面临更大挑战。</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/10/nx-s1-5851837/china-and-north-korea-renew-ties-complicating-u-s-response-to-kims-nuclear-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Israeli leader who pulled out of Lebanon warns against getting stuck again</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>以色列前总理巴拉克警告勿再陷入黎巴嫩泥潭。</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/10/g-s1-126791/israeli-leader-who-pulled-out-of-lebanon-warns-against-getting-stuck-again</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Norway crown princess's son to stay in custody before rape verdict, says court</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>挪威法院裁定，王储妃的儿子在强奸案判决前继续羁押，推翻此前释放决定。</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c621lnee131o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>'I'll never get over watching my home burn': Belfast residents reel after night of unrest</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>贝尔法斯特一夜骚乱后居民被迫逃离家园，起因是北部一起持刀袭击事件引发的抗议。</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cevl9j9y8dmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Three arrested over Glasgow unrest and racist assaults after Belfast knife attack</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>格拉斯哥发生骚乱和种族袭击，三人被捕，警称民众因肤色遭攻击。</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cr5jme6ld54o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>World Cup referee denied US entry arrives home to hero's welcome in Somalia</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>被美国拒入境的索马里世界杯裁判奥马尔·阿尔坦回国受英雄欢迎，誓言执法2030年世界杯。</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c2dylj8kj82o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Stokes out of England squad, Root named captain</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>斯托克斯因夜店事件落选英格兰队，鲁特任临时队长参加第二场对新西兰测试赛。</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/cricket/articles/ce371kq48v7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Lacey Turner confirmed as first Strictly contestant</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>演员莱西·特纳确认成为《舞动奇迹》首位参赛者，因饰演《东区人》角色闻名。</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cg74gvy8lgjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-11
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1193"/>
+  <dimension ref="A1:F1222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38613,6 +38613,934 @@
         </is>
       </c>
     </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260611 21:00</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道习近平外交文选出版、访朝纪实片、国务院会议等多条国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEDlpFYTZZXYNE0dVenXM8260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>[视频]《习近平外交文选》第一卷、第二卷出版发行</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>《习近平外交文选》第一卷、第二卷出版发行，收录习近平关于外交工作的134篇著作。</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEzvkGHrr8MB2HZ6sWjUdk260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>[视频]电视专题片《续写中朝传统友谊崭新篇章——习近平总书记访问朝鲜纪实》今晚播出</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>央视播出专题片，记录习近平总书记访问朝鲜，此访具有里程碑意义。</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDENek0gLb4lPSaxS0TB9vP260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，研究审计整改、科技大会落实及教育“十五五”规划。</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDE8PIB9CRHKO4fBKQOXCU1260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际就日本前众议长河野洋平逝世向遗属致唁电</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>赵乐际就日本前众议长河野洋平逝世向遗属致唁电，肯定其推动中日友好。</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDE8EBWEnHI96Kiad9VFCH1260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】实干担当促发展 推动学习教育见行见效</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>北京西城区、陕西汉中市推进正确政绩观学习教育，解决老旧小区改造等民生问题。</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDE0oFa5uKcHxPrHDwUA7ZC260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>[视频]“2026·全球人权治理高端论坛”在京举办</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>全球人权治理高端论坛在京举办，发布《国家人权行动计划（2026—2030年）》。</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDE6Vt0MUEFB9TwiilfqYAz260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>五位海关代表在国新办记者会上分享为国把关、为民造福的故事。</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDERwQl65XJhkJudH1ZTC5m260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Asylum appeal backlog at record high, new figures show</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>新数据显示英国庇护申请上诉积压达历史新高，尽管决策积压减少，但上诉数量上升。</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwyld5rnw9vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>[视频]我国开展东西部协作30年 成效显著</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>我国东西部协作30年成效显著，引导企业投资7500多亿，助力西部就业与产业发展。</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEwq1HJxYBAhoWoi4qtTtr260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>[视频]前5个月我国工程机械海内外市场快速增长</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>今年前5个月，我国挖掘机、装载机等工程机械国内国际销量同比均实现两位数增长。</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDERqxBHNxNMSwdgm4CL92w260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>南博会开幕；企业数据交易额增39.8%；四部委推创业行动；两部门启动人形机器人实训。</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEnqEUU6qm8fQ4k6sykLJm260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>How 'algorithm' got its name from a 9th-century Persian mathematician</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>“算法”一词源自9世纪波斯数学家穆罕默德·伊本·穆萨·花剌子米。</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/nx-s1-5848013/algorithm-word-week-etymology</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Deadly Sudan drone strike targets funeral procession</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>人权组织指控RSF民兵组织在苏丹内战前线城市杀害平民，无人机袭击葬礼队伍。</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c70yeee2jvqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>US and Iran exchange strikes across Middle East for second day in a row</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>美国和伊朗连续第二天在中东互相打击对方资产，伊朗称袭击了美国在科威特、约旦和巴林的设施。</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4gyp9v0e93o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>军事, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>U.S. launches second day of Iran strikes. And, World Cup facts to know before kickoff</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>美国连续第二天空袭伊朗；世界杯在墨西哥城开幕，紧张局势威胁活动。</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/g-s1-127423/up-first-newsletter-us-iran-war-inflation-rates-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】筑牢地下管网 让城市“里子”更扎实</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>国家投入1600亿元超长期特别国债，推进城市地下管网更新改造。</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDE1QQWNIueqRCsSoj8tYxv260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Weight-loss drug Wegovy to be available in pill form in UK for first time</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>减肥药Wegovy将在英国首次以药片形式提供，制造商称每日药片比每周注射更方便。</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9d2pl10lqzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Japan reactor restart sparks fresh fears over nuclear waste storage</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>日本重启核反应堆，引发核废料储存空间不足及处置计划缺失的担忧。</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/g-s1-127439/japan-reactor-restart-sparks-fresh-fears-over-nuclear-waste-storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>[视频]美军称完成对伊朗新一轮打击 伊朗称打击美军基地重要目标</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>美军称完成对伊朗新一轮打击，伊朗袭击美军基地并宣布关闭霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEcoJ0Wyk6BtNM63MhrB9D260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>以军袭击黎南部；欧洲视美国为盟友比例降至11%；美国5月CPI同比涨4.2%。</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEuarEieMPSWaOzULLlOag260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>El Niño under way and threatens weather extremes, scientists say</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>美国科学家宣布厄尔尼诺现象已正式形成，或将引发极端天气。</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c75ylx7g00xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Nigeria evacuates citizens from South Africa as anti-migrant sentiment rises</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>尼日利亚从南非撤离公民，因反移民情绪上升，继多国之后采取行动。</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq512vgyzl9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Number of people forced to flee their homes has dropped, U.N. report finds</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>联合国报告称全球被迫逃离家园人数下降，难民返乡人数创新高，但部分非自愿。</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/nx-s1-5850270/number-of-people-forced-to-flee-their-homes-has-dropped-u-n-report-finds</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】徐淙祥：多种粮 种好粮</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>74岁老党员徐淙祥扎根田间，钻研科学种田，带领乡亲致富。</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/11/VIDEZyg0R9C50wLKQQxqcpQi260611.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>The furious dispute over what caused Air India flight 171 to crash</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>关于印度航空171航班坠毁原因的激烈争议持续，最终调查结论尚未公布。</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwyk9exxp2qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Police officer, 19, dies from crash injuries</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>一名19岁女警Jess Turnbull因车祸受伤去世，警长称其职业生涯和生活本有光明前景。</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c621l2nkz4ko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>'Mum was killing me': England's Declan Rice on sunburn for his World Cup photoshoot</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>英格兰中场德克兰·赖斯因世界杯宣传照晒伤，笑称妈妈“差点害死我”，球员努力适应炎热天气。</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cq61l6d870vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Greetings from a Seoul museum, where Buddhist masterpieces offer calm away from city bustle</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>首尔国家博物馆的静思室展出韩国国宝级金铜菩萨雕像，提供宁静体验。</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/g-s1-126207/korea-seoul-national-museum-room-of-quiet-contemplation-bodhisattavas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-12
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1222"/>
+  <dimension ref="A1:F1251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39541,6 +39541,934 @@
         </is>
       </c>
     </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260612 19:00</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>缅甸总统将访华；井冈山精神引领发展；社会融资存量458万亿；约谈7家火车票平台。</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEGURMPgkG2APq52hHoYp3260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 缅甸总统将对中国进行国事访问</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>应习近平邀请，缅甸总统敏昂莱将于6月15日至19日访华。</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDE1PPVkNxiLRQjymElMRRr260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>[视频]【牢记初心使命 奋进复兴征程】跨越时空的井冈山精神照亮革命老区高质量发展新路</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>井冈山精神传承不息，推动革命老区高质量发展。</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEovgOUCZPmsW1MnbyuXm5260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际同新加坡国会议长会谈</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>赵乐际同新加坡国会议长会谈，加强立法机构等合作。</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEURUt46jjJzHVmfpPCgnQ260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见新加坡国会议长</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>韩正会见新加坡国会议长，深化中新全方位合作。</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEY9V6Z3tK43dxNEUit4cl260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Discovery of €1.2m jewellery prompts fresh probe into former Spanish PM</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>西班牙前首相因涉嫌未支付珠宝进口关税被调查。</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjeg9p1xqdwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Defence row exposes tensions over how to keep UK safe</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>前国防大臣称英国防务投资计划远未达标，暴露分歧。</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8d2q84y1gno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Ousted South Korean President Yoon given prison term for drone flights over Pyongyang</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>韩国被罢免总统尹锡悦因2024年派无人机飞越平壤加剧紧张被判30年监禁。</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/12/nx-s1-5856122/ousted-south-korean-president-yoon-prison-drone-flights-pyongyang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>[视频]【凝心聚力 真抓实干 奋力实现“十五五”良好开局】科技赋能福建新能源产业建设 云南加快推进“绿电+先进制造”深度融合</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>福建、云南科技赋能新能源，推进绿电与先进制造融合。</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEqmJIitvbVGOzMohdfs8U260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>[视频]5月末社会融资规模存量458.81万亿元</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>5月末社会融资规模存量458.81万亿元，货币增速高于GDP。</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDE5GWRvcF3YCLmZv21zNYL260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】织密全域物流网 畅通经济大动脉</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>我国加速建设内河水运物流网，通过支线航道升级补齐短板，降低物流成本。</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEKO8sNHNNYyPlnjhEy1un260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>大湾区前5月对APEC经济体进出口增长；个人信息保护报告发布；非遗购物月启动。</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDE81blwzh2shM33oAvtAwM260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>[视频]市场监管总局等部门约谈7家涉火车票销售第三方平台</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>市场监管总局约谈7家火车票平台，规范购票行为。</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEtAtjjp36y5eTxGJVDsyA260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国小麦收获过八成 夏播进入高峰</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>全国小麦收获进度过八成，夏播进入高峰，智能农机助力抢收抢种。</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEsGhjIzUCDO9Gz8Y7TqoG260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>[视频]我国不断完善以失能老人照护为重点的基本养老服务体系</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>我国完善失能老人照护体系，发放消费补贴并建立长期护理保险制度。</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEr3Er1py3Wgpywc6uLYcg260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Ministers want 60% of children walking or cycling to school by 2035</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>英国目标2035年60%儿童步行或骑车上学，将建安全通道。</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3wyezwly69o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>[视频]美称美伊或将签署协议 伊称美方不断改变立场影响进程</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>美称与伊朗或将签署协议，伊方指美方立场矛盾影响进程，美袭击油轮致印度船员死亡。</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEERxwMtSlsvVx1G1shLk1260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>欧洲央行近三年来首次加息；全球流离失所者超1.17亿；美中西部遭强风暴。</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEjEVjPriR7NihJmSzflFD260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Tehran says 'nothing' finalised after Trump claims deal to end Iran war near</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>伊朗否认特朗普所称的结束战争协议，称报道是“猜测”。</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78y6w78828o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>London council takes possession of property linked to Sierra Leone's First Lady</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>伦敦南华克议会接管与塞拉利昂第一夫人相关的房产。</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyxkeny8x6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>国际, 政治, 文体</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Trump cancels further Iran strikes. And, U.S. men's soccer takes on Paraguay</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>特朗普取消对伊朗进一步打击，称和平协议将很快达成，但伊朗称尚未定案。美国男足今日迎世界杯首战。</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/12/g-s1-127711/up-first-newsletter-iran-peace-national-intelligence-director-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Trump now says a peace deal will be announced 'soon,' cancels further strikes</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>特朗普称和平协议将很快宣布并取消进一步对伊打击，此前其言论持续升级。</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/nx-s1-5854970/trump-iran-peace-deal-cancel-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>[视频]第48届世界技能大赛将于9月22日至27日在上海举办</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>第48届世界技能大赛将于9月在上海举办，设64个竞赛项目，中国将派71名选手参赛。</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/12/VIDEVbx7FPa2ZBHAcfdDhMf8260612.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>More time needed for deadly Air India crash inquiry, officials say</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>印度航空致命空难调查需更多时间，已获重大进展。</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cnv93899vzqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Grooming survivors left with criminal records still being failed, BBC told</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>性侵幸存者因儿童时被起诉留犯罪记录，报告称仍被忽视。</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cly7jjq8nr1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>The Teddy Bear Doctor treats stuffies in need of care</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>加拿大女子在家中开设“泰迪熊医院”，为破损玩偶提供修复与关爱。</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/11/nx-s1-5777629/the-teddy-bear-doctor-treats-stuffies-in-need-of-care</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Tributes paid to David Hockney, a 'giant' and 'true icon' of British art</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>英国著名艺术家大卫·霍克尼逝世，享年88岁，被视为英国艺术界巨匠。</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgjxdr27z4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Taylor Swift makes tearful 21-minute speech as she joins Songwriters Hall of Fame</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>泰勒·斯威夫特含泪演讲21分钟，入选创作名人堂。</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yzxd0g833o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>She waited decades for Scotland to make the World Cup. At 93, she'll cheer in person</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>93岁苏格兰球迷莫伊拉·布朗将在波士顿现场观看女足世界杯，自称最幸运的人。</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/12/nx-s1-5842854/scotland-world-cup-tartan-army-fans</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-13
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1251"/>
+  <dimension ref="A1:F1284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40469,6 +40469,1062 @@
         </is>
       </c>
     </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260613 19:00</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道文化保护、海峡论坛、抗战精神、海洋生态、铁路旅游融合、人才下乡、算力网及国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEZpZAyP6qk0oSOsNtETif260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>[视频]第十八届海峡论坛大会在厦门举行 王沪宁出席并致辞</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>第十八届海峡论坛在厦门举行，王沪宁强调坚持一个中国原则，推动两岸关系和平发展。</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEWa6X5DghIcttU3tvs3ih260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】铭记烽火历史 传承抗战精神</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>回顾抗日战争历史，强调中国共产党中流砥柱作用，铭记烽火岁月，传承抗战精神。</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDE9DMCbYAsrAj9qu4D2yMx260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Are the Downing Street dominoes about to fall?</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>国防大臣希利辞职，对英国首相造成重大打击。</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c6213rkyp3lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Trump travels to France for the 52nd G7 Summit</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>特朗普赴法参加G7峰会，伊朗战争持续成焦点。</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/13/nx-s1-5854957/trump-travels-to-france-for-the-52nd-g7-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>[视频]多项措施促进铁路与旅游融合发展</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>我国推动铁路旅游融合，改造基础设施、开发主题专列、出台优惠票价，激发消费潜力。</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEAf85dU30QFoXhspobu4N260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Warner Bros $111bn sale to Paramount approved by US justice department</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>美国司法部批准华纳兄弟以1110亿美元出售给派拉蒙。</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjwgled9jxwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>[视频]【一线调研】算力网织就数字经济新底座</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>全国算力网建设加速，应对人工智能算力需求增长，西部地区数据中心密集建设。</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEiQpPXyiCg17EnyPsp5zH260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Anthropic suspends new AI tools over US government security concerns</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Anthropic因美国政府担忧网络安全和黑客风险，暂停新AI工具发布。</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c932g3v3e13o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Trump says U.S. military strike killed leader of Tren de Aragua gang</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>特朗普称美军打击委内瑞拉帮派头目，击毙其“著名领导人”。</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/12/nx-s1-5856611/u-s-military-kill-leader-tren-de-aragua</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>[视频]我国海洋生态保护修复取得新成效</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>我国海洋生态保护修复成效显著，多个海湾水质改善，珍稀物种栖息地得到有效保护。</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEXMUIkOyeXFMa50pmU6bA260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>[视频]各地推动人才下乡 助力乡村振兴</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>各地推行人才下乡政策，吸引青年回乡创业，提供孵化培训，助力乡村振兴。</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEN242L4srTaMa5nugaqIr260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>[视频]伊朗外长披露伊美谅解备忘录草案部分内容</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>伊朗外长披露伊美备忘录草案内容，包括结束冲突、解除封锁等，但尚未最终签署。</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEllvOS5UjeFyWrMW3bZs3260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>黎以新谈判将涉撤军；古巴谴责美国石油封锁；南极半岛出现异常高温。</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEx7Hc2xZTzj1tAC1NqqMr260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Israel carries out air strikes on Lebanon, state media says, as Iran claims deal with US near</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>以色列空袭黎巴嫩，伊朗称与美即将达成结束冲突协议。</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c39y02x98k8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>国际, 政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Switzerland to vote on plan to cap population at 10 million</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>瑞士将公投限制人口不超过1000万的“可持续倡议”。</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx23kz7e76po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>US kills leader of Venezuela's Tren de Aragua gang in airstrike, Trump says</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>特朗普称美军空袭杀死委内瑞拉Tren de Aragua黑帮头目。</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp36z37knlko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Watch: Why is Trump not at the World Cup?</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>北美三国领导人为何均缺席本届世界杯开幕式？</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/ced48dv99lvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>国际, 社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>The trauma and hope behind Haiti's rare World Cup appearance</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>海地52年后重返世界杯，饱受冲突的国家充满希望。</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c23yvvv7kr3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Pope Leo XIV's flight home from Spain was grounded so the king came to his aid</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>教皇专机因故障停飞，西班牙国王提供私人飞机相助。</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/13/nx-s1-5856981/pope-leo-flight-grounded</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】守护文化瑰宝 赓续中华文脉</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>习近平总书记强调文化遗产保护，我国推进系统性保护，廊桥等古迹实现主动预防与数字化保护。</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEmPZS8cfKWiHA1rcG1cG6260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>社会, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>文化和自然遗产日武汉主场活动举行；多部门推动新能源重卡；四部门整治农村出行安全；网信办设AI举报专区。</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEuYUUR0ZM1sRNcIGqw9dy260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Married at First Sight Australia stars not told partners had drug and violence convictions</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>《澳大利亚一见钟情》嘉宾称不知对方有毒品和暴力前科。</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clypy0ndvjlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>David Hockney depicted a 'peaceful, gay paradise' when homosexuality was a crime</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>画家大卫·霍克尼在同性恋非法时期，通过艺术歌颂同性关系打破禁忌。</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpq393dz535o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Royal Family watch Red Arrows flypast on Buckingham Palace balcony</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>王室成员在白金汉宫阳台观看红箭飞行表演，庆祝国王官方生日。</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn07y41kn2wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>In pictures: Trooping the Colour marks King's official birthday</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>国王和王后乘车前往阅兵场，参加庆祝国王官方生日的皇家阅兵仪式。</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpv3mmlg872o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Rugby star Sinfield and authors Blackman and Donaldson lead honours list</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>橄榄球星辛菲尔德及两位女作家获授勋爵位或女爵位。</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4gyx4dnr21o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Staying up to watch the match? Here's how to survive an all-nighter</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>熬夜看球指南：如何为足球比赛通宵做好准备。</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3wyel830w8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>'It's all they're talking about': Scotland gripped by football fever</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>苏格兰时隔28年再战世界杯，民众陷入足球狂热。</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78ydv8er7no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>[视频]文化和自然遗产日</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>新闻联播展示中华文化和自然遗产之美。</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/13/VIDEf9ZwomiaXPVDU3nDRg3B260613.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Niagara Falls: Is there a better spot to watch a World Cup game?</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>球迷在尼亚加拉大瀑布参加美加队世界杯揭幕战观赛派对。</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c62132n53exo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Superstar in Spain, doubted in Brazil: Will Vinicius convince a nation?</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>巴西球星维尼修斯需在世界杯上赢得本国球迷的心。</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c0l2rek0dj4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>体育, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>The costs and challenges facing the 2026 World Cup</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>2026年世界杯面临高温、成本、环境影响和旅行限制等挑战。</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c24ynjvm43qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-14
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1284"/>
+  <dimension ref="A1:F1317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41525,6 +41525,1062 @@
         </is>
       </c>
     </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260614 19:00</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>本期《新闻联播》涵盖红色传承、两岸融合、夏收夏种、铁路货运、公积金调整、北京水生态、党员治沙及国际新闻等。</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEjT8moOsE3WV2YaMrKml2260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>[视频]【牢记初心使命 奋进复兴征程】赓续红色血脉 走好新时代长征路</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>贵州遵义传承遵义会议精神，红色宣讲员活动火热进行，激励老区高质量发展。</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDE6hoSwdflaOTeJ1rAaWzq260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁出席两岸融合发展示范区建设专题推进会</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>王沪宁出席两岸融合发展示范区推进会，强调政策创新与台胞福祉。</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEUikHa4GfISlaWC1NkqwD260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>政治, 文体</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>'Boyfriend duties call,' Trudeau says after skipping Canada match to watch Perry</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>特鲁多看演唱会未观赛，称“男友职责”，女友跑下台与其亲吻。</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cly9eljexnno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Tech firms had 'enough time' says Nandy, ahead of social media announcement</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>英国首相预计周一宣布保护青少年上网措施。</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8jyp78mklo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>政治, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Britain detains sanctioned oil tanker believed to be linked to Russia's shadow fleet</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>英国扣留一艘疑似俄罗斯影子舰队运油船，涉嫌违反制裁。</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/14/nx-s1-5857587/britain-detains-sanctioned-oil-tanker-believed-linked-to-russias-shadow-fleet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>[视频]前5个月铁路客货运量多项指标创新高</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>前5个月铁路客货运量多项指标创新高，发送旅客19.69亿人次，货物16.7亿吨。</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEMxc1gveBNmwl6soRZ9KF260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>经济, 民生, 文体</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>六部门印发金融数据分类指南；我国首次开展蔬菜纯电农机测评；世界献血者日举行活动；上海国际电影节开幕。</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDE6Yrx1JhnDltyGTdBJAvR260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Why the US economy keeps defying the odds</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>美国经济为何在全球冲击下持续优于其他同行？</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy031el03po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>US kills leader of Venezuela's Tren de Aragua gang in air strike, Trump says</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>特朗普称美国空袭击毙委内瑞拉“阿拉瓜火车”黑帮头目。</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp36z37knlko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Royal Marines board Russian shadow fleet oil tanker in English Channel</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>英国皇家海军与犯罪调查局登检英吉利海峡疑似俄“影子舰队”油轮。</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyek039l2vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】各地做好抢收抢种 筑牢丰收基础</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>各地抢收夏粮并抢种秋粮，智能农机助力，全国已收获夏粮2.88亿亩。</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEzpjJk48TvP3nSyCmANVR260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>[视频]各地积极调整优化住房公积金政策</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>超60城优化公积金政策，拓展提取范围至装修、适老化改造等，并推进灵活就业人员缴存。</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEptsqu81XHEixiw3Amwec260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>[视频]建设“清水”北京 享受“亲水”生活</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>北京修复河湖生态，永定河连续六年通水，滨水慢行系统超1000公里。</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEKwwNOdkfHTIYaWCvC0uB260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>[视频]美称14日与伊朗签协议 伊朗称签署时间待定</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>美称14日与伊朗签协议并开放霍尔木兹海峡，伊方否认签署时间，以色列媒体称协议危及以安全利益。</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDE5odF6sIDejk8PFl0drZo260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>以军打击黎贝鲁特真主党目标；美海军“大黄蜂”战机坠毁引发火灾，飞行员弹射逃生。</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEyitWBM1RclslXsBeG3U4260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Trump says US-Iran deal to be signed on Sunday as Tehran casts doubt on timing</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>特朗普称美伊协议周日签署，伊朗对签署时间提出质疑。</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvglmn49xz0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Swiss voters reject 10 million population cap, early projections say</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>瑞士初步计票显示，55%选民反对将人口上限设为1000万的提案。</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20ygjem17zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Teen shot and buses torched in Manhattan after historic NBA win for Knicks</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>尼克斯队NBA夺冠后，曼哈顿发生骚乱，一名青少年被枪击、巴士被烧，至少63人被捕。</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8623n5pq2vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Fifa to pay Somali referee Artan full World Cup fee</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>被拒入境美国的索马里裁判阿尔坦，将获得国际足联全额世界杯酬金。</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c79y10r2plzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Armed men kidnap high-ranking security official in Haiti</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>武装分子在海地绑架一名高级安全官员，系该国近年最高级别绑架案。</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cz9le087414o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Trump says deal to end Iran war will be signed Sunday, as Iran disagrees on timing</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>特朗普称周日签署结束伊朗战争协议，伊方否认时间安排。</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/13/nx-s1-5857149/trump-iran-war-peace-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】侯贵：从沙海一棵树 到绿洲一片林</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>党员侯贵25年坚持植树治沙，将2000多亩沙地变成绿洲，种下30多万株树木。</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEQrNW5xRtgPhil2nZAZcX260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>[视频]【美丽中国行】泥巴山上架起“熊猫廊道”</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>四川泥巴山通过生态修复，为野生大熊猫架起“熊猫廊道”，连续七年记录到熊猫带崽影像，村民转变为生态导赏员。</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEqO0e62xgdID23x9B0wHx260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Tourist train overturns and injures 17 during Cártama tapas festival</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>西班牙小镇旅游列车在节日期间侧翻，17人受伤，无人重伤。</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c14yn10jzyeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Author Chimamanda Adichie accuses hospital of stalling review into son's death</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>作家阿迪契指责医院拖延调查其21个月大儿子在拉各斯医院的死亡。</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgk6jzkr0xvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】薪火相传 秦腔不老</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>秦腔作为西北戏曲代表，通过总台大剧《主角》热播引发关注，易俗社等传承机构推动戏曲在新时代焕发新生。</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/14/VIDEsOsVm3WrC9o9o6bUM5Qc260614.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Why Haiti v Scotland was antidote to the ills of world football</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>苏格兰队战胜海地队，报道称这是世界足球弊病的一剂解药。</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cdjkdmel292o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton wins first grand prix for Ferrari</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>汉密尔顿为法拉利赢得首个大奖赛冠军，领跑者安东内利退赛。</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/formula1/articles/cn8k5n737p4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>The 20-year-old who stole the show on Scotland's World Cup return</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>20岁小将甘农-多克在苏格兰世界杯首秀中表现抢眼，助队取胜。</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/clyrepwp0gno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Jubilation as Scotland fans celebrate win</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>苏格兰球迷清晨聚集酒吧庆祝国家队战胜海地队。</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c78yxr7dl3mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Smaller than Isle of Man &amp; huge Dutch influence: Curacao making history</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>面积小于马恩岛的库拉索岛，受荷兰影响深，正创造世界杯历史。</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cn7p0d1mdrzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Two men charged over theft of England World Cup kit</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>两名男子被指控在堪萨斯城训练基地盗窃英格兰队世界杯装备。</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cm2r35lk8ejo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-15
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1317"/>
+  <dimension ref="A1:F1346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42581,6 +42581,934 @@
         </is>
       </c>
     </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260615 19:00</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>新闻联播报道民生福祉、国务院学习、中越通话、党建座谈、麦收夏播、节能降碳等多项内容。</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEpVsqrt8BBfLrRi9n8UmV260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>[视频]李强主持国务院第二十次专题学习</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>李强主持国务院专题学习，强调强化主体功能区战略，促进区域协调发展。</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDESzdF0kyGgCV7JWyUqJyO260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>[视频]李强同越南总理通电话</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>李强同越南总理通电话，就加强合作、推动中越命运共同体建设达成共识。</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDE25rpERlCJeUWyjpTnol0260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>[视频]全国党建工作座谈会在京召开 蔡奇出席并讲话 李希出席</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>全国党建工作座谈会召开，强调习近平党建思想是新时代党建根本遵循。</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEy87DOkjSyj01JgqGOBXC260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>[视频]中央组织部从代中央管理党费中划拨4.27亿元用于“七一”前夕开展走访慰问活动</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>中央组织部划拨4.27亿元党费，用于七一前夕走访慰问党员和群众。</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEMX8KOOLSRsPvV2EqsJfn260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>[视频]中央纪委办公厅公开通报五起政绩观偏差典型案件</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>中央纪委通报五起政绩观偏差典型案件，涉及违规举债、搞政绩工程等问题，要求严肃纠治。</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEz4FxAxCHanCSVRDYtzl0260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Palestine Action ban is lawful, Court of Appeal rules</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>上诉法院裁定禁止巴勒斯坦行动组织合法。</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4gy927jx88o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>政治, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>U.S. and Iran announce a deal to end the war and reopen the Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>美伊宣布达成结束战争并重开霍尔木兹海峡的协议，但关键问题未解决。</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/15/nx-s1-5858590/us-iran-deal-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>[视频]九大重点行业启动节能降碳改造攻坚行动</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>五部门启动九大重点行业节能降碳改造攻坚行动，目标到2028年累计节能量超1亿吨标准煤。</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEMMCbtwKKpOz7RvPtgROa260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>经济, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>[视频]多元场景引客来 入境游热度攀升</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>今年前5月入境游持续升温，多元场景与便利政策吸引海外游客，外籍人员入境近1910万人次。</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEYSpe8a1Kuxo5iYDdgBBl260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>经济, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>国内联播快讯：节能宣传周启动、深圳港集装箱量创新高、春招提供1268万岗位、硅-28量产成功。</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEEIrTajFq2MQC3awRkNYN260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Social media ban - bold and blunt, but no silver bullet</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>社交媒体禁令虽严厉但非万能，专家讨论对青少年的影响。</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cddl65dp0rdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】持续增进民生福祉 托起百姓稳稳的幸福</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>习近平总书记强调民生为大，各地建设口袋公园等举措增进民生福祉。</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEDsqm8OKH46g8xcef5CUn260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国麦收接近尾声 夏播高效推进</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>全国麦收进度近九成，夏播高效推进，各地推广高效装备保障粮食生产。</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDE22j0umgZ6htzyLMlIMPw260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>[视频]“两重”建设推动一批民生工程落地实施</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>“两重”建设推动灌区改造、城市管网升级等民生工程，改善基础设施和公共服务。</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEe1jU2IYV1WHrQBAVkxH6260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>[视频]中蒙重大合作项目乌兰巴托中央污水处理厂正式启用</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>中蒙合作项目乌兰巴托中央污水处理厂启用，采用中国标准和技术，成为两国友谊标志。</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEDMvQ26ZNl0x2noxHjDHi260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>[视频]美称与伊朗达成协议 伊朗称伊美就结束战争达成谅解备忘录</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>美伊达成和平协议，霍尔木兹海峡将重新开放，伊朗承诺全面停战并开始后续谈判。</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/15/VIDEbXiVJLeRTOadAlJVP3lp260615.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Bowen: Iran deal ends Trump's war that revealed limit of US dominance</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>分析称伊朗协议结束特朗普战争，暴露美国主导地位局限，但双方立场未变，伤亡惨重。</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdr4x3vg347o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Norwegian crown princess's son found guilty of two counts of rape</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>挪威王储妃之子因两项强奸罪被判四年监禁。</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cly9d10l5p4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>MSF staff abused Sudanese refugees in sex-for-food scandal</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>无国界医生工作人员以性换取食物，虐待苏丹难民。</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c74ykjl8mx3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Russia was behind arson attacks targeting PM, BBC reveals</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>BBC揭露俄罗斯策划纵火袭击并利用虚假组织煽动紧张局势。</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8r2l352z2do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Former American businessman detained in Myanmar after alleged financial misconduct</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>美国商人卡斯蒂略因涉嫌金融不当行为在缅甸仰光机场被拘留。</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/15/g-s1-128147/former-american-businessman-detained-in-myanmar-after-alleged-financial-misconduct</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>国际, 政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Trump announces deal to end war in Iran. And, how to stay safe in deadly heat</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>特朗普宣布达成结束美伊战争的协议，并提醒极端高温下的安全措施。</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/15/g-s1-128145/up-first-newsletter-iran-war-g7-summit-ufc-fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Inside Ebola country: NPR reports from eastern DR Congo's outbreak zone</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>刚果（金）东部埃博拉疫情肆虐，恐惧蔓延超过信息传播，医院变隔离点。</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/15/nx-s1-5856414/ebola-congo-bunia-health-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Brazil woman dies after rope-jumping instructors fail to attach cord</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>巴西一名女性因蹦极教练未系绳索而坠桥身亡，三人被捕。</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c5yz4xelnveo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Teacher guilty of sexually abusing and murdering adopted baby</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>教师因性侵并谋杀领养婴儿被判有罪。</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgld0vywpmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Henry Nowak killer's sentence referred to Court of Appeal under unduly lenient scheme</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>亨利·诺瓦克谋杀案嫌犯刑期被提交上诉法院复审。</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8721y4341qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>Britain will ban under-16s from social media apps, including TikTok and YouTube</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>英国将禁止16岁以下青少年使用TikTok、YouTube等社交媒体平台。</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/15/nx-s1-5858644/britain-social-media-ban</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>South African jazz legend Abdullah Ibrahim dies at 91</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>南非爵士乐传奇人物阿卜杜拉·易卜拉欣去世，享年91岁。</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy5vngrq3q5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-16
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1346"/>
+  <dimension ref="A1:F1376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43509,6 +43509,966 @@
         </is>
       </c>
     </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260616 21:00</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>习近平举行仪式欢迎缅甸总统访华，并举行会谈；发布教育科技人才重要文章；报道多项国内政治经济活动及经济数据。</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEf49rMqSUbPphPZRdVLCj260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎缅甸总统访华</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂举行仪式，欢迎缅甸总统敏昂莱访华，21响礼炮，检阅仪仗队。</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEe9WYvZ2nFT63mW2s91Ck260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>[视频]习近平同缅甸总统会谈</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>习近平同缅甸总统会谈，强调中缅胞波情谊，推进中缅经济走廊建设，支持缅方发展与重建。</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEPwCzg5ZcIVVzWYriPPfR260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>[视频]《求是》杂志发表习近平总书记重要文章《一体推进教育科技人才发展》</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>《求是》发表习近平重要文章，强调教育、科技、人才一体化发展，支撑全面建设社会主义现代化国家。</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEUA3KC8odKK9Iaxv8iBT3260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>[视频]以习近平党建思想为指引 推动党的事业不断开创新局面</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>全国党建工作座谈会对学习贯彻习近平党建思想作出部署，引发热烈反响，强调以此推动党的事业新局面。</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDELSZYbUg7ZeMUUMo1lxmN260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>[视频]新华社综述：不断开辟百年大党管党治党、兴党强党新境界——深入学习领会习近平党建思想</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>新华社播发综述，深入阐述习近平党建思想，强调管党治党、兴党强党的新境界。</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDECSZVnKSpx6h3K9Spl3Qs260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>[视频]李强会见缅甸总统</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>李强会见缅甸总统敏昂莱，表示深化中缅贸易投资、执法安全等领域合作，推进经济走廊建设。</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEl8fqrhjBAfl5hR2ZfWCu260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际主持召开十四届全国人大常委会第六十八次委员长会议 决定十四届全国人大常委会第二十三次会议6月23日至26日在京举行</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>赵乐际主持委员长会议，决定十四届全国人大常委会第二十三次会议6月23日至26日举行，将审议多项法律草案。</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEYVYPacUSUVp90tQrQNQV260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见缅甸总统</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>赵乐际会见缅甸总统敏昂莱，称愿深化互利合作，丰富命运共同体内涵。</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDE7KL8gmZEeUiNUXR6Z4Io260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见尼泊尔外交部长</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>王沪宁会见尼泊尔外长，强调深化政治互信与务实合作。</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDE33QByEfB4xoDEHhlFuR6260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>What UK social media ban means for gaming and YouTube</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>英国社交媒体禁令对Roblox、YouTube和WhatsApp等平台的影响尚不明确。</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9824zvpz9po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>[视频]韩正出席第七届跨国公司领导人青岛峰会开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>韩正出席跨国公司领导人峰会，提出四点合作建议，强调扩大开放。</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEuUhIxSG6ntTlK4Ijs8nB260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>[视频]5月份我国经济总体平稳 持续向新向优</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>5月国民经济总体平稳，工业、服务业稳中有升，就业物价稳定。</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDE4dCI7IIqWTb6AlJrfwLS260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>经济, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>前5月综保区进出口增长27.1%；市场监管总局严惩失信；教育部系统升级；光热电站开工。</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEFiHxOQUtxMPp8piSPzOl260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>UK forces face operational cuts without more cash, defence chief warns</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>英防务高官警告：缺乏资金将导致军队作战能力削减。</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20ydx06ym2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>UK investigating reports Russian warship fired warning shots near yacht in English Channel</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>英方调查俄军舰在英吉利海峡向游艇鸣枪示警事件。</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20yzm84r7lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Tehran selling deal with US as victory – but for Iranians it was necessity</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>伊朗向民众宣称与美国达成协议是胜利，但民众更关心物价和战争恐惧。</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4rwzxvl8ko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Fragile quiet in Lebanon as US-Iran truce leaves unanswered questions</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>美伊停火协议下黎巴嫩暂获平静，但民众怀疑以黎冲突能否终结。</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgepl5gdp1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Russian artist and Putin critic shot dead in Poland</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>俄罗斯艺术家、普京批评者在波兰遭枪杀。</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyrzd5g6k2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Three reasons ships are not going through the Strait of Hormuz yet</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>专家称安全、水雷和通行费阻碍船只恢复通行霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4rw784nj2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>In Albania, anger grows against the government for supporting a Kushner-linked luxury resort</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚民众抗议政府批准库什纳关联的豪华度假村项目。</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/16/g-s1-128162/albania-resort-protests-kushner-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>国际, 政治, 文体</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>How Israel could complicate Iran peace negotiations. And, World Cup highlights</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>以色列被排除在美伊协议外，可能破坏伊朗和平谈判。世界杯精彩开局。</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/16/g-s1-128341/up-first-newsletter-iran-israel-g7-primaries-luigi-mangione</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Israeli ambassador to U.S. says Israel is 'not going to withdraw from South Lebanon'</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>以色列驻美大使称以色列不会从南黎巴嫩撤军。</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/16/nx-s1-5858937/israels-ambassador-to-the-u-s-talks-about-u-s-iran-deal-to-end-war</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>G7 leaders meet for first full day of summit Tuesday</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>G7峰会首日，特朗普会见各国领导人及乌克兰、卡塔尔、阿联酋首脑。</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/16/nx-s1-5859260/g7-leaders-meet-for-first-full-day-of-summit-tuesday</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>G7 allies scramble to put Ukraine back atop Trump's agenda as war drags on</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>G7盟友试图让乌克兰议题重回特朗普议程，伊朗冲突抢占了关注度。</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/16/g-s1-128325/g7-leaders-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行文旅领域代表见面会，讲述奋斗故事，弘扬文化自信。</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDE0XDmm7vmKHVw2bgVNBeh260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>[视频]中央宣传部 应急管理部联合发布“最美应急管理工作者”</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>中央宣传部、应急管理部联合发布9名“最美应急管理工作者”。</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEDldHd9AMHJcTsmvp1JnU260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>France's oldest female detainee, 79, goes on trial for in-law's grisly murder</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>法国79岁女囚因1995年塞纳河碎尸案受审，DNA证据近期才将其关联。</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy498llene1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>[视频]第十九届中华图书特殊贡献奖颁奖仪式在京举行</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>第十九届中华图书特殊贡献奖在京颁奖，表彰15位外国作家、翻译家等。</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/16/VIDEbYA7YLQqTXaOkmFaeCms260616.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>文体, 经济</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>'Daylight robbery but worth it' - what fans are spending on World Cup</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>美加墨球迷斥巨资购买世界杯门票、交通和住宿，认为虽贵但值得。</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy73xe2006po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-17
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1376"/>
+  <dimension ref="A1:F1406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44469,6 +44469,966 @@
         </is>
       </c>
     </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260617 19:00</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>新闻联播报道了习近平指示、党建思想、就业规划、夏粮丰收等多项国内要闻。</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEz5W4hdbsZtWPAcJt5TQY260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>[视频]习近平对常态化做好东西部协作工作作出重要指示强调 总结运用闽宁协作等有益经验 不断增强区域发展协调性 推动全体人民共同富裕迈出坚实步伐</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>习近平指示常态化做好东西部协作，总结闽宁经验，推动共同富裕。</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEPgIXw4T4UtupJD1nA16B260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>[视频]学习贯彻习近平党建思想 深入推进新时代党的建设新的伟大工程</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>学习贯彻习近平党建思想，深入推进新时代党的建设新的伟大工程。</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDE4HCh4ShrCXjsliOZwGe7260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：加强新时代党的建设的根本遵循——论学习贯彻习近平党建思想</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>人民日报发表评论员文章，强调习近平党建思想是加强党的建设的根本遵循。</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEZHlwzk4gaAenkag5dZ0Q260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>政治, 文体</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>[视频]中国戏剧家协会第十次全国代表大会、中国民间文艺家协会第十一次全国代表大会、中国书法家协会第九次全国代表大会在北京召开</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>中国戏剧、民间文艺、书法家协会全国代表大会在京召开，要求担当文化使命。</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDErqHdEa0O7nWkA4Ochd35260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>PM warns Burnham against immediate leadership challenge if he wins by-election</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>英首相警告伯纳姆若赢得补选勿立即挑战领袖地位。</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn4dj7n83yqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>Taiwan says Chinese pressure over the island is the "new normal"</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>台湾称中国大陆施压已成“新常态”，学者在肯尼亚被扣留。</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/17/g-s1-128550/taiwan-says-chinese-pressure-over-the-island-is-the-new-normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Trump to face questions at G7 press conference. And, Tuesday's primary results</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>特朗普将在G7记者会上答问并关注初选结果。</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/17/g-s1-128547/up-first-newsletter-tentative-iran-ceasefire-agreement-g7-trump-kevin-warsh-georgia-primaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Trump expected to face questions about Iran war as he wraps up G7 summit</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>特朗普在G7闭幕记者会面临伊朗战争协议与乌克兰援助质疑。</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/17/nx-s1-5860655/trump-expected-to-face-questions-about-iran-war-as-he-wraps-up-g7-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>[视频]多项金融开放举措今天发布</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>多项金融开放举措发布，涉及央行、证监会、外汇局等多项改革。</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEqIkyFiOwXcn1YjW4GfRk260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>财政部在港发行150亿元国债；三部门部署端午安全；外卖补贴规范征求意见。</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEREzuma1Yr9jB0TcbsSlJ260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>BBC announces 550 job cuts as first part of £500m savings plan</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>BBC为节省5亿英镑宣布裁减550个岗位，首批200个。</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgmqrrlej5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>军事, 政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Trump's Iran agreement dominates G7 but big questions remain</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>美以主导的伊朗战争重创全球经济并损害特朗普国内支持。</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/17/nx-s1-5860782/trumps-iran-agreement-dominates-g7-but-big-questions-remain</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《实施就业优先战略“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>国务院印发“十五五”就业规划，聚焦高质量充分就业。</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEMG3LNkeduAfB0rjDPCsJ260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国夏粮丰收成定局</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>全国夏粮丰收已成定局，智能化农机助力减损增产。</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEP8FUsYtJwvCJSds0y6a0260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>[视频]我国荒漠化防治取得显著成效</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>我国荒漠化治理成效显著，沙化土地面积年均缩减1000万亩。</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEjy9Bv0Q5hyt3SRoHjDUh260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见美国前运输部长</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>国家副主席韩正在北京会见美国前运输部长赵小兰。</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEY2QMZ4saqcrulma255Ki260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>[视频]中国政府发布关于全球治理的白皮书</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>中国政府发布全球治理白皮书，阐述中国理念与行动。</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEwAW649qA4MrdYGz7WkVi260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称第二阶段谈判将聚焦核问题及解除制裁 美称与伊朗谈判已进入第二阶段</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>美伊谈判将进入第二阶段，聚焦核问题及解除制裁，伊朗油轮驶出封锁线。</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEDPekdJJvElS8LzNEflJW260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>国际, 军事, 科技</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>俄舰在英吉利海峡向逼近游艇开火示警；德国警告依赖美AI模型存风险。</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDESKkEKrsc3xXxo6bKA7ma260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>Iran sends tankers loaded with oil past US military blockade</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>三艘伊朗油轮载原油突破美军在阿曼湾的封锁线。</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cpq37yxexd9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>Status quo at Jerusalem's holiest site under threat as Israeli nationalists flout rules</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>以色列民族主义者无视规则，挑战耶路撒冷圣地共享现状。</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy0nlv90jno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>Search for six-year-old Ebola patient after armed men storm DR Congo hospital</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>武装分子袭击刚果（金）医院，搜寻6岁埃博拉患者。</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgep4l397eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>Israel launches fresh strikes on Lebanon despite Trump criticism</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>以色列对黎巴嫩发动新袭击，特朗普批评其需更负责。</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c7vyn17g832o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Harry and Meghan to bring children to UK next month</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>哈里和梅根下月将首次带子女回英国，时隔四年。</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce3eqkzy2z4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>国新办举行见面会，四位代表分享文明乡风建设故事。</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDEqbb9NkqGZptlMjK8jJkR260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>Serial killer who murdered eight women in Long Island town imprisoned for life</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>长岛杀害8名女性的连环杀手被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyw29kvlydo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>Greetings from Maputo, Mozambique's capital, shaped by a modernist architecture</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>莫桑比克首都马普托因建筑师潘乔·格迪斯留下现代主义印记。</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/17/nx-s1-5853087/maputo-mozambique-modernist-architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>[视频]第三十二届北京国际图书博览会在京举办</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>第三十二届北京国际图书博览会开幕，82国1700多家展商参展。</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/17/VIDE5FDWmdaFoBSg9LD4ZBQp260617.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>Baby blue tracksuits and no ties - what England's off-pitch looks say about the team</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>专家解读英格兰队世界杯场外时尚：蓝色运动服配无领带。</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9v2e8llnkwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-18
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1406"/>
+  <dimension ref="A1:F1436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45429,6 +45429,966 @@
         </is>
       </c>
     </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260618 19:00</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平回信老党员、党建思想通知、韩正会见外宾、两新资金下达等要闻。</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDECqvYWP6W8gh3Mz0hp3rX260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>[视频]习近平给新华社老党员张连生回信强调 传承红色基因 在新征程上书写优异答卷</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>习近平给102岁老党员张连生回信，强调传承红色基因，在新征程上书写优异答卷。</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEt6xBTw3MyCzErvk5LYYh260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>[视频]以习近平党建思想为指引 奋力谱写中国式现代化新篇章</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>党员干部表示以习近平党建思想为指引，奋力谱写中国式现代化新篇章。</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEahOL91Hsgg4tt4jI9OiD260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>[视频]中央党的建设工作领导小组印发《关于学习贯彻习近平党建思想的通知》</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>中央党的建设工作领导小组印发通知，要求深入学习贯彻习近平党建思想。</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDE1KWowMoBramwGEH5PG75260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：为发展马克思主义建党学说作出重大原创性贡献——论学习贯彻习近平党建思想</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>人民日报评论员文章：习近平党建思想为发展马克思主义建党学说作出重大原创性贡献。</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEdH5dU5Nkykl58HZyerE4260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>政治, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见加拿大、丹麦客人</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>韩正会见加拿大和丹麦客人，讨论经贸合作与健康中国建设。</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEaoMp2XchuY4nVMuiXKoV260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>政治, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>国内快讯：中央预拨1亿救灾资金；海南自贸港封关半年红利释放；西部陆海新通道进出口创新高；首个工业产品碳足迹数据库上线。</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDE5aqPwV13dbre1j1Hn1iQ260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>Hegseth renews Nato criticism and says US will review presence in Europe</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>美防长赫格塞斯再次批评北约，称将审查美国在欧洲的军事部署。</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3vy5l62622o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>Trump signs agreement with Iran. And, the president's approval hits record lows</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>特朗普与伊朗签署初步协议结束战争并开放霍尔木兹海峡，但支持率创新低。</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/18/g-s1-128755/up-first-newsletter-iran-agreement-jay-clayton-bill-pulte-trump-approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>[视频]加快下达“两新”项目资金 持续释放政策效能</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>国家发改委称6月底前下达今年全部2000亿元设备更新项目及第三批625亿元以旧换新资金。</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEeVaW4I6mzp2Pj1EvU2Ub260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>[视频]端午临近 节日市场供应丰富</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>端午临近，时令商品热销，各地推出文旅活动及惠民措施促消费。</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEJLWNmkgkJKLS5kXTfBV5260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>Report: Russia's nuclear-powered 'Skyfall' missile is dirty and dangerous</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>MIT研究称俄核动力‘天降’导弹危险且糟糕，但并非不可行。</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/18/nx-s1-5843252/russia-nuclear-powered-missile-burevestnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>Moscow residents complain of black rain after largest Ukrainian attack hits oil refinery</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>乌克兰大规模无人机袭击莫斯科东南部，炼油厂和购物中心起火，居民抱怨下黑雨。</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c98291g5rr1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>Gunmen attack Niger's biggest airport for second time in months</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>尼日尔最大机场数月内再次遭武装分子袭击，该国反恐已持续十年。</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cdx7krkdqeno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>Ukraine hits a Moscow oil refinery and other sites in a large-scale drone attack</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>乌克兰大规模无人机袭击莫斯科油厂等地，为冲突以来最大规模之一。</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/18/g-s1-128782/moscow-ukraine-drone-attack-russia-oil-refinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>Hegseth announces in Brussels a review of U.S. forces in Europe, and a 'NATO 3.0'</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>美防长抨击北约盟友，宣布审查驻欧美军并呼吁构建‘北约3.0’。</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/18/nx-s1-5862604/hegseth-nato-3-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>[视频]“在高质量发展中保障和改善民生”形势政策系列报告会首场报告会在北京举行</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>“高质量发展中保障和改善民生”系列报告会首场举行，聚焦交通强国建设。</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEZnECg56qATEvNvhC14z8260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>[视频]全国铁路端午假期运输今天启动</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>铁路端午运输启动，预计发送旅客8300万人次，精准投放运力。</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEa8vbfwKSUxEsVecxpOLh260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>[视频]美国总统和伊朗总统远程签署谅解备忘录 正式文本公布</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>美伊远程签署谅解备忘录，内容包括停火、重开霍尔木兹海峡等，巴基斯坦宣布生效。</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEYvASD3cuetQMYKxvKo8v260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>俄称控制顿涅茨克并击落180架无人机；巴勒斯坦谴责以色列扩建定居点；G7峰会第三次未发联合公报。</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEWxqirCiJekngdG9tqXC8260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>Bowen: US-Iran deal raises inescapable question of what the war was for</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>美伊协议引发疑问：伊朗政权不仅未被削弱，反而因战争更加强大。</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyegr2mp8jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>Why Iran believes deal with US leaves it stronger than before</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>伊朗认为当前美伊协议使其比战前更强，但即将面临更艰巨挑战。</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1428" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c932yqz8lggo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>'Do not travel' advice for Dubai dropped</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>美伊战争爆发后，数千英国人滞留中东，官方撤销旅行禁令。</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cddl29lg5gro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>For Lebanon, a U.S.-Iran agreement raises questions beyond Hezbollah</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>美伊协议影响黎巴嫩，前大使解析停火前景及真主党以外的变数。</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/18/nx-s1-5861723/us-iran-agreement-lebanon-reactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】林丹：一辈子做好居民的服务员</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>78岁老党员林丹扎根社区50余年，带领党员服务居民，成为居民的贴心人。</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1431" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEIL8NNNMjnesHYzwSVyGu260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>五位铁路工人代表在国新办见面会上分享开路先锋故事，展现奋斗精神。</t>
+        </is>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1432" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDE4t4utFmgpLqGYwZl7zXD260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>[视频]中国戏剧家协会 中国民间文艺家协会 中国书法家协会选举产生新一届领导机构</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>中国剧协、民协、书协选举产生新一届领导机构和主席。</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1433" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEyjfXABL5a74tHZcrheU6260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>[视频]总台推出特别节目 陪您共度端午假期</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>中央广播电视总台推出多档端午特别节目，陪伴观众共度佳节。</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1434" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/18/VIDEhYw42osNejSCoLi4UbWi260618.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>Man arrested on suspicion of attempted murder after boy injured in crocodile enclosure</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>一名男子因涉嫌谋杀未遂被捕，此前一名三岁男孩在鳄鱼池受重伤。</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1435" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czx50n2vj74o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>Teacher who murdered adopted baby son Preston Davey given whole life prison sentence</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>教师杰米·瓦利因长期性虐并杀害养子普雷斯顿·戴维，被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1436" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/czrx8gj112mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-19
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1436"/>
+  <dimension ref="A1:F1471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46389,6 +46389,1126 @@
         </is>
       </c>
     </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260619 19:00</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>新闻联播报道爱国教育、端午活动、客流高峰、新能源汽车下乡等国内国际要闻。</t>
+        </is>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDEyWcJOt9j24rnkbVy4ayu260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】弘扬爱国主义精神 奋楫民族复兴新征程</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>习近平总书记强调弘扬爱国主义精神，端午佳节传承爱国情，激励奋进新征程。</t>
+        </is>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1438" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDEacPrZWBztlp6zVRjVMNG260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：对强党强国具有重大现实意义和长远指导意义——论学习贯彻习近平党建思想</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>人民日报评论员文章强调习近平党建思想对强党强国意义重大而深远。</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1439" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDELjLpXjfdJDeHsqX3UNDy260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】新中国诞生 东方大国开启新纪元</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>回顾新中国诞生历程，中国共产党领导人民取得胜利，开启民族新纪元。</t>
+        </is>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1440" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDENZluNzD7qE9cL4QHfnKR260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>Zimbabwe MPs pass bill to extend president's time in power</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>津巴布韦议会通过法案，延长总统任期两年并取消直选。</t>
+        </is>
+      </c>
+      <c r="E1441" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20y15m0337o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>In Trump's shadow, Vance becomes face of Iran deal</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>万斯在特朗普阴影下成为伊朗协议代言人，引发2028年参选猜测。</t>
+        </is>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1442" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx23jr133lwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>Henry Zeffman: What does Keir Starmer do next after Andy Burnham's Makerfield win?</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>补选失利后，英国首相斯塔默的未来走向引发讨论。</t>
+        </is>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1443" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3ryp0nejdro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>Historic by-election win sends message to Labour and SNP, says Badenoch</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>苏格兰保守党自1973年来首次赢得补选，从苏格兰民族党手中夺回阿伯丁南部席位。</t>
+        </is>
+      </c>
+      <c r="E1444" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn8q4p34qg4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>Labour's Andy Burnham wins a special election, setting up a showdown with Starmer to lead Britain</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>英国工党伯纳姆赢得特别选举，有望挑战首相斯塔默的领导地位。</t>
+        </is>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1445" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/19/nx-s1-5864087/labour-andy-burnham-wins-special-election</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>[视频]跨国公司深耕中国市场 共享发展新机遇</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>跨国公司在华投资向高技术领域集聚，持续增资扩产，共享中国产业升级机遇。</t>
+        </is>
+      </c>
+      <c r="E1446" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDER9pgnwdMeU1MxYY24LR9260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>经济, 社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>新能源汽车下乡将启动，共155款车型；网信办整治账号名称乱象；动漫节金猴奖揭晓；端午期间长江中下游多雨。</t>
+        </is>
+      </c>
+      <c r="E1447" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDED3gAy5i0ilQ4q3Eaxrwa260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>Asia's richest man Ambani announces what could be India's biggest share sale</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>亚洲首富安巴尼宣布其电信公司可能进行印度最大规模股票发售。</t>
+        </is>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1448" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx2kerpkynko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>Plans to end gazumping with binding agreements in house sales shake-up</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>英国计划改革房产销售，引入具有法律约束力的协议以终止抢房现象，并提前要求卖家提供更多信息。</t>
+        </is>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c6216g52p8wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>[视频]【活力中国调研行】北京：一条连廊 连起产学研</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>北京中关村通过产学研连廊，培养AI人才，推动创新成果转化为产业优势。</t>
+        </is>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1450" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDEx7ELYLK0qItr3RJT8Ozr260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>U.S. strike on an alleged drug boat kills 3 in the eastern Pacific Ocean</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>美国在太平洋东部打击涉嫌运毒船，致3人死亡，累计已超211人。</t>
+        </is>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1451" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/19/nx-s1-5864084/us-strike-alleged-drug-boat-kills-3-eastern-pacific-ocean</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>[视频]假期首日客流现高峰 交通部门增运力</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>端午假期首日客流高峰，全国铁路预计发送1970万人次，交通部门增运力保障出行。</t>
+        </is>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDENvasJIYlXhW1iwFjF5Zg260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>Amber extreme heat warning issued as 35C heatwave approaches</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>英国发布琥珀色极端高温警告，周一周二气温将达35℃，影响健康并可能扰乱交通。</t>
+        </is>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1453" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/cz0jde5xkjvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>[视频]瑞士宣布今日比尔根山美伊谈判取消</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>美伊谈判因以色列袭击黎巴嫩取消；美以就黎南部军事存在分歧；美军解除伊朗海上封锁。</t>
+        </is>
+      </c>
+      <c r="E1454" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDE9pBkHnV0TQ0R2uu3wVwV260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>美国将审查欧洲军力部署，要求欧洲自负防务责任；日本核心CPI连续57个月上涨。</t>
+        </is>
+      </c>
+      <c r="E1455" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1455" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDELSqYuHL97Nqqzn7X1tHl260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>Italy's Meloni says Trump 'made up' story that she 'begged' him for photo at G7</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>意大利总理称特朗普编造其“乞求”合影故事，双方关系因对伊朗战争分歧而紧张。</t>
+        </is>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1456" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20y1ygn707o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>Six-year-old Ebola patient taken from DR Congo hospital found and 'doing well'</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>刚果（金）一名6岁埃博拉患者从医院被带走后已找到，目前状况良好。</t>
+        </is>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1457" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0qyg29wpk2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>Morocco captain Achraf Hakimi to stand trial for rape</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>摩洛哥队长阿什拉夫因2023年强奸指控将在法国受审。</t>
+        </is>
+      </c>
+      <c r="E1458" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1458" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c20y18z7le1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>UK actress charged with importing meth worth almost A$300m into Australia</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>英国女演员因涉嫌将320公斤冰毒伪装成木炭走私至澳大利亚被捕。</t>
+        </is>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1459" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ckg5nq0172no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>国际, 科技</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>US-Iran talks in Switzerland canceled. And, DHS to give police facial recognition app</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>美伊在瑞士的会谈取消；国土安全部计划向地方警察提供ICE人脸识别技术。</t>
+        </is>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/19/g-s1-129076/up-first-newsletter-vice-president-vance-iran-agreement-obama-presidential-center-judicial-system-dhs-facial-recognition</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>What you need to know about the preliminary U.S.-Iran agreement signed by Trump</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>了解特朗普签署的美伊初步协议内容及实现持久和平仍面临的挑战。</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1461" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/19/nx-s1-5863544/trump-us-iran-agreement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>Do Middle East nations still see the U.S. as a reliable ally?</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>探讨中东国家是否仍视美国为可靠盟友，专家接受采访分析。</t>
+        </is>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1462" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/19/nx-s1-5863043/do-middle-east-nations-still-see-the-u-s-as-a-reliable-ally</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>[视频]千舸竞 粽飘香 多彩活动共度端午</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>端午佳节各地举办龙舟赛、包粽子等多彩活动，传承传统文化，感受家国情怀。</t>
+        </is>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1463" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDECUHLkgs65WuGfmzj42vw260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>[视频]中国传统佳节·端午</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>端午佳节，传承屈原爱国主义精神，赛龙舟、吃粽子等习俗体现文化长河生生不息。</t>
+        </is>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1464" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/19/VIDEwZ2YRyudDTcTMzBRNhSq260619.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>Do it at home too, women tell Japanese fans who cleaned World Cup stadium</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>日本女球迷呼吁男性在家也做家务，指其世界杯赛场清洁行为存在双重标准。</t>
+        </is>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1465" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/crel9xlp8r1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>Boy, 12, wins hearts after trying to check sick chicken into Ethiopian hospital</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>12岁男孩为救病鸡试图将其送入埃塞俄比亚医院，感动众人。</t>
+        </is>
+      </c>
+      <c r="E1466" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1466" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy49e7w3rmxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>Mangione's lawyers reverse course on psychiatric defence in state murder trial</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>曼乔内律师在州谋杀案庭审中放弃精神失常辩护，改变策略。</t>
+        </is>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1467" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20y162gpm6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>Boy, 3, hurt at zoo was attacked by a crocodile</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>3岁男童在动物园遭鳄鱼攻击受伤，被捕嫌犯已获保释。</t>
+        </is>
+      </c>
+      <c r="E1468" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1468" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp9l2278m8no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>Thirty rioters sentenced for disorder which saw police officer set on fire</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>三十名骚乱者因2023年卡迪夫青少年死亡引发的暴力事件被判刑，期间一名警察被纵火。</t>
+        </is>
+      </c>
+      <c r="E1469" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1469" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cvgl9z8l271o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>Thousands of HGV drivers given bogus medical tests in the back of vans</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>数千名货车司机在面包车内接受虚假体检，交易标准局称“车轮上的医生”以低价吸引客户。</t>
+        </is>
+      </c>
+      <c r="E1470" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1470" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cy8wqy83q46o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>Rapist who 'catfished' Muslim men on Snapchat and Grindr jailed</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>一名在Snapchat和Grindr上伪装身份强奸穆斯林男子的强奸犯被判刑，警方称还有数十名受害者。</t>
+        </is>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1471" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwyenemwnd9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-20
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1471"/>
+  <dimension ref="A1:F1504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47509,6 +47509,1062 @@
         </is>
       </c>
     </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>[视频]保护传承革命文物 各地红色展馆迎参观热潮</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>七一前夕，全国红色展馆迎参观热潮，革命文物保护传承推动红色基因赓续。</t>
+        </is>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1472" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEt2ulRnnf163TwdJ6OJsJ260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>Talk of Starmer staying on to fight is fading - fast</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>安迪·伯纳姆补选获胜后，首相斯塔默的支持率迅速下滑。</t>
+        </is>
+      </c>
+      <c r="E1473" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1473" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cjeg7p5w4y9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>经济, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260620 19:00</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>端午假期中短途出行活跃，中欧班列开行量增长10.8倍，科技创新与产业融合加快。</t>
+        </is>
+      </c>
+      <c r="E1474" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1474" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDE2flMySL99j9yksI4qlbc260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>[视频]中欧班列年开行量十年间增长10.8倍</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>中欧班列年开行量十年增长10.8倍，已通达欧洲26国236个城市，服务亚欧全境。</t>
+        </is>
+      </c>
+      <c r="E1475" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1475" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDE9TKbcvROrBnXOlZDLrNh260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>[视频]外资机构：越来越开放的中国市场 越来越有吸引力</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>制度型开放持续推进，陆家嘴论坛推出金融开放举措，吸引外资机构深耕中国市场。</t>
+        </is>
+      </c>
+      <c r="E1476" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1476" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEW12WRi4OVSThvTz0H1e3260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>经济, 科技, 社会</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>5月全社会用电量同比增长6.9%，多部门发布平台经济方案，金川水电站投运，暑期档票房破10亿。</t>
+        </is>
+      </c>
+      <c r="E1477" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1477" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDE6vumy63v1IyPpwyegpnA260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>[视频]我国科技创新和产业创新融合发展步伐加快</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>我国科技创新和产业创新融合加快，高技术制造业5月增加值同比增长15.1%。</t>
+        </is>
+      </c>
+      <c r="E1478" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1478" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEaphF9ZnximDAfxd3qIAR260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>Steve Rosenberg: Moscow oil refinery attack brings Russia's war with Ukraine closer to home</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>莫斯科炼油厂遭袭，俄乌战争影响逼近市民生活。</t>
+        </is>
+      </c>
+      <c r="E1479" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1479" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp3xqkxp3x5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>[视频]端午假期第二天 中短途出行活跃</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>端午假期第二天，铁路、公路出行活跃，预计全社会跨区域人员流动量超2亿人次。</t>
+        </is>
+      </c>
+      <c r="E1480" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1480" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEaz3os5g2tl3aEaMyyHXW260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>Extreme heat warning expanded as 36C heatwave approaches UK</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>英国高温预警扩大，下周二气温或达36℃，琥珀色预警生效。</t>
+        </is>
+      </c>
+      <c r="E1481" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1481" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/cp8lye61jk6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>[视频]全球多地举办丰富多彩的端午节活动</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>加拿大、英国、南非、巴西等多国举办龙舟赛、包粽子等活动，共庆端午佳节。</t>
+        </is>
+      </c>
+      <c r="E1482" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1482" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEshp0MYUxqKUZQGcNZctN260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>[视频]日本民众集会反对政府扩军修宪动向</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>上万日本民众在国会前集会，抗议政府扩军修宪等危险动向。</t>
+        </is>
+      </c>
+      <c r="E1483" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1483" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDE6ZfEoGqtPLAsr7QwPtYT260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称启动伊美谈判取决于谅解备忘录相关条款的执行情况</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>伊朗称伊美谈判启动取决于备忘录条款执行，以黎停火协议遭破坏，以色列继续空袭。</t>
+        </is>
+      </c>
+      <c r="E1484" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1484" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDETeVasMMiHZVzBGY6E7Th260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>欧盟称需与俄建立直接沟通渠道；英国贝德福德火车相撞致1死89伤。</t>
+        </is>
+      </c>
+      <c r="E1485" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1485" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEV7a0cXpOVzPoDTHqRLOj260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>Israel and Hezbollah continue strikes despite ceasefire agreement</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>以色列与黎巴嫩真主党停火协议后继续交火，黎南部有人员伤亡报告。</t>
+        </is>
+      </c>
+      <c r="E1486" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1486" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx240k9l112o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>Tourist dies in Dominican Republic luxury resort fire</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>多米尼加度假胜地酒店大火，近1700人被疏散。</t>
+        </is>
+      </c>
+      <c r="E1487" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1487" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c932k8010j1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>Trump hits out at Italy's Meloni after pushback on G7 photo claim</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>特朗普与意大利总理梅洛尼就G7合影事件争执。</t>
+        </is>
+      </c>
+      <c r="E1488" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1488" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgqj77909jpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>Australia confirms first case of H5N1 bird flu as virus reaches every continent</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>澳大利亚确认首例H5N1禽流感，病毒已遍布各大洲。</t>
+        </is>
+      </c>
+      <c r="E1489" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1489" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c4gykxklvl5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>African and Caribbean nations call for formal apology for transatlantic slavery</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>非洲和加勒比国家要求奴隶贸易涉事国正式道歉及补偿。</t>
+        </is>
+      </c>
+      <c r="E1490" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1490" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm2rl8z5x7no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>Fighting persists in Lebanon despite a ceasefire as  U.S.-Iran deal is under threat</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>黎巴嫩南部遭以军袭击致7人死亡，包括2名儿童，此前传停火协议达成。</t>
+        </is>
+      </c>
+      <c r="E1491" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1491" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/20/nx-s1-5865006/fighting-lebanon-despite-ceasefire</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】在文脉赓续中推动城市高质量发展</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>苏州平江历史文化街区游客如织，各地在文脉赓续中推动城市高质量发展。</t>
+        </is>
+      </c>
+      <c r="E1492" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1492" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEzkE9KYjGchK4AsTSdlQk260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>[视频]赏民俗品文化 欢度端午假期</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>端午假期各地举办龙舟赛、民俗体验等活动，民众享受假日生活。</t>
+        </is>
+      </c>
+      <c r="E1493" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1493" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEiuga4rQq96hSNG1XxQHq260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>社会, 经济</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】一枚香包 一脉“香”传</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>江苏徐州马庄村传承香包非遗，带动乡村振兴，年轻一代创新融合，让传统手艺焕发新生。</t>
+        </is>
+      </c>
+      <c r="E1494" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1494" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDErKK3pJ6SCVhPdiLeUabM260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>[视频]端午：千年传承 文脉绵长</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>节目展示端午文化魅力，弘扬家国情怀与奋进精神。</t>
+        </is>
+      </c>
+      <c r="E1495" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1495" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/20/VIDEnEExxxfbgQHfG5aMGhP2260620.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>What we know so far about the collision and how it is affecting travel</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>两列客运火车相撞，致司机死亡多人受伤，旅行受影响。</t>
+        </is>
+      </c>
+      <c r="E1496" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1496" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn75z3nl048o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>'People flew from their seats': Passengers describe how collision unfolded</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>碰撞事故致近90人受伤，其中30多人伤势严重。</t>
+        </is>
+      </c>
+      <c r="E1497" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1497" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cx2j700l5jlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>Video shows scene of crash as passenger describes aftermath</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>周五车祸后，截至周六下午仍有9人情况危急。</t>
+        </is>
+      </c>
+      <c r="E1498" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1498" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/c8d21z2q77do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>These nuns spent a lifetime helping others. In their last years, who will help them?</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>乌干达修女一生助人，晚年却面临无人照料的困境。</t>
+        </is>
+      </c>
+      <c r="E1499" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1499" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/20/g-s1-128632/nuns-convent-africa-hospice</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>Watch: World Cup fans react to US defeating Australia to reach knockout round</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>世界杯美国队2-0胜澳大利亚，球迷反应各异。</t>
+        </is>
+      </c>
+      <c r="E1500" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1500" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/videos/cdxdly41p23o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>James Burrows, legendary director of Cheers and Friends, dies aged 85</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>《欢乐酒店》《老友记》传奇导演詹姆斯·伯罗斯去世，享年85岁。</t>
+        </is>
+      </c>
+      <c r="E1501" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1501" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/ce8k07x523eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>Why Harry Kane is different at this World Cup</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t>前英格兰队长分析凯恩在本次世界杯的显著变化。</t>
+        </is>
+      </c>
+      <c r="E1502" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1502" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/crr87vwrwwlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>Flawed but relentless Scotland show themselves as men of substance</t>
+        </is>
+      </c>
+      <c r="D1503" t="inlineStr">
+        <is>
+          <t>苏格兰队虽败犹荣，展现顽强意志与坚韧品质。</t>
+        </is>
+      </c>
+      <c r="E1503" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1503" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c33y5v4mer3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B1504" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr">
+        <is>
+          <t>Curacao's trailblazer doctor on football's big stage</t>
+        </is>
+      </c>
+      <c r="D1504" t="inlineStr">
+        <is>
+          <t>库拉索男足队医苏珊博士，世界杯史上最小参赛队的医疗主管。</t>
+        </is>
+      </c>
+      <c r="E1504" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1504" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/ckg08ewg9l2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-21
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1504"/>
+  <dimension ref="A1:F1536"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48565,6 +48565,1030 @@
         </is>
       </c>
     </row>
+    <row r="1505">
+      <c r="A1505" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1505" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260621 21:00</t>
+        </is>
+      </c>
+      <c r="D1505" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道东西部协作、改革开放、假日经济、长三角外贸等国内新闻及美伊谈判等国际快讯。</t>
+        </is>
+      </c>
+      <c r="E1505" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1505" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEowfMpCzRa8JHODfkT9M2260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1506" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】山海携手 书写东西部协作崭新篇章</t>
+        </is>
+      </c>
+      <c r="D1506" t="inlineStr">
+        <is>
+          <t>习近平总书记推动东西部协作，闽宁镇发展光伏、农业等产业，实现山海携手共同发展。</t>
+        </is>
+      </c>
+      <c r="E1506" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1506" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDER3eAW6ZUMkJlLZ9C69Rf260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】党的十一届三中全会开启改革开放和社会主义现代化建设新时期</t>
+        </is>
+      </c>
+      <c r="D1507" t="inlineStr">
+        <is>
+          <t>回顾党的十一届三中全会，开启改革开放和社会主义现代化建设新时期，深圳等城市见证发展。</t>
+        </is>
+      </c>
+      <c r="E1507" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1507" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEz4xwGRgwTkM6CteR8LTl260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>政治, 经济, 社会</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1508" t="inlineStr">
+        <is>
+          <t>甘肃天水公祭伏羲，两岸共祭；四部门支持海洋经济就业；房屋建筑将全生命周期一码贯通；2030年多式联运1小时换装率超90%。</t>
+        </is>
+      </c>
+      <c r="E1508" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1508" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEKmSgDj2l0sR4VR59r5wu260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1509" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr">
+        <is>
+          <t>Signs grow that Starmer will resign as government mood shifts</t>
+        </is>
+      </c>
+      <c r="D1509" t="inlineStr">
+        <is>
+          <t>迹象显示英国首相斯塔默将辞职，政府内部氛围转变。</t>
+        </is>
+      </c>
+      <c r="E1509" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1509" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cql10wwy69zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1510" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr">
+        <is>
+          <t>Colombia runoff vote shaped by security fears and conflict warnings</t>
+        </is>
+      </c>
+      <c r="D1510" t="inlineStr">
+        <is>
+          <t>哥伦比亚总统决选：候选人应对武装组织策略分歧，领先者主张强化军事行动。</t>
+        </is>
+      </c>
+      <c r="E1510" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1510" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/21/nx-s1-5862783/colombia-election-conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1511" t="inlineStr">
+        <is>
+          <t>经济, 民生, 文体</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr">
+        <is>
+          <t>[视频]服务消费提质扩容 假日经济活力迸发</t>
+        </is>
+      </c>
+      <c r="D1511" t="inlineStr">
+        <is>
+          <t>端午假期服务消费提质扩容，赛事文旅融合、国潮市集等带动假日经济活力迸发。</t>
+        </is>
+      </c>
+      <c r="E1511" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1511" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDErNe2u9QR14OsIWxY1jEN260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1512" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr">
+        <is>
+          <t>[视频]长三角地区进出口连续15个月保持增长</t>
+        </is>
+      </c>
+      <c r="D1512" t="inlineStr">
+        <is>
+          <t>长三角地区前5个月进出口7.82万亿元，连续15个月增长，高端制造出口强劲。</t>
+        </is>
+      </c>
+      <c r="E1512" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1512" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEvLEqrDDcwWqCiZ1IOqvJ260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1513" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr">
+        <is>
+          <t>[视频]第四届链博会明天开幕 布展工作已全面完成</t>
+        </is>
+      </c>
+      <c r="D1513" t="inlineStr">
+        <is>
+          <t>第四届链博会明天开幕，设六大展区，首次设人工智能专区，首发首展超160项。</t>
+        </is>
+      </c>
+      <c r="E1513" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1513" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDECmtLqyomhtB77E5cQHdD260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1514" t="inlineStr">
+        <is>
+          <t>军事, 国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1514" t="inlineStr">
+        <is>
+          <t>俄称在红利曼夺取据点，乌打击纵深目标；美洛杉矶仓储火灾持续；刚果（金）埃博拉死亡247例。</t>
+        </is>
+      </c>
+      <c r="E1514" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1514" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEhT5kax5VhBnVrE9k0Jle260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1515" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr">
+        <is>
+          <t>Fuel sales halted in occupied Crimea as Ukraine targets oil facilities</t>
+        </is>
+      </c>
+      <c r="D1515" t="inlineStr">
+        <is>
+          <t>乌克兰袭击俄占克里米亚燃料设施，导致燃油销售暂停，此前已因短缺实施配给。</t>
+        </is>
+      </c>
+      <c r="E1515" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1515" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/clyx2lk9d15o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1516" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr">
+        <is>
+          <t>[视频]端午假期全社会跨区域人员流动量预计超6.5亿人次</t>
+        </is>
+      </c>
+      <c r="D1516" t="inlineStr">
+        <is>
+          <t>端午假期全社会跨区域人员流动量预计超6.5亿人次，铁路公路迎来返程高峰。</t>
+        </is>
+      </c>
+      <c r="E1516" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1516" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEROztx9xxR1xxSnrZKPDG260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1517" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr">
+        <is>
+          <t>Tight security as Indian students resit medical exam after alleged paper leak</t>
+        </is>
+      </c>
+      <c r="D1517" t="inlineStr">
+        <is>
+          <t>印度医学生因试卷泄露重考，数百万考生接受生物识别检查，空军出动保障试卷安全。</t>
+        </is>
+      </c>
+      <c r="E1517" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1517" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy0gjqv783o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1518" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr">
+        <is>
+          <t>Extreme heat warning extended to four days as temperatures could hit 38C</t>
+        </is>
+      </c>
+      <c r="D1518" t="inlineStr">
+        <is>
+          <t>英国极端高温警告延长至四天，气温或达38°C。</t>
+        </is>
+      </c>
+      <c r="E1518" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1518" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/weather/articles/c932k0lewygo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1519" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr">
+        <is>
+          <t>[视频]美国与伊朗今日在瑞士举行技术层面谈判</t>
+        </is>
+      </c>
+      <c r="D1519" t="inlineStr">
+        <is>
+          <t>美伊在瑞士进行技术层面谈判，伊朗宣布关闭霍尔木兹海峡，以总理称不会从黎南部撤军。</t>
+        </is>
+      </c>
+      <c r="E1519" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1519" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEqOJKr44CyzeTtcAfDYj7260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1520" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>US and Iran begin talks on initial peace deal in Switzerland</t>
+        </is>
+      </c>
+      <c r="D1520" t="inlineStr">
+        <is>
+          <t>美伊在瑞士开始初步和平谈判，黎巴嫩冲突持续，伊朗声称关闭霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E1520" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1520" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy0q41v1lzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1521" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr">
+        <is>
+          <t>Ukrainian attacks prompt Russian-held Crimea to halt civilian gasoline sales</t>
+        </is>
+      </c>
+      <c r="D1521" t="inlineStr">
+        <is>
+          <t>乌克兰袭击燃料供应，俄占克里米亚暂停民用汽油销售。</t>
+        </is>
+      </c>
+      <c r="E1521" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1521" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/21/g-s1-129200/ukrainian-attacks-russia-crimea-halt-gas-sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1522" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr">
+        <is>
+          <t>What could make a peace deal with Iran viable? One expert weighs in</t>
+        </is>
+      </c>
+      <c r="D1522" t="inlineStr">
+        <is>
+          <t>专家分析美伊谅解备忘录及未来和平协议的关键优先事项。</t>
+        </is>
+      </c>
+      <c r="E1522" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1522" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/21/nx-s1-5863129/what-could-make-a-peace-deal-with-iran-viable-one-expert-weighs-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1523" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr">
+        <is>
+          <t>Cambodia cracked down on scams costing Americans billions. It created a new crisis</t>
+        </is>
+      </c>
+      <c r="D1523" t="inlineStr">
+        <is>
+          <t>柬埔寨打击诈骗中心致数千名外国工人滞留金边街头，引发新危机。</t>
+        </is>
+      </c>
+      <c r="E1523" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1523" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/21/g-s1-128624/freed-from-cambodias-scam-compounds-trafficking-victims-face-a-new-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1524" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】农加贵：烛照深山40年</t>
+        </is>
+      </c>
+      <c r="D1524" t="inlineStr">
+        <is>
+          <t>云南教师农加贵扎根麻风病村小学40年，建设学校并获评全国优秀党员。</t>
+        </is>
+      </c>
+      <c r="E1524" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1524" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEf2TLRurhnOEX1bByl7HD260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1525" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr">
+        <is>
+          <t>[视频]【暖心一瞬】凡人善举暖人心 生活处处有温情</t>
+        </is>
+      </c>
+      <c r="D1525" t="inlineStr">
+        <is>
+          <t>江苏七旬老人雨中为小麦盖防雨布，湖北11岁女孩背4岁走失幼童找警察，善举暖心。</t>
+        </is>
+      </c>
+      <c r="E1525" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1525" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDEXwFVSwRsaj3Y9gKcPmt9260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1526" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr">
+        <is>
+          <t>[视频]二十四节气·夏至</t>
+        </is>
+      </c>
+      <c r="D1526" t="inlineStr">
+        <is>
+          <t>夏至到来，北半球白昼最长，介绍节气文化、习俗及自然之美。</t>
+        </is>
+      </c>
+      <c r="E1526" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1526" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/21/VIDE8mFXtfYuTPJeJ2iXi0cj260621.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1527" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr">
+        <is>
+          <t>France bans alcohol at music festival events under red heatwave alert</t>
+        </is>
+      </c>
+      <c r="D1527" t="inlineStr">
+        <is>
+          <t>法国因红色高温预警，禁止音乐节活动期间售酒，以保护医疗系统在40℃高温下运行。</t>
+        </is>
+      </c>
+      <c r="E1527" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1527" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cgmdw4vn7y2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1528" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr">
+        <is>
+          <t>Former Olympian denies vandalising Washington Reflecting Pool after arrest</t>
+        </is>
+      </c>
+      <c r="D1528" t="inlineStr">
+        <is>
+          <t>前奥运选手否认破坏华盛顿倒影池，称只是出于好奇触摸新油漆。</t>
+        </is>
+      </c>
+      <c r="E1528" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1528" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c8d26051vv2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1529" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr">
+        <is>
+          <t>Low-key funeral held for giant of the art world David Hockney</t>
+        </is>
+      </c>
+      <c r="D1529" t="inlineStr">
+        <is>
+          <t>艺术大师大卫·霍克尼低调安葬，仅伴侣和侄孙参加葬礼。</t>
+        </is>
+      </c>
+      <c r="E1529" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1529" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cn8q6wxy706o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1530" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr">
+        <is>
+          <t>Dutch royals enjoy two big results in one World Cup day</t>
+        </is>
+      </c>
+      <c r="D1530" t="inlineStr">
+        <is>
+          <t>荷兰皇室同一天见证荷兰队和库拉索队双双取胜，尽管两地相距约5000英里。</t>
+        </is>
+      </c>
+      <c r="E1530" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1530" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/c4gydq973nqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1531" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr">
+        <is>
+          <t>Indian cricketer, 15, hits record-breaking 50 in just 11 balls</t>
+        </is>
+      </c>
+      <c r="D1531" t="inlineStr">
+        <is>
+          <t>15岁印度板球手Vaibhav Sooryavanshi创纪录，11球完成50分，同日未入选国家队。</t>
+        </is>
+      </c>
+      <c r="E1531" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1531" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/cricket/articles/czdev6lp8p9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1532" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr">
+        <is>
+          <t>Backstage at Gorillaz' epic, one-off stadium show: 'The vibe is ridiculous'</t>
+        </is>
+      </c>
+      <c r="D1532" t="inlineStr">
+        <is>
+          <t>Gorillaz在巨型体育场举办史诗级单场演出，后台氛围热烈。</t>
+        </is>
+      </c>
+      <c r="E1532" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1532" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cm203gndx0lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1533" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr">
+        <is>
+          <t>William marks 44th birthday as royals celebrate Father's Day</t>
+        </is>
+      </c>
+      <c r="D1533" t="inlineStr">
+        <is>
+          <t>威廉王子44岁生日，凯特王妃与子女送祝福，称其为“世界上最好的爸爸”。</t>
+        </is>
+      </c>
+      <c r="E1533" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1533" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9d2gzlze9po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1534" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr">
+        <is>
+          <t>Stokes to return as captain for third Test, coach McCullum says</t>
+        </is>
+      </c>
+      <c r="D1534" t="inlineStr">
+        <is>
+          <t>英格兰队主帅麦卡勒姆表示，已准备好与重返队长职务的斯托克斯合作。</t>
+        </is>
+      </c>
+      <c r="E1534" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1534" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/cricket/articles/ce8j350k5vro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1535" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr">
+        <is>
+          <t>The records that look set to be broken</t>
+        </is>
+      </c>
+      <c r="D1535" t="inlineStr">
+        <is>
+          <t>2026年世界杯开赛10天已刷新多项足球历史纪录。</t>
+        </is>
+      </c>
+      <c r="E1535" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1535" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/cpv3kkv4z4mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B1536" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr">
+        <is>
+          <t>How many World Cup Golden Boot winners can you name?</t>
+        </is>
+      </c>
+      <c r="D1536" t="inlineStr">
+        <is>
+          <t>世界杯历届金靴奖得主，你能说出多少位？</t>
+        </is>
+      </c>
+      <c r="E1536" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1536" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/sport/football/articles/ckgpjw4wd21o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-22
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1536"/>
+  <dimension ref="A1:F1565"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49589,6 +49589,934 @@
         </is>
       </c>
     </row>
+    <row r="1537">
+      <c r="A1537" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1537" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260622 19:00</t>
+        </is>
+      </c>
+      <c r="D1537" t="inlineStr">
+        <is>
+          <t>本期《新闻联播》涵盖延安精神、领导调研、外资政策、夏播科技、军事训练及多国政经动态。</t>
+        </is>
+      </c>
+      <c r="E1537" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1537" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEulK6G1oOvyswfk9L6age260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1538" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1538" t="inlineStr">
+        <is>
+          <t>[视频]【牢记初心使命 奋进复兴征程】赓续延安精神 书写时代新篇</t>
+        </is>
+      </c>
+      <c r="D1538" t="inlineStr">
+        <is>
+          <t>习近平总书记强调延安精神是宝贵财富，激励新时代奋斗，传承红色基因。</t>
+        </is>
+      </c>
+      <c r="E1538" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1538" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEAyu3ulUyAv1CT6KIYoiO260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1539" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1539" t="inlineStr">
+        <is>
+          <t>[视频]李强将出席第十七届夏季达沃斯论坛</t>
+        </is>
+      </c>
+      <c r="D1539" t="inlineStr">
+        <is>
+          <t>李强将出席大连夏季达沃斯论坛，多国领导人及1700余名代表参会。</t>
+        </is>
+      </c>
+      <c r="E1539" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1539" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDELZtWzYCcES2o4zRnEXNo260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1540" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1540" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁主持召开全国政协主席会议</t>
+        </is>
+      </c>
+      <c r="D1540" t="inlineStr">
+        <is>
+          <t>王沪宁主持政协主席会议，强调贯彻习近平党建思想，聚焦区域协调与产业发展建言献策。</t>
+        </is>
+      </c>
+      <c r="E1540" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1540" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEMK1yLaQ5lNgKK2n73w1U260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1541" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1541" t="inlineStr">
+        <is>
+          <t>[视频]全国人大常委会启动青藏高原生态保护法执法检查</t>
+        </is>
+      </c>
+      <c r="D1541" t="inlineStr">
+        <is>
+          <t>全国人大常委会启动青藏高原生态保护法执法检查，7至8月赴五省区实地检查。</t>
+        </is>
+      </c>
+      <c r="E1541" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1541" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEZEurbb9p90n10RE8mHAE260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1542" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1542" t="inlineStr">
+        <is>
+          <t>Analysis: Everything points to Burnham becoming PM within weeks</t>
+        </is>
+      </c>
+      <c r="D1542" t="inlineStr">
+        <is>
+          <t>分析称安迪·伯纳姆数周内可能成为英国首相，无需等到九月选举。</t>
+        </is>
+      </c>
+      <c r="E1542" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1542" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c20y1zvg50lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1543" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1543" t="inlineStr">
+        <is>
+          <t>Why did Starmer resign and what could happen next?</t>
+        </is>
+      </c>
+      <c r="D1543" t="inlineStr">
+        <is>
+          <t>英国工党领袖斯塔默辞职，称留任首相直至继任者选出。</t>
+        </is>
+      </c>
+      <c r="E1543" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1543" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c0qyllvpkw8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1544" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1544" t="inlineStr">
+        <is>
+          <t>Starmer's premiership in six charts</t>
+        </is>
+      </c>
+      <c r="D1544" t="inlineStr">
+        <is>
+          <t>BBC通过六张图表分析斯塔默自2024年7月上任以来的执政记录。</t>
+        </is>
+      </c>
+      <c r="E1544" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1544" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8p9qellmqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1545" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1545" t="inlineStr">
+        <is>
+          <t>Who is Andy Burnham? Ex-Manchester mayor who wants to lead the country</t>
+        </is>
+      </c>
+      <c r="D1545" t="inlineStr">
+        <is>
+          <t>前大曼彻斯特市长安迪·伯纳姆第三次竞选工党领袖，欲领导国家。</t>
+        </is>
+      </c>
+      <c r="E1545" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1545" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cp8pml5z8p6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1546" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1546" t="inlineStr">
+        <is>
+          <t>Watch and read Starmer's resignation speech in full</t>
+        </is>
+      </c>
+      <c r="D1546" t="inlineStr">
+        <is>
+          <t>斯塔默在唐宁街发表辞职演讲，宣布卸任工党领袖和首相职务。</t>
+        </is>
+      </c>
+      <c r="E1546" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1546" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c621nnq4pm7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1547" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1547" t="inlineStr">
+        <is>
+          <t>UK PM Keir Starmer resigns. And, US and Iran agree to roadmap for final deal</t>
+        </is>
+      </c>
+      <c r="D1547" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默辞职，同时美国和伊朗同意60天内达成最终协议的路线图。</t>
+        </is>
+      </c>
+      <c r="E1547" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1547" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/22/g-s1-129268/up-first-newsletter-keir-starmer-iran-us-vance-trump-reflection-pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1548" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1548" t="inlineStr">
+        <is>
+          <t>Keir Starmer has resigned, paving way for a 7th U.K. prime minister in 10 years</t>
+        </is>
+      </c>
+      <c r="D1548" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默辞职，可能由前市长伯纳姆接任，十年内第七位首相。</t>
+        </is>
+      </c>
+      <c r="E1548" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1548" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/22/nx-s1-5866231/keir-starmer-resigns</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1549" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1549" t="inlineStr">
+        <is>
+          <t>U.K. Prime Minister Keir Starmer announces resignation</t>
+        </is>
+      </c>
+      <c r="D1549" t="inlineStr">
+        <is>
+          <t>英国首相斯塔默宣布辞职，继任者或为曼彻斯特前市长伯纳姆。</t>
+        </is>
+      </c>
+      <c r="E1549" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1549" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/22/nx-s1-5866213/uk-prime-minister-keir-starmer-announces-resignation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1550" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1550" t="inlineStr">
+        <is>
+          <t>[视频]李强在辽宁大连调研</t>
+        </is>
+      </c>
+      <c r="D1550" t="inlineStr">
+        <is>
+          <t>李强在大连调研，强调发展高端装备制造业，加速关键技术突破，建设世界一流造船基地。</t>
+        </is>
+      </c>
+      <c r="E1550" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1550" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEqfgxP9zOXuw30H4zE0h9260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1551" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1551" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥出席第四届中国国际供应链促进博览会开幕式并作主旨讲话</t>
+        </is>
+      </c>
+      <c r="D1551" t="inlineStr">
+        <is>
+          <t>丁薛祥在供应链博览会呼吁维护全球产业链稳定，反对将经贸问题政治化。</t>
+        </is>
+      </c>
+      <c r="E1551" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1551" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDE5xp4VBVbsQ8jasQ9BU2Z260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1552" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1552" t="inlineStr">
+        <is>
+          <t>[视频]国家出台多项举措推动利用外资固稳促优</t>
+        </is>
+      </c>
+      <c r="D1552" t="inlineStr">
+        <is>
+          <t>国家发布《利用外资固稳促优行动方案》，扩大市场准入并优化投资便利度。</t>
+        </is>
+      </c>
+      <c r="E1552" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1552" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEhInGJqTWUzXitAx95j8h260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1553" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1553" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1553" t="inlineStr">
+        <is>
+          <t>中央下达2.19亿救灾资金；公共机构碳排放目标；端午出入境666.7万人次；食品安全平稳。</t>
+        </is>
+      </c>
+      <c r="E1553" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1553" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEASGzx52tcVROKt8tboCW260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1554" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1554" t="inlineStr">
+        <is>
+          <t>Alan Greenspan, the legendary former Federal Reserve chair, dies</t>
+        </is>
+      </c>
+      <c r="D1554" t="inlineStr">
+        <is>
+          <t>前美联储主席艾伦·格林斯潘去世，曾被誉为最佳央行行长，后因金融危机声誉受损。</t>
+        </is>
+      </c>
+      <c r="E1554" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1554" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/22/656930918/alan-greenspan-the-legendary-former-federal-reserve-chair-dies</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1555" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C1555" t="inlineStr">
+        <is>
+          <t>[视频]海军辽宁舰编队完成远海实战化训练</t>
+        </is>
+      </c>
+      <c r="D1555" t="inlineStr">
+        <is>
+          <t>辽宁舰编队完成40余天远海实战化训练，赴南海、西太平洋演练，提升航母编队作战能力。</t>
+        </is>
+      </c>
+      <c r="E1555" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1555" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDE6fgaHShHvTvYSHqXZ9Oo260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1556" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1556" t="inlineStr">
+        <is>
+          <t>Russian troop build-up threatens city seen as key to seizing Ukraine's Donbas</t>
+        </is>
+      </c>
+      <c r="D1556" t="inlineStr">
+        <is>
+          <t>俄军集结威胁顿涅茨克关键城市，若失守乌东最后据点将受冲击。</t>
+        </is>
+      </c>
+      <c r="E1556" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1556" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c9w2g0ewk95o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1557" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1557" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】全国夏播进入高峰 科技赋能提质增效</t>
+        </is>
+      </c>
+      <c r="D1557" t="inlineStr">
+        <is>
+          <t>全国夏播进度过七成，新技术新装备提升播种效率，助力丰产增收。</t>
+        </is>
+      </c>
+      <c r="E1557" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1557" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEK2Z0hY1MugdfwxllhS6v260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1558" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1558" t="inlineStr">
+        <is>
+          <t>[视频]南方多地强降雨 各部门多举措应对</t>
+        </is>
+      </c>
+      <c r="D1558" t="inlineStr">
+        <is>
+          <t>南方多地持续强降雨，各部门启动应急措施，抢排积水，转移群众，抢修基础设施。</t>
+        </is>
+      </c>
+      <c r="E1558" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1558" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEIpdw8D37gbpK7mVhoawp260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1559" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1559" t="inlineStr">
+        <is>
+          <t>[视频]伊美比尔根山首轮谈判结束 建立技术性谈判机制</t>
+        </is>
+      </c>
+      <c r="D1559" t="inlineStr">
+        <is>
+          <t>伊美在瑞士首轮谈判结束，建立技术性谈判机制，讨论核协议、黎巴嫩停火等议题。</t>
+        </is>
+      </c>
+      <c r="E1559" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1559" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEyEGZEoy5L0j4Ue3q8kgc260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1560" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C1560" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1560" t="inlineStr">
+        <is>
+          <t>英首相斯塔默辞职将迎新首相；俄乌互相打击；芝加哥周末枪击致8死38伤。</t>
+        </is>
+      </c>
+      <c r="E1560" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1560" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/22/VIDEu5BQNIdM6V5ri7nlVmVg260622.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1561" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1561" t="inlineStr">
+        <is>
+          <t>Vance says Iran will allow nuclear inspectors back into the country</t>
+        </is>
+      </c>
+      <c r="D1561" t="inlineStr">
+        <is>
+          <t>美国副总统称伊朗将允许核检查员重返，美伊首轮谈判取得重大进展。</t>
+        </is>
+      </c>
+      <c r="E1561" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1561" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3vy3nr63gxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1562" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1562" t="inlineStr">
+        <is>
+          <t>At least 13 killed and dozens injured after Qatar gas explosion</t>
+        </is>
+      </c>
+      <c r="D1562" t="inlineStr">
+        <is>
+          <t>卡塔尔拉斯拉凡工业区液化天然气设施发生技术事故，致13死数十伤。</t>
+        </is>
+      </c>
+      <c r="E1562" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1562" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cwy05llpjpno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1563" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1563" t="inlineStr">
+        <is>
+          <t>Myanmar army killed over 700 civilians in six months, UN says</t>
+        </is>
+      </c>
+      <c r="D1563" t="inlineStr">
+        <is>
+          <t>联合国报告称，缅甸军方半年内杀害超700名平民，含153名儿童。</t>
+        </is>
+      </c>
+      <c r="E1563" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1563" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/cnv97e42r7yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1564" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1564" t="inlineStr">
+        <is>
+          <t>2 students in custody after shooting at high school in Philippines kills 3</t>
+        </is>
+      </c>
+      <c r="D1564" t="inlineStr">
+        <is>
+          <t>菲律宾高中发生枪击案致3死，2名嫌疑人被拘留，自称曾遭校园欺凌。</t>
+        </is>
+      </c>
+      <c r="E1564" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1564" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/22/g-s1-129323/2-students-in-custody-after-shooting-at-high-school-in-philippines-kills-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1565" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1565" t="inlineStr">
+        <is>
+          <t>Clive Davis, music mogul behind Whitney Houston and Bruce Springsteen, dies aged 94</t>
+        </is>
+      </c>
+      <c r="D1565" t="inlineStr">
+        <is>
+          <t>捧红惠特尼·休斯顿等巨星的音乐界传奇克莱夫·戴维斯去世，享年94岁。</t>
+        </is>
+      </c>
+      <c r="E1565" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1565" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/news/articles/c3vy3e6q90qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-23
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1565"/>
+  <dimension ref="A1:F1604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50517,6 +50517,1254 @@
         </is>
       </c>
     </row>
+    <row r="1566">
+      <c r="A1566" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1566" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1566" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260623 19:00</t>
+        </is>
+      </c>
+      <c r="D1566" t="inlineStr">
+        <is>
+          <t>《习近平党建文选》出版发行；李强会见多国总理；人大常委会审议多项法律草案；多国政要活动及国内新闻汇总。</t>
+        </is>
+      </c>
+      <c r="E1566" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1566" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEaxVWsL9teqysa5BPbRxE260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1567" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1567" t="inlineStr">
+        <is>
+          <t>[视频]《习近平党建文选》第一卷、第二卷出版发行</t>
+        </is>
+      </c>
+      <c r="D1567" t="inlineStr">
+        <is>
+          <t>《习近平党建文选》第一、二卷出版发行，收入习近平党建著作102篇。</t>
+        </is>
+      </c>
+      <c r="E1567" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1567" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDE7ueEQSFbabmVvkuvzdzY260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1568" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1568" t="inlineStr">
+        <is>
+          <t>[视频]【牢记初心使命 奋进复兴征程】弘扬西柏坡精神 走好新时代赶考路</t>
+        </is>
+      </c>
+      <c r="D1568" t="inlineStr">
+        <is>
+          <t>弘扬西柏坡精神，重温“两个务必”，激励新时代赶考路。</t>
+        </is>
+      </c>
+      <c r="E1568" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1568" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDER4bD95TQYixKIS05K83G260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1569" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1569" t="inlineStr">
+        <is>
+          <t>[视频]十四届全国人大常委会第二十三次会议在京举行 审议商标法修订草案等 赵乐际主持</t>
+        </is>
+      </c>
+      <c r="D1569" t="inlineStr">
+        <is>
+          <t>全国人大常委会审议商标法、金融法等修订草案及多项议案。</t>
+        </is>
+      </c>
+      <c r="E1569" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1569" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDExJUg9x0w9aZsTQqgpkJj260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1570" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1570" t="inlineStr">
+        <is>
+          <t>[视频]全国政协十四届常委会第十七次会议开幕 王沪宁主持 丁薛祥作报告</t>
+        </is>
+      </c>
+      <c r="D1570" t="inlineStr">
+        <is>
+          <t>全国政协常委会开幕，围绕高质量发展协商议政，丁薛祥作报告。</t>
+        </is>
+      </c>
+      <c r="E1570" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1570" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDE2xZOFdPHNwdt8Mzkivvs260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1571" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1571" t="inlineStr">
+        <is>
+          <t>Peter Murrell jailed for more than five years for embezzling SNP funds</t>
+        </is>
+      </c>
+      <c r="D1571" t="inlineStr">
+        <is>
+          <t>苏格兰民族党前首席执行官默雷尔因贪污公款被判五年以上监禁。</t>
+        </is>
+      </c>
+      <c r="E1571" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1571" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yzlqv4dyeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1572" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1572" t="inlineStr">
+        <is>
+          <t>Farage says £5m gift spending details 'not public's business'</t>
+        </is>
+      </c>
+      <c r="D1572" t="inlineStr">
+        <is>
+          <t>法拉奇称接受5万英镑赠礼细节不属公共知情范围。</t>
+        </is>
+      </c>
+      <c r="E1572" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1572" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn0vx2edk0vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1573" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1573" t="inlineStr">
+        <is>
+          <t>Britain left the EU 10 years ago. Its politics has been an unruly mess</t>
+        </is>
+      </c>
+      <c r="D1573" t="inlineStr">
+        <is>
+          <t>英国脱欧十年，政治陷入混乱，两大政党流失数百万选民给替代政党。</t>
+        </is>
+      </c>
+      <c r="E1573" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1573" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/nx-s1-5867281/brexit-10-years-later</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1574" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1574" t="inlineStr">
+        <is>
+          <t>[视频]我国利用外资结构持续优化</t>
+        </is>
+      </c>
+      <c r="D1574" t="inlineStr">
+        <is>
+          <t>今年前五月我国新设外资企业增长5.3%，高技术产业利用外资增长19.4%，结构持续优化。</t>
+        </is>
+      </c>
+      <c r="E1574" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1574" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEYMUp24QYJ1lalPfFhotk260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1575" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1575" t="inlineStr">
+        <is>
+          <t>[视频]我国将全链条扩大汽车消费</t>
+        </is>
+      </c>
+      <c r="D1575" t="inlineStr">
+        <is>
+          <t>我国将全链条扩大汽车消费，聚焦房车露营等六大领域，推出17条举措。</t>
+        </is>
+      </c>
+      <c r="E1575" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1575" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEG12Iq0T61TQkuNzPwu2O260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1576" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1576" t="inlineStr">
+        <is>
+          <t>Irish government to contribute £197m to cross-border rail services</t>
+        </is>
+      </c>
+      <c r="D1576" t="inlineStr">
+        <is>
+          <t>爱尔兰政府拨款1.97亿英镑用于跨境铁路服务。</t>
+        </is>
+      </c>
+      <c r="E1576" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1576" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd95yd1y050o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1577" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C1577" t="inlineStr">
+        <is>
+          <t>Campaigners consider appeal after Gatwick bids fail</t>
+        </is>
+      </c>
+      <c r="D1577" t="inlineStr">
+        <is>
+          <t>英国高等法院支持盖特威克机场扩建，反对者考虑上诉。</t>
+        </is>
+      </c>
+      <c r="E1577" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1577" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjdg158v185o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1578" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1578" t="inlineStr">
+        <is>
+          <t>Spider which uses spring trap to capture prey discovered in Australia</t>
+        </is>
+      </c>
+      <c r="D1578" t="inlineStr">
+        <is>
+          <t>澳大利亚发现新蜘蛛，用弹簧陷阱捕食危险蚂蚁。</t>
+        </is>
+      </c>
+      <c r="E1578" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1578" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c70y138y995o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1579" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1579" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】以学促干 将学习教育成果落到实处</t>
+        </is>
+      </c>
+      <c r="D1579" t="inlineStr">
+        <is>
+          <t>上海静安、辽宁沈阳开展政绩观学习教育，解决群众急难愁盼问题。</t>
+        </is>
+      </c>
+      <c r="E1579" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1579" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDE5tJKjLPfbUd2CxNi7Fyv260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1580" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1580" t="inlineStr">
+        <is>
+          <t>[视频]2026年黄河调水调沙启动</t>
+        </is>
+      </c>
+      <c r="D1580" t="inlineStr">
+        <is>
+          <t>黄河2026年调水调沙启动，多水库联合调度，为下游水安全提供屏障。</t>
+        </is>
+      </c>
+      <c r="E1580" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1580" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEr2ygt7ENkSQctdpgwJX4260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1581" t="inlineStr">
+        <is>
+          <t>民生, 社会, 科技</t>
+        </is>
+      </c>
+      <c r="C1581" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1581" t="inlineStr">
+        <is>
+          <t>烈士陵园登记完成99.6%；可再生能源新规8月施行；机动车合格证实时共享；西渝高铁隧道贯通。</t>
+        </is>
+      </c>
+      <c r="E1581" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1581" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEgG4evL099lwEVIlHKcSD260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1582" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1582" t="inlineStr">
+        <is>
+          <t>From cool-down spots to chalk on windows - how Europeans are coping with the heat</t>
+        </is>
+      </c>
+      <c r="D1582" t="inlineStr">
+        <is>
+          <t>欧洲民众采取多种措施应对席卷全洲的酷暑高温。</t>
+        </is>
+      </c>
+      <c r="E1582" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1582" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz0j87vpz79o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1583" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1583" t="inlineStr">
+        <is>
+          <t>[视频]李强分别会见几内亚总理、哈萨克斯坦总理、韩国总理、蒙古国总理、黑山总理</t>
+        </is>
+      </c>
+      <c r="D1583" t="inlineStr">
+        <is>
+          <t>李强在大连会见五国总理，推动双边关系与多领域合作。</t>
+        </is>
+      </c>
+      <c r="E1583" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1583" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEXreFZtFOycUO6uXLtXZQ260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1584" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1584" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见南非副总统</t>
+        </is>
+      </c>
+      <c r="D1584" t="inlineStr">
+        <is>
+          <t>韩正会见南非副总统，强调深化政治互信与务实合作。</t>
+        </is>
+      </c>
+      <c r="E1584" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1584" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEfcQ1z3TgP43nQCgXDriW260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1585" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1585" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称各方展开技术性会谈 决定成立多个工作组</t>
+        </is>
+      </c>
+      <c r="D1585" t="inlineStr">
+        <is>
+          <t>伊美技术性会谈设四个工作组；美国放松对伊石油制裁致油价下跌；以色列继续在黎南部行动。</t>
+        </is>
+      </c>
+      <c r="E1585" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1585" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDE6gJC5MMRUJyMvJB0HwT6260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1586" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C1586" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1586" t="inlineStr">
+        <is>
+          <t>俄军在顿涅茨克推进，乌打击俄设施；日元逼近40年低位；卡塔尔天然气工厂爆炸致13死。</t>
+        </is>
+      </c>
+      <c r="E1586" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1586" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/23/VIDEeIDu0OOi2HPKN9bu1VgG260623.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1587" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1587" t="inlineStr">
+        <is>
+          <t>Drowning deaths soar in France as Europe buckles in peak of heatwave</t>
+        </is>
+      </c>
+      <c r="D1587" t="inlineStr">
+        <is>
+          <t>法国热浪致40人溺亡，欧洲遭遇高温高峰。</t>
+        </is>
+      </c>
+      <c r="E1587" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1587" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c79yvw3j114o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1588" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1588" t="inlineStr">
+        <is>
+          <t>Dozens of ships head through Strait of Hormuz after US-Iran deal</t>
+        </is>
+      </c>
+      <c r="D1588" t="inlineStr">
+        <is>
+          <t>美伊协议后，霍尔木兹海峡单日通行42艘船，航运显著增加。</t>
+        </is>
+      </c>
+      <c r="E1588" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1588" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx23rnzdgl8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>Iran says no new commitments on nuclear sites after Vance says inspectors to be invited back</t>
+        </is>
+      </c>
+      <c r="D1589" t="inlineStr">
+        <is>
+          <t>伊朗否认在瑞士核谈中作出新承诺，坚称未让步。</t>
+        </is>
+      </c>
+      <c r="E1589" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1589" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3vy3nr63gxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr">
+        <is>
+          <t>UN commission of inquiry says Israel committing genocide in Gaza by deliberately targeting children</t>
+        </is>
+      </c>
+      <c r="D1590" t="inlineStr">
+        <is>
+          <t>联合国指控以色列在加沙实施种族灭绝，以方驳斥。</t>
+        </is>
+      </c>
+      <c r="E1590" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1590" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0jy96w6pw2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr">
+        <is>
+          <t>Trump anticipates better relationship with Colombia under new leader</t>
+        </is>
+      </c>
+      <c r="D1591" t="inlineStr">
+        <is>
+          <t>特朗普称与哥伦比亚新当选总统关系将改善。</t>
+        </is>
+      </c>
+      <c r="E1591" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1591" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9v278ny9meo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>Stop pretending EU's new border system is working, says airports chief</t>
+        </is>
+      </c>
+      <c r="D1592" t="inlineStr">
+        <is>
+          <t>欧洲机场协会负责人称欧盟新边境系统不成熟，担忧夏季运营。</t>
+        </is>
+      </c>
+      <c r="E1592" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1592" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn4rlzrdj14o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>Afghan Taliban hold first, closed-door talks with EU on deportations</t>
+        </is>
+      </c>
+      <c r="D1593" t="inlineStr">
+        <is>
+          <t>阿富汗塔利班与欧盟就驱逐问题举行首次闭门会谈，人权组织批评此举损害欧盟人权义务。</t>
+        </is>
+      </c>
+      <c r="E1593" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1593" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/g-s1-129648/afghan-taliban-hold-first-closed-door-talks-with-eu-on-deportations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>U.S. lifts Iran oil sanctions. And, federal judge rules SAVE voter tool unlawful</t>
+        </is>
+      </c>
+      <c r="D1594" t="inlineStr">
+        <is>
+          <t>美国临时解除对伊朗石油制裁，同时联邦法官裁定特朗普政府SAVE选民工具违法。</t>
+        </is>
+      </c>
+      <c r="E1594" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1594" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/g-s1-129603/up-first-newsletter-iran-oil-sanctions-trump-economy-minnesota-subpoenas-save-voter-info</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>Iran's president heads to Pakistan as the U.S. and Iran work on a war-ending deal</t>
+        </is>
+      </c>
+      <c r="D1595" t="inlineStr">
+        <is>
+          <t>伊朗总统访问巴基斯坦，美伊技术团队正敲定结束战争的协议细节。</t>
+        </is>
+      </c>
+      <c r="E1595" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1595" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/nx-s1-5867322/us-iran-finalize-war-ending-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>国际, 军事, 民生</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>Lebanese struggle to get by in an ancient city under Israeli evacuation order</t>
+        </is>
+      </c>
+      <c r="D1596" t="inlineStr">
+        <is>
+          <t>黎巴嫩古城居民在以色列撤离令下艰难求生，古城曾遭亚历山大大帝围困。</t>
+        </is>
+      </c>
+      <c r="E1596" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1596" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/g-s1-128783/lebanon-israel-tyre-hezbollah-war</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>Zambia ex-president's family wins latest legal battle over what should happen to his body</t>
+        </is>
+      </c>
+      <c r="D1597" t="inlineStr">
+        <is>
+          <t>赞比亚前总统遗体处置案，家属与政府再起法律争端。</t>
+        </is>
+      </c>
+      <c r="E1597" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1597" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8r2yryr5mvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>US top court says Rastafarian man cannot sue prison guards for shaving his dreadlocks</t>
+        </is>
+      </c>
+      <c r="D1598" t="inlineStr">
+        <is>
+          <t>美最高法院裁定，拉斯特法里教徒不得起诉狱警剪其发辫。</t>
+        </is>
+      </c>
+      <c r="E1598" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1598" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx247v39r1no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>社会, 军事</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>Montreal shooting leaves officer, civilian and suspect dead</t>
+        </is>
+      </c>
+      <c r="D1599" t="inlineStr">
+        <is>
+          <t>蒙特利尔枪击致警官、平民和嫌疑人死亡，24年来首次。</t>
+        </is>
+      </c>
+      <c r="E1599" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1599" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz3lv015qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>Bright Horizons nursery chain served safeguarding notice by Ofsted</t>
+        </is>
+      </c>
+      <c r="D1600" t="inlineStr">
+        <is>
+          <t>英国教育标准局向Bright Horizons幼儿园连锁发出安全整改通知。</t>
+        </is>
+      </c>
+      <c r="E1600" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1600" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9321qq5y8jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>Major incident declared after bus crash near roundabout in Wales</t>
+        </is>
+      </c>
+      <c r="D1601" t="inlineStr">
+        <is>
+          <t>威尔士卡马森郡一巴士环岛附近发生车祸，宣布重大事件。</t>
+        </is>
+      </c>
+      <c r="E1601" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1601" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20ye768v6lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>A red alert over France, and heat that may rewrite the record books</t>
+        </is>
+      </c>
+      <c r="D1602" t="inlineStr">
+        <is>
+          <t>法国遭遇极端高温，大部分地区发布红色警报，高温将持续至本周末。</t>
+        </is>
+      </c>
+      <c r="E1602" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1602" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/g-s1-129586/france-red-heat-wave-alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>社会, 军事</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>Gunman kills an officer at a Montreal hotel before being shot dead, police say</t>
+        </is>
+      </c>
+      <c r="D1603" t="inlineStr">
+        <is>
+          <t>蒙特利尔酒店发生枪击，一名警察被持长枪嫌犯杀害，嫌犯被警方击毙。</t>
+        </is>
+      </c>
+      <c r="E1603" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1603" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/23/g-s1-129576/montreal-officer-killed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>World Cup 2026: Will England fans in Boston follow Scotland's lead?</t>
+        </is>
+      </c>
+      <c r="D1604" t="inlineStr">
+        <is>
+          <t>2026世界杯：英格兰球迷能否效仿苏格兰征服波士顿？</t>
+        </is>
+      </c>
+      <c r="E1604" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1604" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c8x2rev41ydo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-24
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1604"/>
+  <dimension ref="A1:F1642"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51765,6 +51765,1222 @@
         </is>
       </c>
     </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260624 19:00</t>
+        </is>
+      </c>
+      <c r="D1605" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道习近平考察山东、李强出席达沃斯论坛、人大常委会会议等国内要闻。</t>
+        </is>
+      </c>
+      <c r="E1605" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1605" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDErYllUbVdL8Ya63cJTrDn260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>[视频]习近平在山东德州考察时强调 以扎实举措推进农业农村现代化 用勤劳和智慧创造更加美好生活</t>
+        </is>
+      </c>
+      <c r="D1606" t="inlineStr">
+        <is>
+          <t>习近平在山东德州考察，强调以扎实举措推进农业农村现代化，保障粮食稳定供给。</t>
+        </is>
+      </c>
+      <c r="E1606" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1606" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDERIngxa94yVqMRtGqjwNM260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>[视频]【央视快评】用勤劳和智慧创造更加美好生活</t>
+        </is>
+      </c>
+      <c r="D1607" t="inlineStr">
+        <is>
+          <t>央视快评《用勤劳和智慧创造更加美好生活》播发。</t>
+        </is>
+      </c>
+      <c r="E1607" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1607" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDE3MObH1u1TqDApYC9awXM260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>[视频]十四届全国人大常委会第二十三次会议举行联组会议 审议国务院关于建设全国统一大市场工作情况的报告并开展专题询问 赵乐际出席</t>
+        </is>
+      </c>
+      <c r="D1608" t="inlineStr">
+        <is>
+          <t>十四届全国人大常委会举行联组会议，审议全国统一大市场建设情况并开展专题询问。</t>
+        </is>
+      </c>
+      <c r="E1608" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1608" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEK0zsJ7peb2jwFsnn8XCm260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际同全国人大常委会会议列席代表座谈</t>
+        </is>
+      </c>
+      <c r="D1609" t="inlineStr">
+        <is>
+          <t>赵乐际同全国人大代表座谈，强调人大代表要深入学习宣传习近平法治思想。</t>
+        </is>
+      </c>
+      <c r="E1609" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1609" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEjEUycsCXXpEXuv5h7hTI260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>[视频]全国政协十四届常委会第十七次会议举行全体会议 围绕“坚持高质量发展，推动经济持续健康发展和社会全面进步”进行大会发言 王沪宁出席</t>
+        </is>
+      </c>
+      <c r="D1610" t="inlineStr">
+        <is>
+          <t>全国政协常委会围绕高质量发展进行大会发言，涉及科技创新、产业体系等议题。</t>
+        </is>
+      </c>
+      <c r="E1610" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1610" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEeRlYsBPruzlW8zbzdbqO260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>[视频]全国政协十四届常委会第十七次会议闭幕 王沪宁主持并讲话</t>
+        </is>
+      </c>
+      <c r="D1611" t="inlineStr">
+        <is>
+          <t>全国政协十四届常委会第十七次会议闭幕，聚焦高质量发展，王沪宁讲话强调凝聚共识。</t>
+        </is>
+      </c>
+      <c r="E1611" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1611" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEx7OfS1D17cFlin5XKdx9260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行新闻发布会 介绍民族团结进步促进法</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>国新办介绍民族团结进步促进法，该法是新时代首部民族领域专门法律，7月1日起施行。</t>
+        </is>
+      </c>
+      <c r="E1612" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1612" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDELA4dKtSB6vlJ81Aj1f1e260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>Clean sweep for Mamdani-backed candidates in New York's Democratic primary</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>马姆达尼支持候选人在纽约民主党初选中大胜，显露加沙战争分歧。</t>
+        </is>
+      </c>
+      <c r="E1613" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1613" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clye652m41po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>Burnham on course to be PM, but what would his No 10 operation look like?</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>伯纳姆有望成为首相，其核心团队正在组建，但政策优先项仍存疑问。</t>
+        </is>
+      </c>
+      <c r="E1614" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1614" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp3xv2j7gepo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>IAEA chief says inspectors will visit nuclear sites under Iran-U.S. interim deal</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>国际原子能机构总干事称，将根据美伊临时协议派员视察伊朗核设施。</t>
+        </is>
+      </c>
+      <c r="E1615" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1615" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/g-s1-129770/iran-nuclear-inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>政治, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>As U.S. government looks to leverage food aid, producers seek other delivery methods</t>
+        </is>
+      </c>
+      <c r="D1616" t="inlineStr">
+        <is>
+          <t>美国调整粮食援助方式，将其作为外交工具，同时探索其他分发途径。</t>
+        </is>
+      </c>
+      <c r="E1616" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1616" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/nx-s1-5843163/as-u-s-government-looks-to-leverage-food-aid-producers-seek-other-delivery-methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>[视频]李强出席2026年夏季达沃斯论坛开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D1617" t="inlineStr">
+        <is>
+          <t>李强在大连出席2026年夏季达沃斯论坛开幕式并致辞，强调创新驱动与全球合作。</t>
+        </is>
+      </c>
+      <c r="E1617" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1617" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEkLmeXjIaA3rmN6VWgW45260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>[视频]李强出席2026年夏季达沃斯论坛工商界代表座谈会</t>
+        </is>
+      </c>
+      <c r="D1618" t="inlineStr">
+        <is>
+          <t>李强出席达沃斯论坛工商界座谈会，称中国将深化开放合作，为各国企业带来新机遇。</t>
+        </is>
+      </c>
+      <c r="E1618" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1618" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEaYsKz4wFYDNkmedtwG6s260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr">
+        <is>
+          <t>[视频]链博会与会嘉宾：中国开辟全球供应链合作新机遇</t>
+        </is>
+      </c>
+      <c r="D1619" t="inlineStr">
+        <is>
+          <t>第四届链博会吸引多国嘉宾，认为中国经济为全球供应链合作带来新机遇。</t>
+        </is>
+      </c>
+      <c r="E1619" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1619" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEa69nlkzkdFYJZbOkG6e6260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1620" t="inlineStr">
+        <is>
+          <t>审计整改1.41万亿元；前5月财政收入超10万亿元；中国超算“灵晟”登顶全球500强。</t>
+        </is>
+      </c>
+      <c r="E1620" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1620" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDE5EHb2rporZYwdu1bRcPn260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>经济, 文体</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>GTA 6 will cost $80 - and physical edition will not contain a disc</t>
+        </is>
+      </c>
+      <c r="D1621" t="inlineStr">
+        <is>
+          <t>《侠盗猎车手6》售价80美元，实体版不含光盘，仅提供数字下载码。</t>
+        </is>
+      </c>
+      <c r="E1621" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1621" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjrg52egw1ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr">
+        <is>
+          <t>军事, 民生</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr">
+        <is>
+          <t>Biggest city in Crimea without power after Ukraine strikes</t>
+        </is>
+      </c>
+      <c r="D1622" t="inlineStr">
+        <is>
+          <t>乌克兰袭击后，克里米亚最大城市塞瓦斯托波尔断电至晚间。</t>
+        </is>
+      </c>
+      <c r="E1622" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1622" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3ryv72pjqno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1623" t="inlineStr">
+        <is>
+          <t>国新办举行民政系统代表见面会，分享社会救助、养老护理等为民服务故事。</t>
+        </is>
+      </c>
+      <c r="E1623" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1623" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDE3v7oR7Bw62nh5yEZ56q2260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr">
+        <is>
+          <t>Power outages hit France as record heatwave set to peak</t>
+        </is>
+      </c>
+      <c r="D1624" t="inlineStr">
+        <is>
+          <t>法国布列塔尼约6.8万户因创纪录热浪停电，电力预计周三晚恢复。</t>
+        </is>
+      </c>
+      <c r="E1624" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1624" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c78y4102n1zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr">
+        <is>
+          <t>Air conditioning creates political divide after France records hottest day</t>
+        </is>
+      </c>
+      <c r="D1625" t="inlineStr">
+        <is>
+          <t>法国高温创纪录，引发对空调使用的政治分歧与反思。</t>
+        </is>
+      </c>
+      <c r="E1625" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1625" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyqldl3p5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr">
+        <is>
+          <t>Why this heatwave feels worse than the last one</t>
+        </is>
+      </c>
+      <c r="D1626" t="inlineStr">
+        <is>
+          <t>多重因素共同导致本次热浪比以往更令人不适。</t>
+        </is>
+      </c>
+      <c r="E1626" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1626" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/c3vyzly206no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr">
+        <is>
+          <t>[视频]伊朗称伊美谈判不会涉及伊朗弹道导弹议题</t>
+        </is>
+      </c>
+      <c r="D1627" t="inlineStr">
+        <is>
+          <t>伊朗称伊美谈判不涉及弹道导弹；美参议院要求结束对伊军事行动。</t>
+        </is>
+      </c>
+      <c r="E1627" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1627" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEwAWCWMEJNRzBKvSSn33K260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1628" t="inlineStr">
+        <is>
+          <t>俄总统称愿特定条件下与乌和谈；德国铁路因通信故障一度停运；美犹他州林火蔓延。</t>
+        </is>
+      </c>
+      <c r="E1628" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1628" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/24/VIDEyAnOBM9hafRWhgT1GHCU260624.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr">
+        <is>
+          <t>UN nuclear chief says inspectors will visit Iran sites as part of war deal</t>
+        </is>
+      </c>
+      <c r="D1629" t="inlineStr">
+        <is>
+          <t>国际原子能机构总干事称将访伊核设施，伊朗称需最终协议。</t>
+        </is>
+      </c>
+      <c r="E1629" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1629" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpd395zv81vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr">
+        <is>
+          <t>France confirms first Ebola case</t>
+        </is>
+      </c>
+      <c r="D1630" t="inlineStr">
+        <is>
+          <t>法国确认首例埃博拉病例，患者曾在刚果（金）工作。</t>
+        </is>
+      </c>
+      <c r="E1630" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1630" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj9gzr9rdjlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1631" t="inlineStr">
+        <is>
+          <t>King meets women's cricket team that is not allowed to exist</t>
+        </is>
+      </c>
+      <c r="D1631" t="inlineStr">
+        <is>
+          <t>查尔斯国王会见已被禁止参加正式比赛的阿富汗女子板球队以示支持。</t>
+        </is>
+      </c>
+      <c r="E1631" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1631" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gykxdn6gwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1632" t="inlineStr">
+        <is>
+          <t>Greetings from sweltering Switzerland</t>
+        </is>
+      </c>
+      <c r="D1632" t="inlineStr">
+        <is>
+          <t>瑞士卢塞恩湖畔，球迷通过巨型电视观看世界杯，当地天气湿热如热带。</t>
+        </is>
+      </c>
+      <c r="E1632" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1632" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/nx-s1-5867606/lucerne-switzerland-world-cup-heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1633" t="inlineStr">
+        <is>
+          <t>Inside the gold-mining town where the Ebola outbreak likely started</t>
+        </is>
+      </c>
+      <c r="D1633" t="inlineStr">
+        <is>
+          <t>刚果金金矿小镇蒙布瓦卢是埃博拉疫情源头，当地物资匮乏且居民质疑病毒真实性。</t>
+        </is>
+      </c>
+      <c r="E1633" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1633" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/nx-s1-5863157/ebola-outbreak-democratic-republic-congo-health-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1634" t="inlineStr">
+        <is>
+          <t>French woman allegedly held captive by husband for 12 years rescued in Pakistan</t>
+        </is>
+      </c>
+      <c r="D1634" t="inlineStr">
+        <is>
+          <t>法国女子被丈夫囚禁12年，在巴基斯坦与五名子女一同获救。</t>
+        </is>
+      </c>
+      <c r="E1634" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1634" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj0g71pnv3no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1635" t="inlineStr">
+        <is>
+          <t>Sydney woman wakes from induced coma more than a week after shark attack</t>
+        </is>
+      </c>
+      <c r="D1635" t="inlineStr">
+        <is>
+          <t>悉尼女子遭鲨鱼袭击一周多后，从诱导昏迷中苏醒。</t>
+        </is>
+      </c>
+      <c r="E1635" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1635" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy8drk2dk3no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr">
+        <is>
+          <t>社会, 军事</t>
+        </is>
+      </c>
+      <c r="C1636" t="inlineStr">
+        <is>
+          <t>Eight sentenced to 450 years in prison over anti-ICE riot where officer was shot</t>
+        </is>
+      </c>
+      <c r="D1636" t="inlineStr">
+        <is>
+          <t>八人因反ICE暴乱中枪击警官被判450年监禁，检察官称涉Antifa。</t>
+        </is>
+      </c>
+      <c r="E1636" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1636" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyedgnyn4mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1637" t="inlineStr">
+        <is>
+          <t>Bondi Beach shooting hero pleads not guilty to alleged assault on his father</t>
+        </is>
+      </c>
+      <c r="D1637" t="inlineStr">
+        <is>
+          <t>英雄在犹太活动枪击案中制服一名枪手，现被指控袭击其父亲，他不认罪。</t>
+        </is>
+      </c>
+      <c r="E1637" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1637" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn8q33gdgjjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1638" t="inlineStr">
+        <is>
+          <t>Baby deaths and toxic culture - the Nottingham maternity report at a glance</t>
+        </is>
+      </c>
+      <c r="D1638" t="inlineStr">
+        <is>
+          <t>诺丁汉孕产服务审查报告指出存在系统性失误和不良文化。</t>
+        </is>
+      </c>
+      <c r="E1638" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1638" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyd8kkjnx2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1639" t="inlineStr">
+        <is>
+          <t>Train passed red signal before fatal crash, says report</t>
+        </is>
+      </c>
+      <c r="D1639" t="inlineStr">
+        <is>
+          <t>独立铁路事故调查处发布初步报告，称列车在致命撞车前闯了红灯。</t>
+        </is>
+      </c>
+      <c r="E1639" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1639" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly90nqpryko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1640" t="inlineStr">
+        <is>
+          <t>Police took eight minutes to find Henry Nowak's fatal stab wound</t>
+        </is>
+      </c>
+      <c r="D1640" t="inlineStr">
+        <is>
+          <t>警方在手铐控制南安普顿学生八分钟后才发现其致命刀伤，该生死亡。</t>
+        </is>
+      </c>
+      <c r="E1640" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1640" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2v02r105jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1641" t="inlineStr">
+        <is>
+          <t>Archaeologists find huge Viking textile production site in Denmark</t>
+        </is>
+      </c>
+      <c r="D1641" t="inlineStr">
+        <is>
+          <t>丹麦发现千年维京时代大型纺织品生产基地，揭示其社会复杂性。</t>
+        </is>
+      </c>
+      <c r="E1641" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1641" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/g-s1-129750/viking-textile-production-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1642" t="inlineStr">
+        <is>
+          <t>Scotland on 'brink of history', fans say ahead of Brazil World Cup tie</t>
+        </is>
+      </c>
+      <c r="D1642" t="inlineStr">
+        <is>
+          <t>世界杯小组赛末轮，苏格兰队将对阵巴西，球迷称球队处于历史边缘。</t>
+        </is>
+      </c>
+      <c r="E1642" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1642" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdejr7gey9do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-25
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1642"/>
+  <dimension ref="A1:F1684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52981,6 +52981,1350 @@
         </is>
       </c>
     </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1643" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260625 19:00</t>
+        </is>
+      </c>
+      <c r="D1643" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平山东考察反响、李强会见孟加拉国总理、人大常委会会议等国内外大事。</t>
+        </is>
+      </c>
+      <c r="E1643" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1643" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEifTWzARn895XaoK4Ldny260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1644" t="inlineStr">
+        <is>
+          <t>[视频]用勤劳和智慧创造更加美好生活——习近平总书记在山东德州考察引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D1644" t="inlineStr">
+        <is>
+          <t>习近平在山东德州考察农业农村，强调保障粮食安全、推进乡村振兴，引发热烈反响。</t>
+        </is>
+      </c>
+      <c r="E1644" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1644" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEcaXaWSTfM25vJsP2NqS2260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1645" t="inlineStr">
+        <is>
+          <t>[视频]李强举行仪式欢迎孟加拉国总理访华</t>
+        </is>
+      </c>
+      <c r="D1645" t="inlineStr">
+        <is>
+          <t>国务院总理李强在北京人民大会堂举行仪式，欢迎孟加拉国总理塔里克访华。</t>
+        </is>
+      </c>
+      <c r="E1645" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1645" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEsxmifBsJC2D4M0neuU4J260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr">
+        <is>
+          <t>政治, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1646" t="inlineStr">
+        <is>
+          <t>[视频]李强同孟加拉国总理会谈</t>
+        </is>
+      </c>
+      <c r="D1646" t="inlineStr">
+        <is>
+          <t>李强与孟加拉国总理会谈，强调深化“一带一路”合作，拓展经贸、新能源等领域合作。</t>
+        </is>
+      </c>
+      <c r="E1646" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1646" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDE3QGehiuAQ4xOC5EsriX7260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1647" t="inlineStr">
+        <is>
+          <t>[视频]十四届全国人大常委会举行第六十九次委员长会议</t>
+        </is>
+      </c>
+      <c r="D1647" t="inlineStr">
+        <is>
+          <t>十四届全国人大常委会举行委员长会议，审议商标法修订草案、中央决算等议题。</t>
+        </is>
+      </c>
+      <c r="E1647" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1647" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEJ8goTuaHsS1mNCPMmlQ9260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1648" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见柬埔寨人民党主席、参议院主席洪森</t>
+        </is>
+      </c>
+      <c r="D1648" t="inlineStr">
+        <is>
+          <t>赵乐际会见柬埔寨人民党主席洪森，强调加强战略协作和立法机构交流。</t>
+        </is>
+      </c>
+      <c r="E1648" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1648" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEH1TxWaSdK2WA9KnOgpRU260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C1649" t="inlineStr">
+        <is>
+          <t>[视频]“在高质量发展中保障和改善民生”形势政策系列报告会第二场报告会在京举行</t>
+        </is>
+      </c>
+      <c r="D1649" t="inlineStr">
+        <is>
+          <t>科技部党组书记阴和俊表示，科技创新对增进民生福祉、支撑现代化产业体系作用更加有力，要加快实现高水平科技自立自强。</t>
+        </is>
+      </c>
+      <c r="E1649" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1649" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEd2R0czzvhXjWchmaKmxO260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1650" t="inlineStr">
+        <is>
+          <t>Trump asks Congress for billions for Iran war, after tension with Republicans</t>
+        </is>
+      </c>
+      <c r="D1650" t="inlineStr">
+        <is>
+          <t>特朗普向国会申请数十亿美元用于对伊战争，与共和党关系紧张。</t>
+        </is>
+      </c>
+      <c r="E1650" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1650" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1eydwldzdjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1651" t="inlineStr">
+        <is>
+          <t>Key figure in South Africa police corruption scandal pleads guilty</t>
+        </is>
+      </c>
+      <c r="D1651" t="inlineStr">
+        <is>
+          <t>南非警方腐败案关键人物认罪，将提供高官涉案证据。</t>
+        </is>
+      </c>
+      <c r="E1651" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1651" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2j4g5k52jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>Supreme Court allows Trump to restrict asylum seekers at border</t>
+        </is>
+      </c>
+      <c r="D1652" t="inlineStr">
+        <is>
+          <t>最高法院允许特朗普恢复针对边境寻求庇护者的限制政策。</t>
+        </is>
+      </c>
+      <c r="E1652" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1652" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4g8ym422lko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>Trump airs grievances with NATO chief over alliance's lack of Iran war support</t>
+        </is>
+      </c>
+      <c r="D1653" t="inlineStr">
+        <is>
+          <t>特朗普与北约秘书长会面，抱怨盟友未支持对伊朗战争。</t>
+        </is>
+      </c>
+      <c r="E1653" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1653" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/nx-s1-5869806/trump-airs-grievances-with-nato-chief-over-alliances-lack-of-iran-war-support</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>Former U.S. ambassador to NATO on the relationship between the alliance and Trump</t>
+        </is>
+      </c>
+      <c r="D1654" t="inlineStr">
+        <is>
+          <t>前美国驻北约大使分析北约与特朗普的关系动态。</t>
+        </is>
+      </c>
+      <c r="E1654" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1654" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/nx-s1-5869554/former-u-s-ambassador-to-nato-on-the-relationship-between-the-alliance-and-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>经济, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥出席第九届中国—亚欧博览会开幕式并会见与会外国政要</t>
+        </is>
+      </c>
+      <c r="D1655" t="inlineStr">
+        <is>
+          <t>第九届中国—亚欧博览会在新疆开幕，丁薛祥致辞提出加强亚欧合作四点建议。</t>
+        </is>
+      </c>
+      <c r="E1655" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1655" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEZDFD4NdA1WZEBWGDzng9260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>[视频]我国土地资源利用效率全面提升</t>
+        </is>
+      </c>
+      <c r="D1656" t="inlineStr">
+        <is>
+          <t>全国土地日发布数据：我国土地资源利用效率提升，盘活存量土地198万亩。</t>
+        </is>
+      </c>
+      <c r="E1656" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1656" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEjnDP63keZHolb87jcHvM260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>[视频]发电装机突破40亿千瓦 电力供给能力迈上新台阶</t>
+        </is>
+      </c>
+      <c r="D1657" t="inlineStr">
+        <is>
+          <t>截至5月底，全国发电装机容量突破40亿千瓦居世界首位，电力供给更绿色，非化石能源占比达62%。</t>
+        </is>
+      </c>
+      <c r="E1657" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1657" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDErm8nD0yb4gsmoBqnXvRk260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>[视频]前4个月我国新兴产业和未来产业新设企业37.3万户</t>
+        </is>
+      </c>
+      <c r="D1658" t="inlineStr">
+        <is>
+          <t>前4月我国新兴产业和未来产业新设企业37.3万户，生成式人工智能领域同比增长24.9%。</t>
+        </is>
+      </c>
+      <c r="E1658" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1658" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEMMIGUrn6AlOZORw9GNBo260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>[视频]【新闻特写】中国创新为全球发展注入新机遇</t>
+        </is>
+      </c>
+      <c r="D1659" t="inlineStr">
+        <is>
+          <t>第十七届夏季达沃斯论坛闭幕，中国创新成果成为焦点，为全球提供发展机遇。</t>
+        </is>
+      </c>
+      <c r="E1659" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1659" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDExg45FVl9LShAn8X517vR260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>Oil price falls back to pre-Iran war levels</t>
+        </is>
+      </c>
+      <c r="D1660" t="inlineStr">
+        <is>
+          <t>霍尔木兹海峡航运逐步恢复，油价回落至对伊开战前水平。</t>
+        </is>
+      </c>
+      <c r="E1660" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1660" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0jy7d7wzv4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>IBM hails new 'block of flats' design breakthrough for ultra tiny chips</t>
+        </is>
+      </c>
+      <c r="D1661" t="inlineStr">
+        <is>
+          <t>IBM宣称突破1纳米以下芯片技术，但量产尚需时日。</t>
+        </is>
+      </c>
+      <c r="E1661" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1661" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg7vpyn5pxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>Anthropic accuses Chinese rival Alibaba of illicitly extracting AI capabilities</t>
+        </is>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>Anthropic指控中国阿里非法获取其AI模型数据。</t>
+        </is>
+      </c>
+      <c r="E1662" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1662" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyklykn5dwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>The science behind the back-to-back earthquakes that struck northern Venezuela</t>
+        </is>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>专家解析委内瑞拉、日本及加州连续地震的科学原因。</t>
+        </is>
+      </c>
+      <c r="E1663" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1663" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/nx-s1-5869928/the-science-behind-the-back-to-back-earthquakes-that-struck-northern-venezuela</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr">
+        <is>
+          <t>How is Moscow dealing with Ukraine's stepped-up drone attacks?</t>
+        </is>
+      </c>
+      <c r="D1664" t="inlineStr">
+        <is>
+          <t>莫斯科应对乌克兰无人机攻击加剧的局面。</t>
+        </is>
+      </c>
+      <c r="E1664" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1664" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/nx-s1-5869503/how-is-moscow-dealing-with-ukraines-stepped-up-drone-attacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1665" t="inlineStr">
+        <is>
+          <t>第12批药品集采启动；平陆运河枢纽工程进入有水联调；拉林铁路运客超625万；毒品犯罪下降。</t>
+        </is>
+      </c>
+      <c r="E1665" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1665" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEDqfvQXiSP5i9kMrFhFZl260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr">
+        <is>
+          <t>Ryanair says it will reluctantly not charge parents to sit next to children</t>
+        </is>
+      </c>
+      <c r="D1666" t="inlineStr">
+        <is>
+          <t>瑞安航空将不再向带幼童家长收取选座费。</t>
+        </is>
+      </c>
+      <c r="E1666" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1666" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdr4zy4e1n1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr">
+        <is>
+          <t>Number of children getting special educational needs support hits another record high</t>
+        </is>
+      </c>
+      <c r="D1667" t="inlineStr">
+        <is>
+          <t>英国获得特殊教育支持儿童数量创历史新高。</t>
+        </is>
+      </c>
+      <c r="E1667" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1667" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj4g18gy14no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr">
+        <is>
+          <t>[视频]委内瑞拉发生7级以上强震 至少164人遇难</t>
+        </is>
+      </c>
+      <c r="D1668" t="inlineStr">
+        <is>
+          <t>委内瑞拉发生7级以上强震，已致164人遇难、971人受伤，全国进入紧急状态。</t>
+        </is>
+      </c>
+      <c r="E1668" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1668" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDE90hyY98hTDQSiFPY2jY8260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr">
+        <is>
+          <t>[视频]日本岩手县附近海域发生强震</t>
+        </is>
+      </c>
+      <c r="D1669" t="inlineStr">
+        <is>
+          <t>日本岩手县附近海域发生7.2级地震，造成至少6人受伤，部分新干线暂停运行。</t>
+        </is>
+      </c>
+      <c r="E1669" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1669" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEGjUckx9jgU37XwwMD4iH260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr">
+        <is>
+          <t>[视频]美巴官员表示美伊技术性谈判本月底继续</t>
+        </is>
+      </c>
+      <c r="D1670" t="inlineStr">
+        <is>
+          <t>美伊技术性谈判将于月底继续；国际油价跌破70美元，金价跌破4000美元。</t>
+        </is>
+      </c>
+      <c r="E1670" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1670" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDE5o35PWUA3uKwTbuQB0XJ260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>国际, 军事, 民生</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1671" t="inlineStr">
+        <is>
+          <t>俄乌互有打击；欧洲高温破纪录；国际奥委会修改宪章强调体育中立。</t>
+        </is>
+      </c>
+      <c r="E1671" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1671" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/25/VIDEYHwqNZXoZM0mX0glFt2M260625.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr">
+        <is>
+          <t>'I thought I was going to die' - Venezuelans describe earthquake panic</t>
+        </is>
+      </c>
+      <c r="D1672" t="inlineStr">
+        <is>
+          <t>委内瑞拉首都加拉加斯地震导致建筑倒塌，废墟下有呼救声。</t>
+        </is>
+      </c>
+      <c r="E1672" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1672" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czj8vjvmz38o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr">
+        <is>
+          <t>Earthquake is devastating blow to Venezuela at time of uncertainty</t>
+        </is>
+      </c>
+      <c r="D1673" t="inlineStr">
+        <is>
+          <t>委内瑞拉接连遭遇两次地震，前领导人马杜罗半年前被美军抓捕。</t>
+        </is>
+      </c>
+      <c r="E1673" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1673" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3vynpw7rk4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr">
+        <is>
+          <t>Europe's heatwave shifts east as France raises health alert to highest level</t>
+        </is>
+      </c>
+      <c r="D1674" t="inlineStr">
+        <is>
+          <t>欧洲热浪东移，德国气温或达40℃，法国高温已致年轻人死亡。</t>
+        </is>
+      </c>
+      <c r="E1674" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1674" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwy0pdq89zno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr">
+        <is>
+          <t>Families lay flowers on barbed wire barricade on anniversary of deadly Kenya protests</t>
+        </is>
+      </c>
+      <c r="D1675" t="inlineStr">
+        <is>
+          <t>肯尼亚抗议周年，家属在铁丝网献花要求为死难者伸张正义。</t>
+        </is>
+      </c>
+      <c r="E1675" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1675" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgqjl8kj8wpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr">
+        <is>
+          <t>People flee as building collapses on Caracas outskirts</t>
+        </is>
+      </c>
+      <c r="D1676" t="inlineStr">
+        <is>
+          <t>委内瑞拉首都附近建筑因强震倒塌，居民逃离。</t>
+        </is>
+      </c>
+      <c r="E1676" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1676" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c78y1e3606vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr">
+        <is>
+          <t>TikTok influencer charged with Dubai murder</t>
+        </is>
+      </c>
+      <c r="D1677" t="inlineStr">
+        <is>
+          <t>23岁英国TikTok网红因刺死伴侣在迪拜被控谋杀。</t>
+        </is>
+      </c>
+      <c r="E1677" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1677" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwy0p813jn7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr">
+        <is>
+          <t>2 earthquakes in Venezuela kill at least 164. And, Trump cancels housing bill signing</t>
+        </is>
+      </c>
+      <c r="D1678" t="inlineStr">
+        <is>
+          <t>委内瑞拉两次地震致164人死亡；特朗普取消住房法案签署。</t>
+        </is>
+      </c>
+      <c r="E1678" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1678" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/g-s1-130184/up-first-newsletter-venezuela-earthquakes-trump-senate-tensions-chris-donahue</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr">
+        <is>
+          <t>'They can kill you': Immigrants fear a surge in xenophobic violence in South Africa</t>
+        </is>
+      </c>
+      <c r="D1679" t="inlineStr">
+        <is>
+          <t>南非移民恐惧排外暴力激增，多起袭击致人死亡。</t>
+        </is>
+      </c>
+      <c r="E1679" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1679" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/25/nx-s1-5866241/they-can-kill-you-immigrants-fear-a-surge-in-xenophobic-violence-in-south-africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr">
+        <is>
+          <t>'Disruptive' passenger restrained on Jet2 flight dies</t>
+        </is>
+      </c>
+      <c r="D1680" t="inlineStr">
+        <is>
+          <t>Jet2航班上被制服的“扰乱”乘客在机上死亡。</t>
+        </is>
+      </c>
+      <c r="E1680" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1680" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c17ypedelk9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr">
+        <is>
+          <t>Teenager cleared of murdering nine-year-old girl</t>
+        </is>
+      </c>
+      <c r="D1681" t="inlineStr">
+        <is>
+          <t>16岁少年被布里斯托法院裁定谋杀9岁女孩罪名不成立。</t>
+        </is>
+      </c>
+      <c r="E1681" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1681" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9320y90lnno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr">
+        <is>
+          <t>Council sorry for parking fines after fatal train crash near Bedford</t>
+        </is>
+      </c>
+      <c r="D1682" t="inlineStr">
+        <is>
+          <t>贝德福德致命火车事故后，被困乘客车辆被贴罚单，议会致歉。</t>
+        </is>
+      </c>
+      <c r="E1682" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1682" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c70y8128w1wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr">
+        <is>
+          <t>The death toll rises to 164 after major Venezuela earthquakes topple many buildings</t>
+        </is>
+      </c>
+      <c r="D1683" t="inlineStr">
+        <is>
+          <t>委内瑞拉连续强震致164死971伤，多栋建筑倒塌。</t>
+        </is>
+      </c>
+      <c r="E1683" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1683" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/24/nx-s1-5869817/2-major-earthquakes-strike-northern-venezuela-near-caracas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr">
+        <is>
+          <t>The games that show the flaws in a 48-team World Cup</t>
+        </is>
+      </c>
+      <c r="D1684" t="inlineStr">
+        <is>
+          <t>小组赛最后两场可默契打平，暴露48队世界杯赛制缺陷。</t>
+        </is>
+      </c>
+      <c r="E1684" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1684" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cgev2vdzjvvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-26
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1684"/>
+  <dimension ref="A1:F1728"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54325,6 +54325,1414 @@
         </is>
       </c>
     </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>政治, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260626 19:00</t>
+        </is>
+      </c>
+      <c r="D1685" t="inlineStr">
+        <is>
+          <t>习近平会见柬埔寨、孟加拉国领导人；签署主席令；就委内瑞拉地震致慰问电；国内多领域进展及国际新闻。</t>
+        </is>
+      </c>
+      <c r="E1685" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1685" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDE9fFr2DOnONHI02XxdBAx260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见柬埔寨人民党主席、参议院主席洪森</t>
+        </is>
+      </c>
+      <c r="D1686" t="inlineStr">
+        <is>
+          <t>习近平会见柬埔寨人民党主席洪森，强调筑牢战略互信，推动中柬命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E1686" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1686" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEtqMwBVyENaFQXg4LkPJO260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见孟加拉国总理</t>
+        </is>
+      </c>
+      <c r="D1687" t="inlineStr">
+        <is>
+          <t>习近平会见孟加拉国总理，宣布构建新时代中孟命运共同体，深化合作。</t>
+        </is>
+      </c>
+      <c r="E1687" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1687" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEQsoUlsFJhrBwrcdQQBZ3260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr">
+        <is>
+          <t>[视频]习近平签署国家主席令</t>
+        </is>
+      </c>
+      <c r="D1688" t="inlineStr">
+        <is>
+          <t>习近平签署主席令，公布修订后的商标法、修改注册会计师法决定及人事任免。</t>
+        </is>
+      </c>
+      <c r="E1688" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1688" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEY0DThpVaNmkG17kkrvIw260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr">
+        <is>
+          <t>[视频]李强会见柬埔寨人民党主席、参议院主席洪森</t>
+        </is>
+      </c>
+      <c r="D1689" t="inlineStr">
+        <is>
+          <t>李强会见柬埔寨人民党主席洪森，同意深化政治互信与多领域合作。</t>
+        </is>
+      </c>
+      <c r="E1689" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1689" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDE5wbCaWX1q51xHiGIElwI260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr">
+        <is>
+          <t>[视频]十四届全国人大常委会第二十三次会议在京闭幕</t>
+        </is>
+      </c>
+      <c r="D1690" t="inlineStr">
+        <is>
+          <t>十四届全国人大常委会闭幕，通过商标法修订等多项法律及人事任免。</t>
+        </is>
+      </c>
+      <c r="E1690" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1690" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEOheNiXjwOYdoIObOZvm4260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见孟加拉国总理</t>
+        </is>
+      </c>
+      <c r="D1691" t="inlineStr">
+        <is>
+          <t>赵乐际会见孟加拉国总理，强调深化政治互信与立法机构交流。</t>
+        </is>
+      </c>
+      <c r="E1691" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1691" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEg6QoJYxPbeSKokgj9XCl260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥在新疆调研</t>
+        </is>
+      </c>
+      <c r="D1692" t="inlineStr">
+        <is>
+          <t>丁薛祥在新疆调研，强调推动高质量发展，加强能源保供和中欧班列建设。</t>
+        </is>
+      </c>
+      <c r="E1692" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1692" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEOUloIqJmO17eASUDEdz5260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>How transparent are the royals being about money?</t>
+        </is>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>国王公开纳税情况后，王室财务透明度仍遭质疑。</t>
+        </is>
+      </c>
+      <c r="E1693" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1693" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c77yzgnp5lvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>Ex-Trump adviser John Bolton pleads guilty to mishandling classified documents</t>
+        </is>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>前特朗普顾问博尔顿对不当处理机密文件认罪，面临最高5年监禁和225万美元罚款。</t>
+        </is>
+      </c>
+      <c r="E1694" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1694" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czxqwg4nrvlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>Mahmood restricts minister's access to documents as Home Office row escalates</t>
+        </is>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>内政部长马哈茂德限制大臣文件查阅权，因对其文章内容不满，首相正在考虑建议。</t>
+        </is>
+      </c>
+      <c r="E1695" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1695" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj9g7w0xnnjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>South Korean ex-first lady sentenced to 7 years for bribery scandal</t>
+        </is>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>韩国前第一夫人因贿赂案被判7年，此前另一涉及统一教的案件已判4年。</t>
+        </is>
+      </c>
+      <c r="E1696" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1696" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/g-s1-130372/south-korean-ex-first-lady-sentenced-to-7-years-for-bribery-scandal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】到2030年我国将初步建成新型能源体系</t>
+        </is>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>我国规划到2030年初步建成新型能源体系，新能源装机将成主体。</t>
+        </is>
+      </c>
+      <c r="E1697" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1697" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEzet2k1sG2kAZbOzbBXrm260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>经济, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>联播快讯：发布工业产品清单、设立养老服务师、AI微短剧新规、天台抽水蓄能电站投产。</t>
+        </is>
+      </c>
+      <c r="E1698" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1698" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEmAeUo2rjG53EtoGFyp1W260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>Asia stock markets slide as tech shares slump</t>
+        </is>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>亚洲股市因科技股暴跌下滑，韩国Kospi指数本周第三次暂停交易以防恐慌抛售。</t>
+        </is>
+      </c>
+      <c r="E1699" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1699" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce8jz40k00ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>Senior Ukrainian intelligence official jailed for life for spying for Russia</t>
+        </is>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>乌克兰高级情报官员因长期向俄罗斯泄密被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E1700" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1700" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cg4w3wyxzzno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>Ukraine unleashes one of its heaviest drone bombardments, as Russia strikes Ukraine</t>
+        </is>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>乌克兰对俄罗斯多地发动大规模无人机袭击，俄方也攻击乌克兰多地区，战事持续。</t>
+        </is>
+      </c>
+      <c r="E1701" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1701" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/nx-s1-5872256/russia-ukraine-war-drone-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr">
+        <is>
+          <t>[视频]习近平就委内瑞拉发生强烈地震向委内瑞拉代总统致慰问电</t>
+        </is>
+      </c>
+      <c r="D1702" t="inlineStr">
+        <is>
+          <t>习近平就委内瑞拉强烈地震致慰问电，表示中方将提供救灾和重建帮助。</t>
+        </is>
+      </c>
+      <c r="E1702" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1702" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEDdL2dswGXGwwUdsZCbHq260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr">
+        <is>
+          <t>[视频]委内瑞拉强震遇难人数升至235人 救援持续进行</t>
+        </is>
+      </c>
+      <c r="D1703" t="inlineStr">
+        <is>
+          <t>委内瑞拉强震致235人遇难，救援持续，政府宣布多项应对措施。</t>
+        </is>
+      </c>
+      <c r="E1703" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1703" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEc0c3YKN2mKyHcWrVfQnK260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr">
+        <is>
+          <t>[视频]伊朗和阿曼两国外长通话讨论霍尔木兹海峡问题</t>
+        </is>
+      </c>
+      <c r="D1704" t="inlineStr">
+        <is>
+          <t>伊朗与阿曼通话讨论霍尔木兹海峡管理，海湾国家强调航行自由。</t>
+        </is>
+      </c>
+      <c r="E1704" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1704" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEU9WumuP25pnvb7GRjNXA260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1705" t="inlineStr">
+        <is>
+          <t>以称将无限期驻留黎南部等地；白俄罗斯警告乌克兰勿激化局势。</t>
+        </is>
+      </c>
+      <c r="E1705" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1705" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEDjK0fMAQhkCfEMl388tQ260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr">
+        <is>
+          <t>Earthquake is devastating blow to Venezuela at time of uncertainty</t>
+        </is>
+      </c>
+      <c r="D1706" t="inlineStr">
+        <is>
+          <t>委内瑞拉发生双震，政局本已因前领导人被美军抓捕而不稳。</t>
+        </is>
+      </c>
+      <c r="E1706" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1706" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3vynpw7rk4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr">
+        <is>
+          <t>Aerial footage reveals destruction in coastal Venezuela</t>
+        </is>
+      </c>
+      <c r="D1707" t="inlineStr">
+        <is>
+          <t>航拍显示委内瑞拉沿海城市拉瓜伊拉在地震中多栋高楼倒塌。</t>
+        </is>
+      </c>
+      <c r="E1707" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1707" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c75y1kd16qdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr">
+        <is>
+          <t>UN pauses Strait of Hormuz evacuation plan after cargo ship attacked</t>
+        </is>
+      </c>
+      <c r="D1708" t="inlineStr">
+        <is>
+          <t>货船在阿曼附近被不明弹丸袭击，联合国暂停霍尔木兹海峡疏散计划。</t>
+        </is>
+      </c>
+      <c r="E1708" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1708" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjwg9np904qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr">
+        <is>
+          <t>US sanctions Rwanda gold refinery accused of smuggling DR Congo's minerals</t>
+        </is>
+      </c>
+      <c r="D1709" t="inlineStr">
+        <is>
+          <t>美国制裁卢旺达一家金矿精炼厂，指控其2026年初走私至少60公斤刚果黄金。</t>
+        </is>
+      </c>
+      <c r="E1709" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1709" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9d268xy90xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr">
+        <is>
+          <t>Rescuers scramble to find Venezuela earthquake survivors. And, SCOTUS rules on asylum</t>
+        </is>
+      </c>
+      <c r="D1710" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震后救援人员搜寻数千失踪者；美国最高法院裁定可拒绝边境庇护申请。</t>
+        </is>
+      </c>
+      <c r="E1710" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1710" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/g-s1-130361/up-first-newsletter-venezuela-earthquakes-asylum-claims-farmers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr">
+        <is>
+          <t>Aid worker says hundreds remain trapped after Venezuela earthquakes</t>
+        </is>
+      </c>
+      <c r="D1711" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震致首都多栋建筑倒塌，数百人被困，救援队正全力搜救。</t>
+        </is>
+      </c>
+      <c r="E1711" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1711" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/nx-s1-5870683/venezuela-earthquakes-rescue-efforts</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr">
+        <is>
+          <t>Venezuela reels from earthquakes, as death toll more than doubles</t>
+        </is>
+      </c>
+      <c r="D1712" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震死亡人数翻倍，经济与医疗系统瘫痪加剧救援困难。</t>
+        </is>
+      </c>
+      <c r="E1712" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1712" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/nx-s1-5870651/venezuela-earthquakes-caracas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr">
+        <is>
+          <t>UN agency pauses evacuation of ships through the Strait of Hormuz after attack on vessel</t>
+        </is>
+      </c>
+      <c r="D1713" t="inlineStr">
+        <is>
+          <t>英国称船只遭袭击后，联合国机构暂停霍尔木兹海峡船舶撤离。</t>
+        </is>
+      </c>
+      <c r="E1713" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1713" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/nx-s1-5871963/un-agency-pauses-evacuation-of-ships-through-strait-of-hormuz-after-attack-vessel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr">
+        <is>
+          <t>King Charles III will not live at Buckingham Palace after its costly refurbishment</t>
+        </is>
+      </c>
+      <c r="D1714" t="inlineStr">
+        <is>
+          <t>查尔斯三世因白金汉宫翻修费用高昂，决定不再居住于此。</t>
+        </is>
+      </c>
+      <c r="E1714" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1714" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/g-s1-130347/king-charles-buckingham-palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr">
+        <is>
+          <t>[视频]红色旅游升温 汇聚奋进力量</t>
+        </is>
+      </c>
+      <c r="D1715" t="inlineStr">
+        <is>
+          <t>“七一”临近，各地红色旅游升温，人们通过参观学习传承革命精神。</t>
+        </is>
+      </c>
+      <c r="E1715" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1715" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEEc1WnjmbHGwe2hLMxwhL260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr">
+        <is>
+          <t>[视频]国际禁毒日：各地开展形式多样的禁毒主题宣传活动</t>
+        </is>
+      </c>
+      <c r="D1716" t="inlineStr">
+        <is>
+          <t>国际禁毒日各地开展以防范青少年药物滥用为主题的宣传活动。</t>
+        </is>
+      </c>
+      <c r="E1716" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1716" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/26/VIDEJPuhrvFMYhfD1LXaH8Cn260626.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr">
+        <is>
+          <t>Christmas market attacker jailed for life for murdering six in Germany</t>
+        </is>
+      </c>
+      <c r="D1717" t="inlineStr">
+        <is>
+          <t>德国圣诞市场驾车袭击案凶手因谋杀6人被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E1717" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1717" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy06y63y6lno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr">
+        <is>
+          <t>Reflecting Pool liner cut with sharp knife or razor, National Park Service says</t>
+        </is>
+      </c>
+      <c r="D1718" t="inlineStr">
+        <is>
+          <t>美国国家公园管理局称倒影池衬垫被利刃割破，特朗普此前指责人为破坏。</t>
+        </is>
+      </c>
+      <c r="E1718" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1718" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn8qxz6qypyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr">
+        <is>
+          <t>Four men held over child-marriage in Sierra Leone set to appear in landmark court case</t>
+        </is>
+      </c>
+      <c r="D1719" t="inlineStr">
+        <is>
+          <t>塞拉利昂四名男子因涉及17岁女孩童婚案将首次出庭受审。</t>
+        </is>
+      </c>
+      <c r="E1719" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1719" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9q212y8p21o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr">
+        <is>
+          <t>New bodycam footage shows Henry Nowak killer's arrest and repeated lies to police</t>
+        </is>
+      </c>
+      <c r="D1720" t="inlineStr">
+        <is>
+          <t>新执法记录仪视频显示，亨利·诺瓦克杀手被捕时向警方反复撒谎。</t>
+        </is>
+      </c>
+      <c r="E1720" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1720" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yzl5xl3gjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr">
+        <is>
+          <t>Court rules 13 men who allegedly helped rapist drug and abuse wife can be named</t>
+        </is>
+      </c>
+      <c r="D1721" t="inlineStr">
+        <is>
+          <t>法院裁定13名涉嫌帮助强奸犯对妻子下药并施虐的男子身份可公开。</t>
+        </is>
+      </c>
+      <c r="E1721" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1721" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cnv9er181lno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr">
+        <is>
+          <t>Watch: Moment woman pulled from rubble alive</t>
+        </is>
+      </c>
+      <c r="D1722" t="inlineStr">
+        <is>
+          <t>在拉瓜伊拉，救援人员从倒塌建筑废墟中成功救出一名生还者。</t>
+        </is>
+      </c>
+      <c r="E1722" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1722" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/clyxgxr2672o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr">
+        <is>
+          <t>Tate brothers lose court bid to be told names of their UK accusers</t>
+        </is>
+      </c>
+      <c r="D1723" t="inlineStr">
+        <is>
+          <t>泰特兄弟败诉，无法获知英国指控者姓名，将面临强奸等多项指控。</t>
+        </is>
+      </c>
+      <c r="E1723" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1723" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2dyrw36gzjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr">
+        <is>
+          <t>Plane crashes into Beijing's tallest building; damage reported</t>
+        </is>
+      </c>
+      <c r="D1724" t="inlineStr">
+        <is>
+          <t>一架飞机撞上北京最高建筑造成损坏，原因未获独立证实，当局尚未回应。</t>
+        </is>
+      </c>
+      <c r="E1724" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1724" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/g-s1-130388/beijings-tallest-building-is-damaged-after-small-airplane-reportedly-crashed-into-it</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr">
+        <is>
+          <t>Australia plans to strengthen laws banning children from social media</t>
+        </is>
+      </c>
+      <c r="D1725" t="inlineStr">
+        <is>
+          <t>澳大利亚计划加强禁止儿童使用社交媒体的法律，因现有禁令被指执行不力。</t>
+        </is>
+      </c>
+      <c r="E1725" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1725" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/26/g-s1-130375/australia-plans-to-strengthen-laws-banning-children-from-social-media</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr">
+        <is>
+          <t>Canada eligible to join Eurovision competition</t>
+        </is>
+      </c>
+      <c r="D1726" t="inlineStr">
+        <is>
+          <t>加拿大总理在2025年预算中提议加入欧洲歌唱大赛，获参赛资格。</t>
+        </is>
+      </c>
+      <c r="E1726" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1726" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy06yzp4r0eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr">
+        <is>
+          <t>BBC DJ and presenter Trevor Nelson taking a break from work due to health issues</t>
+        </is>
+      </c>
+      <c r="D1727" t="inlineStr">
+        <is>
+          <t>BBC主持人特雷弗·纳尔逊因健康问题暂停工作，称将专注康复。</t>
+        </is>
+      </c>
+      <c r="E1727" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1727" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gykyenweyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr">
+        <is>
+          <t>Rainbow flags await Egypt and Iran at Pride Match</t>
+        </is>
+      </c>
+      <c r="D1728" t="inlineStr">
+        <is>
+          <t>伊朗与埃及在关键小组赛相遇，伊朗教练拒绝讨论在西雅图的骄傲庆祝活动。</t>
+        </is>
+      </c>
+      <c r="E1728" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1728" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/ckg4k0ddg5go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-27
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1728"/>
+  <dimension ref="A1:F1764"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -55733,6 +55733,1158 @@
         </is>
       </c>
     </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260627 19:00</t>
+        </is>
+      </c>
+      <c r="D1729" t="inlineStr">
+        <is>
+          <t>本期《新闻联播》主要报道高质量发展、政绩观教育、红色旅游、基层党建、文艺界大会、工业企业利润增长及夏粮收购等。</t>
+        </is>
+      </c>
+      <c r="E1729" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1729" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDE2wKH0GTCokDZLb8J73cm260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】促发展 惠民生 各地推动学习教育见行见效</t>
+        </is>
+      </c>
+      <c r="D1730" t="inlineStr">
+        <is>
+          <t>海口、郴州等地推动政绩观学习教育，化解信访积案，优化医保拨付，惠民生促发展。</t>
+        </is>
+      </c>
+      <c r="E1730" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1730" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEiaX4M2c06lI3c1VczN5B260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】筑牢基层战斗堡垒 建设幸福和美乡村</t>
+        </is>
+      </c>
+      <c r="D1731" t="inlineStr">
+        <is>
+          <t>河南兰考代庄村通过党建引领，发展“共富工坊”等产业，从软弱涣散村变为乡村振兴样板。</t>
+        </is>
+      </c>
+      <c r="E1731" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1731" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEKNdYQ47Gum2nZdzeONMp260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr">
+        <is>
+          <t>Billionaire Leon Black walks out of Epstein investigation hearing</t>
+        </is>
+      </c>
+      <c r="D1732" t="inlineStr">
+        <is>
+          <t>亿万富翁Leon Black因爱泼斯坦调查听证会拒绝作证，遭众议院传票要求宣誓录像作证。</t>
+        </is>
+      </c>
+      <c r="E1732" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1732" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn948lwyl3jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr">
+        <is>
+          <t>Ex-Trump adviser John Bolton pleads guilty to mishandling classified documents</t>
+        </is>
+      </c>
+      <c r="D1733" t="inlineStr">
+        <is>
+          <t>前特朗普顾问John Bolton承认处理机密文件不当，面临最高五年监禁及225万美元罚款。</t>
+        </is>
+      </c>
+      <c r="E1733" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1733" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czxqwg4nrvlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr">
+        <is>
+          <t>Mahmood announces new refugee sponsorship route into UK</t>
+        </is>
+      </c>
+      <c r="D1734" t="inlineStr">
+        <is>
+          <t>英内政大臣宣布新难民庇护路线，称上限安全合法途径将恢复庇护系统信心。</t>
+        </is>
+      </c>
+      <c r="E1734" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1734" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz952dm74o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr">
+        <is>
+          <t>Is Andy Burnham Labour's saviour, or just its best bet?</t>
+        </is>
+      </c>
+      <c r="D1735" t="inlineStr">
+        <is>
+          <t>工党内部评价安迪·伯纳姆被视为取代斯塔默的首相人选。</t>
+        </is>
+      </c>
+      <c r="E1735" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1735" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621e13n2dvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】以高质量发展引领中国经济航船破浪前行</t>
+        </is>
+      </c>
+      <c r="D1736" t="inlineStr">
+        <is>
+          <t>以习近平同志为核心的党中央加强党对经济工作的领导，中国经济跃上新台阶，GDP突破140万亿元。</t>
+        </is>
+      </c>
+      <c r="E1736" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1736" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEtu9yY2U3lnx7PqiKKu5m260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr">
+        <is>
+          <t>[视频]今年前5个月工业企业利润实现较快增长</t>
+        </is>
+      </c>
+      <c r="D1737" t="inlineStr">
+        <is>
+          <t>1-5月全国规上工业企业利润同比增18.8%，高技术制造业利润增44.7%，电子行业贡献突出。</t>
+        </is>
+      </c>
+      <c r="E1737" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1737" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEHjDRpJkdp5eMAiHkL9BI260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr">
+        <is>
+          <t>[视频]夏粮收购陆续展开 质优价稳购销两旺</t>
+        </is>
+      </c>
+      <c r="D1738" t="inlineStr">
+        <is>
+          <t>夏粮收购进展顺利，累计超4000万吨，AI检测提速，市场质优价稳、购销两旺。</t>
+        </is>
+      </c>
+      <c r="E1738" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1738" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEJSZYhd7vmbEOIfPJq0Y0260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr">
+        <is>
+          <t>Just how much trouble is Canada's economy in?</t>
+        </is>
+      </c>
+      <c r="D1739" t="inlineStr">
+        <is>
+          <t>五张图表揭示加拿大经济困境，并对比其他富裕国家的表现。</t>
+        </is>
+      </c>
+      <c r="E1739" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1739" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c70y1y909pdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr">
+        <is>
+          <t>A historian analyzes whether Ukraine has a localized advantage in modern combat power</t>
+        </is>
+      </c>
+      <c r="D1740" t="inlineStr">
+        <is>
+          <t>历史学家分析乌克兰在现代作战中是否拥有局部优势。</t>
+        </is>
+      </c>
+      <c r="E1740" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1740" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/nx-s1-5869693/a-historian-analyzes-whether-ukraine-has-a-localized-advantage-in-modern-combat-power</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr">
+        <is>
+          <t>Inside a secretive Ukrainian team launching deep drone strikes at Russia</t>
+        </is>
+      </c>
+      <c r="D1741" t="inlineStr">
+        <is>
+          <t>乌克兰秘密行动组深入俄境内1200公里，用远程无人机袭击炼油设施。</t>
+        </is>
+      </c>
+      <c r="E1741" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1741" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/g-s1-129704/ukraine-long-range-drones-russia-war</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr">
+        <is>
+          <t>U.S. strikes Iran in response to a drone attack on a ship</t>
+        </is>
+      </c>
+      <c r="D1742" t="inlineStr">
+        <is>
+          <t>美军为报复无人机袭击商船，打击伊朗目标，考验美伊临时协议。</t>
+        </is>
+      </c>
+      <c r="E1742" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1742" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/nx-s1-5872954/us-strikes-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>民生, 科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1743" t="inlineStr">
+        <is>
+          <t>5月全国空气质量改善；美丽中国建设计划出台；核聚变超导磁体获突破；西康高铁联调联试；全球南方电力合作。</t>
+        </is>
+      </c>
+      <c r="E1743" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1743" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDElXw7wkG1vauAfeRFMl9O260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr">
+        <is>
+          <t>Hundreds of Heathrow and Gatwick flights delayed due to thunderstorms</t>
+        </is>
+      </c>
+      <c r="D1744" t="inlineStr">
+        <is>
+          <t>希思罗和盖特威克机场因雷暴延误，超800架航班受影响。</t>
+        </is>
+      </c>
+      <c r="E1744" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1744" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjwgynnwyw2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr">
+        <is>
+          <t>Are we in for a summer of serial heatwaves?</t>
+        </is>
+      </c>
+      <c r="D1745" t="inlineStr">
+        <is>
+          <t>预报称今夏可能比往年更热，出现连续热浪的风险增加。</t>
+        </is>
+      </c>
+      <c r="E1745" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1745" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/cgrk4w57e74o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr">
+        <is>
+          <t>[视频]中方：绝不允许“新型军国主义”成势为患</t>
+        </is>
+      </c>
+      <c r="D1746" t="inlineStr">
+        <is>
+          <t>中方在联合国强调绝不允许“新型军国主义”成势为患。</t>
+        </is>
+      </c>
+      <c r="E1746" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1746" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDE9FkDaogaLpSixH8BOA8Z260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr">
+        <is>
+          <t>[视频]委内瑞拉强震遇难人数升至920人</t>
+        </is>
+      </c>
+      <c r="D1747" t="inlineStr">
+        <is>
+          <t>委内瑞拉强震致920人遇难，含7名中国公民；政府实施军事化管理救灾。</t>
+        </is>
+      </c>
+      <c r="E1747" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDELczsl8h8yMx3dWN15aPC260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr">
+        <is>
+          <t>[视频]美称对伊朗目标实施打击 伊朗称已回击</t>
+        </is>
+      </c>
+      <c r="D1748" t="inlineStr">
+        <is>
+          <t>美打击伊朗目标，伊朗回击；黎以美达成停火撤军三方框架协议。</t>
+        </is>
+      </c>
+      <c r="E1748" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1748" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEDzGnmhg4i4Q9KPhJju7y260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>国际, 政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1749" t="inlineStr">
+        <is>
+          <t>欧盟回应美关税威胁；布基纳法索与法国断交；日本本州岛5.1级地震致17伤。</t>
+        </is>
+      </c>
+      <c r="E1749" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1749" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDExGvSrIdP0BK7qfQdE8Z6260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr">
+        <is>
+          <t>US strikes Iran after attack on cargo ship</t>
+        </is>
+      </c>
+      <c r="D1750" t="inlineStr">
+        <is>
+          <t>伊朗指控美国违反协议并称已袭击美军相关目标。</t>
+        </is>
+      </c>
+      <c r="E1750" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1750" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ckg590wqxwpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1751" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr">
+        <is>
+          <t>Venezuela earthquakes kill 920 people as international rescue teams arrive</t>
+        </is>
+      </c>
+      <c r="D1751" t="inlineStr">
+        <is>
+          <t>委内瑞拉强震致920人遇难，国际救援队抵达，数百人恐仍被困。</t>
+        </is>
+      </c>
+      <c r="E1751" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1751" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c39y79g7gzko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1752" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr">
+        <is>
+          <t>Newborn baby rescued from Venezuela earthquake rubble</t>
+        </is>
+      </c>
+      <c r="D1752" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震后，一名新生婴儿从废墟中被救出，地震致至少920人死亡。</t>
+        </is>
+      </c>
+      <c r="E1752" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1752" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/cm2d0vzp3ngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1753" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr">
+        <is>
+          <t>In Caracas, this feels like the hardest moment in Venezuela's modern history</t>
+        </is>
+      </c>
+      <c r="D1753" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震救援持续，但希望渺茫，民众愤怒情绪增长。</t>
+        </is>
+      </c>
+      <c r="E1753" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1753" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdjk8zwe7z3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1754" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr">
+        <is>
+          <t>Iran takes swipe at US' 'unfair treatment' and throws down gauntlet to Fifa</t>
+        </is>
+      </c>
+      <c r="D1754" t="inlineStr">
+        <is>
+          <t>伊朗教练指责美国在世界杯期间不公平对待，并向国际足联提出挑战。</t>
+        </is>
+      </c>
+      <c r="E1754" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1754" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cze98ywdwlgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr">
+        <is>
+          <t>Venezuelans in Colombia scramble to send aid as earthquakes death toll increases</t>
+        </is>
+      </c>
+      <c r="D1755" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震致近千人死亡，救援迟缓，旅哥侨胞紧急送物资。</t>
+        </is>
+      </c>
+      <c r="E1755" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1755" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/nx-s1-5872951/venezuela-earthquakes-colombia-aid</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr">
+        <is>
+          <t>[视频]传承红色基因 各地红色旅游升温</t>
+        </is>
+      </c>
+      <c r="D1756" t="inlineStr">
+        <is>
+          <t>七一临近，各地红色旅游升温，游客在纪念馆、革命旧址重温历史，传承革命精神。</t>
+        </is>
+      </c>
+      <c r="E1756" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1756" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDEpydaPUtouU9sA7Nuszb5260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr">
+        <is>
+          <t>Religion row as Texas makes Bible stories required reading in schools</t>
+        </is>
+      </c>
+      <c r="D1757" t="inlineStr">
+        <is>
+          <t>得州将圣经故事列为学校必修阅读，批评者称其侵犯宗教自由。</t>
+        </is>
+      </c>
+      <c r="E1757" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1757" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ckg8m2xkg84o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1758" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr">
+        <is>
+          <t>Pete Buttigieg briefly separated from children after false police report</t>
+        </is>
+      </c>
+      <c r="D1758" t="inlineStr">
+        <is>
+          <t>Pete Buttigieg因虚假报警与孩子短暂分离，称这是人生最黑暗的时刻之一。</t>
+        </is>
+      </c>
+      <c r="E1758" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwydx95kjx0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1759" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr">
+        <is>
+          <t>How completing the World Cup sticker book is like having a second job</t>
+        </is>
+      </c>
+      <c r="D1759" t="inlineStr">
+        <is>
+          <t>收集世界杯贴纸簿需大量时间和金钱，家庭通过停车场交易和小组省钱。</t>
+        </is>
+      </c>
+      <c r="E1759" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1759" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3eyv0v28gwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1760" t="inlineStr">
+        <is>
+          <t>文体, 政治</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr">
+        <is>
+          <t>[视频]中国音乐家协会第十次全国代表大会、中国舞蹈家协会第十二次全国代表大会、中国杂技家协会第九次全国代表大会在北京召开</t>
+        </is>
+      </c>
+      <c r="D1760" t="inlineStr">
+        <is>
+          <t>中国音协、舞协、杂协全国代表大会在京召开，强调锚定文化强国目标，推动艺术创作。</t>
+        </is>
+      </c>
+      <c r="E1760" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1760" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/27/VIDE6x3GyJG1WhG6x5o3kToe260627.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1761" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr">
+        <is>
+          <t>Who are the Panama players England need to look out for?</t>
+        </is>
+      </c>
+      <c r="D1761" t="inlineStr">
+        <is>
+          <t>BBC分析巴拿马关键球员，他们欲在世界杯小组赛爆冷击败英格兰。</t>
+        </is>
+      </c>
+      <c r="E1761" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1761" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/articles/cr47wd2d3ero?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1762" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr">
+        <is>
+          <t>Scotland's World Cup hopes at 0.07% - these are results they need</t>
+        </is>
+      </c>
+      <c r="D1762" t="inlineStr">
+        <is>
+          <t>苏格兰世界杯出线概率仅0.07%，负于巴西后需看其他赛果。</t>
+        </is>
+      </c>
+      <c r="E1762" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1762" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cx23rx038w1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1763" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr">
+        <is>
+          <t>Uzbekistan makes its World Cup debut, a first for Central Asia</t>
+        </is>
+      </c>
+      <c r="D1763" t="inlineStr">
+        <is>
+          <t>乌兹别克斯坦成为首个晋级世界杯的中亚国家，球迷展示国家文化。</t>
+        </is>
+      </c>
+      <c r="E1763" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1763" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/g-s1-129705/uzbekistan-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B1764" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr">
+        <is>
+          <t>There's a beef about beef at the World Cup, as Argentina fans pour into Texas</t>
+        </is>
+      </c>
+      <c r="D1764" t="inlineStr">
+        <is>
+          <t>阿根廷球迷涌入德州观战世界杯，引发美阿牛肉烹饪文化之争。</t>
+        </is>
+      </c>
+      <c r="E1764" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1764" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/27/nx-s1-5873328/beef-about-beef-world-cup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-28
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1764"/>
+  <dimension ref="A1:F1797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56885,6 +56885,1062 @@
         </is>
       </c>
     </row>
+    <row r="1765">
+      <c r="A1765" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1765" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260628 19:00</t>
+        </is>
+      </c>
+      <c r="D1765" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道党建、经济、军事、外交等多领域要闻，含以旧换新资金下达及国际动态。</t>
+        </is>
+      </c>
+      <c r="E1765" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDELu1LocjfYAPhyPSYiw8p260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1766" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】以习近平党建思想为引领 奋力走好新时代“赶考”路</t>
+        </is>
+      </c>
+      <c r="D1766" t="inlineStr">
+        <is>
+          <t>强调以习近平党建思想引领，推进新时代党的建设，开展正确政绩观学习教育。</t>
+        </is>
+      </c>
+      <c r="E1766" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1766" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDECNmpJNvjV4DIEb5jfq2u260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1767" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr">
+        <is>
+          <t>[视频]各地开展主题党日活动迎“七一”</t>
+        </is>
+      </c>
+      <c r="D1767" t="inlineStr">
+        <is>
+          <t>各地开展主题党日活动，新党员宣誓、瞻仰红船等，迎接“七一”建党节。</t>
+        </is>
+      </c>
+      <c r="E1767" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1767" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEjK2H7h8hkYkHKJzkJoyC260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1768" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr">
+        <is>
+          <t>[视频]中央层面树立和践行正确政绩观学习教育工作专班 中央纪委办公厅公开通报广西壮族自治区南宁市、甘肃省酒泉市新城区、浙江省杭州市萧山区3起政绩观偏差问题</t>
+        </is>
+      </c>
+      <c r="D1768" t="inlineStr">
+        <is>
+          <t>中央通报广西、甘肃、浙江三起政绩观偏差问题，涉及虚增财政、骗取国债等。</t>
+        </is>
+      </c>
+      <c r="E1768" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1768" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDE0bLRieM8snOr1yjYBuFS260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1769" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr">
+        <is>
+          <t>[视频]中国音乐家协会 中国舞蹈家协会 中国杂技家协会选举产生新一届领导机构</t>
+        </is>
+      </c>
+      <c r="D1769" t="inlineStr">
+        <is>
+          <t>中国音协、舞协、杂技家协会在京闭幕，选举产生新一届领导机构。</t>
+        </is>
+      </c>
+      <c r="E1769" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1769" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEFtkjbpSodeSxSfDzA1Ll260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1770" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr">
+        <is>
+          <t>Uganda's leading media outlets shut down by army chief</t>
+        </is>
+      </c>
+      <c r="D1770" t="inlineStr">
+        <is>
+          <t>乌干达陆军总部门令关闭主要媒体NTV和《每日观察报》。</t>
+        </is>
+      </c>
+      <c r="E1770" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1770" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj9gyk1z7ngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1771" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr">
+        <is>
+          <t>Senior Labour figures say party is united behind Andy Burnham</t>
+        </is>
+      </c>
+      <c r="D1771" t="inlineStr">
+        <is>
+          <t>工党高层称党内团结支持伯纳姆，无需竞争。</t>
+        </is>
+      </c>
+      <c r="E1771" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1771" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn0vkle1q5ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr">
+        <is>
+          <t>[视频]新一批支持消费品以旧换新资金下达</t>
+        </is>
+      </c>
+      <c r="D1772" t="inlineStr">
+        <is>
+          <t>第三批625亿元超长期国债支持消费品以旧换新，已带动销售额超1万亿元。</t>
+        </is>
+      </c>
+      <c r="E1772" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1772" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEnwzORzgmz3en9375q7uD260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr">
+        <is>
+          <t>[视频]前五个月我国物流运行结构优化 质效提升</t>
+        </is>
+      </c>
+      <c r="D1773" t="inlineStr">
+        <is>
+          <t>前5月全国物流总额146.6万亿元同比增5.2%，高端制造物流需求增长快。</t>
+        </is>
+      </c>
+      <c r="E1773" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1773" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEYjpfQWwxb8ffLZvucHvy260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>经济, 民生, 文体</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1774" t="inlineStr">
+        <is>
+          <t>1-5月农业保险赔付370亿；黄河三角洲生态补水启动；内地与香港贸易年均增长6.7%；暑期档票房超15亿。</t>
+        </is>
+      </c>
+      <c r="E1774" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1774" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEiETvkzRCdC6eHBKA7RI1260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号乘组在轨满月 各项任务进展顺利</t>
+        </is>
+      </c>
+      <c r="D1775" t="inlineStr">
+        <is>
+          <t>神舟二十三号乘组在轨满月，完成细胞实验、出舱安装及应急演练，状态良好。</t>
+        </is>
+      </c>
+      <c r="E1775" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1775" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEm5Et1ti3BXWKP30SPDzZ260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr">
+        <is>
+          <t>[视频]空军航空兵某团：锻造制胜空天的铁翼鲲鹏</t>
+        </is>
+      </c>
+      <c r="D1776" t="inlineStr">
+        <is>
+          <t>空军航空兵某团列装运油-20系列，创新训练模式提升战略投送与实战能力。</t>
+        </is>
+      </c>
+      <c r="E1776" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1776" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDEITFrjWYPkPpYmhNOXf8D260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr">
+        <is>
+          <t>Sort Your Life Out: The four most common cluttering mistakes and how to fix them</t>
+        </is>
+      </c>
+      <c r="D1777" t="inlineStr">
+        <is>
+          <t>整理专家分享厨房、客厅和衣物最常见的四种杂乱问题及解决方法。</t>
+        </is>
+      </c>
+      <c r="E1777" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1777" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgd54yvjz1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr">
+        <is>
+          <t>[视频]国际人士：中国共产党领导中国取得瞩目成就 对世界和平与发展意义重大</t>
+        </is>
+      </c>
+      <c r="D1778" t="inlineStr">
+        <is>
+          <t>国际人士称赞中国共产党领导中国取得瞩目成就，对世界和平与发展意义重大。</t>
+        </is>
+      </c>
+      <c r="E1778" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1778" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDE7YO07P3iCbcsmtVBkVXJ260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1779" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr">
+        <is>
+          <t>[视频]委内瑞拉强震遇难人数升至1430人</t>
+        </is>
+      </c>
+      <c r="D1779" t="inlineStr">
+        <is>
+          <t>委内瑞拉强震遇难人数升至1430人，含8名中国公民，搜救工作仍在进行。</t>
+        </is>
+      </c>
+      <c r="E1779" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1779" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDE3jG7FBj3INyeZ7bEaj4b260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>[视频]美国和伊朗分别打击对方目标 互指对方违反停火承诺</t>
+        </is>
+      </c>
+      <c r="D1780" t="inlineStr">
+        <is>
+          <t>美国和伊朗相互打击对方目标，互指对方违反停火承诺，局势紧张。</t>
+        </is>
+      </c>
+      <c r="E1780" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1780" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDECuhdDx1c7ucHpBg1EXQz260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1781" t="inlineStr">
+        <is>
+          <t>黎真主党拒认三方协议；美国肯塔基州洪灾致4死；意大利埃特纳火山喷发。</t>
+        </is>
+      </c>
+      <c r="E1781" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1781" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/28/VIDE8nfwVXrdxdWfCUF72OEA260628.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>Two boys rescued from Venezuela earthquake rubble after days of being trapped</t>
+        </is>
+      </c>
+      <c r="D1782" t="inlineStr">
+        <is>
+          <t>委内瑞拉强震后，两名被困数日的男孩被成功救出。</t>
+        </is>
+      </c>
+      <c r="E1782" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1782" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr47dvywvy5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>US and Iran exchange strikes and accuse each other of violating ceasefire</t>
+        </is>
+      </c>
+      <c r="D1783" t="inlineStr">
+        <is>
+          <t>伊朗对美军在科威特和巴林的目标发动报复性打击，美伊互指违约。</t>
+        </is>
+      </c>
+      <c r="E1783" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1783" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdxdwkgqgq0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>Eleven killed after plane carrying skydivers crashes in eastern France</t>
+        </is>
+      </c>
+      <c r="D1784" t="inlineStr">
+        <is>
+          <t>法国东部一架载有跳伞者的飞机坠毁，造成11人死亡。</t>
+        </is>
+      </c>
+      <c r="E1784" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1784" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz9yj9x74o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>Australian man charged with murder after girl found dead in suitcase in Thailand</t>
+        </is>
+      </c>
+      <c r="D1785" t="inlineStr">
+        <is>
+          <t>澳大利亚男子因泰国行李箱藏尸案被控谋杀，死者为17岁少女。</t>
+        </is>
+      </c>
+      <c r="E1785" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1785" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd0my5zy821o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>Harry reconsiders bringing Meghan and children on UK trip</t>
+        </is>
+      </c>
+      <c r="D1786" t="inlineStr">
+        <is>
+          <t>因警方拒绝安保请求，哈里重新考虑带家人访英。</t>
+        </is>
+      </c>
+      <c r="E1786" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gy6ywg73wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>27 flights, 24 matches: The carbon cost of Fifa president's World Cup tour</t>
+        </is>
+      </c>
+      <c r="D1787" t="inlineStr">
+        <is>
+          <t>国际足联主席世界杯之旅产生大量碳排放。</t>
+        </is>
+      </c>
+      <c r="E1787" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1787" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cgev5wy0zg3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>'If you are alive, make any noise': Venezuela searches rubble on day 4</t>
+        </is>
+      </c>
+      <c r="D1788" t="inlineStr">
+        <is>
+          <t>委内瑞拉双震已致超1400死，数万人失踪，救援队争分夺秒搜救。</t>
+        </is>
+      </c>
+      <c r="E1788" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1788" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/28/nx-s1-5873413/venezuela-earthquake</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr">
+        <is>
+          <t>117 dead dogs found at California 'no-kill' animal rescue - many with gunshot wounds</t>
+        </is>
+      </c>
+      <c r="D1789" t="inlineStr">
+        <is>
+          <t>加州“无杀”动物收容所发现117具狗尸，部分有枪伤，数百只失踪。</t>
+        </is>
+      </c>
+      <c r="E1789" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1789" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj4gqz5lx1eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>I'm in therapy for my 14-hour-a-day phone addiction and I'm determined to beat it</t>
+        </is>
+      </c>
+      <c r="D1790" t="inlineStr">
+        <is>
+          <t>男子因每日14小时手机成瘾接受治疗，成瘾中心称求助者增多。</t>
+        </is>
+      </c>
+      <c r="E1790" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1790" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg7v7j3wqwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>These women said no to having kids - here's why</t>
+        </is>
+      </c>
+      <c r="D1791" t="inlineStr">
+        <is>
+          <t>女性因经济、环境担忧等原因选择不生育，讲述背后故事。</t>
+        </is>
+      </c>
+      <c r="E1791" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1791" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz0jx2z2l41o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>Bad Bunny lights up London with history-making stadium show</t>
+        </is>
+      </c>
+      <c r="D1792" t="inlineStr">
+        <is>
+          <t>坏兔兔成为首位在英国体育场演出的拉丁艺人，现场充满自豪与狂欢。</t>
+        </is>
+      </c>
+      <c r="E1792" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1792" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2dyrk56dg9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>World Cup knockouts are here - what is England's path to the final?</t>
+        </is>
+      </c>
+      <c r="D1793" t="inlineStr">
+        <is>
+          <t>分析英格兰队世界杯淘汰赛晋级决赛的路径。</t>
+        </is>
+      </c>
+      <c r="E1793" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1793" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c5yz0zkzw39o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>England top group - but they will not win World Cup unless they improve</t>
+        </is>
+      </c>
+      <c r="D1794" t="inlineStr">
+        <is>
+          <t>评论：英格兰小组头名出线，但若不改进难赢世界杯。</t>
+        </is>
+      </c>
+      <c r="E1794" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cg4wnp592z1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>Clarke leaves strong Scotland legacy but exit brings sense of relief</t>
+        </is>
+      </c>
+      <c r="D1795" t="inlineStr">
+        <is>
+          <t>克拉克留强苏格兰足球遗产，但球队止步小组赛。</t>
+        </is>
+      </c>
+      <c r="E1795" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1795" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cn4d1eg5eqeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>Best team, moments, matches and players of the group stage</t>
+        </is>
+      </c>
+      <c r="D1796" t="inlineStr">
+        <is>
+          <t>BBC记者评选世界杯小组赛最佳队伍、瞬间等。</t>
+        </is>
+      </c>
+      <c r="E1796" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1796" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/ce3e256752qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>How to win a World Cup penalty shootout</t>
+        </is>
+      </c>
+      <c r="D1797" t="inlineStr">
+        <is>
+          <t>分析世界杯点球大战历史数据以寻求取胜策略。</t>
+        </is>
+      </c>
+      <c r="E1797" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1797" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cd9px47g8jlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-29
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1797"/>
+  <dimension ref="A1:F1823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57941,6 +57941,838 @@
         </is>
       </c>
     </row>
+    <row r="1798">
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260629 19:00</t>
+        </is>
+      </c>
+      <c r="D1798" t="inlineStr">
+        <is>
+          <t>本期节目包含习近平会见白俄总统、民生福祉、国务院常务会议、教育规划及建党105周年活动等要闻。</t>
+        </is>
+      </c>
+      <c r="E1798" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1798" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEL3m7e9oVuTyCOlDr3dpt260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见白俄罗斯总统</t>
+        </is>
+      </c>
+      <c r="D1799" t="inlineStr">
+        <is>
+          <t>习近平在北京会见白俄罗斯总统卢卡申科，强调深化全天候全面战略伙伴关系。</t>
+        </is>
+      </c>
+      <c r="E1799" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1799" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEGPrq7wtTHX6gmtLCBhel260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>[视频]各地举行活动庆祝建党105周年</t>
+        </is>
+      </c>
+      <c r="D1800" t="inlineStr">
+        <is>
+          <t>各地举行活动庆祝建党105周年，包括宣誓、参观红色基地等，坚定理想信念。</t>
+        </is>
+      </c>
+      <c r="E1800" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEtBOeJldZzy9hAUdtQrV8260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】山海之间的家国坚守</t>
+        </is>
+      </c>
+      <c r="D1801" t="inlineStr">
+        <is>
+          <t>讲述王继才夫妇守岛32年及布茹玛汗·毛勒朵护边的故事，彰显党员家国坚守。</t>
+        </is>
+      </c>
+      <c r="E1801" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1801" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEyDDlwLgPrCZwR3kfyAXS260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>[视频]国际人士：中国共产党以人民为中心 成就发展奇迹</t>
+        </is>
+      </c>
+      <c r="D1802" t="inlineStr">
+        <is>
+          <t>国际人士称赞中国共产党以人民为中心，领导中国取得辉煌成就，为世界注入稳定性。</t>
+        </is>
+      </c>
+      <c r="E1802" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1802" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDE9vjkSMlD2Q1tBC0VmIJn260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>New 'No 10 North' plan will rebalance power in Britain, Burnham promises</t>
+        </is>
+      </c>
+      <c r="D1803" t="inlineStr">
+        <is>
+          <t>伯纳姆承诺新计划将重新平衡英国各地权力。</t>
+        </is>
+      </c>
+      <c r="E1803" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1803" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2jw5q5pdzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>Henry Zeffman: Andy Burnham offers a blueprint for his premiership</t>
+        </is>
+      </c>
+      <c r="D1804" t="inlineStr">
+        <is>
+          <t>伯纳姆勾勒首相任期蓝图，但未提供详细计划。</t>
+        </is>
+      </c>
+      <c r="E1804" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1804" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpq3yy48zglo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D1805" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，部署人工智能发展、外贸工作，并通过碳达峰及健康规划。</t>
+        </is>
+      </c>
+      <c r="E1805" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDETvYwNNxUmmYNXggNLPHE260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁出席建设强大国内市场调研协商座谈会</t>
+        </is>
+      </c>
+      <c r="D1806" t="inlineStr">
+        <is>
+          <t>王沪宁出席建设强大国内市场调研协商座谈会，强调凝聚共识推动高质量发展。</t>
+        </is>
+      </c>
+      <c r="E1806" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEZSYRmGVtgcUWJSIXd4jy260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>[视频]2025年我国文化及相关产业营业收入规模突破20万亿元</t>
+        </is>
+      </c>
+      <c r="D1807" t="inlineStr">
+        <is>
+          <t>2025年我国文化产业营收突破20万亿元，新业态贡献近六成增长，研发投入增长12.1%。</t>
+        </is>
+      </c>
+      <c r="E1807" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1807" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEjJ73IcGpH6vDXJiSlAUv260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>Frank Gardner: Navy plans reflect sea change in how wars are fought</t>
+        </is>
+      </c>
+      <c r="D1808" t="inlineStr">
+        <is>
+          <t>海军新计划反映无人机战争带来的作战方式巨变。</t>
+        </is>
+      </c>
+      <c r="E1808" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1808" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz9lv0xkz42o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】以人民为中心 持续增进民生福祉</t>
+        </is>
+      </c>
+      <c r="D1809" t="inlineStr">
+        <is>
+          <t>报道中国共产党以人民为中心，持续增进民生福祉，通过河北阜平乡村振兴案例展现。</t>
+        </is>
+      </c>
+      <c r="E1809" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1809" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEA06yvH18aqjR11fnn3vo260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《教育发展“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D1810" t="inlineStr">
+        <is>
+          <t>国务院印发《教育发展“十五五”规划》，部署23项重点任务和15个重大项目。</t>
+        </is>
+      </c>
+      <c r="E1810" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1810" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDEhxg4YYUluM82oxtooo3i260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>国际, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1811" t="inlineStr">
+        <is>
+          <t>第四届中国-中东欧新闻发言人对话会举行；工会部署送清凉；东北首座光热电站投产。</t>
+        </is>
+      </c>
+      <c r="E1811" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1811" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDERiwZNOLy4aMqZMnP9mIt260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1812" t="inlineStr">
+        <is>
+          <t>美伊同意停止互袭继续谈判；委内瑞拉强震1450人遇难；美国犹他州林火蔓延。</t>
+        </is>
+      </c>
+      <c r="E1812" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1812" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/29/VIDENtghXZFYapZVMF0O7EBA260629.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>Mum rescued from Venezuela rubble with newborn baby tells BBC how he helped her survive</t>
+        </is>
+      </c>
+      <c r="D1813" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震中，一名18天大的婴儿奇迹获救，成为希望象征。</t>
+        </is>
+      </c>
+      <c r="E1813" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1813" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyw3rkj2p7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>Sixth person dies after shooting at youth welfare centre in Germany</t>
+        </is>
+      </c>
+      <c r="D1814" t="inlineStr">
+        <is>
+          <t>德国一家青少年福利中心发生枪击，致6人死亡，警方已介入调查。</t>
+        </is>
+      </c>
+      <c r="E1814" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1814" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c17yzzw1vkjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>Supreme Court rejects Trump's appeal of E Jean Carroll's sexual abuse case</t>
+        </is>
+      </c>
+      <c r="D1815" t="inlineStr">
+        <is>
+          <t>美国最高法院驳回特朗普上诉，维持其需赔偿性侵案受害者500万美元的判决。</t>
+        </is>
+      </c>
+      <c r="E1815" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1815" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn8q2z5wpn2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>DR Congo bans mass gatherings in the  capital to prevent spread of Ebola</t>
+        </is>
+      </c>
+      <c r="D1816" t="inlineStr">
+        <is>
+          <t>刚果（金）禁止首都大规模集会防埃博拉，反对派指责政府以此阻挠抗议。</t>
+        </is>
+      </c>
+      <c r="E1816" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1816" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c992k7zk981o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>US says it has agreed to 'stand down' after exchange of strikes with Iran</t>
+        </is>
+      </c>
+      <c r="D1817" t="inlineStr">
+        <is>
+          <t>美伊周末互指违反停火协议并相互攻击。</t>
+        </is>
+      </c>
+      <c r="E1817" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1817" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c872rjw17qpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>Pakistani airstrikes kill 36 civilians in Afghanistan and wound 160, officials say</t>
+        </is>
+      </c>
+      <c r="D1818" t="inlineStr">
+        <is>
+          <t>巴基斯坦空袭阿富汗致36死160伤，阿方谴责。</t>
+        </is>
+      </c>
+      <c r="E1818" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1818" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/g-s1-130826/pakistani-airstrikes-kill-36-civilians-in-afghanistan-and-wound-160-officials-say</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>U.S. and Iran exchange fire despite ceasefire. And, Trump nominates a new head of ICE</t>
+        </is>
+      </c>
+      <c r="D1819" t="inlineStr">
+        <is>
+          <t>美伊周末交火危及停火；特朗普提名ICE新负责人。</t>
+        </is>
+      </c>
+      <c r="E1819" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1819" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/g-s1-130793/up-first-newsletter-iran-war-ceasefire-venezuela-earthquakes-ice-lance-schroyer</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>Trump says the U.S. and Iran will meet in Qatar after weekend attacks</t>
+        </is>
+      </c>
+      <c r="D1820" t="inlineStr">
+        <is>
+          <t>特朗普称美伊将在卡塔尔会谈，伊朗未确认参与。</t>
+        </is>
+      </c>
+      <c r="E1820" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1820" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/nx-s1-5874618/us-iran-talks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>Former Iran nuclear deal negotiator on what U.S.-Iran 'new normal' looks like</t>
+        </is>
+      </c>
+      <c r="D1821" t="inlineStr">
+        <is>
+          <t>前伊朗核协议谈判代表谈美伊“新常态”及停火谈判。</t>
+        </is>
+      </c>
+      <c r="E1821" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1821" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/nx-s1-5873990/us-iran-ceasefire-new-normal-gulf-flareups</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>Could neo-Nazi youth, or 'active clubs,' have played a role in Belfast riots?</t>
+        </is>
+      </c>
+      <c r="D1822" t="inlineStr">
+        <is>
+          <t>北爱尔兰骚乱中，新纳粹青年组织“活跃俱乐部”被指参与。</t>
+        </is>
+      </c>
+      <c r="E1822" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/nx-s1-5871337/violence-belfast-northern-ireland-white-supremacy-riots-active-clubs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>Tributes paid to 'comic genius' Penelope Keith after her death aged 86</t>
+        </is>
+      </c>
+      <c r="D1823" t="inlineStr">
+        <is>
+          <t>喜剧天才女演员佩内洛普·基思去世，享年86岁。</t>
+        </is>
+      </c>
+      <c r="E1823" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1823" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2ey1pjx0z9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-06-30
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1823"/>
+  <dimension ref="A1:F1862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58773,6 +58773,1254 @@
         </is>
       </c>
     </row>
+    <row r="1824">
+      <c r="A1824" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260630 19:00</t>
+        </is>
+      </c>
+      <c r="D1824" t="inlineStr">
+        <is>
+          <t>中共中央政治局部署防汛抗旱；庆祝建党105周年音乐会举行等多项要闻。</t>
+        </is>
+      </c>
+      <c r="E1824" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEXi5z3cZYJAuyL4CNi2mM260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>[视频]中共中央政治局召开会议 研究部署防汛抗旱工作 中共中央总书记习近平主持会议</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr">
+        <is>
+          <t>中共中央政治局会议研究部署防汛抗旱工作，强调人民生命安全。</t>
+        </is>
+      </c>
+      <c r="E1825" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1825" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEBDRZCR3PUdNXo3W0QKz3260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>政治, 文体</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>[视频]庆祝中国共产党成立105周年音乐会《人民至上》在京举行</t>
+        </is>
+      </c>
+      <c r="D1826" t="inlineStr">
+        <is>
+          <t>庆祝建党105周年音乐会《人民至上》在京举行，党和国家领导人出席。</t>
+        </is>
+      </c>
+      <c r="E1826" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1826" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEC2swR7agEZYhbHYOySOJ260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>[视频]习近平同塞舌尔总统就中塞建交50周年互致贺电</t>
+        </is>
+      </c>
+      <c r="D1827" t="inlineStr">
+        <is>
+          <t>习近平同塞舌尔总统互致贺电，庆祝中塞建交50周年。</t>
+        </is>
+      </c>
+      <c r="E1827" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1827" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEjOBFwGxdIjT5w5MXDFdc260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr">
+        <is>
+          <t>[视频]庆祝中国共产党成立105周年大会7月1日上午在京隆重举行 习近平将向“七一勋章”获得者颁授勋章并发表重要讲话</t>
+        </is>
+      </c>
+      <c r="D1828" t="inlineStr">
+        <is>
+          <t>庆祝建党105周年大会7月1日举行，习近平将颁授“七一勋章”。</t>
+        </is>
+      </c>
+      <c r="E1828" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1828" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDETegOChUamALR3PP0F2LZ260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr">
+        <is>
+          <t>[视频]人民日报社论：砥砺初心使命 书写时代答卷——热烈庆祝中国共产党成立105周年</t>
+        </is>
+      </c>
+      <c r="D1829" t="inlineStr">
+        <is>
+          <t>人民日报社论庆祝建党105周年，题为《砥砺初心使命 书写时代答卷》。</t>
+        </is>
+      </c>
+      <c r="E1829" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1829" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEPvCuSlSeaGEp8eLj5Sb0260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr">
+        <is>
+          <t>[视频]人民日报任仲平文章：把握历史主动 实现伟大复兴——写在中国共产党成立105周年之际</t>
+        </is>
+      </c>
+      <c r="D1830" t="inlineStr">
+        <is>
+          <t>人民日报任仲平文章写于建党105周年之际，题为《把握历史主动 实现伟大复兴》。</t>
+        </is>
+      </c>
+      <c r="E1830" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1830" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEoPCGoqIGbxGgjJynxX0f260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：坚持以习近平党建思想为指引，奋力走好新的赶考之路——热烈庆祝中国共产党成立105周年</t>
+        </is>
+      </c>
+      <c r="D1831" t="inlineStr">
+        <is>
+          <t>央视快评强调以习近平党建思想为指引，奋力走好新的赶考之路。</t>
+        </is>
+      </c>
+      <c r="E1831" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1831" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEvrWxo0oem7t2z0xaGjqT260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr">
+        <is>
+          <t>[视频]李强签署国务院令 公布《退役军人就业创业促进条例》</t>
+        </is>
+      </c>
+      <c r="D1832" t="inlineStr">
+        <is>
+          <t>李强签署国务院令，公布《退役军人就业创业促进条例》，自2026年8月1日起施行。</t>
+        </is>
+      </c>
+      <c r="E1832" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1832" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEwfZZYN9UdpcZ0gHae1s3260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr">
+        <is>
+          <t>[视频]中国共产党最新党内统计数据发布</t>
+        </is>
+      </c>
+      <c r="D1833" t="inlineStr">
+        <is>
+          <t>截至2025年底，中国共产党党员总数为10128.6万名，比上年净增101.5万名。</t>
+        </is>
+      </c>
+      <c r="E1833" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1833" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEdIcX0foDZP96p3qPKwe7260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr">
+        <is>
+          <t>[视频]各地举办多样活动 庆祝建党105周年</t>
+        </is>
+      </c>
+      <c r="D1834" t="inlineStr">
+        <is>
+          <t>各地开展多样活动庆祝建党105周年，弘扬伟大建党精神。</t>
+        </is>
+      </c>
+      <c r="E1834" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1834" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDELYDKiza8hSGwbX5lczQm260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr">
+        <is>
+          <t>[视频]国际人士：中国共产党为各国政党建设和国家治理提供重要借鉴</t>
+        </is>
+      </c>
+      <c r="D1835" t="inlineStr">
+        <is>
+          <t>国际人士赞扬中国共产党领导中国取得成就，为各国提供重要借鉴。</t>
+        </is>
+      </c>
+      <c r="E1835" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1835" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEPw2cnNtdITNUlI5COx8T260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr">
+        <is>
+          <t>Supreme Court's birthright ruling is major blow to Trump</t>
+        </is>
+      </c>
+      <c r="D1836" t="inlineStr">
+        <is>
+          <t>美最高法院关于出生公民权的裁决对特朗普构成重大打击。</t>
+        </is>
+      </c>
+      <c r="E1836" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1836" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c9w2nprzq5ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr">
+        <is>
+          <t>US Supreme Court upholds bans on transgender women in female school and college sports</t>
+        </is>
+      </c>
+      <c r="D1837" t="inlineStr">
+        <is>
+          <t>美最高法院支持禁止跨性别女性参加女性学校及大学体育比赛。</t>
+        </is>
+      </c>
+      <c r="E1837" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1837" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj40x888d9go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr">
+        <is>
+          <t>Senegalese MPs move to clip presidential powers as tensions mount</t>
+        </is>
+      </c>
+      <c r="D1838" t="inlineStr">
+        <is>
+          <t>塞内加尔议员提议削弱总统权力，引发议会外抗议。</t>
+        </is>
+      </c>
+      <c r="E1838" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1838" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgl352xjgngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr">
+        <is>
+          <t>Founder of Asian super-app Gojek sentenced to years in jail for corruption</t>
+        </is>
+      </c>
+      <c r="D1839" t="inlineStr">
+        <is>
+          <t>Gojek创始人因在担任教育部长期间涉及笔记本电脑交易腐败被判刑。</t>
+        </is>
+      </c>
+      <c r="E1839" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1839" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c79yvw23yr9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr">
+        <is>
+          <t>Government 'cannot deport' grooming gang ringleader</t>
+        </is>
+      </c>
+      <c r="D1840" t="inlineStr">
+        <is>
+          <t>因55年旧法律，政府无法驱逐犯罪团伙头目沙比尔·艾哈迈德。</t>
+        </is>
+      </c>
+      <c r="E1840" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1840" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2wl6ynn2no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>Burnham plans to work some days in Manchester as PM</t>
+        </is>
+      </c>
+      <c r="D1841" t="inlineStr">
+        <is>
+          <t>前大曼彻斯特市长计划若成为工党领袖，将在曼彻斯特设首相办公室。</t>
+        </is>
+      </c>
+      <c r="E1841" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1841" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1ey985nyqpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>Refugees would be told to repay around £10,000 under new asylum bill</t>
+        </is>
+      </c>
+      <c r="D1842" t="inlineStr">
+        <is>
+          <t>新法案规定难民需偿还约1万英镑的庇护支持费用。</t>
+        </is>
+      </c>
+      <c r="E1842" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1842" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cddlgqlm7q2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>SCOTUS to rule on birthright citizenship. And, U.S. murder rate nears new low</t>
+        </is>
+      </c>
+      <c r="D1843" t="inlineStr">
+        <is>
+          <t>美最高法院预计就出生公民权做出裁决，同时美国谋杀率接近新低。</t>
+        </is>
+      </c>
+      <c r="E1843" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1843" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/30/g-s1-131004/up-first-newsletter-supreme-court-tps-birthright-citizenship-iran-war-us-murder-rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>Chinese billionaire Guo Wengui gets 30 years in U.S. prison for fraud conviction</t>
+        </is>
+      </c>
+      <c r="D1844" t="inlineStr">
+        <is>
+          <t>中国富豪郭文贵因诈骗被判30年美国监禁，法官斥其挥霍投资者资金。</t>
+        </is>
+      </c>
+      <c r="E1844" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1844" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/29/g-s1-130976/chinese-billionaire-guo-wengui-gets-30-years-in-u-s-prison-for-fraud-conviction</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>[视频]2025年我国水运多项指标稳居世界第一</t>
+        </is>
+      </c>
+      <c r="D1845" t="inlineStr">
+        <is>
+          <t>2025年我国水运多项指标稳居世界第一，港口货物和集装箱吞吐量领先。</t>
+        </is>
+      </c>
+      <c r="E1845" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1845" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDE0qDXc4sfPmYl4x8r5INL260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>[视频]中国制造业采购经理指数升至50.3%</t>
+        </is>
+      </c>
+      <c r="D1846" t="inlineStr">
+        <is>
+          <t>6月份中国制造业采购经理指数升至50.3%，制造业发展动能增强。</t>
+        </is>
+      </c>
+      <c r="E1846" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1846" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEzhw0o7WBe7u4vJLIZNdr260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>[视频]【在希望的田野上】夏播粮食近八成 夏管全面展开</t>
+        </is>
+      </c>
+      <c r="D1847" t="inlineStr">
+        <is>
+          <t>全国夏播粮食进度近八成，夏季田间管理全面展开，夯实秋粮丰收基础。</t>
+        </is>
+      </c>
+      <c r="E1847" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1847" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEOKBNuDzFUHIiOSOjdDHG260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>民生, 社会, 科技</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1848" t="inlineStr">
+        <is>
+          <t>国内联播快讯：液态食品散装运输新规、首个流域型排放标准发布、防汛应急响应等。</t>
+        </is>
+      </c>
+      <c r="E1848" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1848" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEcuzw1Rg3kdXzbhoKrYGX260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr">
+        <is>
+          <t>Flooding hits Ghana's capital killing 13 people - with another storm forecast</t>
+        </is>
+      </c>
+      <c r="D1849" t="inlineStr">
+        <is>
+          <t>加纳首都洪灾致13人死亡，气象预报另一场风暴即将来临。</t>
+        </is>
+      </c>
+      <c r="E1849" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1849" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn4r8zlv8edo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>Government promises to act on maternity care failings which 'shame our society'</t>
+        </is>
+      </c>
+      <c r="D1850" t="inlineStr">
+        <is>
+          <t>政府承诺解决产科护理中不可接受的种族歧视问题。</t>
+        </is>
+      </c>
+      <c r="E1850" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1850" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cddlgqpg7mzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见沙特外交大臣</t>
+        </is>
+      </c>
+      <c r="D1851" t="inlineStr">
+        <is>
+          <t>韩正会见沙特外交大臣，强调深化中沙关系，维护地区和平稳定。</t>
+        </is>
+      </c>
+      <c r="E1851" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1851" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEITpuWhBxQAEANv7XRoE2260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>国际, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1852" t="inlineStr">
+        <is>
+          <t>委内瑞拉发生余震致地铁停运，伊朗称单独执行霍尔木兹排雷，日元汇率跌至近40年最低。</t>
+        </is>
+      </c>
+      <c r="E1852" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1852" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/06/30/VIDEQp6AbAHWUuSoqzNVKUqt260630.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>Angry Venezuelans accuse government of negligence over earthquake response</t>
+        </is>
+      </c>
+      <c r="D1853" t="inlineStr">
+        <is>
+          <t>委内瑞拉民众指责政府在地震救援中疏忽，要求更多支持。</t>
+        </is>
+      </c>
+      <c r="E1853" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1853" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yzd18dxzxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>Manhunt after bomb injures Ukrainian oligarch in Monaco</t>
+        </is>
+      </c>
+      <c r="D1854" t="inlineStr">
+        <is>
+          <t>摩纳哥发生爆炸致乌克兰富豪受伤，当局展开搜捕。</t>
+        </is>
+      </c>
+      <c r="E1854" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1854" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpv37wx03v7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>US envoys in Doha to meet mediators but not Iranians, Qatar says</t>
+        </is>
+      </c>
+      <c r="D1855" t="inlineStr">
+        <is>
+          <t>卡塔尔称美国特使将与调解人会面，但不会与伊朗直接会谈。</t>
+        </is>
+      </c>
+      <c r="E1855" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1855" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpd38x1dy4no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>Chinese tycoon sentenced to 30 years in US jail</t>
+        </is>
+      </c>
+      <c r="D1856" t="inlineStr">
+        <is>
+          <t>中国商人郭文贵因欺诈在美国被判30年监禁。</t>
+        </is>
+      </c>
+      <c r="E1856" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1856" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjeg15vw3z9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>Another UK heatwave could be on the way</t>
+        </is>
+      </c>
+      <c r="D1857" t="inlineStr">
+        <is>
+          <t>欧洲多国高温持续，本周末英国可能再次迎来热浪。</t>
+        </is>
+      </c>
+      <c r="E1857" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1857" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/cql14kwex2wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>Venezuelans deported from the U.S. were killed hours later in powerful quakes</t>
+        </is>
+      </c>
+      <c r="D1858" t="inlineStr">
+        <is>
+          <t>146名委内瑞拉人被美驱逐出境后数小时，在酒店遭遇强烈地震。</t>
+        </is>
+      </c>
+      <c r="E1858" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1858" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/30/nx-s1-5875287/venezuela-deportees-us-quakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>国际, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>Iran war supercharges pivot to renewable energy</t>
+        </is>
+      </c>
+      <c r="D1859" t="inlineStr">
+        <is>
+          <t>伊朗战争及高油价推动全球可再生能源和电动汽车普及。</t>
+        </is>
+      </c>
+      <c r="E1859" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1859" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/30/nx-s1-5869701/iran-war-supercharges-pivot-to-renewable-energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>Explosion in Monaco injures 3, including Ukrainian tycoon</t>
+        </is>
+      </c>
+      <c r="D1860" t="inlineStr">
+        <is>
+          <t>摩纳哥爆炸致三人受伤，包括一名乌克兰大亨，嫌疑人仍在逃。</t>
+        </is>
+      </c>
+      <c r="E1860" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1860" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/30/g-s1-130990/explosion-monaco-ukrainian-tycoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>Thousands of anti-migrant protesters march in South Africa amid heavy police presence</t>
+        </is>
+      </c>
+      <c r="D1861" t="inlineStr">
+        <is>
+          <t>南非数千名反移民抗议者游行，警方严密戒备，部分外国人已撤离。</t>
+        </is>
+      </c>
+      <c r="E1861" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1861" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy4eq1l184po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>France superstars thriving thanks to Deschamps' bold changes</t>
+        </is>
+      </c>
+      <c r="D1862" t="inlineStr">
+        <is>
+          <t>德尚调整人员和阵型，助法国队在本届世界杯再创佳绩。</t>
+        </is>
+      </c>
+      <c r="E1862" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1862" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cg53ggg03nno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-01
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1862"/>
+  <dimension ref="A1:F1894"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -60021,6 +60021,1030 @@
         </is>
       </c>
     </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260701 21:00</t>
+        </is>
+      </c>
+      <c r="D1863" t="inlineStr">
+        <is>
+          <t>庆祝中国共产党成立105周年大会在京举行；《求是》发表习近平重要文章；习近平致贺电祝贺哥伦比亚总统当选。</t>
+        </is>
+      </c>
+      <c r="E1863" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1863" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEnXWst1pzgRcXVcc9PRX4260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>[视频]庆祝中国共产党成立105周年大会在京隆重举行</t>
+        </is>
+      </c>
+      <c r="D1864" t="inlineStr">
+        <is>
+          <t>庆祝中国共产党成立105周年大会在京举行，习近平发表重要讲话并颁授“七一勋章”。</t>
+        </is>
+      </c>
+      <c r="E1864" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1864" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEQoMGbfTGORicHogyPemA260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>[视频]《求是》杂志发表习近平总书记重要文章《做焦裕禄式的县委书记》</t>
+        </is>
+      </c>
+      <c r="D1865" t="inlineStr">
+        <is>
+          <t>《求是》杂志重新发表习近平重要文章《做焦裕禄式的县委书记》，强调县委书记要心中有党。</t>
+        </is>
+      </c>
+      <c r="E1865" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1865" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDE2AQVYBgtJVKysuDBIo2h260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>[视频]习近平致电祝贺德拉埃斯普列亚当选哥伦比亚总统</t>
+        </is>
+      </c>
+      <c r="D1866" t="inlineStr">
+        <is>
+          <t>习近平致电祝贺德拉埃斯普列亚当选哥伦比亚总统，强调深化中哥战略伙伴关系。</t>
+        </is>
+      </c>
+      <c r="E1866" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1866" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEbJzAmoGacYr8vZ4kYWZv260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>[视频]践行初心使命 不断创造无愧于时代和人民的新业绩——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D1867" t="inlineStr">
+        <is>
+          <t>习近平在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响，激励奋进新征程。</t>
+        </is>
+      </c>
+      <c r="E1867" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1867" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEMirLMpx0pRY815vn1EZS260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：牢记“三个务必” 奋力创造新的历史辉煌</t>
+        </is>
+      </c>
+      <c r="D1868" t="inlineStr">
+        <is>
+          <t>央视快评强调牢记“三个务必”，奋力创造新的历史辉煌。</t>
+        </is>
+      </c>
+      <c r="E1868" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1868" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEgm7yTL2848AzFPBlV2rx260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>[视频]世界政党政要热烈祝贺中国共产党成立105周年</t>
+        </is>
+      </c>
+      <c r="D1869" t="inlineStr">
+        <is>
+          <t>多国政党和政府领导人致贺中国共产党成立105周年，高度评价中国成就。</t>
+        </is>
+      </c>
+      <c r="E1869" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1869" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEPXMTXLLLAhQRupl01tfL260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>[视频]香港举行升旗仪式庆祝回归祖国29周年</t>
+        </is>
+      </c>
+      <c r="D1870" t="inlineStr">
+        <is>
+          <t>香港特区政府在金紫荆广场举行升旗仪式，庆祝回归祖国29周年。</t>
+        </is>
+      </c>
+      <c r="E1870" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1870" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEHFzQ4rArPkfhriWpfddK260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>政治, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D1871" t="inlineStr">
+        <is>
+          <t>中央档案馆开放4.4万余件档案；全国铁路暑运预计发送10.1亿人次；我国全面进入主汛期；北京市郊铁路城市副中心线西段开通。</t>
+        </is>
+      </c>
+      <c r="E1871" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1871" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDECjLu6SxDOqLHQXNwTsNa260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>US Supreme Court upholds birthright citizenship in blow to Trump</t>
+        </is>
+      </c>
+      <c r="D1872" t="inlineStr">
+        <is>
+          <t>美最高法院支持出生公民权，打击特朗普移民议程，民权组织欢迎。</t>
+        </is>
+      </c>
+      <c r="E1872" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1872" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgmepnx1wzzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>Badenoch accuses Starmer of leaving defence spending 'mess' for Burnham</t>
+        </is>
+      </c>
+      <c r="D1873" t="inlineStr">
+        <is>
+          <t>保守党领袖巴德诺赫指责斯塔默国防投资计划存在50亿英镑缺口。</t>
+        </is>
+      </c>
+      <c r="E1873" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1873" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy9rgg9ddw2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>Is Burnham facing a £5bn defence 'black hole'?</t>
+        </is>
+      </c>
+      <c r="D1874" t="inlineStr">
+        <is>
+          <t>BBC核查政府国防投资计划的50亿英镑资金缺口是否属实。</t>
+        </is>
+      </c>
+      <c r="E1874" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1874" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c14ymy41v5go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>Trump made more than $1bn from crypto in first year back in office</t>
+        </is>
+      </c>
+      <c r="D1875" t="inlineStr">
+        <is>
+          <t>特朗普重返白宫首年，加密货币收入超10亿美元，远超其他业务。</t>
+        </is>
+      </c>
+      <c r="E1875" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1875" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgmv98ez3zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>Up to 150 ex-WHSmith High Street stores to close as rescue deal approved</t>
+        </is>
+      </c>
+      <c r="D1876" t="inlineStr">
+        <is>
+          <t>WHSmith高街店最多关闭150家，法院批准重组并大幅削减租金。</t>
+        </is>
+      </c>
+      <c r="E1876" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1876" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn751pkmgyxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>Anthropic says US lifts export ban on its advanced AI tools</t>
+        </is>
+      </c>
+      <c r="D1877" t="inlineStr">
+        <is>
+          <t>Anthropic称美国取消对其先进AI工具的出口禁令。</t>
+        </is>
+      </c>
+      <c r="E1877" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1877" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdr42623e1do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>Teachers in England to get 3.5% pay rise</t>
+        </is>
+      </c>
+      <c r="D1878" t="inlineStr">
+        <is>
+          <t>英格兰教师将获3.5%加薪，工会称经费紧张将加剧预算压力。</t>
+        </is>
+      </c>
+      <c r="E1878" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1878" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2d41vlvzlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>Fire at Antwerp apartment block kills at least six</t>
+        </is>
+      </c>
+      <c r="D1879" t="inlineStr">
+        <is>
+          <t>比利时安特卫普一公寓楼发生火灾，至少6人死亡，约200人居住。</t>
+        </is>
+      </c>
+      <c r="E1879" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1879" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621dx0vl7xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>Three-year-old rescued and taken to hospital six days after Venezuela quake</t>
+        </is>
+      </c>
+      <c r="D1880" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震六天后，一名3岁儿童从废墟中被救出并送医。</t>
+        </is>
+      </c>
+      <c r="E1880" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1880" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1jykwk8n18o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>Canada to make Eurovision Song Contest debut in 2027</t>
+        </is>
+      </c>
+      <c r="D1881" t="inlineStr">
+        <is>
+          <t>加拿大将于2027年首次参加欧洲歌唱大赛，为2015年来首个新参赛国。</t>
+        </is>
+      </c>
+      <c r="E1881" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1881" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8x2y2vwqn1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>Sudan's RSF committed crimes against humanity in el-Fasher, Amnesty says</t>
+        </is>
+      </c>
+      <c r="D1882" t="inlineStr">
+        <is>
+          <t>大赦国际报告称，苏丹快速支援部队在法希尔犯下危害人类罪。</t>
+        </is>
+      </c>
+      <c r="E1882" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1882" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz9lqvx0z1vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>Man guilty of attempted murder of three children in Dublin</t>
+        </is>
+      </c>
+      <c r="D1883" t="inlineStr">
+        <is>
+          <t>男子否认2023年11月在都柏林试图谋杀三名儿童和袭击四人。</t>
+        </is>
+      </c>
+      <c r="E1883" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1883" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c78yjgpr5j3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>Funerals held for 14 Pakistani children killed in tutoring center collapse</t>
+        </is>
+      </c>
+      <c r="D1884" t="inlineStr">
+        <is>
+          <t>巴基斯坦14名儿童在补习中心倒塌事故中遇难，警方调查是否因施工疏忽。</t>
+        </is>
+      </c>
+      <c r="E1884" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1884" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/01/g-s1-131537/funerals-held-for-14-pakistani-children-killed-in-tutoring-center-collapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>Mexico ends a 40-year knockout drought, beats Ecuador to advance in World Cup</t>
+        </is>
+      </c>
+      <c r="D1885" t="inlineStr">
+        <is>
+          <t>墨西哥1-0胜厄瓜多尔，终结40年世界杯淘汰赛无胜绩。</t>
+        </is>
+      </c>
+      <c r="E1885" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1885" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/01/nx-s1-5877257/mexico-beats-ecuador-advance-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>Three die in Mexico City World Cup celebrations</t>
+        </is>
+      </c>
+      <c r="D1886" t="inlineStr">
+        <is>
+          <t>超百万民众在墨西哥城街头庆祝国家队战胜厄瓜多尔，三人丧生。</t>
+        </is>
+      </c>
+      <c r="E1886" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1886" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2xjwj8p39o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>Judge 'wrong' to spare boy rapists from custody, court told</t>
+        </is>
+      </c>
+      <c r="D1887" t="inlineStr">
+        <is>
+          <t>上诉法院审理称法官错误判决三名少年强奸犯免于拘留。</t>
+        </is>
+      </c>
+      <c r="E1887" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1887" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clye2enp0lxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>England's warmest June on record following historic heatwave</t>
+        </is>
+      </c>
+      <c r="D1888" t="inlineStr">
+        <is>
+          <t>英格兰经历有记录以来最温暖的六月，英国整体为第二暖。</t>
+        </is>
+      </c>
+      <c r="E1888" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1888" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/cjdg98g8lg8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr">
+        <is>
+          <t>Nowak case officers face gross misconduct investigation</t>
+        </is>
+      </c>
+      <c r="D1889" t="inlineStr">
+        <is>
+          <t>警察因亨利·诺瓦克案中不当行为面临严重渎职调查。</t>
+        </is>
+      </c>
+      <c r="E1889" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1889" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd6ezln069vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr">
+        <is>
+          <t>Greetings from London, where Banksy's flag man is a warning cry</t>
+        </is>
+      </c>
+      <c r="D1890" t="inlineStr">
+        <is>
+          <t>班克西新雕像：举旗人前行中旗子反吹脸上，警示危险坠落。</t>
+        </is>
+      </c>
+      <c r="E1890" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1890" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/01/nx-s1-5867594/banksy-flag-man-statue-london</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr">
+        <is>
+          <t>[视频]庆祝中国共产党成立105周年音乐会今晚播出</t>
+        </is>
+      </c>
+      <c r="D1891" t="inlineStr">
+        <is>
+          <t>庆祝中国共产党成立105周年音乐会《人民至上》今晚在总台多个平台播出。</t>
+        </is>
+      </c>
+      <c r="E1891" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1891" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/01/VIDEBFhEDSN2cwkfMcJ58NPg260701.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr">
+        <is>
+          <t>Tens of thousands rush for tickets to see Bayeux Tapestry in UK</t>
+        </is>
+      </c>
+      <c r="D1892" t="inlineStr">
+        <is>
+          <t>数万人抢票观看贝叶挂毯首次从法国来英国展出。</t>
+        </is>
+      </c>
+      <c r="E1892" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1892" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4g49q5qyjxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr">
+        <is>
+          <t>Williams' knee injury leaves Wimbledon doubles in doubt</t>
+        </is>
+      </c>
+      <c r="D1893" t="inlineStr">
+        <is>
+          <t>塞雷娜·威廉姆斯膝伤可能影响温网双打比赛。</t>
+        </is>
+      </c>
+      <c r="E1893" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1893" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/tennis/articles/cx2kr12ggv9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr">
+        <is>
+          <t>Village People frontman Victor Willis dies aged 74</t>
+        </is>
+      </c>
+      <c r="D1894" t="inlineStr">
+        <is>
+          <t>村民乐队主唱维克多·威利斯去世，享年74岁。</t>
+        </is>
+      </c>
+      <c r="E1894" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1894" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cddlnqy8zmqo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-02
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1894"/>
+  <dimension ref="A1:F1928"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61045,6 +61045,1094 @@
         </is>
       </c>
     </row>
+    <row r="1895">
+      <c r="A1895" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260702 19:00</t>
+        </is>
+      </c>
+      <c r="D1895" t="inlineStr">
+        <is>
+          <t>习近平建党105周年讲话引反响；《习近平谈治国理政》第五卷在土耳其推介；各地庆祝建党；外贸数据公布；防汛防台风工作推进。</t>
+        </is>
+      </c>
+      <c r="E1895" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1895" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEAX4aFkplTaQGigeTkwAs260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr">
+        <is>
+          <t>[视频]奋进新征程 建功新时代 奋力创造新的历史辉煌——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D1896" t="inlineStr">
+        <is>
+          <t>习近平讲话在中央和国家机关引发热烈反响，强调奋进新征程、建功新时代的信心与决心。</t>
+        </is>
+      </c>
+      <c r="E1896" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1896" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDER5SZxFrBNAUaXwv1J1iS260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr">
+        <is>
+          <t>[视频]《习近平谈治国理政》第五卷土耳其推介会在安卡拉举行</t>
+        </is>
+      </c>
+      <c r="D1897" t="inlineStr">
+        <is>
+          <t>《习近平谈治国理政》第五卷在土耳其安卡拉举行推介会，促进中土治国理政经验交流。</t>
+        </is>
+      </c>
+      <c r="E1897" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1897" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEqipVMTSzzIbpDwjQyX2G260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr">
+        <is>
+          <t>[视频]各地庆祝建党105周年 凝聚新征程奋进力量</t>
+        </is>
+      </c>
+      <c r="D1898" t="inlineStr">
+        <is>
+          <t>各地以重温誓词、参观展览等方式庆祝建党105周年，汲取奋进力量。</t>
+        </is>
+      </c>
+      <c r="E1898" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1898" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEJfFK4QNQ2G0o9AqjrgpU260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1899" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr">
+        <is>
+          <t>[视频]国际人士高度评价习近平在庆祝中国共产党成立105周年大会上的重要讲话</t>
+        </is>
+      </c>
+      <c r="D1899" t="inlineStr">
+        <is>
+          <t>国际人士高度评价习近平在庆祝建党105周年大会上的重要讲话，赞扬中国共产党坚持人民至上理念。</t>
+        </is>
+      </c>
+      <c r="E1899" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1899" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEfQMvVt0Zqke1OUJB9HOJ260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr">
+        <is>
+          <t>Labour failed to prepare for power, admits PM's former top aide</t>
+        </is>
+      </c>
+      <c r="D1900" t="inlineStr">
+        <is>
+          <t>英国首相前助手承认工党执政后未能迅速兑现承诺。</t>
+        </is>
+      </c>
+      <c r="E1900" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1900" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce8j2e38zzgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr">
+        <is>
+          <t>'The shame is not yours': Starmer apologises for state's role in forced adoptions</t>
+        </is>
+      </c>
+      <c r="D1901" t="inlineStr">
+        <is>
+          <t>英首相为1949-1976年国家主导的强制收养政策道歉。</t>
+        </is>
+      </c>
+      <c r="E1901" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1901" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20yq332018o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr">
+        <is>
+          <t>Trump denies conflict of interest over crypto. And, Vatican excommunicates rebel group</t>
+        </is>
+      </c>
+      <c r="D1902" t="inlineStr">
+        <is>
+          <t>特朗普否认加密货币利益冲突；梵蒂冈驱逐传统派团体。</t>
+        </is>
+      </c>
+      <c r="E1902" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1902" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/02/g-s1-131702/up-first-newsletter-trump-crypto-earnings-society-pope-pius-venezuela-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr">
+        <is>
+          <t>[视频]前5个月我国知识密集型服务出口增长12.2%</t>
+        </is>
+      </c>
+      <c r="D1903" t="inlineStr">
+        <is>
+          <t>前5个月我国知识密集型服务出口增长12.2%，旅行服务出口增长31.3%。</t>
+        </is>
+      </c>
+      <c r="E1903" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1903" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDErLh5WJTDN1Dmemeuq9lh260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr">
+        <is>
+          <t>[视频]机电产品出口增势良好 外贸发展质效双升</t>
+        </is>
+      </c>
+      <c r="D1904" t="inlineStr">
+        <is>
+          <t>机电产品出口连续15个月增势良好，AI产业链相关产品贡献增量超五成。</t>
+        </is>
+      </c>
+      <c r="E1904" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1904" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDE67YlxDim7EMLQDvUfbK3260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr">
+        <is>
+          <t>Alleged Scattered Spider hacker arrested in Finland</t>
+        </is>
+      </c>
+      <c r="D1905" t="inlineStr">
+        <is>
+          <t>19岁美国-爱沙尼亚双重国籍黑客在芬兰被捕并引渡至美国。</t>
+        </is>
+      </c>
+      <c r="E1905" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1905" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwy0we4yw1lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr">
+        <is>
+          <t>'Most massive' Russian attack on Kyiv kills at least 20</t>
+        </is>
+      </c>
+      <c r="D1906" t="inlineStr">
+        <is>
+          <t>俄罗斯对基辅发动大规模空袭，致至少20人死亡，市长宣布哀悼。</t>
+        </is>
+      </c>
+      <c r="E1906" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1906" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyv05gk4do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr">
+        <is>
+          <t>A major Russian attack kills 17 in Kyiv as Ukraine keeps striking Moscow's oil sector</t>
+        </is>
+      </c>
+      <c r="D1907" t="inlineStr">
+        <is>
+          <t>俄军大规模袭击基辅致17人死亡，乌方持续打击莫斯科石油设施。</t>
+        </is>
+      </c>
+      <c r="E1907" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1907" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/02/g-s1-131681/russian-attack-ukraine</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr">
+        <is>
+          <t>[视频]各地采取有力措施做好防汛防台风工作</t>
+        </is>
+      </c>
+      <c r="D1908" t="inlineStr">
+        <is>
+          <t>各地加强防汛防台风，安徽、重庆应对强降雨，南海热带低压将影响华南沿海。</t>
+        </is>
+      </c>
+      <c r="E1908" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1908" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEjlwuJ4ZwzehZeEZIGTPV260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1909" t="inlineStr">
+        <is>
+          <t>民生, 经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1909" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1909" t="inlineStr">
+        <is>
+          <t>人社部启动青年就业服务；市监局扩容食品抽检队伍；北京发布AI赋能科研方案；中老铁路货值破900亿。</t>
+        </is>
+      </c>
+      <c r="E1909" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1909" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEAef8DpP40uw11UYIrQF1260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr">
+        <is>
+          <t>Government may now allow pubs to extend hours for 1am England clash</t>
+        </is>
+      </c>
+      <c r="D1910" t="inlineStr">
+        <is>
+          <t>政府可能允许酒吧为英格兰比赛延长营业时间至凌晨1点。</t>
+        </is>
+      </c>
+      <c r="E1910" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1910" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1kyr8747m9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr">
+        <is>
+          <t>Exam board sorry for delay to Sats results in England</t>
+        </is>
+      </c>
+      <c r="D1911" t="inlineStr">
+        <is>
+          <t>考试局为英格兰Sats成绩延迟致歉，工会要求确保最终结果准确。</t>
+        </is>
+      </c>
+      <c r="E1911" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1911" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cewq7d4yxq2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1912" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1912" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1912" t="inlineStr">
+        <is>
+          <t>俄称美在日部署导弹破坏亚太稳定；美不同意续签美墨加协定；德国起诉“北溪”爆炸案乌克兰嫌疑人。</t>
+        </is>
+      </c>
+      <c r="E1912" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1912" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEznzTcs6dMSyFQMPpH0co260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1913" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1913" t="inlineStr">
+        <is>
+          <t>South Africa and Ghana in diplomatic row over killing of migrant</t>
+        </is>
+      </c>
+      <c r="D1913" t="inlineStr">
+        <is>
+          <t>南非否认在开普敦反移民抗议中杀害一名加纳公民的说法。</t>
+        </is>
+      </c>
+      <c r="E1913" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1913" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c982k1j3d70o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1914" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1914" t="inlineStr">
+        <is>
+          <t>Aunt of Venezuelan boy pulled from rubble tells BBC she will give him 'mother's warmth'</t>
+        </is>
+      </c>
+      <c r="D1914" t="inlineStr">
+        <is>
+          <t>委内瑞拉2岁男童在地震六天后获救，其姑姑表示将给予他母爱。</t>
+        </is>
+      </c>
+      <c r="E1914" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1914" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c05yv34qlnlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1915" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1915" t="inlineStr">
+        <is>
+          <t>Residents of Ethiopian town forced to kill hundreds of their own dogs after rabies deaths</t>
+        </is>
+      </c>
+      <c r="D1915" t="inlineStr">
+        <is>
+          <t>埃塞俄比亚镇居民因狂犬病致死被迫自行处决数百只狗。</t>
+        </is>
+      </c>
+      <c r="E1915" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1915" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1wy4d5p4pxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1916" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1916" t="inlineStr">
+        <is>
+          <t>Nine Thai monks killed after 11-year-old driver collides with procession</t>
+        </is>
+      </c>
+      <c r="D1916" t="inlineStr">
+        <is>
+          <t>泰国11岁司机撞向僧侣队伍，致9名僧侣死亡。</t>
+        </is>
+      </c>
+      <c r="E1916" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1916" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c23y90lygpzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1917" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1917" t="inlineStr">
+        <is>
+          <t>Watch: BBC at site of deadly Russian attack on Kyiv flats</t>
+        </is>
+      </c>
+      <c r="D1917" t="inlineStr">
+        <is>
+          <t>BBC记者报道俄罗斯致命袭击基辅公寓楼的现场。</t>
+        </is>
+      </c>
+      <c r="E1917" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1917" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c33yl1l8dkro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1918" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1918" t="inlineStr">
+        <is>
+          <t>Vatican declares Society of St. Pius X in schism, excommunicates bishops</t>
+        </is>
+      </c>
+      <c r="D1918" t="inlineStr">
+        <is>
+          <t>梵蒂冈宣布圣庇护十世会分裂，开除其主教和神父教籍。</t>
+        </is>
+      </c>
+      <c r="E1918" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1918" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/02/nx-s1-5878916/vatican-society-of-st-pius-x-in-schism</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1919" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C1919" t="inlineStr">
+        <is>
+          <t>Russia hits Ukraine's capital with a massive drone and missile attack, killing at least 18</t>
+        </is>
+      </c>
+      <c r="D1919" t="inlineStr">
+        <is>
+          <t>俄罗斯大规模无人机和导弹袭击基辅，致至少18人死亡。</t>
+        </is>
+      </c>
+      <c r="E1919" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1919" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/02/nx-s1-5878894/russia-attacks-ukraines-capital-killing-more-than-a-dozen-people</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1920" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1920" t="inlineStr">
+        <is>
+          <t>U.S. and Iran hold separate meetings in Qatar and agree to continue discussions</t>
+        </is>
+      </c>
+      <c r="D1920" t="inlineStr">
+        <is>
+          <t>美伊通过卡塔尔和巴基斯坦调解分别会谈，同意继续讨论并取得积极进展。</t>
+        </is>
+      </c>
+      <c r="E1920" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1920" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/02/nx-s1-5878887/us-iran-meetings-qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1921" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1921" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者马善祥：矛盾化解践初心</t>
+        </is>
+      </c>
+      <c r="D1921" t="inlineStr">
+        <is>
+          <t>“七一勋章”获得者马善祥30多年化解2500多件矛盾，总结“老马工作法”服务基层。</t>
+        </is>
+      </c>
+      <c r="E1921" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1921" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/02/VIDEXgPgKMgmGTPp6OqITw0e260702.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1922" t="inlineStr">
+        <is>
+          <t>Venezuela quake survivor pulled out alive after eight days</t>
+        </is>
+      </c>
+      <c r="D1922" t="inlineStr">
+        <is>
+          <t>委内瑞拉一名男子在建筑倒塌被困八天后获救生还。</t>
+        </is>
+      </c>
+      <c r="E1922" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1922" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce375v12z0qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C1923" t="inlineStr">
+        <is>
+          <t>People smuggler convicted in France found by BBC living in UK and seeking asylum</t>
+        </is>
+      </c>
+      <c r="D1923" t="inlineStr">
+        <is>
+          <t>在法国被判有罪的人口走私头目，被BBC发现生活在英国并寻求庇护。</t>
+        </is>
+      </c>
+      <c r="E1923" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1923" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clye9zn0y1ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1924" t="inlineStr">
+        <is>
+          <t>Canadian boy, 11, dies of rabies after waking to bat on his face</t>
+        </is>
+      </c>
+      <c r="D1924" t="inlineStr">
+        <is>
+          <t>加拿大11岁男孩因被蝙蝠咬伤后死于狂犬病，该国1924年以来仅28例死亡。</t>
+        </is>
+      </c>
+      <c r="E1924" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1924" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c982m1m95q9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1925" t="inlineStr">
+        <is>
+          <t>China says pilot crashed small plane into skyscraper for 'personal reasons'</t>
+        </is>
+      </c>
+      <c r="D1925" t="inlineStr">
+        <is>
+          <t>中国官方称飞行员因个人原因将小型飞机撞入摩天大楼，其已死亡且日记提及轻生。</t>
+        </is>
+      </c>
+      <c r="E1925" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1925" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr47129ky6do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1926" t="inlineStr">
+        <is>
+          <t>Gary Glitter charged with historical sexual offences</t>
+        </is>
+      </c>
+      <c r="D1926" t="inlineStr">
+        <is>
+          <t>前歌手加里·格利特因历史性性犯罪被指控。</t>
+        </is>
+      </c>
+      <c r="E1926" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1926" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2lywez0zddo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1927" t="inlineStr">
+        <is>
+          <t>Grooming gang leader released from prison</t>
+        </is>
+      </c>
+      <c r="D1927" t="inlineStr">
+        <is>
+          <t>性犯罪团伙头目沙比尔·艾哈迈德获释出狱。</t>
+        </is>
+      </c>
+      <c r="E1927" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1927" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyx0vldrlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1928" t="inlineStr">
+        <is>
+          <t>Support floods in for influencer Nara Smith after daughter's cancer diagnosis</t>
+        </is>
+      </c>
+      <c r="D1928" t="inlineStr">
+        <is>
+          <t>网红娜拉·史密斯的女儿确诊癌症后，获得大量支持。</t>
+        </is>
+      </c>
+      <c r="E1928" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1928" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyd3nxr5ggo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-03
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1928"/>
+  <dimension ref="A1:F1966"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62133,6 +62133,1222 @@
         </is>
       </c>
     </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1929" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260703 19:00</t>
+        </is>
+      </c>
+      <c r="D1929" t="inlineStr">
+        <is>
+          <t>中央军委举行晋升上将军衔仪式，习近平颁发命令状；多部门学习贯彻习近平建党105周年讲话。</t>
+        </is>
+      </c>
+      <c r="E1929" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1929" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEcTNEq7lYlINRUm5tZqrU260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C1930" t="inlineStr">
+        <is>
+          <t>[视频]中央军委举行晋升上将军衔仪式 习近平颁发命令状并向晋衔的军官表示祝贺</t>
+        </is>
+      </c>
+      <c r="D1930" t="inlineStr">
+        <is>
+          <t>中央军委举行仪式，习近平向张曙光、王刚颁发晋升上将军衔命令状。</t>
+        </is>
+      </c>
+      <c r="E1930" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1930" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEZQQue6pdTmCNLV8OhN4c260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1931" t="inlineStr">
+        <is>
+          <t>[视频]习近平《在庆祝中国共产党成立105周年大会上的讲话》单行本出版</t>
+        </is>
+      </c>
+      <c r="D1931" t="inlineStr">
+        <is>
+          <t>习近平在庆祝中国共产党成立105周年大会上的讲话单行本出版发行。</t>
+        </is>
+      </c>
+      <c r="E1931" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1931" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDE0m2GTimuQ79AebOWnFKm260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr">
+        <is>
+          <t>[视频]应习近平邀请 纳米比亚总统将访华</t>
+        </is>
+      </c>
+      <c r="D1932" t="inlineStr">
+        <is>
+          <t>应习近平邀请，纳米比亚总统将于7月5日至11日对中国进行国事访问。</t>
+        </is>
+      </c>
+      <c r="E1932" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1932" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDE2SPf4sfFK4ZsyuvprUmP260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr">
+        <is>
+          <t>[视频]为以中国式现代化全面推进强国建设、民族复兴伟业而不懈奋斗——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D1933" t="inlineStr">
+        <is>
+          <t>习近平在建党105周年大会上的讲话引发热烈反响，鼓舞人民奋进新征程。</t>
+        </is>
+      </c>
+      <c r="E1933" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1933" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEufTwuxXH1Z1h9pgPtX8i260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院党组会议 学习贯彻习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话精神和习近平党建思想 丁薛祥出席</t>
+        </is>
+      </c>
+      <c r="D1934" t="inlineStr">
+        <is>
+          <t>李强主持召开国务院党组会议，学习贯彻习近平建党105周年讲话和党建思想。</t>
+        </is>
+      </c>
+      <c r="E1934" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1934" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEQcb2Wbak4xunFP3cTzwG260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr">
+        <is>
+          <t>[视频]全国人大常委会党组举行会议 学习贯彻习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话精神和习近平党建思想 赵乐际主持并讲话</t>
+        </is>
+      </c>
+      <c r="D1935" t="inlineStr">
+        <is>
+          <t>全国人大常委会党组举行会议，赵乐际主持学习贯彻习近平建党105周年讲话。</t>
+        </is>
+      </c>
+      <c r="E1935" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1935" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEcGjxOMomcqnfAhvhGrj1260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr">
+        <is>
+          <t>[视频]中共全国政协党组理论学习中心组举行2026年第三次集体学习 学习贯彻习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话精神和习近平党建思想 王沪宁主持并讲话</t>
+        </is>
+      </c>
+      <c r="D1936" t="inlineStr">
+        <is>
+          <t>全国政协党组理论学习中心组学习习近平建党105周年讲话及党建思想。</t>
+        </is>
+      </c>
+      <c r="E1936" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1936" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEU7qjxiDpSk58QBJMvviO260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr">
+        <is>
+          <t>[视频]中央和国家机关“两优一先”表彰大会在京召开 蔡奇出席并讲话</t>
+        </is>
+      </c>
+      <c r="D1937" t="inlineStr">
+        <is>
+          <t>中央国家机关“两优一先”表彰大会在京召开，蔡奇强调学习贯彻习近平党建思想。</t>
+        </is>
+      </c>
+      <c r="E1937" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1937" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDE0tGrzeLhQdzyahFa6bc2260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>[视频]李希主持召开中央纪委常委会会议 学习贯彻习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话精神和习近平党建思想</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr">
+        <is>
+          <t>李希主持中央纪委常委会，要求贯彻习近平重要讲话和党建思想，推动纪检监察工作高质量发展。</t>
+        </is>
+      </c>
+      <c r="E1938" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1938" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEDuBtqvcc5qJmwv2yHLHT260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr">
+        <is>
+          <t>Iran begins public mourning for Ayatollah killed in February</t>
+        </is>
+      </c>
+      <c r="D1939" t="inlineStr">
+        <is>
+          <t>伊朗为二月遇袭身亡的领袖开始公开哀悼，遗体将停放大清真寺。</t>
+        </is>
+      </c>
+      <c r="E1939" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1939" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2k4k7jqeno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr">
+        <is>
+          <t>Ex-HK bookseller Lam Wing-kee, detained by China in 2015, dies in Taiwan at 70</t>
+        </is>
+      </c>
+      <c r="D1940" t="inlineStr">
+        <is>
+          <t>2015年被中国拘留的香港书店老板林荣基在台湾去世，终年70岁。</t>
+        </is>
+      </c>
+      <c r="E1940" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1940" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/03/g-s1-131904/ex-hk-bookseller-lam-wing-kee-detained-by-china-in-2015-dies-in-taiwan-at-70</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr">
+        <is>
+          <t>[视频]今年2000亿元设备更新资金已全部下达</t>
+        </is>
+      </c>
+      <c r="D1941" t="inlineStr">
+        <is>
+          <t>今年2000亿元设备更新资金已全部下达，支持22个领域约1.1万个项目。</t>
+        </is>
+      </c>
+      <c r="E1941" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1941" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEHVCzO6XU7NIObXTCM9SG260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>经济, 民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D1942" t="inlineStr">
+        <is>
+          <t>公平竞争审查制度十年审查188万件；启动招聘专项行动与网络整治；长三角发布首批国际标准联合项目。</t>
+        </is>
+      </c>
+      <c r="E1942" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1942" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEb63ykW7LPPU5vAFHPQYn260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D1943" t="inlineStr">
+        <is>
+          <t>五位“最美科技工作者”代表在国新办记者会分享投身科技强国建设的故事。</t>
+        </is>
+      </c>
+      <c r="E1943" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1943" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDE82EEzEgYszYkRamgZSSQ260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr">
+        <is>
+          <t>Nasa launches mission to save falling space telescope</t>
+        </is>
+      </c>
+      <c r="D1944" t="inlineStr">
+        <is>
+          <t>NASA发射机器人任务，拯救即将烧毁的太空望远镜。</t>
+        </is>
+      </c>
+      <c r="E1944" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1944" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0ry4xx7rk8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>军事, 社会</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr">
+        <is>
+          <t>[视频]舰艇编队首个开放日迎来众多香港青少年学生参观</t>
+        </is>
+      </c>
+      <c r="D1945" t="inlineStr">
+        <is>
+          <t>海军舰艇编队在港开放，众多香港青少年登舰参观，感受海军风采。</t>
+        </is>
+      </c>
+      <c r="E1945" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1945" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEieUOAgCRLjxwK7nrhyDO260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr">
+        <is>
+          <t>US withdraws troops from Nigeria after Islamic State mission</t>
+        </is>
+      </c>
+      <c r="D1946" t="inlineStr">
+        <is>
+          <t>美军完成在尼日利亚的反恐任务后撤军，称行动成功。</t>
+        </is>
+      </c>
+      <c r="E1946" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1946" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwylkvpl80xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>'Most massive' Russian attack on Kyiv kills at least 30</t>
+        </is>
+      </c>
+      <c r="D1947" t="inlineStr">
+        <is>
+          <t>俄军对基辅发动最大规模袭击，致至少30人死亡。</t>
+        </is>
+      </c>
+      <c r="E1947" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1947" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyv05gk4do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《美丽中国建设“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D1948" t="inlineStr">
+        <is>
+          <t>国务院印发《美丽中国建设“十五五”规划》，部署绿色转型和生态保护重点任务。</t>
+        </is>
+      </c>
+      <c r="E1948" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1948" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEHxB3KBqY94yNppsqscfc260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>[视频]今年第10号台风“美莎克”在海南登陆</t>
+        </is>
+      </c>
+      <c r="D1949" t="inlineStr">
+        <is>
+          <t>今年第10号台风“美莎克”在海南登陆，多地有大到暴雨，各部门做好防范。</t>
+        </is>
+      </c>
+      <c r="E1949" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1949" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDE3HOiJTqj1BJCRlk41UmC260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>NHS to reward people who walk 30 minutes a day</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr">
+        <is>
+          <t>英国NHS将奖励每日步行30分钟的人，明年启动计划。</t>
+        </is>
+      </c>
+      <c r="E1950" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1950" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj6g0rdy40jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>'Less than 10% sheep': How millions may have unknowingly eaten goat, skin and fat kebabs</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr">
+        <is>
+          <t>数百万人在不知情下吃了用山羊皮和脂肪做的“羊肉”烤肉串。</t>
+        </is>
+      </c>
+      <c r="E1951" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1951" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce95y1zlzyxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>German row over plan for workers to need sick note on first day of illness</t>
+        </is>
+      </c>
+      <c r="D1952" t="inlineStr">
+        <is>
+          <t>德国拟要求工人病假首日提交证明，医生组织称此举“近乎疯狂”。</t>
+        </is>
+      </c>
+      <c r="E1952" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1952" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyxnj38m1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>[视频]韩正出席第十四届世界和平论坛开幕式并致辞</t>
+        </is>
+      </c>
+      <c r="D1953" t="inlineStr">
+        <is>
+          <t>韩正在世界和平论坛致辞，提出坚定维护联合国权威、深化多边合作等四点建议。</t>
+        </is>
+      </c>
+      <c r="E1953" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1953" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/03/VIDEf75Oedrbq9VBkesaf6kJ260703.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>France records 2,025 excess deaths at peak of heatwave as Europe braces for more extreme weather</t>
+        </is>
+      </c>
+      <c r="D1954" t="inlineStr">
+        <is>
+          <t>法国热浪高峰期死亡人数超2025人，欧洲面临更极端天气预警。</t>
+        </is>
+      </c>
+      <c r="E1954" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1954" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3ry307rxqro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr">
+        <is>
+          <t>Ukrainian suspect hunted by police after Monaco bomb attack was 'disguised as a man'</t>
+        </is>
+      </c>
+      <c r="D1955" t="inlineStr">
+        <is>
+          <t>摩纳哥爆炸案嫌疑人伪装成男性，警方怀疑其有同伙并事先侦察。</t>
+        </is>
+      </c>
+      <c r="E1955" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1955" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gy603z2qlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1956" t="inlineStr">
+        <is>
+          <t>Instagram running ads promoting child sexual abuse material in India, BBC finds</t>
+        </is>
+      </c>
+      <c r="D1956" t="inlineStr">
+        <is>
+          <t>BBC发现Instagram在印度推送含“强奸”“儿童视频”等词条的性剥削广告。</t>
+        </is>
+      </c>
+      <c r="E1956" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1956" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgm4e0316zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1957" t="inlineStr">
+        <is>
+          <t>Venezuela quake survivor pulled out alive after eight days</t>
+        </is>
+      </c>
+      <c r="D1957" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震八天后，一名被困停车场废墟的男子被救出。</t>
+        </is>
+      </c>
+      <c r="E1957" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1957" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce375v12z0qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1958" t="inlineStr">
+        <is>
+          <t>At least 32 dead after overcrowded bus plunges into ravine in Pakistan</t>
+        </is>
+      </c>
+      <c r="D1958" t="inlineStr">
+        <is>
+          <t>巴基斯坦一辆超载巴士坠入峡谷，至少32人死亡。</t>
+        </is>
+      </c>
+      <c r="E1958" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1958" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czrxezg60x1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1959" t="inlineStr">
+        <is>
+          <t>Bomb blast at Damascus cafe kills nine, Syrian state media say</t>
+        </is>
+      </c>
+      <c r="D1959" t="inlineStr">
+        <is>
+          <t>叙利亚大马士革咖啡馆发生炸弹爆炸，9人死亡。</t>
+        </is>
+      </c>
+      <c r="E1959" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1959" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn0vwxyz40zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1960" t="inlineStr">
+        <is>
+          <t>Greek man found guilty of murdering Scottish woman on Greek island in 2009</t>
+        </is>
+      </c>
+      <c r="D1960" t="inlineStr">
+        <is>
+          <t>希腊男子因2009年杀害苏格兰女子被判10年监禁。</t>
+        </is>
+      </c>
+      <c r="E1960" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1960" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2xwd68l1eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1961" t="inlineStr">
+        <is>
+          <t>UK in talks with Pakistan about deporting grooming gang leader</t>
+        </is>
+      </c>
+      <c r="D1961" t="inlineStr">
+        <is>
+          <t>英国与巴基斯坦商议遣送一名犯罪团伙头目。</t>
+        </is>
+      </c>
+      <c r="E1961" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1961" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8e2j0z7xgxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C1962" t="inlineStr">
+        <is>
+          <t>July 4th events threatened by heat wave. And, Russia strikes on Ukraine's capital</t>
+        </is>
+      </c>
+      <c r="D1962" t="inlineStr">
+        <is>
+          <t>美国独立日活动受热浪威胁，俄罗斯袭击乌克兰首都基辅致多人死亡。</t>
+        </is>
+      </c>
+      <c r="E1962" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1962" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/03/g-s1-131920/up-first-newsletter-america-250-heat-wave-ukraine-russia-democratic-party</t>
+        </is>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1963" t="inlineStr">
+        <is>
+          <t>Police criticise timing of decision on pubs staying open for England match</t>
+        </is>
+      </c>
+      <c r="D1963" t="inlineStr">
+        <is>
+          <t>警方批评酒吧为英格兰比赛延至凌晨5点营业的决定。</t>
+        </is>
+      </c>
+      <c r="E1963" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1963" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd95v388k5jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1964" t="inlineStr">
+        <is>
+          <t>Three men found not guilty of Lyra McKee murder</t>
+        </is>
+      </c>
+      <c r="D1964" t="inlineStr">
+        <is>
+          <t>三名男子被裁定无罪，未参与2019年记者莱拉·麦基谋杀案。</t>
+        </is>
+      </c>
+      <c r="E1964" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1964" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpd357j7020o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C1965" t="inlineStr">
+        <is>
+          <t>'Start work at 11' - but will other bosses be as flexible over England's 1am match?</t>
+        </is>
+      </c>
+      <c r="D1965" t="inlineStr">
+        <is>
+          <t>公司被鼓励允许员工灵活上班，以观看英格兰凌晨1点的比赛。</t>
+        </is>
+      </c>
+      <c r="E1965" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1965" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8x27k180x8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1966" t="inlineStr">
+        <is>
+          <t>Australian officials ask fans to respect the privacy of Neil, a trouble-making seal</t>
+        </is>
+      </c>
+      <c r="D1966" t="inlineStr">
+        <is>
+          <t>澳大利亚官员呼吁民众尊重网红海豹尼尔的隐私，它因捣乱行为走红。</t>
+        </is>
+      </c>
+      <c r="E1966" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1966" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/03/g-s1-131911/australia-trouble-making-seal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-04
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1966"/>
+  <dimension ref="A1:F2001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63349,6 +63349,1126 @@
         </is>
       </c>
     </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C1967" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260704 19:00</t>
+        </is>
+      </c>
+      <c r="D1967" t="inlineStr">
+        <is>
+          <t>庆祝建党105周年重要讲话引发热烈反响；循环经济体系加快建设；各地应对强降雨。</t>
+        </is>
+      </c>
+      <c r="E1967" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1967" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEa8TEsh6IFMghlKtThJg3260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1968" t="inlineStr">
+        <is>
+          <t>[视频]牢记初心使命 勇担时代重任——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D1968" t="inlineStr">
+        <is>
+          <t>习近平在建党105周年大会上的讲话引发中管企业、金融企业及各地干部群众热烈反响。</t>
+        </is>
+      </c>
+      <c r="E1968" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1968" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEnpHM70N0Q1cSyQMMPbyv260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1969" t="inlineStr">
+        <is>
+          <t>[视频]为中华民族伟大复兴凝聚磅礴力量——习近平主席重要讲话引发港澳台人士热烈反响</t>
+        </is>
+      </c>
+      <c r="D1969" t="inlineStr">
+        <is>
+          <t>习近平主席讲话引发港澳台人士热烈反响，凝聚中华民族伟大复兴的磅礴力量。</t>
+        </is>
+      </c>
+      <c r="E1969" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1969" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEp0HIXti7UfXNcsAOaxoF260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr">
+        <is>
+          <t>[视频]《习近平谈治国理政》第五卷中斯读者会在斯里兰卡首都科伦坡举行</t>
+        </is>
+      </c>
+      <c r="D1970" t="inlineStr">
+        <is>
+          <t>《习近平谈治国理政》第五卷中斯读者会在斯里兰卡科伦坡举行，促进中斯命运共同体。</t>
+        </is>
+      </c>
+      <c r="E1970" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1970" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDE4aFGH3nUJLUPhH57dpI3260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1971" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者李连成：当干部就应该能吃亏</t>
+        </is>
+      </c>
+      <c r="D1971" t="inlineStr">
+        <is>
+          <t>“七一勋章”获得者李连成30多年带领村民致富，践行“当干部就该能吃亏”信念。</t>
+        </is>
+      </c>
+      <c r="E1971" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1971" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDESv6magE1sfZgRV6mVuhX260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C1972" t="inlineStr">
+        <is>
+          <t>[视频]多国人士高度评价习近平在庆祝中国共产党成立105周年大会上的重要讲话</t>
+        </is>
+      </c>
+      <c r="D1972" t="inlineStr">
+        <is>
+          <t>多国人士高度评价习近平在庆祝中国共产党成立105周年大会上的重要讲话。</t>
+        </is>
+      </c>
+      <c r="E1972" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1972" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEVCxtam1ay8fyCPJbmiSg260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1973" t="inlineStr">
+        <is>
+          <t>Keiko Fujimori declared winner of Peru's presidential election weeks after vote</t>
+        </is>
+      </c>
+      <c r="D1973" t="inlineStr">
+        <is>
+          <t>藤森庆子在大选近一个月后被宣布赢得秘鲁总统选举。</t>
+        </is>
+      </c>
+      <c r="E1973" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1973" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr5jpvv06e1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C1974" t="inlineStr">
+        <is>
+          <t>The massive scramble behind the scenes before the new PM arrives</t>
+        </is>
+      </c>
+      <c r="D1974" t="inlineStr">
+        <is>
+          <t>新首相即将上任，白宫内职位争夺激烈，议员称场面混乱。</t>
+        </is>
+      </c>
+      <c r="E1974" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1974" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj4g0n0p15xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C1975" t="inlineStr">
+        <is>
+          <t>Fireworks, flyovers and a 'really long' Trump speech ahead as US celebrates 250th</t>
+        </is>
+      </c>
+      <c r="D1975" t="inlineStr">
+        <is>
+          <t>美国250周年庆典将燃放85万烟花，特朗普发表长篇演讲。</t>
+        </is>
+      </c>
+      <c r="E1975" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1975" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp36l4e6v9po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C1976" t="inlineStr">
+        <is>
+          <t>[视频]我国加快建设循环经济高质量发展体系</t>
+        </is>
+      </c>
+      <c r="D1976" t="inlineStr">
+        <is>
+          <t>我国将推新举措建设循环经济体系，目标2030年建成全球最大体系，产值达8万亿元。</t>
+        </is>
+      </c>
+      <c r="E1976" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1976" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEqZIPfhgZL9EDTrrruYiD260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C1977" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D1977" t="inlineStr">
+        <is>
+          <t>四部门延续稳岗扩岗政策；国际科技组织成立指引出台；西渝高铁隧道贯通；全球数字经济案例发布。</t>
+        </is>
+      </c>
+      <c r="E1977" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1977" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEK5r7NMFrssuF1ugkXow8260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C1978" t="inlineStr">
+        <is>
+          <t>[视频]【活力中国调研行】天津：打通科研成果转化“最后一公里”</t>
+        </is>
+      </c>
+      <c r="D1978" t="inlineStr">
+        <is>
+          <t>天津天开园打通科研成果转化“最后一公里”，助初创企业半年实现规模化量产。</t>
+        </is>
+      </c>
+      <c r="E1978" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1978" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEf0CgRuTuA1FaSKvdfmaU260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr">
+        <is>
+          <t>军事</t>
+        </is>
+      </c>
+      <c r="C1979" t="inlineStr">
+        <is>
+          <t>[视频]俄称控制重镇康斯坦丁诺夫卡 乌称袭击圣彼得堡</t>
+        </is>
+      </c>
+      <c r="D1979" t="inlineStr">
+        <is>
+          <t>俄称控制顿涅茨克重镇，乌称袭击圣彼得堡，双方战况激烈。</t>
+        </is>
+      </c>
+      <c r="E1979" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1979" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEFp1AsWyLwhS46JimhHzG260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C1980" t="inlineStr">
+        <is>
+          <t>Ukraine hits major oil terminal in Russia's St Petersburg</t>
+        </is>
+      </c>
+      <c r="D1980" t="inlineStr">
+        <is>
+          <t>乌克兰袭击俄罗斯圣彼得堡一主要石油终端。</t>
+        </is>
+      </c>
+      <c r="E1980" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1980" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8j2vmzxezro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1981" t="inlineStr">
+        <is>
+          <t>China's military promotes 2 new generals after anti-corruption purge thins ranks</t>
+        </is>
+      </c>
+      <c r="D1981" t="inlineStr">
+        <is>
+          <t>中国军方在反腐行动后提拔两名新将军，以确保军队对党和领导人的忠诚。</t>
+        </is>
+      </c>
+      <c r="E1981" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1981" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/04/g-s1-131994/chinas-military-promotes-2-new-generals-after-anti-corruption-purge-thins-ranks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C1982" t="inlineStr">
+        <is>
+          <t>[视频]各地积极应对强降雨天气</t>
+        </is>
+      </c>
+      <c r="D1982" t="inlineStr">
+        <is>
+          <t>全国多地遭遇强降雨、台风天气，各部门积极应对，保障生产生活秩序。</t>
+        </is>
+      </c>
+      <c r="E1982" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1982" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDENocjlxExAvwvIFcae1pH260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1983" t="inlineStr">
+        <is>
+          <t>Row after Indian state drops eggs from school lunch menu</t>
+        </is>
+      </c>
+      <c r="D1983" t="inlineStr">
+        <is>
+          <t>印度西孟加拉邦取消学校午餐鸡蛋引发争议。</t>
+        </is>
+      </c>
+      <c r="E1983" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1983" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c33yldyd62po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C1984" t="inlineStr">
+        <is>
+          <t>What could new rights for unmarried couples mean for your money?</t>
+        </is>
+      </c>
+      <c r="D1984" t="inlineStr">
+        <is>
+          <t>英国政府拟提案，为非婚同居夫妇分手时提供更多法律保护。</t>
+        </is>
+      </c>
+      <c r="E1984" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1984" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2vx4dvgzno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C1985" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D1985" t="inlineStr">
+        <is>
+          <t>伊朗举行哈梅内伊遗体告别仪式；美国高温限电；西班牙林火影响近万人。</t>
+        </is>
+      </c>
+      <c r="E1985" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1985" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDE8cCK6lszkI2TtwyrwWoV260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1986" t="inlineStr">
+        <is>
+          <t>Brutal heat cancels Fourth of July events, from DC to Philadelphia</t>
+        </is>
+      </c>
+      <c r="D1986" t="inlineStr">
+        <is>
+          <t>美国超1.65亿人遭受极端高温，多地独立日庆祝活动被取消。</t>
+        </is>
+      </c>
+      <c r="E1986" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1986" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cevlkzer7vdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1987" t="inlineStr">
+        <is>
+          <t>Large crowds gather in Tehran on first day of Ayatollah Khamenei's funeral</t>
+        </is>
+      </c>
+      <c r="D1987" t="inlineStr">
+        <is>
+          <t>大批民众聚集德黑兰参加哈梅内伊葬礼首日活动。</t>
+        </is>
+      </c>
+      <c r="E1987" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1987" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0ky2zen1kgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1988" t="inlineStr">
+        <is>
+          <t>'Flamingo Revolution' takes off as thousands demand Albanian PM's resignation</t>
+        </is>
+      </c>
+      <c r="D1988" t="inlineStr">
+        <is>
+          <t>“火烈鸟革命”爆发，数千人要求阿尔巴尼亚总理辞职。</t>
+        </is>
+      </c>
+      <c r="E1988" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1988" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8925jnl0z3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C1989" t="inlineStr">
+        <is>
+          <t>Pope urges Europe to do more for migrants while visiting gateway island</t>
+        </is>
+      </c>
+      <c r="D1989" t="inlineStr">
+        <is>
+          <t>教皇在访问兰佩杜萨岛时呼吁欧洲为移民做更多。</t>
+        </is>
+      </c>
+      <c r="E1989" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1989" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz83n7q5no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C1990" t="inlineStr">
+        <is>
+          <t>Prince Harry will not be joined by Meghan and children on London trip</t>
+        </is>
+      </c>
+      <c r="D1990" t="inlineStr">
+        <is>
+          <t>哈里王子伦敦行程变动，梅根与孩子因无公费安保不会同行。</t>
+        </is>
+      </c>
+      <c r="E1990" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1990" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr5jpzn2814o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C1991" t="inlineStr">
+        <is>
+          <t>Dayslong funeral for slain Supreme Leader Ayatollah Ali Khamenei begins in Tehran</t>
+        </is>
+      </c>
+      <c r="D1991" t="inlineStr">
+        <is>
+          <t>伊朗最高领袖哈梅内伊遇袭身亡，葬礼在德黑兰开始，持续数日。</t>
+        </is>
+      </c>
+      <c r="E1991" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F1991" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/04/nx-s1-5882083/iran-funeral-ayatollah-ali-khamenei</t>
+        </is>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1992" t="inlineStr">
+        <is>
+          <t>[视频]【暖心一瞬】危急时刻伸援手 凡人善举暖人心</t>
+        </is>
+      </c>
+      <c r="D1992" t="inlineStr">
+        <is>
+          <t>江苏、山东等地热心市民在危急关头挺身而出，合力救人灭火。</t>
+        </is>
+      </c>
+      <c r="E1992" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1992" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEDyoBiUvivrOkPua8wCcH260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C1993" t="inlineStr">
+        <is>
+          <t>Boy, 3, had five surgeries after crocodile attack</t>
+        </is>
+      </c>
+      <c r="D1993" t="inlineStr">
+        <is>
+          <t>3岁男孩遭鳄鱼攻击后接受五次手术，手臂活动情况不确定。</t>
+        </is>
+      </c>
+      <c r="E1993" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1993" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gy0k2d491o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>社会, 科技</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr">
+        <is>
+          <t>'Hotter and hotter and hotter' - Europe's new climate in seven charts</t>
+        </is>
+      </c>
+      <c r="D1994" t="inlineStr">
+        <is>
+          <t>欧洲六月气温破纪录，科学家警告气候变化将加剧。</t>
+        </is>
+      </c>
+      <c r="E1994" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1994" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8e2j0j87reo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr">
+        <is>
+          <t>The schools starting late after 1am England kick-off to 'reduce pressure' on parents</t>
+        </is>
+      </c>
+      <c r="D1995" t="inlineStr">
+        <is>
+          <t>部分学校为配合凌晨球赛推迟上课，获家长支持。</t>
+        </is>
+      </c>
+      <c r="E1995" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F1995" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621j2qj50do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr">
+        <is>
+          <t>[视频]“七一”前后红色文艺作品集中上演 传承革命精神</t>
+        </is>
+      </c>
+      <c r="D1996" t="inlineStr">
+        <is>
+          <t>七一前后红色文艺作品集中上演，创新表达吸引年轻人传承革命精神。</t>
+        </is>
+      </c>
+      <c r="E1996" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F1996" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/04/VIDEbvNxYWgrNe5spD5bGu6z260704.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr">
+        <is>
+          <t>Taylor Swift marries Travis Kelce in NYC ceremony officiated by Adam Sandler</t>
+        </is>
+      </c>
+      <c r="D1997" t="inlineStr">
+        <is>
+          <t>泰勒·斯威夫特与特拉维斯·凯尔西在纽约结婚，亚当·桑德勒主持。</t>
+        </is>
+      </c>
+      <c r="E1997" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1997" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c982ry2pen3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr">
+        <is>
+          <t>Dior dress, Adam Sandler and a man of honour: What we know about Taylor and Travis's wedding</t>
+        </is>
+      </c>
+      <c r="D1998" t="inlineStr">
+        <is>
+          <t>泰勒和特拉维斯在纽约完婚，婚礼细节曝光。</t>
+        </is>
+      </c>
+      <c r="E1998" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1998" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg5zn58nj2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr">
+        <is>
+          <t>In pictures: Stars and fans celebrate Taylor Swift and Travis Kelce's wedding</t>
+        </is>
+      </c>
+      <c r="D1999" t="inlineStr">
+        <is>
+          <t>明星和粉丝庆祝泰勒·斯威夫特和特拉维斯·凯尔西的婚礼。</t>
+        </is>
+      </c>
+      <c r="E1999" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F1999" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c7vyqgy4r5lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr">
+        <is>
+          <t>Cape Verde's historic World Cup ride ends after pushing Argentina to the brink</t>
+        </is>
+      </c>
+      <c r="D2000" t="inlineStr">
+        <is>
+          <t>佛得角世界杯首秀虽未赢球，但与阿根廷激战至最后一刻，令人难忘。</t>
+        </is>
+      </c>
+      <c r="E2000" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2000" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/04/nx-s1-5882086/cape-verde-world-cup-ends</t>
+        </is>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>体育</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr">
+        <is>
+          <t>Pubs and police brace for England-Mexico 1am kick-off after Fifa U-turn</t>
+        </is>
+      </c>
+      <c r="D2001" t="inlineStr">
+        <is>
+          <t>英格兰世界杯16强赛因国际足联改期，将于周一凌晨1点开球。</t>
+        </is>
+      </c>
+      <c r="E2001" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2001" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy9r2x4pz1wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-05
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2001"/>
+  <dimension ref="A1:F2029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64469,6 +64469,902 @@
         </is>
       </c>
     </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>政治, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260705 19:00</t>
+        </is>
+      </c>
+      <c r="D2002" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道了习近平论述摘编出版、生态建设、强军反响、七一勋章、强降雨应对、香港空间站载荷等新闻。</t>
+        </is>
+      </c>
+      <c r="E2002" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2002" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDE8chc5JgDZc9DPXQIC9PG260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>[视频]《习近平关于基层工作方法论述摘编》出版发行</t>
+        </is>
+      </c>
+      <c r="D2003" t="inlineStr">
+        <is>
+          <t>《习近平关于基层工作方法论述摘编》出版发行，摘自1983年至2026年期间重要讲话。</t>
+        </is>
+      </c>
+      <c r="E2003" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2003" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEkpuaf9zNHOEqwIhy5DQS260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：坚定信心、接续奋斗，不断创造无愧于时代和人民的新业绩——论学习贯彻习近平总书记在庆祝中国共产党成立105周年大会上重要讲话</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>人民日报发表评论员文章，论学习贯彻习近平在建党105周年大会上的重要讲话。</t>
+        </is>
+      </c>
+      <c r="E2004" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2004" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEdurcZppGKbeDsk260FCN260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>How Iran's new regime is very different to what came before</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>伊朗新政权与以往截然不同，哈梅内伊葬礼凸显变化，新领导层意图不明。</t>
+        </is>
+      </c>
+      <c r="E2005" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2005" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cg534ryp660o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>Reform denies rules broken by Farage after benefits from ally not declared</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>改革党否认法拉奇违规，但未申报一名有欺诈前科的加密货币商人的支持。</t>
+        </is>
+      </c>
+      <c r="E2006" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2006" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy0424end7vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>Pastor freed from prison in China weeks after Trump requested his release</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>特朗普向习近平提及后，中国释放了一名被拘留的地下教会牧师。</t>
+        </is>
+      </c>
+      <c r="E2007" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2007" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/05/nx-s1-5882784/pastor-freed-prison-china-trump-request</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>经济, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr">
+        <is>
+          <t>快递量破千亿、电子信息制造业增长、国际航空货运航线新增、核电并网、电影票房破20亿。</t>
+        </is>
+      </c>
+      <c r="E2008" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2008" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDErPPoHYJsgFfbTKB68wPu260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>[视频]香港首个空间站科学载荷“天韵相机”完成部署</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>香港首个空间站科学载荷“天韵相机”在神舟任务中完成部署，监测温室气体。</t>
+        </is>
+      </c>
+      <c r="E2009" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2009" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEMhyvPYqcRbCxScNEKA0F260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>军事, 政治</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>[视频]铸牢听党指挥的强军之魂 攻坚建军百年奋斗目标——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话在全军引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>习近平在建党105周年大会讲话在全军引发热烈反响，强调绝对领导与强军目标。</t>
+        </is>
+      </c>
+      <c r="E2010" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2010" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEKv1ufLcSBdnyDm4fjVcF260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】践行绿色发展理念 绘就生态中国壮美画卷</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>践行绿色发展理念，中国在生态修复和绿色能源等方面取得举世瞩目的生态奇迹。</t>
+        </is>
+      </c>
+      <c r="E2011" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2011" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEInEqxjlXJ2TAFa1EKmse260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>[视频]各地采取有效措施 积极应对强降雨天气</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>华南至长江中下游持续强降雨，各地积极组织抢险并转移被困群众。</t>
+        </is>
+      </c>
+      <c r="E2012" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2012" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDETOjTPZUXiS0vwwxtsQjI260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>'Start work at 11' - but will other bosses be as flexible over England's 1am match?</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>呼吁雇主灵活安排员工凌晨看球，允许11点开始工作。</t>
+        </is>
+      </c>
+      <c r="E2013" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2013" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8x27k180x8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>[视频]国际人士高度评价习近平在庆祝中国共产党成立105周年大会上的重要讲话</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>国际人士高度评价习近平讲话，认为为世界贡献中国智慧。</t>
+        </is>
+      </c>
+      <c r="E2014" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2014" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEHRdQXeNU3ZZtSKN7LlRR260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>伊朗警告勿干涉霍尔木兹海峡；以色列承认在阿联酋部署“铁穹”；极端高温或影响环法赛。</t>
+        </is>
+      </c>
+      <c r="E2015" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2015" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDE8CBiwUCo3sdc9bsxigDW260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>Iran's supreme leader absent as senior officials attend ayatollah's funeral</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>伊朗最高领袖缺席高级官员葬礼，其子哈梅内伊自父亲遇袭后未公开露面。</t>
+        </is>
+      </c>
+      <c r="E2016" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2016" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cevllyj9vv3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>国际, 政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>US marks 250th birthday with fireworks, flyovers and extreme weather</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>美国纪念250周年生日，特朗普演讲涉及政治议程并致敬老兵。</t>
+        </is>
+      </c>
+      <c r="E2017" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2017" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp9lppvkmz5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>Evacuations in Guam as super typhoon Bavi approaches</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>超强台风巴维逼近关岛，风速超160英里/时，居民紧急疏散。</t>
+        </is>
+      </c>
+      <c r="E2018" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2018" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr7xpgx50jxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>国际, 科技</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>Australia probes mystery space balls that washed up on beach</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>澳大利亚调查在昆士兰海滩发现的六块神秘太空残骸。</t>
+        </is>
+      </c>
+      <c r="E2019" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2019" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1jyydr7jnjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>Chinese underground church figure Jin Mingri freed from prison</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>中国地下教会领袖金明日获释，此前特朗普向习近平提出请求。</t>
+        </is>
+      </c>
+      <c r="E2020" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2020" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gy51ky75vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>Nigeria says two nationals killed in South Africa amid rise of anti-migrant attacks</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr">
+        <is>
+          <t>尼日利亚称一名国民在南非被警方用残忍审讯手段杀害，反移民袭击增多。</t>
+        </is>
+      </c>
+      <c r="E2021" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2021" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cqj11lxwnn0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者吴亚琴：温暖一方邻里 守住万家灯火</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr">
+        <is>
+          <t>“七一勋章”获得者吴亚琴扎根基层30年，将老旧社区建成花园社区。</t>
+        </is>
+      </c>
+      <c r="E2022" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2022" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/05/VIDEiYwc5oUqunN7KyFeOr5H260705.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>Scorching heat and delays: How Washington DC marked America 250</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>美国庆祝250周年国庆，烟花、飞行表演与酷热天气并存。</t>
+        </is>
+      </c>
+      <c r="E2023" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2023" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/cwyk2ypj014o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>France survive Paraguay's 'disgraceful' and 'embarrassing' dark arts</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>法国队在本届世界杯遭遇巴拉圭队的“黑暗艺术”战术，艰难取胜引争议。</t>
+        </is>
+      </c>
+      <c r="E2024" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2024" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cn4dpd11v1eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>England battling history as well as Mexican nation in Azteca cauldron</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>英格兰队将在阿兹台克球场对阵墨西哥，不仅要对抗历史还要对抗整个国家。</t>
+        </is>
+      </c>
+      <c r="E2025" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2025" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cvg7z7zxkw9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>文体, 民生</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>Staying up for the match? How to handle a 1am kick-off</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>如何应对凌晨1点开球的比赛？提供观赛战术建议。</t>
+        </is>
+      </c>
+      <c r="E2026" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2026" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3wyel830w8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>England enter the Azteca - where football kings are crowned</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>英格兰队将在世界杯迎战墨西哥，BBC探索阿兹台克球场的历史与文化影响力。</t>
+        </is>
+      </c>
+      <c r="E2027" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2027" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cg74e324835o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>Mexico return luxury watches gifted by YouTuber</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>墨西哥队因违反国际足联规定，退还了YouTuber赠送的豪华手表。</t>
+        </is>
+      </c>
+      <c r="E2028" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2028" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/clyrpy3kn9po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>Stay humble - the Premier League feud about to hit world stage</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>哈兰德与加布里埃尔的英超恩怨将在世界杯挪威对巴西的比赛中上演。</t>
+        </is>
+      </c>
+      <c r="E2029" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2029" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c2ky2x52kwlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-06
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2029"/>
+  <dimension ref="A1:F2056"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65365,6 +65365,870 @@
         </is>
       </c>
     </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>政治, 民生, 经济</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260706 19:00</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>中国领导人致贺电；庆祝建党105周年；物流业扩张；广西水库险情；多领域动态。</t>
+        </is>
+      </c>
+      <c r="E2030" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2030" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEdBf3ibWxj9LWxXUjShiC260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>[视频]习近平致电祝贺藤森庆子当选秘鲁总统</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>习近平致电祝贺藤森庆子当选秘鲁总统，强调建交55周年，推动双边关系发展。</t>
+        </is>
+      </c>
+      <c r="E2031" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2031" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEAtaVpVkKOpnjcYnYtCuH260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>[视频]习近平同黑山总统就中国同黑山建交20周年互致贺电</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>习近平与黑山总统互致贺电，庆祝两国建交20周年，愿深化互利合作。</t>
+        </is>
+      </c>
+      <c r="E2032" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2032" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDE3PtY1qAzxvViFoPXVGej260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>[视频]【伟大征程】携手构建人类命运共同体 谱写和平发展新篇章</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>阐述构建人类命运共同体理念，强调中国全球视野与和平发展，迎密集访华潮。</t>
+        </is>
+      </c>
+      <c r="E2033" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2033" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDE3UodOsA4CW0DHwAQEOto260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>[视频]勠力同心 团结奋斗 汇聚强国建设民族复兴伟业磅礴力量——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>习近平建党105周年讲话在民主党派中引发热烈反响，强调团结奋斗推进中国式现代化。</t>
+        </is>
+      </c>
+      <c r="E2034" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2034" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEMsWuaVqjZpxjfRp15EKa260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>[视频]“在高质量发展中保障和改善民生”形势政策系列报告会第三场报告会在京举行</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>形势政策报告会在京举行，强调以高水平法治服务高质量发展，保障民生安全。</t>
+        </is>
+      </c>
+      <c r="E2035" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2035" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEReiiRVL8vsMnB08lnh1n260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>政治, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>中宣部新命名77个爱国主义教育示范基地；国务院部署安全生产；中国援助委内瑞拉物资启运；黄河调水调沙。</t>
+        </is>
+      </c>
+      <c r="E2036" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2036" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDETRN2jAMkzZStZUgNSrM1260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>Chris Mason: Accusations around Farage leave him looking vulnerable to his rivals</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>围绕法拉奇的指控令其在权力、透明度和金钱问题上显得脆弱。</t>
+        </is>
+      </c>
+      <c r="E2037" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2037" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c04yyx15xngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>政治, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>Trump, Mamdani give contrasting July 4th speeches. And, U.S. faces Belgium in World Cup</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>特朗普与马姆达尼在独立日发表对立演讲，美国队将与比利时进行世界杯比赛。</t>
+        </is>
+      </c>
+      <c r="E2038" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2038" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/06/g-s1-132097/up-first-newsletter-america-250-trump-democrats-iran-israel-world-cup-folarin-balogun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>政治, 国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>Huge crowds of mourners join a funeral procession for Iran's Ayatollah Ali Khamenei</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>伊朗为遇袭身亡的哈梅内伊举行葬礼，大批民众参加送葬队伍。</t>
+        </is>
+      </c>
+      <c r="E2039" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2039" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/06/nx-s1-5877741/ayatollahs-funeral-procession-begins-in-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>Trump won spending promises from NATO last year. This week, he'll try to enforce them</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>特朗普赴北约峰会，试图强制盟友兑现去年做出的军费承诺。</t>
+        </is>
+      </c>
+      <c r="E2040" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2040" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/06/g-s1-132082/trump-nato-turkey-spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>[视频]今年“两重”建设项目清单全部下达完毕</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>今年“两重”建设项目清单全部下达，共8000亿元支持1417个重大项目建设。</t>
+        </is>
+      </c>
+      <c r="E2041" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2041" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDETxZNUEhmI6vPRYWNftM7260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>[视频]6月份中国物流业景气指数加快扩张</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>6月中国物流业景气指数升至50.6%，需求与投资持续回升，电子设备等物流需求增长良好。</t>
+        </is>
+      </c>
+      <c r="E2042" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2042" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDElaA0vnHdMZKeKIIuh8w7260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>Ukraine warns of interceptor missile shortage as 22 killed in Kyiv region</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>乌克兰警告拦截导弹短缺，基辅遭俄大规模导弹和无人机袭击致22人死亡。</t>
+        </is>
+      </c>
+      <c r="E2043" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2043" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cewqqnd7zdwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>Russian missile and drone attack on Ukraine's capital kills at least 12</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>俄军对基辅发动导弹无人机袭击，至少12人死亡，暴露乌防空漏洞。</t>
+        </is>
+      </c>
+      <c r="E2044" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2044" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/06/g-s1-132088/russian-missile-drone-attack-kyiv-kills-at-least-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>[视频]广西南宁多个水库出现险情 抢险救援加紧进行</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>广西南宁多个水库因台风出现险情，抢险救援加紧，国家防总提升应急响应至二级。</t>
+        </is>
+      </c>
+      <c r="E2045" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2045" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDElOoPKv7NTUgOh1Dawovz260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>[视频]伊媒称伊朗与卡塔尔恢复海上贸易</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>伊朗与卡塔尔恢复海上贸易；内塔尼亚胡称不让伊朗拥核；以军称全面控制黎南部关键区域。</t>
+        </is>
+      </c>
+      <c r="E2046" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2046" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDELuzrJvRTzmCVwqAVsn9l260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>俄大规模打击乌军工设施；欧佩克+决定8月增产；法国林火致万人撤离；刚果（金）埃博拉死亡超500例。</t>
+        </is>
+      </c>
+      <c r="E2047" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2047" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEpKF0hvNyifVCZDZRQFpd260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>Huge crowds fill Tehran streets for Khamenei's funeral procession</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>大量民众涌入德黑兰街头参加哈梅内伊的葬礼游行，挥舞旗帜与复仇横幅。</t>
+        </is>
+      </c>
+      <c r="E2048" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2048" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdejj44kl70o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者王於昌：恪守忠诚 居功不显</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>介绍90岁退伍老兵王於昌，曾击落U-2侦察机立一等功，转业后默默奉献。</t>
+        </is>
+      </c>
+      <c r="E2049" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2049" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/06/VIDEejQ4G2zw61Fe5YC8mW5q260706.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>Wildfire in southern France forces evacuation of 10,000 people</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>法国南部野火蔓延，迫使上万人撤离，环法自行车赛第三赛段禁止观众入场。</t>
+        </is>
+      </c>
+      <c r="E2050" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2050" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crlwweye9glo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>'I ate ketchup and cheese,' says Venezuelan girl trapped under quake rubble for 32 hours</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>委内瑞拉地震中，一名被困废墟32小时的女孩称靠番茄酱和奶酪维生。</t>
+        </is>
+      </c>
+      <c r="E2051" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2051" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9922x87nj8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>Buckingham Palace says Prince Harry will not stay there despite his team announcing he would</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>白金汉宫称哈里王子未在截止日期前回复住宿邀请，将不会入住。</t>
+        </is>
+      </c>
+      <c r="E2052" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2052" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c77yykl87yno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>Amber heat-health alerts issued as UK could see 10 consecutive days of temperatures over 30C</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>英国面临今夏第三波热浪，或连续10天高温超30℃，发布高温健康预警。</t>
+        </is>
+      </c>
+      <c r="E2053" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2053" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/cly77zjey40o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>Trump confirms he asked Fifa to review Balogun ban</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>特朗普确认要求国际足联审查美国前锋巴洛贡的世界杯禁赛处罚。</t>
+        </is>
+      </c>
+      <c r="E2054" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2054" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c1myykx0gmxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>All-nighters, phone bans and school screenings - how you watched England's epic win</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>英格兰队精彩获胜，球迷们在不同地点熬夜观战，包括学校和酒吧。</t>
+        </is>
+      </c>
+      <c r="E2055" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2055" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9q22p2v9dxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>Y si sí: the phrase uniting Mexico during the World Cup</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr">
+        <is>
+          <t>墨西哥世界杯之旅催生全国流行口号“Y si sí?”，意为“如果我们能呢？”。</t>
+        </is>
+      </c>
+      <c r="E2056" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2056" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/05/nx-s1-5881076/y-si-si-the-phrase-uniting-mexicos-world-cup-fans</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-07
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2056"/>
+  <dimension ref="A1:F2094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66229,6 +66229,1222 @@
         </is>
       </c>
     </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>政治, 民生, 军事</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260707 19:00</t>
+        </is>
+      </c>
+      <c r="D2057" t="inlineStr">
+        <is>
+          <t>习近平指示防汛救灾，强调全力抢险、确保群众安全；科技自强、抗战纪念等多条要闻。</t>
+        </is>
+      </c>
+      <c r="E2057" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2057" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEnps8BjXeDHxmjk1JoOi9260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>[视频]习近平对防汛救灾工作作出重要指示强调 要全力组织抢险救援、伤员救治、群众安置 扎实做好防灾救灾各项工作 确保人民群众生命财产安全 李强作出批示</t>
+        </is>
+      </c>
+      <c r="D2058" t="inlineStr">
+        <is>
+          <t>习近平对防汛救灾作指示，要求全力组织抢险救援，确保群众生命财产安全。</t>
+        </is>
+      </c>
+      <c r="E2058" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2058" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDENBDrsCZFeIwOfRfEIZg7260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>[视频]只争朝夕 不负韶华 在新征程上跑好历史接力赛——习近平总书记在庆祝中国共产党成立105周年大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2059" t="inlineStr">
+        <is>
+          <t>习近平建党105周年讲话引发青年热烈反响，激励在新征程上跑好接力赛。</t>
+        </is>
+      </c>
+      <c r="E2059" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2059" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDE6lF1tAIBVswqkh7ocf1d260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>[视频]全国政协召开主席会议成员务虚会 王沪宁主持并讲话</t>
+        </is>
+      </c>
+      <c r="D2060" t="inlineStr">
+        <is>
+          <t>全国政协召开务虚会，王沪宁强调聚焦中心任务，为推进中国式现代化凝聚力量。</t>
+        </is>
+      </c>
+      <c r="E2060" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2060" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDE9qM3MiNZVTaAU57xGbj8260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>[视频]中共中央组织部印发《关于在防汛救灾工作中充分发挥基层党组织战斗堡垒作用和广大党员先锋模范作用的通知》</t>
+        </is>
+      </c>
+      <c r="D2061" t="inlineStr">
+        <is>
+          <t>中组部印发通知，要求基层党组织和党员在防汛救灾中发挥先锋模范作用。</t>
+        </is>
+      </c>
+      <c r="E2061" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2061" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEY1uIxe1y9Kod5slnQBAg260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>[视频]陕西省委原常委、西安市委原书记方红卫严重违纪违法被开除党籍和公职</t>
+        </is>
+      </c>
+      <c r="D2062" t="inlineStr">
+        <is>
+          <t>陕西省委原常委、西安市委原书记方红卫严重违纪违法被开除党籍和公职。</t>
+        </is>
+      </c>
+      <c r="E2062" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2062" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDENMd3EiKkORF07IWDc1e3260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>Marine Le Pen found guilty, but court clears way for presidential run if she wears tag</t>
+        </is>
+      </c>
+      <c r="D2063" t="inlineStr">
+        <is>
+          <t>法国极右翼领导人勒庞被判有罪，但法院允许其佩戴电子标签参选总统。</t>
+        </is>
+      </c>
+      <c r="E2063" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2063" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly85qjg45no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>Resistance and revenge - Iran wanted to send a message with its farewell to Khamenei</t>
+        </is>
+      </c>
+      <c r="D2064" t="inlineStr">
+        <is>
+          <t>伊朗通过三天哀悼向世界传递反抗与报复的讯息。</t>
+        </is>
+      </c>
+      <c r="E2064" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2064" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c07yy3j3nljo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>Public to be asked who should pay for social care as part of major review</t>
+        </is>
+      </c>
+      <c r="D2065" t="inlineStr">
+        <is>
+          <t>重大审查将询问公众谁应支付社会护理费用，当前体系被称不可能。</t>
+        </is>
+      </c>
+      <c r="E2065" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2065" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg49lq1jw6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>Woman accuses Graham Platner of sexual assault. And, NATO summit begins</t>
+        </is>
+      </c>
+      <c r="D2066" t="inlineStr">
+        <is>
+          <t>女子指控格拉汉姆性侵，其参议院竞选面临压力；特朗普在峰会前对北约表达不满。</t>
+        </is>
+      </c>
+      <c r="E2066" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2066" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/g-s1-132281/up-first-newsletter-graham-platner-nato-trump-climate-change-us-roads</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>One million more UK homeowners set  to face higher mortgages</t>
+        </is>
+      </c>
+      <c r="D2067" t="inlineStr">
+        <is>
+          <t>逾百万英国房主面临房贷上涨，平均月供增45英镑。</t>
+        </is>
+      </c>
+      <c r="E2067" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2067" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cze9kpxx6d8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>经济, 社会</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>Online gamblers betting more than £1,000 to face new checks</t>
+        </is>
+      </c>
+      <c r="D2068" t="inlineStr">
+        <is>
+          <t>监管机构规定，24小时内在线下注超1000英镑者需接受评估。</t>
+        </is>
+      </c>
+      <c r="E2068" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2068" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cqj1xvy44xno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】加快高水平科技自立自强 奋进科技强国建设</t>
+        </is>
+      </c>
+      <c r="D2069" t="inlineStr">
+        <is>
+          <t>我国加快科技自立自强，研发投入稳居世界第二，正向科技强国目标迈进。</t>
+        </is>
+      </c>
+      <c r="E2069" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2069" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDE9EMg8pMiMvPHj6kKZI5V260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>科技, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>[视频]联播快讯</t>
+        </is>
+      </c>
+      <c r="D2070" t="inlineStr">
+        <is>
+          <t>2026世界人工智能大会将举办；中国6月仓储指数回升；云端招聘月提供超20万岗位；伊朗回应美威胁。</t>
+        </is>
+      </c>
+      <c r="E2070" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2070" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEQsOlh7SAnHqGPhOiefY6260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>Two tests set to speed up diagnosis of endometriosis</t>
+        </is>
+      </c>
+      <c r="D2071" t="inlineStr">
+        <is>
+          <t>两项检测有望加速诊断子宫内膜异位症，缩短九年等待期。</t>
+        </is>
+      </c>
+      <c r="E2071" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2071" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyy8jdn3eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>军事, 社会</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>[视频]纪念全民族抗战爆发89周年仪式在京举行</t>
+        </is>
+      </c>
+      <c r="D2072" t="inlineStr">
+        <is>
+          <t>纪念全民族抗战爆发89周年仪式在京举行，各界代表敬献花束缅怀先烈。</t>
+        </is>
+      </c>
+      <c r="E2072" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2072" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDETwbRZvfopLMSp2gdxhjM260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>军事, 社会</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>[视频]各地举行活动纪念全民族抗战爆发89周年</t>
+        </is>
+      </c>
+      <c r="D2073" t="inlineStr">
+        <is>
+          <t>全国各地及部队举行活动纪念抗战爆发89周年，警示勿忘国耻、传承精神。</t>
+        </is>
+      </c>
+      <c r="E2073" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2073" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEadiRGyPiWDZLtLat5QWI260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>Zelensky presses Nato for air defence systems after intense Russian strikes</t>
+        </is>
+      </c>
+      <c r="D2074" t="inlineStr">
+        <is>
+          <t>泽连斯基在俄密集空袭后敦促北约在土耳其峰会提供防空系统。</t>
+        </is>
+      </c>
+      <c r="E2074" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2074" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9d227e5zj6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>Ukraine to press NATO for anti-ballistic air defense after latest Russian attacks</t>
+        </is>
+      </c>
+      <c r="D2075" t="inlineStr">
+        <is>
+          <t>乌克兰敦促北约提供反弹道防空系统，此前俄军袭击致20余人死亡。</t>
+        </is>
+      </c>
+      <c r="E2075" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2075" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5883932/ukraine-to-press-nato-for-anti-ballistic-air-defense-after-latest-russian-attacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>China test-launches a ballistic missile in the South Pacific and raises regional concerns</t>
+        </is>
+      </c>
+      <c r="D2076" t="inlineStr">
+        <is>
+          <t>中国在南太平洋试射弹道导弹，引发地区关注。</t>
+        </is>
+      </c>
+      <c r="E2076" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2076" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5884537/china-ballistic-missile-south-pacific</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>[视频]中央组织部从代中央管理党费中划拨6000万元 用于支持广西、甘肃等5省区防汛救灾工作</t>
+        </is>
+      </c>
+      <c r="D2077" t="inlineStr">
+        <is>
+          <t>中组部从党费中划拨6000万元，支持广西、甘肃等5省区防汛救灾工作。</t>
+        </is>
+      </c>
+      <c r="E2077" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2077" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEIuA4jTISPE0JHuYujcv4260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>[视频]极端天气影响我国多地 各方全力组织抢险救援</t>
+        </is>
+      </c>
+      <c r="D2078" t="inlineStr">
+        <is>
+          <t>极端天气致广西、湖北等地受灾，各方全力抢险救援、安置群众。</t>
+        </is>
+      </c>
+      <c r="E2078" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2078" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEQpVM4g5s19KULgyMvyri260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>Woman suspected of Monaco bomb attack found dead in Ukraine</t>
+        </is>
+      </c>
+      <c r="D2079" t="inlineStr">
+        <is>
+          <t>涉嫌摩纳哥炸弹袭击的乌克兰女子在乌克兰被发现死亡。</t>
+        </is>
+      </c>
+      <c r="E2079" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2079" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz3770yg8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>Explosions injure 18 in Damascus during Macron's visit</t>
+        </is>
+      </c>
+      <c r="D2080" t="inlineStr">
+        <is>
+          <t>大马士革发生爆炸，18人受伤，时值法国总统马克龙访问叙利亚。</t>
+        </is>
+      </c>
+      <c r="E2080" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2080" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2eylx1jj9ko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>国际, 政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>Why some African nations are turning down Trump aid money</t>
+        </is>
+      </c>
+      <c r="D2081" t="inlineStr">
+        <is>
+          <t>部分非洲国家拒绝特朗普援助，认为交易不公。</t>
+        </is>
+      </c>
+      <c r="E2081" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2081" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ckg0921y8kdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>Trump's NATO pressure campaign continues as summit begins</t>
+        </is>
+      </c>
+      <c r="D2082" t="inlineStr">
+        <is>
+          <t>特朗普抵达安卡拉出席北约峰会，或再次施加压力。</t>
+        </is>
+      </c>
+      <c r="E2082" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2082" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5884055/trumps-nato-pressure-campaign-continues-as-summit-begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>Explosions rock Damascus, wounding 18, as French President Macron visits Syria</t>
+        </is>
+      </c>
+      <c r="D2083" t="inlineStr">
+        <is>
+          <t>大马士革发生爆炸致18人伤，马克龙访叙行程未受影响。</t>
+        </is>
+      </c>
+      <c r="E2083" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2083" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5884579/damascus-explosions-macron</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>NATO summit set to begin in Turkey</t>
+        </is>
+      </c>
+      <c r="D2084" t="inlineStr">
+        <is>
+          <t>北约峰会前夕，欧洲意识到无法安抚特朗普，被迫加强自身防务。</t>
+        </is>
+      </c>
+      <c r="E2084" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2084" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5879166/nato-summit-set-to-begin-in-turkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>Former U.S. ambassador on Turkey hosting the NATO summit</t>
+        </is>
+      </c>
+      <c r="D2085" t="inlineStr">
+        <is>
+          <t>前美驻土大使就土耳其主办北约峰会发表评论。</t>
+        </is>
+      </c>
+      <c r="E2085" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2085" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/nx-s1-5883847/former-u-s-ambassador-on-turkey-hosting-the-nato-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>2 ships are hit in the latest attacks in the Strait of Hormuz, the U.K. military says</t>
+        </is>
+      </c>
+      <c r="D2086" t="inlineStr">
+        <is>
+          <t>霍尔木兹海峡两船遭袭，伊朗称其一船无视警告。</t>
+        </is>
+      </c>
+      <c r="E2086" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2086" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/07/g-s1-132265/tanker-attack-strait-of-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>[视频]二十四节气·小暑</t>
+        </is>
+      </c>
+      <c r="D2087" t="inlineStr">
+        <is>
+          <t>二十四节气小暑到来，天气炎热但未至极，万物生长，心静自然凉。</t>
+        </is>
+      </c>
+      <c r="E2087" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2087" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/07/VIDEga6WNoAHYjjGBszcRULs260707.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>Watch: Moment rare tornado lashes central Chinese cities</t>
+        </is>
+      </c>
+      <c r="D2088" t="inlineStr">
+        <is>
+          <t>罕见龙卷风袭击中国中部城市，碎片飞散，视频记录现场。</t>
+        </is>
+      </c>
+      <c r="E2088" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2088" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/cq61d22ved2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>Zimbabwean football star survives gun attack in South Africa</t>
+        </is>
+      </c>
+      <c r="D2089" t="inlineStr">
+        <is>
+          <t>津巴布韦足球明星在南非遭枪击，警方调查未逮捕任何人。</t>
+        </is>
+      </c>
+      <c r="E2089" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2089" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1my1rvy28do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>Erika Kirk comes face-to-face in court with husband's alleged killer</t>
+        </is>
+      </c>
+      <c r="D2090" t="inlineStr">
+        <is>
+          <t>埃里卡·柯克在法庭上与涉嫌杀害其丈夫的凶手对峙。</t>
+        </is>
+      </c>
+      <c r="E2090" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2090" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1myyyyjvx5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>India's landmark Ram temple overhauls board after alleged theft of donations</t>
+        </is>
+      </c>
+      <c r="D2091" t="inlineStr">
+        <is>
+          <t>印度罗摩庙董事会重组，因涉嫌信众捐赠现金珠宝被盗。</t>
+        </is>
+      </c>
+      <c r="E2091" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2091" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c872ngz405xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>Murder inquiry after mother and children found dead</t>
+        </is>
+      </c>
+      <c r="D2092" t="inlineStr">
+        <is>
+          <t>警方称一名母亲及其两名儿童被发现死于一处房产内。</t>
+        </is>
+      </c>
+      <c r="E2092" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2092" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgdlnvg2n5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr">
+        <is>
+          <t>Salah v Messi: A World Cup meeting of two national icons</t>
+        </is>
+      </c>
+      <c r="D2093" t="inlineStr">
+        <is>
+          <t>萨拉赫与梅西将在世界杯16强赛相遇，两国希望寄托于他们。</t>
+        </is>
+      </c>
+      <c r="E2093" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2093" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cvg55yl9xj4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr">
+        <is>
+          <t>9.1m people stay up to watch England's epic win over Mexico</t>
+        </is>
+      </c>
+      <c r="D2094" t="inlineStr">
+        <is>
+          <t>910万人熬夜观看英格兰队战胜墨西哥队，挺进世界杯八强。</t>
+        </is>
+      </c>
+      <c r="E2094" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2094" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cdejw7xxe23o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-08
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2094"/>
+  <dimension ref="A1:F2133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67445,6 +67445,1254 @@
         </is>
       </c>
     </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260708 19:00</t>
+        </is>
+      </c>
+      <c r="D2095" t="inlineStr">
+        <is>
+          <t>国家科技奖励大会召开，习近平强调推进科技强国建设；铁路货运增长，防汛救灾进行。</t>
+        </is>
+      </c>
+      <c r="E2095" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2095" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEIMD5INrAduYCdx9htTM0260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr">
+        <is>
+          <t>[视频]国家科学技术奖励大会 两院院士大会 中国科协第十一次全国代表大会在京召开 习近平发表重要讲话</t>
+        </is>
+      </c>
+      <c r="D2096" t="inlineStr">
+        <is>
+          <t>习近平在科技奖励大会上强调抓住攻坚期，加快推进高水平科技自立自强。</t>
+        </is>
+      </c>
+      <c r="E2096" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2096" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEI0jBPpoIt78qeAzG3QE6260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr">
+        <is>
+          <t>[视频]《习近平关于基层工作方法的重要论述学习读本》出版发行</t>
+        </is>
+      </c>
+      <c r="D2097" t="inlineStr">
+        <is>
+          <t>《习近平关于基层工作方法的重要论述学习读本》出版发行。</t>
+        </is>
+      </c>
+      <c r="E2097" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2097" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDE4CST2kkIGsn7XVwrSORK260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr">
+        <is>
+          <t>[视频]中国科协第十一次全国代表大会举行第二次全体会议 蔡奇到会祝贺并代表党中央致词</t>
+        </is>
+      </c>
+      <c r="D2098" t="inlineStr">
+        <is>
+          <t>蔡奇在科协代表大会致词，号召科技工作者助力科技强国建设。</t>
+        </is>
+      </c>
+      <c r="E2098" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2098" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDECaH4oRtT3DtJTaVOi8k5260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>政治, 科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“新征程上的奋斗者”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D2099" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行中外记者见面会，五位工信领域基层代表分享奋斗故事。</t>
+        </is>
+      </c>
+      <c r="E2099" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2099" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEiNJDwPpzbmfSzvADcR5Y260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr">
+        <is>
+          <t>Nigeria's president demands to know how fake agency was allegedly set up in his office</t>
+        </is>
+      </c>
+      <c r="D2100" t="inlineStr">
+        <is>
+          <t>尼日利亚总统要求查明其办公室内疑似设立虚假机构案件。</t>
+        </is>
+      </c>
+      <c r="E2100" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2100" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621xrrp6jeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr">
+        <is>
+          <t>Chris Mason: It's far from certain whether by-election will strengthen Farage</t>
+        </is>
+      </c>
+      <c r="D2101" t="inlineStr">
+        <is>
+          <t>改革英国党领袖法拉奇面临伯爵垃圾桶挑战，主要政党放弃参选。</t>
+        </is>
+      </c>
+      <c r="E2101" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2101" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9d2882jj3yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr">
+        <is>
+          <t>Le Pen says she'll run for French presidency next year despite court-ordered monitor</t>
+        </is>
+      </c>
+      <c r="D2102" t="inlineStr">
+        <is>
+          <t>法国极右翼领袖勒庞宣布参选总统，尽管因贪污被判佩戴电子监控。</t>
+        </is>
+      </c>
+      <c r="E2102" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2102" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/g-s1-132467/le-pen-court-ordered-monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr">
+        <is>
+          <t>[视频]今年上半年铁路货运量稳步增长 服务全国统一大市场</t>
+        </is>
+      </c>
+      <c r="D2103" t="inlineStr">
+        <is>
+          <t>上半年铁路货运量稳步增长，多式联运和中欧班列表现突出。</t>
+        </is>
+      </c>
+      <c r="E2103" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2103" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEkY8vjXY2HkZ3XbFbrmmC260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr">
+        <is>
+          <t>TV licence fee is 'yesterday's model', new BBC director general says</t>
+        </is>
+      </c>
+      <c r="D2104" t="inlineStr">
+        <is>
+          <t>新任BBC总监称电视许可费模式过时。</t>
+        </is>
+      </c>
+      <c r="E2104" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2104" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20yjjm7n87o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：扎扎实实以科技创新支撑和引领中国式现代化</t>
+        </is>
+      </c>
+      <c r="D2105" t="inlineStr">
+        <is>
+          <t>央视快评强调以科技创新支撑和引领中国式现代化。</t>
+        </is>
+      </c>
+      <c r="E2105" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2105" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDE8A95mtxTd0YizhJvxDc0260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥接见国际科技合作奖获奖外国专家</t>
+        </is>
+      </c>
+      <c r="D2106" t="inlineStr">
+        <is>
+          <t>丁薛祥接见国际科技合作奖获奖外国专家，颁发奖章。</t>
+        </is>
+      </c>
+      <c r="E2106" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2106" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEx7IUKKQrAx6DoDC56twy260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr">
+        <is>
+          <t>Trains and emergency calls affected after major outage at Australia's largest telecoms company</t>
+        </is>
+      </c>
+      <c r="D2107" t="inlineStr">
+        <is>
+          <t>澳洲最大电信公司故障致火车延误及紧急呼叫受影响，原因待查。</t>
+        </is>
+      </c>
+      <c r="E2107" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2107" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgevw0d95pdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr">
+        <is>
+          <t>Outcry as Meta lets users make AI images from public Instagram profile pics</t>
+        </is>
+      </c>
+      <c r="D2108" t="inlineStr">
+        <is>
+          <t>Meta允许用户用公开Instagram头像生成AI图像，引发隐私抗议。</t>
+        </is>
+      </c>
+      <c r="E2108" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2108" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp9lee19y1yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr">
+        <is>
+          <t>Nato allies announce £37bn for new missile project</t>
+        </is>
+      </c>
+      <c r="D2109" t="inlineStr">
+        <is>
+          <t>北约盟国宣布370亿英镑新导弹项目，英首相将召集多国讨论。</t>
+        </is>
+      </c>
+      <c r="E2109" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2109" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ckg4e3lwzqzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr">
+        <is>
+          <t>[视频]桂鄂甘等地防汛救灾工作加紧进行</t>
+        </is>
+      </c>
+      <c r="D2110" t="inlineStr">
+        <is>
+          <t>广西、湖北、甘肃等地加紧防汛救灾，转移安置群众。</t>
+        </is>
+      </c>
+      <c r="E2110" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2110" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEF7APsI5hniQMvtpoMUHw260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】党员民警冲锋在前 全力救援被困群众</t>
+        </is>
+      </c>
+      <c r="D2111" t="inlineStr">
+        <is>
+          <t>广西台风强降雨致灾，党员民警冲锋在前，成功救援被困群众。</t>
+        </is>
+      </c>
+      <c r="E2111" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2111" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEgX66gncwSmJWrEJRZdQ2260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr">
+        <is>
+          <t>Ofsted promises to penalise councils using illegal children's homes</t>
+        </is>
+      </c>
+      <c r="D2112" t="inlineStr">
+        <is>
+          <t>英国教育标准局承诺处罚使用非法儿童寄宿场所的议会。</t>
+        </is>
+      </c>
+      <c r="E2112" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2112" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ced4j357jd9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr">
+        <is>
+          <t>More protein or less? The foods to get you through a heatwave</t>
+        </is>
+      </c>
+      <c r="D2113" t="inlineStr">
+        <is>
+          <t>推荐热浪期间取代烤箱和沙拉的高蛋白饮食。</t>
+        </is>
+      </c>
+      <c r="E2113" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2113" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyw89g3443o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr">
+        <is>
+          <t>[视频]美伊再度相互打击对方目标 美国恢复对伊朗石油制裁</t>
+        </is>
+      </c>
+      <c r="D2114" t="inlineStr">
+        <is>
+          <t>美伊相互打击对方目标，美国恢复对伊石油制裁，伊朗称不屈服。</t>
+        </is>
+      </c>
+      <c r="E2114" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2114" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEzYNeBZWuWv90dJeVJIR2260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr">
+        <is>
+          <t>[视频]国际奥委会暂时恢复俄奥委会会员资格</t>
+        </is>
+      </c>
+      <c r="D2115" t="inlineStr">
+        <is>
+          <t>国际奥委会暂时恢复俄奥委会会员资格，为俄运动员回归赛场扫清障碍。</t>
+        </is>
+      </c>
+      <c r="E2115" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2115" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/08/VIDEXggo7gG0F8dV3oeluVQC260708.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr">
+        <is>
+          <t>Trump says ceasefire is 'over' after US and Iran trade strikes</t>
+        </is>
+      </c>
+      <c r="D2116" t="inlineStr">
+        <is>
+          <t>特朗普称美伊停火已结束，但美方仍愿与伊朗继续谈判。</t>
+        </is>
+      </c>
+      <c r="E2116" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2116" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyw8w1g409o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr">
+        <is>
+          <t>US strikes target Iranian military boats</t>
+        </is>
+      </c>
+      <c r="D2117" t="inlineStr">
+        <is>
+          <t>美方打击伊朗快艇，报复其对霍尔木兹海峡油轮的袭击。</t>
+        </is>
+      </c>
+      <c r="E2117" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2117" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/cn94nqzwpxwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr">
+        <is>
+          <t>Will Le Pen rise again? French nationalist leader defiant after court's ruling</t>
+        </is>
+      </c>
+      <c r="D2118" t="inlineStr">
+        <is>
+          <t>法国民粹领袖勒庞上诉失败后，数小时内即宣布启动总统竞选。</t>
+        </is>
+      </c>
+      <c r="E2118" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2118" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgdlprp1r3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr">
+        <is>
+          <t>Eight killed after landslide hits girls' school in Bangladesh</t>
+        </is>
+      </c>
+      <c r="D2119" t="inlineStr">
+        <is>
+          <t>孟加拉国山体滑坡致女子学校8人死亡，救援工作持续。</t>
+        </is>
+      </c>
+      <c r="E2119" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2119" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2wkzww20ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr">
+        <is>
+          <t>Khamenei's coffin carried through Shia shrines as ceremonies held in Iraq</t>
+        </is>
+      </c>
+      <c r="D2120" t="inlineStr">
+        <is>
+          <t>伊朗已故最高领袖哈梅内伊棺椁被抬至伊拉克圣陵，葬礼第五日。</t>
+        </is>
+      </c>
+      <c r="E2120" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2120" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp9le3kjj8eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>国际, 政治, 文体</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr">
+        <is>
+          <t>Trump says he believes the Iran ceasefire is 'over.' And, IOC lifts Russia's suspension</t>
+        </is>
+      </c>
+      <c r="D2121" t="inlineStr">
+        <is>
+          <t>特朗普称美伊停火已结束；国际奥委会为俄运动员参加2028年奥运会铺路。</t>
+        </is>
+      </c>
+      <c r="E2121" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2121" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/g-s1-132474/up-first-newsletter-trump-iran-ceasefire-nato-graham-platner-ioc-russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr">
+        <is>
+          <t>At NATO summit in Turkey, Trump says he believes ceasefire with Iran is 'over'</t>
+        </is>
+      </c>
+      <c r="D2122" t="inlineStr">
+        <is>
+          <t>特朗普在北约峰会上称美伊停火已结束，双方近期冲突加剧紧张局势。</t>
+        </is>
+      </c>
+      <c r="E2122" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2122" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/nx-s1-5883929/trump-nato-iran-strikes-press-conference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr">
+        <is>
+          <t>Trump says ceasefire between the U.S. and Iran is over</t>
+        </is>
+      </c>
+      <c r="D2123" t="inlineStr">
+        <is>
+          <t>特朗普在土耳其宣布美伊停火结束，但未排除继续谈判的可能性。</t>
+        </is>
+      </c>
+      <c r="E2123" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2123" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/nx-s1-5884779/trump-says-ceasefire-between-the-u-s-and-iran-is-over</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr">
+        <is>
+          <t>The state of the NATO alliance amid Trump's second term</t>
+        </is>
+      </c>
+      <c r="D2124" t="inlineStr">
+        <is>
+          <t>专家分析特朗普第二任期北约峰会情况及联盟现状。</t>
+        </is>
+      </c>
+      <c r="E2124" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2124" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/nx-s1-5884818/the-state-of-the-nato-alliance-amid-trumps-second-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr">
+        <is>
+          <t>Tehran targets Bahrain and Kuwait after U.S. strikes</t>
+        </is>
+      </c>
+      <c r="D2125" t="inlineStr">
+        <is>
+          <t>德黑兰针对巴林和科威特采取行动，中东停火协议面临破裂风险。</t>
+        </is>
+      </c>
+      <c r="E2125" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2125" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/g-s1-132460/us-iran-attacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr">
+        <is>
+          <t>German doctor jailed for murder of 15 patients and suspected of more</t>
+        </is>
+      </c>
+      <c r="D2126" t="inlineStr">
+        <is>
+          <t>德国一名姑息治疗医生因杀害15名患者被判终身监禁。</t>
+        </is>
+      </c>
+      <c r="E2126" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2126" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cq819jyp2g7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr">
+        <is>
+          <t>Teenager arrested after two girls, 13, seriously injured in German school attack</t>
+        </is>
+      </c>
+      <c r="D2127" t="inlineStr">
+        <is>
+          <t>德国一名青少年被捕，涉嫌在学校袭击致两名13岁女孩重伤。</t>
+        </is>
+      </c>
+      <c r="E2127" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2127" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0qyvkgndzpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr">
+        <is>
+          <t>Ruth Ellis, last woman to be hanged in UK, gets conditional posthumous pardon</t>
+        </is>
+      </c>
+      <c r="D2128" t="inlineStr">
+        <is>
+          <t>英国最后一名被绞死女性露丝·埃利斯获有条件的死后赦免。</t>
+        </is>
+      </c>
+      <c r="E2128" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2128" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crel4rj801do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr">
+        <is>
+          <t>Police name man wanted over murders of wife and daughters</t>
+        </is>
+      </c>
+      <c r="D2129" t="inlineStr">
+        <is>
+          <t>警方通缉谋杀妻子和女儿的男子，其已通过希思罗机场离境。</t>
+        </is>
+      </c>
+      <c r="E2129" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2129" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8e2njxnn7jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr">
+        <is>
+          <t>Neo-Nazi who planned gun attack jailed after MI5 sting</t>
+        </is>
+      </c>
+      <c r="D2130" t="inlineStr">
+        <is>
+          <t>22岁新纳粹分子阿尔菲·科尔曼因策划枪击案被判刑。</t>
+        </is>
+      </c>
+      <c r="E2130" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2130" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c39yex3v1ryo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr">
+        <is>
+          <t>Greetings from a Syrian church, infused with a mix of sweet fruit and diverse faiths</t>
+        </is>
+      </c>
+      <c r="D2131" t="inlineStr">
+        <is>
+          <t>叙利亚马穆萨修道院提供美味桑葚，其礼拜融合东正教和苏菲派习俗。</t>
+        </is>
+      </c>
+      <c r="E2131" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2131" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/08/nx-s1-5884694/syria-church-interfaith-fruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr">
+        <is>
+          <t>Multiple cakes and stolen keepsakes: Greg James spills the tea on Taylor Swift's wedding</t>
+        </is>
+      </c>
+      <c r="D2132" t="inlineStr">
+        <is>
+          <t>DJ格雷格·詹姆斯在节目中爆料泰勒·斯威夫特婚礼细节。</t>
+        </is>
+      </c>
+      <c r="E2132" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2132" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2kd1de8l5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>体育</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr">
+        <is>
+          <t>Egypt want officials kicked out of World Cup</t>
+        </is>
+      </c>
+      <c r="D2133" t="inlineStr">
+        <is>
+          <t>埃及足协投诉国际足联，要求调查阿根廷比赛判罚双标。</t>
+        </is>
+      </c>
+      <c r="E2133" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2133" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c5yzdd070r3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-09
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2133"/>
+  <dimension ref="A1:F2171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68693,6 +68693,1222 @@
         </is>
       </c>
     </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>政治, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260709 19:00</t>
+        </is>
+      </c>
+      <c r="D2134" t="inlineStr">
+        <is>
+          <t>习近平就鞋厂火灾作指示，强调安全生产；科技大会反响热烈；李强会见纳米比亚总统；国务院印发碳达峰方案等。</t>
+        </is>
+      </c>
+      <c r="E2134" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2134" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEzrouN6SjvEnQmqtBYPCz260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr">
+        <is>
+          <t>[视频]习近平对福建泉州晋江市一鞋厂火灾事故作出重要指示强调 深入排查整治各类风险隐患 抓实抓细安全生产措施落实 坚决防止重特大事故发生 李强作出批示</t>
+        </is>
+      </c>
+      <c r="D2135" t="inlineStr">
+        <is>
+          <t>习近平对福建鞋厂火灾作指示，要求深入排查隐患，坚决防止重特大事故，李强作批示。</t>
+        </is>
+      </c>
+      <c r="E2135" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2135" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEPmCg01y1kcYLhzjBEe7b260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr">
+        <is>
+          <t>[视频]李强会见纳米比亚总统</t>
+        </is>
+      </c>
+      <c r="D2136" t="inlineStr">
+        <is>
+          <t>李强会见纳米比亚总统，深化贸易、基建、矿业等领域合作，推动多边主义。</t>
+        </is>
+      </c>
+      <c r="E2136" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2136" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE10XtMKmKQzTIy8NZHiem260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr">
+        <is>
+          <t>[视频]“习近平新时代中国特色社会主义思想与世界”国际研讨会在银川举行</t>
+        </is>
+      </c>
+      <c r="D2137" t="inlineStr">
+        <is>
+          <t>习近平新时代中国特色社会主义思想国际研讨会银川举行，50多国代表聚焦中国减贫经验。</t>
+        </is>
+      </c>
+      <c r="E2137" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2137" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE2gzTlsZQkuicg4Q2PXt4260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr">
+        <is>
+          <t>Democrat Graham Platner suspends campaign for key US Senate race after assault allegation</t>
+        </is>
+      </c>
+      <c r="D2138" t="inlineStr">
+        <is>
+          <t>美民主党候选人普拉特纳因性侵指控暂停参议员竞选，其否认指控。</t>
+        </is>
+      </c>
+      <c r="E2138" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2138" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9v229434p2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr">
+        <is>
+          <t>Platner's disastrous candidacy exposes rifts that could dampen Democrats' Senate hopes</t>
+        </is>
+      </c>
+      <c r="D2139" t="inlineStr">
+        <is>
+          <t>普拉特纳灾难性竞选暴露党内裂痕，可能削弱民主党参议院希望。</t>
+        </is>
+      </c>
+      <c r="E2139" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2139" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20ylnn8wqgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr">
+        <is>
+          <t>Restore Britain leader describes Dunblane school shooting as 'one murder'</t>
+        </is>
+      </c>
+      <c r="D2140" t="inlineStr">
+        <is>
+          <t>重建英国领导人将邓布兰校园枪击案称为“一起谋杀”。</t>
+        </is>
+      </c>
+      <c r="E2140" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2140" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj3gdj300lyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr">
+        <is>
+          <t>Burnham on path to No 10 with Labour nominations under way</t>
+        </is>
+      </c>
+      <c r="D2141" t="inlineStr">
+        <is>
+          <t>伯纳姆在工党提名中无对手，有望接替斯塔默任首相。</t>
+        </is>
+      </c>
+      <c r="E2141" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2141" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c77y0n7k801o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr">
+        <is>
+          <t>Graham Platner ends Senate bid. And, why Nolan Wells' death captured national attention</t>
+        </is>
+      </c>
+      <c r="D2142" t="inlineStr">
+        <is>
+          <t>民主党人普拉特纳退出参院竞选；民权律师介入诺兰·威尔斯死亡案。</t>
+        </is>
+      </c>
+      <c r="E2142" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2142" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/09/g-s1-132694/up-first-newsletter-graham-platner-trump-iran-israel-nolan-wells</t>
+        </is>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr">
+        <is>
+          <t>How England's class divide shaped Andy Burnham, the U.K.'s likely next prime minister</t>
+        </is>
+      </c>
+      <c r="D2143" t="inlineStr">
+        <is>
+          <t>曼彻斯特市长伯纳姆可能成为英国下一任首相，其阶级背景引人关注。</t>
+        </is>
+      </c>
+      <c r="E2143" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2143" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/09/nx-s1-5876065/andy-burnham-england-uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>政治, 国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr">
+        <is>
+          <t>Trump wraps NATO summit on a positive note,  after meeting Zelenskyy</t>
+        </is>
+      </c>
+      <c r="D2144" t="inlineStr">
+        <is>
+          <t>特朗普在北约峰会会见泽连斯基，称将授权乌克兰生产爱国者系统。</t>
+        </is>
+      </c>
+      <c r="E2144" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/09/nx-s1-5887053/trump-nato-zelenskyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《“十五五”碳达峰行动方案》</t>
+        </is>
+      </c>
+      <c r="D2145" t="inlineStr">
+        <is>
+          <t>国务院印发“十五五”碳达峰行动方案，部署能源结构调整和绿色低碳转型。</t>
+        </is>
+      </c>
+      <c r="E2145" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2145" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEU5Awq5ePUzHAkqtgNheC260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr">
+        <is>
+          <t>[视频]上半年物价运行总体平稳</t>
+        </is>
+      </c>
+      <c r="D2146" t="inlineStr">
+        <is>
+          <t>上半年CPI同比上涨1.0%，PPI同比上涨1.5%，物价运行总体平稳。</t>
+        </is>
+      </c>
+      <c r="E2146" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2146" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE8K9fJHURBNbKcLEKKLKR260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr">
+        <is>
+          <t>[视频]上半年新能源汽车产销量双超700万辆</t>
+        </is>
+      </c>
+      <c r="D2147" t="inlineStr">
+        <is>
+          <t>上半年新能源汽车产销量均超740万辆，出口同比增长120%。</t>
+        </is>
+      </c>
+      <c r="E2147" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2147" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEsxQaG5eVXwHbFjrQjpwR260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr">
+        <is>
+          <t>[视频]2026年亚太经合组织工商咨询理事会第三次会议举行</t>
+        </is>
+      </c>
+      <c r="D2148" t="inlineStr">
+        <is>
+          <t>亚太经合组织工商咨询理事会第三次会议曼谷举行，聚焦区域经济一体化与数字创新。</t>
+        </is>
+      </c>
+      <c r="E2148" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2148" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE9P08pVo4W7zyDrzSpyw9260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>经济, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2149" t="inlineStr">
+        <is>
+          <t>IMF上调中国经济增长预期至4.6%；俄乌互称打击对方目标；欧洲反对美国控制格陵兰岛言论。</t>
+        </is>
+      </c>
+      <c r="E2149" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2149" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEU1dg28Umnd6tLHwyQzpe260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr">
+        <is>
+          <t>Big fall in Strait of Hormuz tanker and cargo ship sailings after new strikes</t>
+        </is>
+      </c>
+      <c r="D2150" t="inlineStr">
+        <is>
+          <t>新打击后，霍尔木兹海峡油轮和货船航行量大幅下降。</t>
+        </is>
+      </c>
+      <c r="E2150" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2150" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621k5r8764o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr">
+        <is>
+          <t>[视频]勇攀世界科学高峰 为建设科技强国多立新功——习近平总书记在国家科学技术奖励大会 两院院士大会 中国科协第十一次全国代表大会上的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2151" t="inlineStr">
+        <is>
+          <t>习近平总书记科技大会讲话引发热烈反响，强调科技强国建设，推动高水平科技自立自强。</t>
+        </is>
+      </c>
+      <c r="E2151" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2151" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEBIvEjAM7SGb1bvEgSpd0260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：扎扎实实以科技创新支撑和引领中国式现代化——论学习贯彻习近平总书记在国家科学技术奖励大会、两院院士大会、中国科协十一大上重要讲话</t>
+        </is>
+      </c>
+      <c r="D2152" t="inlineStr">
+        <is>
+          <t>人民日报发表评论员文章，论以科技创新支撑和引领中国式现代化。</t>
+        </is>
+      </c>
+      <c r="E2152" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2152" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE2cazWtseCnEn7BgFWOXl260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>科技, 政治</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr">
+        <is>
+          <t>[视频]丁薛祥在两院院士大会第二次全体会议上强调 全力抓好党中央关于科技事业各项部署的落实 加快推进高水平科技自立自强</t>
+        </is>
+      </c>
+      <c r="D2153" t="inlineStr">
+        <is>
+          <t>丁薛祥在两院院士大会上强调落实科技部署，加快推进高水平科技自立自强。</t>
+        </is>
+      </c>
+      <c r="E2153" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2153" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEwg9SAzZfZrPLvOzyy72M260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr">
+        <is>
+          <t>[视频]日内瓦“全球治理之友小组”举办人工智能向善普惠发展研讨会</t>
+        </is>
+      </c>
+      <c r="D2154" t="inlineStr">
+        <is>
+          <t>日内瓦举办人工智能向善普惠发展研讨会，中国呼吁加强全球治理协作。</t>
+        </is>
+      </c>
+      <c r="E2154" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2154" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEeksBXCSs5ygDYkxSh8gE260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr">
+        <is>
+          <t>[视频]美军连续两天对伊朗发动军事打击 伊朗称袭击多处美军基地</t>
+        </is>
+      </c>
+      <c r="D2155" t="inlineStr">
+        <is>
+          <t>美军连续两天打击伊朗约90个军事目标，伊朗袭击美军基地报复，国际社会呼吁降级。</t>
+        </is>
+      </c>
+      <c r="E2155" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2155" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDE37B3FNnG0pQEls79Ck4Z260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr">
+        <is>
+          <t>Tehran launches more strikes after explosions reported in southern Iran</t>
+        </is>
+      </c>
+      <c r="D2156" t="inlineStr">
+        <is>
+          <t>美军称击中伊朗90个目标，伊朗卫生部称自周二以来14人死亡。</t>
+        </is>
+      </c>
+      <c r="E2156" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2156" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz75zjj5wp8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr">
+        <is>
+          <t>Ukraine strikes Russian ships near Crimea, escalating attacks on fuel supplies</t>
+        </is>
+      </c>
+      <c r="D2157" t="inlineStr">
+        <is>
+          <t>乌克兰打击克里米亚附近俄舰，升级对燃料供给的袭击。</t>
+        </is>
+      </c>
+      <c r="E2157" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2157" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c70yd1g67z5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr">
+        <is>
+          <t>The U.S. launches new airstrikes on Iran and Tehran fires back at Gulf Arab states</t>
+        </is>
+      </c>
+      <c r="D2158" t="inlineStr">
+        <is>
+          <t>美国对伊朗发动新空袭，伊朗报复攻击美盟友，战争风险加剧。</t>
+        </is>
+      </c>
+      <c r="E2158" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2158" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/09/g-s1-132670/us-iran-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr">
+        <is>
+          <t>[视频]中共中央办公厅、国务院办公厅印发《关于全力做好防汛抗旱工作的通知》</t>
+        </is>
+      </c>
+      <c r="D2159" t="inlineStr">
+        <is>
+          <t>中办国办印发通知，要求全力做好防汛抗旱工作，全面压实责任确保安全。</t>
+        </is>
+      </c>
+      <c r="E2159" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2159" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDESSk1ZRhnn5M6NZ0jssIR260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2160" t="inlineStr">
+        <is>
+          <t>我国将加大医疗数据安全供给，2030年形成现代零售体系，三级养老网络2029年建成。</t>
+        </is>
+      </c>
+      <c r="E2160" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2160" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEx10Mzt1juGBJvMuxI8av260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr">
+        <is>
+          <t>More buildings to receive dangerous cladding removal funding</t>
+        </is>
+      </c>
+      <c r="D2161" t="inlineStr">
+        <is>
+          <t>更多建筑将获得危险覆层拆除资金，此前低于35英尺的房产无此资格。</t>
+        </is>
+      </c>
+      <c r="E2161" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2161" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yz54xk12qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr">
+        <is>
+          <t>How can I get air conditioning in my home and how much does it cost?</t>
+        </is>
+      </c>
+      <c r="D2162" t="inlineStr">
+        <is>
+          <t>英国夏季变热，家用空调是否该普及成为讨论焦点。</t>
+        </is>
+      </c>
+      <c r="E2162" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2162" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2ey1p0jnmxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr">
+        <is>
+          <t>International court tells BBC of breakthrough in Sudan war crimes probe</t>
+        </is>
+      </c>
+      <c r="D2163" t="inlineStr">
+        <is>
+          <t>国际刑事法院告知BBC在苏丹战争罪行调查中取得突破。</t>
+        </is>
+      </c>
+      <c r="E2163" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2163" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9928zr2m5xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr">
+        <is>
+          <t>No contact from UK about on-the-run murder suspect, say Zimbabwe police</t>
+        </is>
+      </c>
+      <c r="D2164" t="inlineStr">
+        <is>
+          <t>津巴布韦警方称未收到英国关于在逃谋杀嫌疑人的联系。</t>
+        </is>
+      </c>
+      <c r="E2164" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2164" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyr4l1p6d4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr">
+        <is>
+          <t>[视频]台风“巴威”逼近 相关地区部署防御</t>
+        </is>
+      </c>
+      <c r="D2165" t="inlineStr">
+        <is>
+          <t>超强台风“巴威”逼近，浙江福建等地启动防御，转移船舶和人员。</t>
+        </is>
+      </c>
+      <c r="E2165" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2165" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEfcEKdagBdfiIhp7D51LG260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】党员冲锋艇“孤岛救援”</t>
+        </is>
+      </c>
+      <c r="D2166" t="inlineStr">
+        <is>
+          <t>广西贵港内涝，党员冲锋艇救援1万多名被困师生，全部安全转移。</t>
+        </is>
+      </c>
+      <c r="E2166" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2166" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/09/VIDEJgPYPcUgUvWW1tZwSy77260709.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr">
+        <is>
+          <t>Factory fire kills at least 28 in China's 'shoe capital'</t>
+        </is>
+      </c>
+      <c r="D2167" t="inlineStr">
+        <is>
+          <t>中国“鞋都”一工厂火灾致至少28人死亡。</t>
+        </is>
+      </c>
+      <c r="E2167" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2167" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2vz51v2pjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr">
+        <is>
+          <t>Most popular baby names for boys and girls in 2025 revealed</t>
+        </is>
+      </c>
+      <c r="D2168" t="inlineStr">
+        <is>
+          <t>2025年最受欢迎婴儿名公布：奥莉维亚和穆罕默德居首。</t>
+        </is>
+      </c>
+      <c r="E2168" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2168" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cevlw4wnlmxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr">
+        <is>
+          <t>Prince Harry gets UK trip back on track with hospital visit</t>
+        </is>
+      </c>
+      <c r="D2169" t="inlineStr">
+        <is>
+          <t>哈里王子访问伯明翰儿童医院，修复英国之行。</t>
+        </is>
+      </c>
+      <c r="E2169" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2169" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czdezv3j7zeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr">
+        <is>
+          <t>'Heartbroken' Catherine Zeta-Jones leads tributes to singer Bonnie Tyler</t>
+        </is>
+      </c>
+      <c r="D2170" t="inlineStr">
+        <is>
+          <t>凯瑟琳·泽塔-琼斯心碎悼念歌手邦妮·泰勒。</t>
+        </is>
+      </c>
+      <c r="E2170" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2170" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clypqj2z1zpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr">
+        <is>
+          <t>Egypt complains officials were biased in World Cup loss to Argentina</t>
+        </is>
+      </c>
+      <c r="D2171" t="inlineStr">
+        <is>
+          <t>埃及足协投诉裁判不公，称世界杯输阿根廷因偏袒判罚。</t>
+        </is>
+      </c>
+      <c r="E2171" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2171" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/09/nx-s1-5887063/egypt-complain-world-cup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-10
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2171"/>
+  <dimension ref="A1:F2206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69909,6 +69909,1126 @@
         </is>
       </c>
     </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260710 21:00</t>
+        </is>
+      </c>
+      <c r="D2172" t="inlineStr">
+        <is>
+          <t>今日新闻联播报道习近平会见纳米比亚总统、朝鲜总理，夏粮丰收，长征十号乙完成海上回收等要闻。</t>
+        </is>
+      </c>
+      <c r="E2172" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2172" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEAimxyb2gLhA0q72AIcnm260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr">
+        <is>
+          <t>[视频]习近平举行仪式欢迎纳米比亚总统访华</t>
+        </is>
+      </c>
+      <c r="D2173" t="inlineStr">
+        <is>
+          <t>习近平在人民大会堂举行仪式，欢迎纳米比亚总统恩代特瓦访华。</t>
+        </is>
+      </c>
+      <c r="E2173" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2173" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEh0pnqsKX5lbpBtG23asg260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr">
+        <is>
+          <t>[视频]习近平同纳米比亚总统会谈</t>
+        </is>
+      </c>
+      <c r="D2174" t="inlineStr">
+        <is>
+          <t>习近平同纳米比亚总统会谈，两国关系提升为新时代中纳命运共同体。</t>
+        </is>
+      </c>
+      <c r="E2174" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2174" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEb5VYonBKTr1cEah8aQmX260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见朝鲜内阁总理</t>
+        </is>
+      </c>
+      <c r="D2175" t="inlineStr">
+        <is>
+          <t>习近平会见朝鲜内阁总理朴泰成，强调巩固中朝传统友好关系。</t>
+        </is>
+      </c>
+      <c r="E2175" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2175" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDECaJFkeEogTNcUE1hokJN260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：加快推进高水平科技自立自强——论学习贯彻习近平总书记在国家科学技术奖励大会、两院院士大会、中国科协十一大上重要讲话</t>
+        </is>
+      </c>
+      <c r="D2176" t="inlineStr">
+        <is>
+          <t>人民日报将发表评论员文章，论学习贯彻习近平总书记关于科技自立自强的重要讲话。</t>
+        </is>
+      </c>
+      <c r="E2176" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2176" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDE4Co1pNe8xuUYTUkhZqxY260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D2177" t="inlineStr">
+        <is>
+          <t>李强主持国务院常务会议，部署防汛抗洪救灾和数字中国建设工作。</t>
+        </is>
+      </c>
+      <c r="E2177" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2177" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDE0s9H0RN2Y3nHI1WCfkmQ260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际分别会见纳米比亚总统、朝鲜内阁总理</t>
+        </is>
+      </c>
+      <c r="D2178" t="inlineStr">
+        <is>
+          <t>赵乐际分别会见纳米比亚总统和朝鲜内阁总理，加强双边合作与立法机构交流。</t>
+        </is>
+      </c>
+      <c r="E2178" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2178" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEmknx6kmBb8hc0NqTStF5260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁出席建设现代化产业体系调研协商座谈会</t>
+        </is>
+      </c>
+      <c r="D2179" t="inlineStr">
+        <is>
+          <t>王沪宁出席建设现代化产业体系调研协商座谈会，强调高质量建言献策。</t>
+        </is>
+      </c>
+      <c r="E2179" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2179" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEDdhUfv2U2vviadsn7o3B260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr">
+        <is>
+          <t>[视频]中央层面整治形式主义为基层减负专项工作机制会议在京召开 蔡奇出席并讲话</t>
+        </is>
+      </c>
+      <c r="D2180" t="inlineStr">
+        <is>
+          <t>中央层面整治形式主义为基层减负专项工作机制会议在京召开，蔡奇出席并讲话。</t>
+        </is>
+      </c>
+      <c r="E2180" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2180" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEkEVkYKx5TDQKuPmEwkTd260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr">
+        <is>
+          <t>Met police investigating Reform over election donations - reports</t>
+        </is>
+      </c>
+      <c r="D2181" t="inlineStr">
+        <is>
+          <t>伦敦警察厅调查英国改革党选举捐款，涉及一名诈骗犯的母亲。</t>
+        </is>
+      </c>
+      <c r="E2181" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2181" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3eyq2np7qgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr">
+        <is>
+          <t>Count Binface: The intergalactic warrior who could upend Britain's strangest election</t>
+        </is>
+      </c>
+      <c r="D2182" t="inlineStr">
+        <is>
+          <t>垃圾桶伯爵挑战法拉奇，英国最奇特的选举或将因财务问题被颠覆。</t>
+        </is>
+      </c>
+      <c r="E2182" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2182" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/nx-s1-5887550/count-binface-the-intergalactic-warrior-who-could-upend-britains-strangest-election</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr">
+        <is>
+          <t>[视频]夏粮丰收 产量首次突破3000亿斤</t>
+        </is>
+      </c>
+      <c r="D2183" t="inlineStr">
+        <is>
+          <t>2026年我国夏粮产量首次突破3000亿斤，达3014.9亿斤，奠定全年粮食生产基础。</t>
+        </is>
+      </c>
+      <c r="E2183" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2183" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEBlrOygmyHBHnNWsdUyNq260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr">
+        <is>
+          <t>Chip giant SK Hynix raises $26.5bn in mega US share sale</t>
+        </is>
+      </c>
+      <c r="D2184" t="inlineStr">
+        <is>
+          <t>韩国芯片巨头SK海力士在美上市，募资265亿美元创纪录。</t>
+        </is>
+      </c>
+      <c r="E2184" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2184" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gym70r0y4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr">
+        <is>
+          <t>[视频]历史性突破 长征十号乙完成全球首次海上网系回收</t>
+        </is>
+      </c>
+      <c r="D2185" t="inlineStr">
+        <is>
+          <t>长征十号乙火箭完成全球首次海上网系回收，我国是唯一实践该技术的国家。</t>
+        </is>
+      </c>
+      <c r="E2185" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2185" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDExc4Z0fbcF0l5A5NLolHi260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr">
+        <is>
+          <t>China lands reusable rocket for first time, state media says</t>
+        </is>
+      </c>
+      <c r="D2186" t="inlineStr">
+        <is>
+          <t>中国首次实现可重复使用火箭着陆，追赶SpaceX等公司。</t>
+        </is>
+      </c>
+      <c r="E2186" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2186" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cm2rmmx86pdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr">
+        <is>
+          <t>Pioneering treatment saves identical twins from rare pregnancy condition</t>
+        </is>
+      </c>
+      <c r="D2187" t="inlineStr">
+        <is>
+          <t>世界首例医学试验：开创性治疗在子宫内拯救了一对罕见妊娠并发症的双胞胎。</t>
+        </is>
+      </c>
+      <c r="E2187" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2187" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2eyl3zkpwko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr">
+        <is>
+          <t>U.S.-Iran fighting appears to pause. And, life inside Israel's military zones in Gaza</t>
+        </is>
+      </c>
+      <c r="D2188" t="inlineStr">
+        <is>
+          <t>美伊冲突在两天交火后暂停；加沙以色列军事区内生活现状。</t>
+        </is>
+      </c>
+      <c r="E2188" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2188" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/g-s1-132943/up-first-newsletter-iran-us-tps-haitians-syrians-eac-gaza-israel-hamas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr">
+        <is>
+          <t>Shelling at night, gunfire by day in Israel's expanding zone of control in Gaza</t>
+        </is>
+      </c>
+      <c r="D2189" t="inlineStr">
+        <is>
+          <t>以色列在加沙扩大控制区，夜间炮击白天枪击，巴勒斯坦人付出惨重代价。</t>
+        </is>
+      </c>
+      <c r="E2189" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2189" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/nx-s1-5887357/israel-gaza-war-trump-ceasefire-military-control</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr">
+        <is>
+          <t>[视频]张国清在广西指导支持受灾群众生活保障和灾后抢修恢复工作</t>
+        </is>
+      </c>
+      <c r="D2190" t="inlineStr">
+        <is>
+          <t>张国清赴广西指导受灾群众生活保障和灾后抢修恢复工作。</t>
+        </is>
+      </c>
+      <c r="E2190" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2190" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEPLQan4Q33sWIemNGreY8260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr">
+        <is>
+          <t>We've saved £6,000 on holidays by swapping homes with strangers</t>
+        </is>
+      </c>
+      <c r="D2191" t="inlineStr">
+        <is>
+          <t>英国兴起换房度假，称已省下6000英镑旅行费用。</t>
+        </is>
+      </c>
+      <c r="E2191" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2191" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce8kkerxz74o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr">
+        <is>
+          <t>'People don't realise how at risk they are': A day with an ambulance service in a heatwave</t>
+        </is>
+      </c>
+      <c r="D2192" t="inlineStr">
+        <is>
+          <t>英国遭遇持续热浪，BBC跟随急救人员记录高温下的救护工作与风险。</t>
+        </is>
+      </c>
+      <c r="E2192" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2192" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg4y289ppjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr">
+        <is>
+          <t>[视频]伊朗媒体称布什尔核电站周边区域遭美军袭击 伊朗称打击美指挥中心</t>
+        </is>
+      </c>
+      <c r="D2193" t="inlineStr">
+        <is>
+          <t>伊朗称布什尔核电站周边遭美军袭击，伊朗打击美指挥中心，美伊仍在核问题谈判。</t>
+        </is>
+      </c>
+      <c r="E2193" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2193" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEKBRMmWoaidezPsZNt5GT260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr">
+        <is>
+          <t>[视频]俄称在红利曼战斗进入收尾阶段 乌称对俄海上目标实施打击</t>
+        </is>
+      </c>
+      <c r="D2194" t="inlineStr">
+        <is>
+          <t>俄称红利曼战斗进入收尾阶段；乌称击中俄海上目标；美将许可乌生产“爱国者”系统。</t>
+        </is>
+      </c>
+      <c r="E2194" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2194" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEH9a9qmwtVp3WRkJtkfJZ260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2195" t="inlineStr">
+        <is>
+          <t>East Asia braces for destructive typhoon as landslides kill 15 in Philippines</t>
+        </is>
+      </c>
+      <c r="D2195" t="inlineStr">
+        <is>
+          <t>东亚面临破坏性台风“巴威”，已致菲律宾15人死于山体滑坡。</t>
+        </is>
+      </c>
+      <c r="E2195" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2195" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c04y6wr03gxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2196" t="inlineStr">
+        <is>
+          <t>One of Spain's deadliest wildfires kills at least 12 people, with 23 others missing</t>
+        </is>
+      </c>
+      <c r="D2196" t="inlineStr">
+        <is>
+          <t>西班牙南部度假胜地发生致命野火，至少12人遇难，23人失踪。</t>
+        </is>
+      </c>
+      <c r="E2196" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2196" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/nx-s1-5888160/southern-spain-wildfire-almeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2197" t="inlineStr">
+        <is>
+          <t>Ebola death toll reaches 600, as new cases suspected in other parts of Congo</t>
+        </is>
+      </c>
+      <c r="D2197" t="inlineStr">
+        <is>
+          <t>刚果埃博拉死亡人数达600，新疑似病例出现在未受影响地区。</t>
+        </is>
+      </c>
+      <c r="E2197" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2197" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/g-s1-132930/ebola-outbreak-congo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2198" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2198" t="inlineStr">
+        <is>
+          <t>U.S. and Iran exchange intensifying fire across Mideast, threatening ceasefire deal</t>
+        </is>
+      </c>
+      <c r="D2198" t="inlineStr">
+        <is>
+          <t>美伊在中东激烈交火，威胁停火协议，周四冲突规模升级。</t>
+        </is>
+      </c>
+      <c r="E2198" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2198" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/10/g-s1-132927/us-iran-war</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr">
+        <is>
+          <t>社会, 经济</t>
+        </is>
+      </c>
+      <c r="C2199" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2199" t="inlineStr">
+        <is>
+          <t>上半年全国出入境3.69亿人次创历史新高；铁路暑运发送超1.2亿人次；用电负荷创历史新高。</t>
+        </is>
+      </c>
+      <c r="E2199" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2199" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/10/VIDEMj4ACMmGTAC1G7Y8UDGC260710.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2200" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2200" t="inlineStr">
+        <is>
+          <t>Man nearly sucked out of window mid-air on Ryanair plane, passengers say</t>
+        </is>
+      </c>
+      <c r="D2200" t="inlineStr">
+        <is>
+          <t>瑞安航空一航班发生事故，乘客险些被吸出窗外，接受治疗。</t>
+        </is>
+      </c>
+      <c r="E2200" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2200" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgk65knkyzdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2201" t="inlineStr">
+        <is>
+          <t>Top Boy actor Micheal Ward found not guilty of rape</t>
+        </is>
+      </c>
+      <c r="D2201" t="inlineStr">
+        <is>
+          <t>《伦敦黑帮》演员沃德被判强奸罪名不成立。</t>
+        </is>
+      </c>
+      <c r="E2201" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2201" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cewq9vznzz5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2202" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2202" t="inlineStr">
+        <is>
+          <t>Bayeux Tapestry arrives in UK for first time in 900 years under police guard</t>
+        </is>
+      </c>
+      <c r="D2202" t="inlineStr">
+        <is>
+          <t>贝叶挂毯900年来首次抵英，将在九月展出。</t>
+        </is>
+      </c>
+      <c r="E2202" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2202" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly9r54e5r4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2203" t="inlineStr">
+        <is>
+          <t>UK bakes in 35C highs as millions under hosepipe bans</t>
+        </is>
+      </c>
+      <c r="D2203" t="inlineStr">
+        <is>
+          <t>英国高温达35°C，数百万人面临软管限水令。</t>
+        </is>
+      </c>
+      <c r="E2203" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2203" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/c0my38l4ex3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2204" t="inlineStr">
+        <is>
+          <t>Longest-serving Archers star Patricia Greene dies aged 95</t>
+        </is>
+      </c>
+      <c r="D2204" t="inlineStr">
+        <is>
+          <t>英国广播四台长寿肥皂剧《阿彻一家》演员帕特丽夏·格林去世，享年95岁。</t>
+        </is>
+      </c>
+      <c r="E2204" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2204" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy04erw9y42o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2205" t="inlineStr">
+        <is>
+          <t>Prince Harry plays pickleball at Invictus Games event, but no Meghan</t>
+        </is>
+      </c>
+      <c r="D2205" t="inlineStr">
+        <is>
+          <t>哈里王子独自参加不屈运动会，打匹克球，妻子梅根未同行。</t>
+        </is>
+      </c>
+      <c r="E2205" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2205" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2dyw9lp02wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2206" t="inlineStr">
+        <is>
+          <t>Arthur Fery's Wimbledon run ended by Alexander Zverev in semi-finals</t>
+        </is>
+      </c>
+      <c r="D2206" t="inlineStr">
+        <is>
+          <t>英国选手费里在温网半决赛被兹维列夫淘汰。</t>
+        </is>
+      </c>
+      <c r="E2206" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2206" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/tennis/articles/ckg475qdnd7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-11
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2206"/>
+  <dimension ref="A1:F2242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -71029,6 +71029,1158 @@
         </is>
       </c>
     </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C2207" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260711 21:00</t>
+        </is>
+      </c>
+      <c r="D2207" t="inlineStr">
+        <is>
+          <t>中朝互致贺电庆祝条约65周年；李强蔡奇会见朝鲜总理；各地防台风转移220万人；多领域政策与建设进展。</t>
+        </is>
+      </c>
+      <c r="E2207" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2207" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEEyq6H0u2EhzVOUrbSf5W260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2208" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2208" t="inlineStr">
+        <is>
+          <t>[视频]习近平同朝鲜劳动党总书记、国务委员会委员长金正恩就《中朝友好合作互助条约》签订65周年互致贺电</t>
+        </is>
+      </c>
+      <c r="D2208" t="inlineStr">
+        <is>
+          <t>习近平与金正恩就《中朝友好合作互助条约》签订65周年互致贺电，强调世代友好与战略合作。</t>
+        </is>
+      </c>
+      <c r="E2208" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2208" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEbloDn9jk5Ip2Xbh7uIFP260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2209" t="inlineStr">
+        <is>
+          <t>[视频]李强举行仪式欢迎朝鲜内阁总理访华</t>
+        </is>
+      </c>
+      <c r="D2209" t="inlineStr">
+        <is>
+          <t>李强在北京人民大会堂举行仪式，欢迎朝鲜内阁总理朴泰成正式访华。</t>
+        </is>
+      </c>
+      <c r="E2209" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2209" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEnLjdMLUl8Or18kjOfRAX260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2210" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2210" t="inlineStr">
+        <is>
+          <t>[视频]李强同朝鲜内阁总理会谈</t>
+        </is>
+      </c>
+      <c r="D2210" t="inlineStr">
+        <is>
+          <t>李强与朝鲜总理朴泰成会谈，强调深化中朝关系，拓展经贸及民生领域合作。</t>
+        </is>
+      </c>
+      <c r="E2210" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2210" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDETQS7lofgRoFueJddxoF4260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2211" t="inlineStr">
+        <is>
+          <t>[视频]蔡奇出席《中朝友好合作互助条约》签订65周年纪念招待会</t>
+        </is>
+      </c>
+      <c r="D2211" t="inlineStr">
+        <is>
+          <t>蔡奇与朝鲜总理朴泰成共同出席纪念招待会，强调赓续中朝传统友谊与合作。</t>
+        </is>
+      </c>
+      <c r="E2211" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2211" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDE24YUlVonFJv5BJhUB2QZ260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2212" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2212" t="inlineStr">
+        <is>
+          <t>[视频]日本民众举行集会 反对高市政权扩军修宪</t>
+        </is>
+      </c>
+      <c r="D2212" t="inlineStr">
+        <is>
+          <t>日本民众在东京集会，反对高市政权解禁杀伤性武器出口和扩军修宪。</t>
+        </is>
+      </c>
+      <c r="E2212" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2212" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEo0QhMGQNwDPbp48SyMj4260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2213" t="inlineStr">
+        <is>
+          <t>Landmark US housing bill becomes law despite Trump protest</t>
+        </is>
+      </c>
+      <c r="D2213" t="inlineStr">
+        <is>
+          <t>美国里程碑式住房法案在总统反对下仍成为法律，旨在降低成本和增加供应。</t>
+        </is>
+      </c>
+      <c r="E2213" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2213" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn8qwj611qxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2214" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2214" t="inlineStr">
+        <is>
+          <t>Reeves tells BBC: Burnham needs worked-through plan to govern from the start</t>
+        </is>
+      </c>
+      <c r="D2214" t="inlineStr">
+        <is>
+          <t>财政大臣里夫斯表示，将向即将上任的首相移交稳定经济。</t>
+        </is>
+      </c>
+      <c r="E2214" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2214" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwykdvgv4d4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2215" t="inlineStr">
+        <is>
+          <t>[视频]今年前五个月我国高端船型出口量大幅增长</t>
+        </is>
+      </c>
+      <c r="D2215" t="inlineStr">
+        <is>
+          <t>今年前五月我国高端液货船出口额同比增长188.8%，达到643亿元。</t>
+        </is>
+      </c>
+      <c r="E2215" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2215" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEimlEX4gnEVZmVNFg43Ch260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2216" t="inlineStr">
+        <is>
+          <t>[视频]人民日报评论员文章：向着到2035年建成科技强国的目标坚定迈进——论学习贯彻习近平总书记在国家科学技术奖励大会、两院院士大会、中国科协十一大上重要讲话</t>
+        </is>
+      </c>
+      <c r="D2216" t="inlineStr">
+        <is>
+          <t>人民日报发表评论员文章，号召坚定迈向2035年建成科技强国的目标。</t>
+        </is>
+      </c>
+      <c r="E2216" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2216" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEepO6WxQpa1bsidpuBr1g260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2217" t="inlineStr">
+        <is>
+          <t>[视频]陈立泉：五十载坚守 让中国锂电池领跑世界</t>
+        </is>
+      </c>
+      <c r="D2217" t="inlineStr">
+        <is>
+          <t>陈立泉院士获国家最高科学技术奖，他带领中国锂电池从无到有并领跑世界。</t>
+        </is>
+      </c>
+      <c r="E2217" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2217" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEU7o2V5SE7LgdpYob6Q5q260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C2218" t="inlineStr">
+        <is>
+          <t>New dinosaur species as long as cricket pitch discovered in Thailand</t>
+        </is>
+      </c>
+      <c r="D2218" t="inlineStr">
+        <is>
+          <t>泰国发现新恐龙物种，体长如板球场，约生活在1.5亿年前。</t>
+        </is>
+      </c>
+      <c r="E2218" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2218" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crely7g8xepo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2219" t="inlineStr">
+        <is>
+          <t>Meta pulls new AI image feature after days of backlash</t>
+        </is>
+      </c>
+      <c r="D2219" t="inlineStr">
+        <is>
+          <t>Meta发布AI图像编辑功能后遭强烈反对，现已撤下该功能。</t>
+        </is>
+      </c>
+      <c r="E2219" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2219" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2dy6e8klw0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2220" t="inlineStr">
+        <is>
+          <t>See if you can spot an AI deepfake with our test</t>
+        </is>
+      </c>
+      <c r="D2220" t="inlineStr">
+        <is>
+          <t>阿伯丁研究人员测试能否训练人们识别AI生成的深度伪造面部图像。</t>
+        </is>
+      </c>
+      <c r="E2220" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2220" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9d2wgvg55jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2221" t="inlineStr">
+        <is>
+          <t>[视频]各地各部门积极应对台风“巴威”</t>
+        </is>
+      </c>
+      <c r="D2221" t="inlineStr">
+        <is>
+          <t>台风“巴威”将登陆浙江沿海，各地转移群众超221万人，停航停课积极应对。</t>
+        </is>
+      </c>
+      <c r="E2221" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2221" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEKSgv84ODvsxFhOv6XHRR260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2222" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】浙江苍南：台风来临前的大转移</t>
+        </is>
+      </c>
+      <c r="D2222" t="inlineStr">
+        <is>
+          <t>浙江苍南党员干部在台风前紧急转移群众12万人，坚守防台风一线。</t>
+        </is>
+      </c>
+      <c r="E2222" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2222" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDESCyeckqTs5sr2zYeamNT260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2223" t="inlineStr">
+        <is>
+          <t>[视频]支持政策多点发力 我国持续减轻家庭生养负担</t>
+        </is>
+      </c>
+      <c r="D2223" t="inlineStr">
+        <is>
+          <t>我国多措并举减轻家庭生养负担，包括生育津贴、育儿补贴、医保报销和普惠托育等。</t>
+        </is>
+      </c>
+      <c r="E2223" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2223" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEzVrNBs3hl7G7UgQXonDq260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2224" t="inlineStr">
+        <is>
+          <t>民生, 经济, 社会</t>
+        </is>
+      </c>
+      <c r="C2224" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2224" t="inlineStr">
+        <is>
+          <t>两部门预拨8000万元救灾资金支持广西；公路运力扩容；暑期文旅消费季启动等。</t>
+        </is>
+      </c>
+      <c r="E2224" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2224" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDEO7wMpwxA70vJzW2MN6Ix260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2225" t="inlineStr">
+        <is>
+          <t>China braced for second typhoon in a week as Bavi approaches landfall</t>
+        </is>
+      </c>
+      <c r="D2225" t="inlineStr">
+        <is>
+          <t>台风“巴威”逼近中国浙江，数十万人从东部省份撤离。</t>
+        </is>
+      </c>
+      <c r="E2225" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2225" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdxd3wkp2rzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2226" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2226" t="inlineStr">
+        <is>
+          <t>Most people who need glasses don't have them. Can the post office change that?</t>
+        </is>
+      </c>
+      <c r="D2226" t="inlineStr">
+        <is>
+          <t>印度部分邮局为视力模糊的访客提供免费验光服务，以解决多数人无眼镜的问题。</t>
+        </is>
+      </c>
+      <c r="E2226" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2226" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/11/nx-s1-5887653/reading-glasses-post-office-india</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2227" t="inlineStr">
+        <is>
+          <t>[视频]美称已同意伊朗请求继续谈判 伊朗称从未提出谈判请求</t>
+        </is>
+      </c>
+      <c r="D2227" t="inlineStr">
+        <is>
+          <t>美称伊朗请求谈判被否认，美伊局势紧张；国际能源署称市场前景蒙阴。</t>
+        </is>
+      </c>
+      <c r="E2227" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2227" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDElZ4dNe3B7JARpOfspB26260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2228" t="inlineStr">
+        <is>
+          <t>国际, 军事, 政治</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2228" t="inlineStr">
+        <is>
+          <t>俄乌冲突持续；土或转让俄制S-400系统；欧盟初步认定Meta平台违规。</t>
+        </is>
+      </c>
+      <c r="E2228" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2228" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/11/VIDE0yt5H4kpOdxJ7s4OyXZE260711.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr">
+        <is>
+          <t>US wants Iran to pledge to stop shooting at ships in Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D2229" t="inlineStr">
+        <is>
+          <t>美国要求伊朗承诺停止在霍尔木兹海峡向船只射击。</t>
+        </is>
+      </c>
+      <c r="E2229" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2229" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crelyq79x71o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2230" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr">
+        <is>
+          <t>Indian tourists among 15 killed as speedboat capsizes in Vietnam</t>
+        </is>
+      </c>
+      <c r="D2230" t="inlineStr">
+        <is>
+          <t>越南一艘快艇在南海倾覆，15人死亡含印度游客，21人获救。</t>
+        </is>
+      </c>
+      <c r="E2230" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2230" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyd7x22lp1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr">
+        <is>
+          <t>US pays out $3m to victims of mystery Havana Syndrome condition reported by spies</t>
+        </is>
+      </c>
+      <c r="D2231" t="inlineStr">
+        <is>
+          <t>美国向“哈瓦那综合征”受害者支付300万美元，该病影响外交官及家属。</t>
+        </is>
+      </c>
+      <c r="E2231" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2231" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr7xyl78vnko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2232" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr">
+        <is>
+          <t>Watch: 'We escaped Spanish wildfire, but our friends lost their lives'</t>
+        </is>
+      </c>
+      <c r="D2232" t="inlineStr">
+        <is>
+          <t>西班牙南部数百名消防员与致命野火搏斗，有人幸存但朋友遇难。</t>
+        </is>
+      </c>
+      <c r="E2232" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2232" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c07y357zvl1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr">
+        <is>
+          <t>Trump threatens Iran after Ayatollah Ali Khamenei's funeral saw calls for his killing</t>
+        </is>
+      </c>
+      <c r="D2233" t="inlineStr">
+        <is>
+          <t>在伊朗最高领袖葬礼出现刺杀呼声后，特朗普威胁伊朗并要求其保证霍尔木兹海峡开放。</t>
+        </is>
+      </c>
+      <c r="E2233" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2233" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/11/nx-s1-5890029/trump-threatens-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2234" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr">
+        <is>
+          <t>Spain battles to contain one of its deadliest wildfires as at least 12 killed</t>
+        </is>
+      </c>
+      <c r="D2234" t="inlineStr">
+        <is>
+          <t>西班牙遭遇致命野火，至少12人死亡，包括4名英国人，另有23人失踪。</t>
+        </is>
+      </c>
+      <c r="E2234" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2234" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1wyv383j2xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr">
+        <is>
+          <t>Australian killer's final police interview footage released</t>
+        </is>
+      </c>
+      <c r="D2235" t="inlineStr">
+        <is>
+          <t>澳大利亚杀人犯默多克最终警方采访视频公布，他未透露受害者遗骸位置。</t>
+        </is>
+      </c>
+      <c r="E2235" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2235" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvglj4k03w4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2236" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr">
+        <is>
+          <t>TV presenter Dermot Murnaghan dies aged 68</t>
+        </is>
+      </c>
+      <c r="D2236" t="inlineStr">
+        <is>
+          <t>前BBC、ITV和天空新闻主持人德莫特·穆尔纳汉因前列腺癌去世，享年68岁。</t>
+        </is>
+      </c>
+      <c r="E2236" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2236" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20yvg13nqpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr">
+        <is>
+          <t>South Africa World Cup midfielder Adams dies aged 25</t>
+        </is>
+      </c>
+      <c r="D2237" t="inlineStr">
+        <is>
+          <t>南非世界杯中场球员亚当斯去世，年仅25岁。</t>
+        </is>
+      </c>
+      <c r="E2237" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2237" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cr47y5nvrqlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2238" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr">
+        <is>
+          <t>Pubs can stay open for full Norway game - even if kick-off delayed</t>
+        </is>
+      </c>
+      <c r="D2238" t="inlineStr">
+        <is>
+          <t>酒吧获准在挪威比赛期间延长营业，即使开球延迟也能看完整场。</t>
+        </is>
+      </c>
+      <c r="E2238" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2238" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cm204lgrv10o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr">
+        <is>
+          <t>Hey Jude: Bellingham's return to England indispensability</t>
+        </is>
+      </c>
+      <c r="D2239" t="inlineStr">
+        <is>
+          <t>资深记者报道贝林厄姆在世界杯上对英格兰队的重要回归与出色表现。</t>
+        </is>
+      </c>
+      <c r="E2239" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2239" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/ckg47l8nl7jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2240" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr">
+        <is>
+          <t>Is it time to give record-breaker Pickford the credit he deserves?</t>
+        </is>
+      </c>
+      <c r="D2240" t="inlineStr">
+        <is>
+          <t>英格兰门将皮克福德创世界杯纪录，文章呼吁给予他应有的赞誉。</t>
+        </is>
+      </c>
+      <c r="E2240" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2240" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cj9gknxm91vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>体育</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr">
+        <is>
+          <t>Quarter‑final turns into endurance test as England meet heat‑hardened Norway</t>
+        </is>
+      </c>
+      <c r="D2241" t="inlineStr">
+        <is>
+          <t>英格兰队将在高温的迈阿密迎战适应热环境的挪威队，世界杯四分之一决赛成耐力考验。</t>
+        </is>
+      </c>
+      <c r="E2241" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2241" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cx2jzl3zxpzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B2242" t="inlineStr">
+        <is>
+          <t>体育</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr">
+        <is>
+          <t>Spain edges Belgium and will face France in World Cup semifinal</t>
+        </is>
+      </c>
+      <c r="D2242" t="inlineStr">
+        <is>
+          <t>西班牙险胜比利时，将在世界杯半决赛对阵同样不败的法国队。</t>
+        </is>
+      </c>
+      <c r="E2242" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2242" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/11/nx-s1-5890030/spain-will-face-france-world-cup-semifinal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-12
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2242"/>
+  <dimension ref="A1:F2272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72181,6 +72181,966 @@
         </is>
       </c>
     </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>政治, 民生, 国际</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260712 19:00</t>
+        </is>
+      </c>
+      <c r="D2243" t="inlineStr">
+        <is>
+          <t>新闻联播报道耕地保护、政绩观教育、台风应对、经济指标、新材料突破、国防科技、治安形势等国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E2243" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2243" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDE10xymttB14WZJn1JbbsJ260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2244" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】直面问题抓整改 推动学习教育走深走实</t>
+        </is>
+      </c>
+      <c r="D2244" t="inlineStr">
+        <is>
+          <t>河北邢台、湖北武汉学习教育，优化营商环境，解决群众急难愁盼问题。</t>
+        </is>
+      </c>
+      <c r="E2244" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2244" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEAEaEpoGOEDAOqJLJzzj2260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr">
+        <is>
+          <t>[视频]上半年多项先行指标企稳回升</t>
+        </is>
+      </c>
+      <c r="D2245" t="inlineStr">
+        <is>
+          <t>上半年先行指标企稳回升，工业生产、投资消费稳步增长。</t>
+        </is>
+      </c>
+      <c r="E2245" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2245" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEH8pvCaKk9RPobOry52kO260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2246" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2246" t="inlineStr">
+        <is>
+          <t>我国推进能源节能降碳；期货市场成交额同比增42%；中国石化完成对中国航油重组。</t>
+        </is>
+      </c>
+      <c r="E2246" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2246" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDExgcdiRTRcSwChXu8uoKf260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr">
+        <is>
+          <t>How Aldi is taking on US supermarkets with its $4 almond butter</t>
+        </is>
+      </c>
+      <c r="D2247" t="inlineStr">
+        <is>
+          <t>德国超市Aldi以4美元杏仁酱进军美国市场，挑战沃尔玛折扣模式。</t>
+        </is>
+      </c>
+      <c r="E2247" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2247" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly0l5d5xn7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2248" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr">
+        <is>
+          <t>[视频]我国新材料领域持续取得新突破</t>
+        </is>
+      </c>
+      <c r="D2248" t="inlineStr">
+        <is>
+          <t>我国新材料领域取得突破，新型智能材料、碳纤维等助力产业升级。</t>
+        </is>
+      </c>
+      <c r="E2248" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2248" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDE6eEc180KjLJ24EQB7u1h260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>科技, 军事</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr">
+        <is>
+          <t>[视频]贲德：用毕生精力铸就国防“火眼金睛”</t>
+        </is>
+      </c>
+      <c r="D2249" t="inlineStr">
+        <is>
+          <t>雷达专家贲德获国家最高科技奖，研制相控阵雷达等国防利器。</t>
+        </is>
+      </c>
+      <c r="E2249" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2249" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDE85Yi0DHKvtbGqMXYAWGG260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2250" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr">
+        <is>
+          <t>People flee as Russian strike hits near Ukraine coffee shop</t>
+        </is>
+      </c>
+      <c r="D2250" t="inlineStr">
+        <is>
+          <t>俄军袭击乌克兰苏梅市咖啡店附近，民众惊慌躲避奔跑。</t>
+        </is>
+      </c>
+      <c r="E2250" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2250" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c8r27drk1nxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】严守耕地红线 筑牢国家粮食安全根基</t>
+        </is>
+      </c>
+      <c r="D2251" t="inlineStr">
+        <is>
+          <t>各地严守耕地红线，推进高标准农田建设，夏粮首次突破3000亿斤。</t>
+        </is>
+      </c>
+      <c r="E2251" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2251" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEagvQIyOQmoHXWBMTyNrj260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2252" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr">
+        <is>
+          <t>[视频]台风“巴威”登陆 各地全力应对</t>
+        </is>
+      </c>
+      <c r="D2252" t="inlineStr">
+        <is>
+          <t>台风巴威登陆浙江，各地紧急转移人员，抢险救灾保障群众安全。</t>
+        </is>
+      </c>
+      <c r="E2252" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2252" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEKUPi9o1VuZ1kojYXMAFC260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】风雨之夜的守护</t>
+        </is>
+      </c>
+      <c r="D2253" t="inlineStr">
+        <is>
+          <t>党员干部在台风夜里巡查抢险，转移群众，守护人民生命财产安全。</t>
+        </is>
+      </c>
+      <c r="E2253" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2253" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDES4QCIOQ24qSXm1BHQOPz260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2254" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr">
+        <is>
+          <t>[视频]我国社会治安形势持续向好 群众安全感稳步提升</t>
+        </is>
+      </c>
+      <c r="D2254" t="inlineStr">
+        <is>
+          <t>全国刑事案件和治安案件立案数同比双降超10%，电诈发案数连续8个月下降，群众安全感提升。</t>
+        </is>
+      </c>
+      <c r="E2254" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2254" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEuMNFultn5cCD2vorOywU260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr">
+        <is>
+          <t>China evacuates nearly two million people as powerful typhoon makes landfall</t>
+        </is>
+      </c>
+      <c r="D2255" t="inlineStr">
+        <is>
+          <t>台风登陆中国浙江，近两百万人被疏散，学校及交通暂停。</t>
+        </is>
+      </c>
+      <c r="E2255" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2255" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdxd3wkp2rzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2256" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr">
+        <is>
+          <t>We are living fewer years in good health: Is the NHS part of the problem?</t>
+        </is>
+      </c>
+      <c r="D2256" t="inlineStr">
+        <is>
+          <t>英国人健康寿命缩短，报道质疑国民医疗服务体系是否成问题源头。</t>
+        </is>
+      </c>
+      <c r="E2256" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2256" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8r2nz82z3vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr">
+        <is>
+          <t>[视频]美称对伊朗展开本周第三轮打击 伊朗称打击美在中东地区目标</t>
+        </is>
+      </c>
+      <c r="D2257" t="inlineStr">
+        <is>
+          <t>美对伊朗发动第三轮打击，伊朗打击美军基地并宣布关闭霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E2257" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2257" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEHvwqZt8GUxVswA43r4nK260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2258" t="inlineStr">
+        <is>
+          <t>国际, 军事, 社会</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2258" t="inlineStr">
+        <is>
+          <t>俄打击乌无人机企业，乌称击落千余架无人机；世卫警告刚果（金）埃博拉疫情可能被低估。</t>
+        </is>
+      </c>
+      <c r="E2258" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2258" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/12/VIDEHo9Sj9ZVMcpoa5Z4xGwO260712.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr">
+        <is>
+          <t>US launches fresh strikes as Iran closes Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D2259" t="inlineStr">
+        <is>
+          <t>美国发动新一轮打击，伊朗关闭霍尔木兹海峡。</t>
+        </is>
+      </c>
+      <c r="E2259" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2259" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj9gkpp0dkeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2260" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr">
+        <is>
+          <t>US senator and close Trump ally Lindsey Graham dies after 'brief and sudden illness'</t>
+        </is>
+      </c>
+      <c r="D2260" t="inlineStr">
+        <is>
+          <t>美国参议员、特朗普亲密盟友林赛·格雷厄姆因突发疾病去世。</t>
+        </is>
+      </c>
+      <c r="E2260" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2260" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgj25j6nmeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr">
+        <is>
+          <t>Badly burned British couple rescued from ravine during Spain wildfires, reports say</t>
+        </is>
+      </c>
+      <c r="D2261" t="inlineStr">
+        <is>
+          <t>西班牙山火中一对严重烧伤的英国夫妇从峡谷中被救出。</t>
+        </is>
+      </c>
+      <c r="E2261" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2261" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2x7441762o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2262" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr">
+        <is>
+          <t>U.S. launches fresh strikes on Iran as Tehran says it has closed Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D2262" t="inlineStr">
+        <is>
+          <t>美国对伊朗发动新空袭，打击140个目标；伊朗关闭霍尔木兹海峡并反击。</t>
+        </is>
+      </c>
+      <c r="E2262" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2262" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/11/g-s1-133212/us-iran-vessel-attack-strait-hormuz-gulf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr">
+        <is>
+          <t>At least two killed in Toronto street festival shooting</t>
+        </is>
+      </c>
+      <c r="D2263" t="inlineStr">
+        <is>
+          <t>多伦多街头节日庆典发生枪击，至少两人死亡，警方已找回两把枪支。</t>
+        </is>
+      </c>
+      <c r="E2263" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2263" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce3e66e1x3go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2264" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr">
+        <is>
+          <t>Muslim judge in India faces death threats after convicting 'cow vigilantes'</t>
+        </is>
+      </c>
+      <c r="D2264" t="inlineStr">
+        <is>
+          <t>印度穆斯林女法官因定罪“护牛私刑者”遭死亡威胁与网络辱骂。</t>
+        </is>
+      </c>
+      <c r="E2264" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2264" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd6e9zq87xvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr">
+        <is>
+          <t>Police say no suggestion of political motive in Widdecombe killing after new arrest</t>
+        </is>
+      </c>
+      <c r="D2265" t="inlineStr">
+        <is>
+          <t>警方称新逮捕嫌犯后，威德科姆案无政治动机，不再追查他人。</t>
+        </is>
+      </c>
+      <c r="E2265" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2265" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8628q3eqdeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2266" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr">
+        <is>
+          <t>Bill for Hillsborough Law set to be approved by MPs</t>
+        </is>
+      </c>
+      <c r="D2266" t="inlineStr">
+        <is>
+          <t>1989年FA杯半决赛踩踏事故致97名球迷死亡，相关法案即将获批。</t>
+        </is>
+      </c>
+      <c r="E2266" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2266" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz754eey3xeo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr">
+        <is>
+          <t>Tuchel angry at 'lucky' England - but Bellingham defends players</t>
+        </is>
+      </c>
+      <c r="D2267" t="inlineStr">
+        <is>
+          <t>英格兰主帅图赫尔批评球队“侥幸”胜挪威，贝林厄姆为队友辩护。</t>
+        </is>
+      </c>
+      <c r="E2267" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2267" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/ckg474ekv58o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2268" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr">
+        <is>
+          <t>McCullum sacked as England Test head coach</t>
+        </is>
+      </c>
+      <c r="D2268" t="inlineStr">
+        <is>
+          <t>英格兰板球队主教练麦卡勒姆被解雇，球队面临无帅无队长局面。</t>
+        </is>
+      </c>
+      <c r="E2268" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2268" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c8028vm2g9ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr">
+        <is>
+          <t>Tuchel wasn't happy with the performance. So why do England keep winning?</t>
+        </is>
+      </c>
+      <c r="D2269" t="inlineStr">
+        <is>
+          <t>尽管图赫尔不满表现，英格兰队仍连胜，专家分析原因。</t>
+        </is>
+      </c>
+      <c r="E2269" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2269" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c7vy25lqll6o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2270" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr">
+        <is>
+          <t>'Animals', Hand of God and Beckham: Argentina and England's World Cup rivalry</t>
+        </is>
+      </c>
+      <c r="D2270" t="inlineStr">
+        <is>
+          <t>英格兰与阿根廷的世界杯半决赛前夕，回顾双方足球恩怨史。</t>
+        </is>
+      </c>
+      <c r="E2270" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2270" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c621y75w2x2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr">
+        <is>
+          <t>'We should all be excited' - Messi set for first England meeting</t>
+        </is>
+      </c>
+      <c r="D2271" t="inlineStr">
+        <is>
+          <t>梅西随阿根廷晋级世界杯半决赛，将首次对阵英格兰队。</t>
+        </is>
+      </c>
+      <c r="E2271" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2271" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cvgexz4qdlgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B2272" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr">
+        <is>
+          <t>Alvarez's 112th-minute goal helps lift Argentina past Switzerland 3-1 and into World Cup semifinals</t>
+        </is>
+      </c>
+      <c r="D2272" t="inlineStr">
+        <is>
+          <t>阿尔瓦雷斯加时赛第112分钟进球，助阿根廷3-1胜瑞士晋级四强。</t>
+        </is>
+      </c>
+      <c r="E2272" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2272" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/12/nx-s1-5890774/argentina-switzerland-3-1-world-cup-semifinals</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-13
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2272"/>
+  <dimension ref="A1:F2308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73141,6 +73141,1158 @@
         </is>
       </c>
     </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>政治, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260713 19:00</t>
+        </is>
+      </c>
+      <c r="D2273" t="inlineStr">
+        <is>
+          <t>习近平将出席世界人工智能大会；国务院印发国民健康规划；台风巴威北上各地应对。</t>
+        </is>
+      </c>
+      <c r="E2273" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2273" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEqVGNumex1YNeUCK1Vavy260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2274" t="inlineStr">
+        <is>
+          <t>政治, 科技</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr">
+        <is>
+          <t>[视频]习近平将出席2026世界人工智能大会暨人工智能全球治理高级别会议开幕式并发表主旨讲话</t>
+        </is>
+      </c>
+      <c r="D2274" t="inlineStr">
+        <is>
+          <t>习近平将出席2026世界人工智能大会开幕式并发表主旨讲话。</t>
+        </is>
+      </c>
+      <c r="E2274" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2274" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEJekOK1rPLMG3ba74MVyG260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见第十一届世界华侨华人社团联谊大会全体代表</t>
+        </is>
+      </c>
+      <c r="D2275" t="inlineStr">
+        <is>
+          <t>王沪宁会见第十一届世界华侨华人社团联谊大会全体代表，强调侨胞助力民族复兴。</t>
+        </is>
+      </c>
+      <c r="E2275" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2275" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEWrNCT6IjAb3COxS8k8yC260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2276" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr">
+        <is>
+          <t>[视频]中共中央办公厅 国务院办公厅印发《关于完善自然资源资产管理制度体系的意见》</t>
+        </is>
+      </c>
+      <c r="D2276" t="inlineStr">
+        <is>
+          <t>中办国办印发意见，完善自然资源资产管理制度体系，明确2030年、2035年目标。</t>
+        </is>
+      </c>
+      <c r="E2276" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2276" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDENFJVnJQs3sVAvKMaFXdS260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr">
+        <is>
+          <t>Senator Lindsey Graham died of aortic tear, examiner says</t>
+        </is>
+      </c>
+      <c r="D2277" t="inlineStr">
+        <is>
+          <t>参议员林赛·格雷厄姆因主动脉撕裂去世，终年71岁。</t>
+        </is>
+      </c>
+      <c r="E2277" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2277" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn75083d472o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2278" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr">
+        <is>
+          <t>UK bans support for Iran's Islamic Revolutionary Guard Corps</t>
+        </is>
+      </c>
+      <c r="D2278" t="inlineStr">
+        <is>
+          <t>英国禁止支持伊朗伊斯兰革命卫队，因其涉英国本土恐吓活动。</t>
+        </is>
+      </c>
+      <c r="E2278" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2278" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz0jkj7e87go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr">
+        <is>
+          <t>Former top official Robbins takes legal action over sacking</t>
+        </is>
+      </c>
+      <c r="D2279" t="inlineStr">
+        <is>
+          <t>前高官罗宾斯因曼德尔森勋爵任驻美大使审查事宜被解雇，现已采取法律行动。</t>
+        </is>
+      </c>
+      <c r="E2279" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2279" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjegqpwxk98o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2280" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开经济形势专家和企业家座谈会</t>
+        </is>
+      </c>
+      <c r="D2280" t="inlineStr">
+        <is>
+          <t>李强主持召开经济形势座谈会，强调加大逆周期调节力度，巩固经济稳中向好态势。</t>
+        </is>
+      </c>
+      <c r="E2280" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2280" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEUVdpmVP9I1PZigrtG5QA260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr">
+        <is>
+          <t>[视频]上半年铁路客运多项指标创新高 激发消费潜能</t>
+        </is>
+      </c>
+      <c r="D2281" t="inlineStr">
+        <is>
+          <t>上半年全国铁路发送旅客23.48亿人次创历史新高，多项并举推动铁路旅游消费。</t>
+        </is>
+      </c>
+      <c r="E2281" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2281" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEOFycie7WoE0GvDAvpaCA260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2282" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr">
+        <is>
+          <t>[视频]金融多向发力 确保夏粮收购平稳有序</t>
+        </is>
+      </c>
+      <c r="D2282" t="inlineStr">
+        <is>
+          <t>金融机构备足信贷资金，创新服务保障夏粮收购，已累计收购小麦超4000万吨。</t>
+        </is>
+      </c>
+      <c r="E2282" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2282" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEBIGlwks1gosaRoYoNyc1260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>经济, 科技, 民生</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2283" t="inlineStr">
+        <is>
+          <t>上半年创新药对外授权交易额超千亿美元；电商物流指数连续四个月回升；塔里木油田供气突破4000亿立方米。</t>
+        </is>
+      </c>
+      <c r="E2283" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2283" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEbXTxx4taFYHfMHlC2xZX260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2284" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】人工智能蓬勃兴起 锻造高质量发展新引擎</t>
+        </is>
+      </c>
+      <c r="D2284" t="inlineStr">
+        <is>
+          <t>我国人工智能产业加速壮大，核心产业规模突破1.2万亿元，综合实力跻身世界第一梯队。</t>
+        </is>
+      </c>
+      <c r="E2284" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2284" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEQe34fGEauaTbkMIsABVg260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>科技, 社会</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者陈俊武：许国七十载 志为石化梦</t>
+        </is>
+      </c>
+      <c r="D2285" t="inlineStr">
+        <is>
+          <t>“七一勋章”获得者陈俊武献身石油工业七十载，攻克炼油技术难题，建成世界首套甲醇制烯烃装置。</t>
+        </is>
+      </c>
+      <c r="E2285" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2285" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEj1FwuUBGWo2zqpgRvlvs260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2286" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr">
+        <is>
+          <t>[视频]美军称打击伊朗防空系统 伊朗称打击美军基地设施</t>
+        </is>
+      </c>
+      <c r="D2286" t="inlineStr">
+        <is>
+          <t>美军打击伊朗防空系统，伊朗反击美军基地，美伊双方对霍尔木兹海峡通行情况说法不一。</t>
+        </is>
+      </c>
+      <c r="E2286" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2286" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEpEMXlwaqdMiZy3d2T6tM260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>军事, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2287" t="inlineStr">
+        <is>
+          <t>俄打击乌港口设施，乌袭击俄炼油厂；国际足联探讨2030年前将世界杯扩至64支球队。</t>
+        </is>
+      </c>
+      <c r="E2287" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2287" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEhAoGje9PBpYTh7P9FfSL260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2288" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr">
+        <is>
+          <t>[视频]国务院印发《国民健康“十五五”规划》</t>
+        </is>
+      </c>
+      <c r="D2288" t="inlineStr">
+        <is>
+          <t>国务院印发《国民健康“十五五”规划》，部署24项重点任务，推动健康中国建设。</t>
+        </is>
+      </c>
+      <c r="E2288" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2288" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEnwAE3nPKNMQ6tQ0x9kcF260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr">
+        <is>
+          <t>[视频]台风“巴威”北上 各地各部门全力应对</t>
+        </is>
+      </c>
+      <c r="D2289" t="inlineStr">
+        <is>
+          <t>台风巴威北上，多地强降雨，各地全力应对，提前转移群众，开展抢险救援。</t>
+        </is>
+      </c>
+      <c r="E2289" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2289" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEXmuxy6aA6UuCYesJvB8Q260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2290" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr">
+        <is>
+          <t>Heatwave to intensify in second week as wildfires burn across UK</t>
+        </is>
+      </c>
+      <c r="D2290" t="inlineStr">
+        <is>
+          <t>英国热浪本周加剧，多地山火肆虐，气温短暂下降后回升。</t>
+        </is>
+      </c>
+      <c r="E2290" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2290" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/c0jyx16ww8jo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr">
+        <is>
+          <t>At least 28 killed, 25 critically injured after fire engulfs Bangkok bar</t>
+        </is>
+      </c>
+      <c r="D2291" t="inlineStr">
+        <is>
+          <t>曼谷一家酒吧起火，造成至少28人死亡、25人重伤，消防员到场时顾客正穿过火焰逃生。</t>
+        </is>
+      </c>
+      <c r="E2291" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2291" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c24yev53q06o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2292" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr">
+        <is>
+          <t>Men disguised as police kill Ecuadorean drug lord's brother</t>
+        </is>
+      </c>
+      <c r="D2292" t="inlineStr">
+        <is>
+          <t>厄瓜多尔毒枭兄弟戴维·马西亚斯遭假扮警察者杀害。</t>
+        </is>
+      </c>
+      <c r="E2292" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2292" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c20yx84g103o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr">
+        <is>
+          <t>German court convicts Iraqi couple of enslaving Yazidi girls</t>
+        </is>
+      </c>
+      <c r="D2293" t="inlineStr">
+        <is>
+          <t>德国法院判一对伊拉克夫妇犯有奴役雅兹迪女孩罪。</t>
+        </is>
+      </c>
+      <c r="E2293" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2293" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cg53rp4e2j4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2294" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr">
+        <is>
+          <t>Heavy rains and flash floods in Bangladesh leave 51 dead</t>
+        </is>
+      </c>
+      <c r="D2294" t="inlineStr">
+        <is>
+          <t>孟加拉国暴雨洪水致51人死亡，数千人无家可归。</t>
+        </is>
+      </c>
+      <c r="E2294" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2294" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce8k7e75k7go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr">
+        <is>
+          <t>Irish police to engage with Jordanian force in murder investigation</t>
+        </is>
+      </c>
+      <c r="D2295" t="inlineStr">
+        <is>
+          <t>爱尔兰警方与约旦警方合作调查贾米·卡尼谋杀案。</t>
+        </is>
+      </c>
+      <c r="E2295" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2295" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c621p1zne6qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2296" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr">
+        <is>
+          <t>British couple return to village at heart of deadly Spanish wildfire</t>
+        </is>
+      </c>
+      <c r="D2296" t="inlineStr">
+        <is>
+          <t>英国夫妇返回西班牙致命野火中心村庄，13人遇难。</t>
+        </is>
+      </c>
+      <c r="E2296" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2296" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx24e09x79no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr">
+        <is>
+          <t>Witness says he crawled for exit as flames swept through Bangkok bar</t>
+        </is>
+      </c>
+      <c r="D2297" t="inlineStr">
+        <is>
+          <t>曼谷酒吧火灾中，一名音乐家爬行逃生，爆炸后被人抛出。</t>
+        </is>
+      </c>
+      <c r="E2297" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2297" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crr8gnx01d7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2298" t="inlineStr">
+        <is>
+          <t>国际, 政治, 军事</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr">
+        <is>
+          <t>The U.S.-Iran ceasefire grows more distant. And, Congress faces a consequential week</t>
+        </is>
+      </c>
+      <c r="D2298" t="inlineStr">
+        <is>
+          <t>美伊在霍尔木兹海峡交火，停火前景渺茫；美国国会面临紧迫议程。</t>
+        </is>
+      </c>
+      <c r="E2298" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2298" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/13/g-s1-133269/up-first-newsletter-us-iran-war-congress-lindsey-graham-gaza-israel-hussam-abu-safiya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr">
+        <is>
+          <t>[视频]【党旗在基层一线高高飘扬】无惧急流 紧急转移被困群众</t>
+        </is>
+      </c>
+      <c r="D2299" t="inlineStr">
+        <is>
+          <t>河北承德消防党员突击队紧急转移被困急流群众，消防员孙聪等人组成人墙，成功解救被困女子。</t>
+        </is>
+      </c>
+      <c r="E2299" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2299" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/13/VIDEdm3YKvL3zva7HOKRj4H3260713.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2300" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr">
+        <is>
+          <t>Wildfire raging south of Paris could have been set deliberately, says minister</t>
+        </is>
+      </c>
+      <c r="D2300" t="inlineStr">
+        <is>
+          <t>巴黎南部野火疑人为纵火，消防飞机首次从南部调往巴黎地区。</t>
+        </is>
+      </c>
+      <c r="E2300" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2300" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clye4z168edo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr">
+        <is>
+          <t>Counter terrorism police take over investigation into Ann Widdecombe's death</t>
+        </is>
+      </c>
+      <c r="D2301" t="inlineStr">
+        <is>
+          <t>反恐警方接手安·威德库姆死亡案，拘留嫌疑人因涉嫌恐怖主义活动。</t>
+        </is>
+      </c>
+      <c r="E2301" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2301" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0mydjl12mwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2302" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr">
+        <is>
+          <t>Twelve arrested over alleged right-wing terror threat to UK Islamic event, police say</t>
+        </is>
+      </c>
+      <c r="D2302" t="inlineStr">
+        <is>
+          <t>英国警方逮捕12人，涉嫌策划对伊斯兰活动的极右翼恐怖袭击。</t>
+        </is>
+      </c>
+      <c r="E2302" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2302" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgl20x1ggpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr">
+        <is>
+          <t>UK seeking extradition of man suspected of killing wife and two daughters</t>
+        </is>
+      </c>
+      <c r="D2303" t="inlineStr">
+        <is>
+          <t>英国寻求引渡一名涉嫌杀害妻子和两名女儿的男子。</t>
+        </is>
+      </c>
+      <c r="E2303" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2303" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy8w61qz873o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2304" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr">
+        <is>
+          <t>Pilot writes 'I'm bored' in sky during flight</t>
+        </is>
+      </c>
+      <c r="D2304" t="inlineStr">
+        <is>
+          <t>飞行员在飞行途中用航迹写出“我很无聊”，被飞行追踪软件爱好者发现。</t>
+        </is>
+      </c>
+      <c r="E2304" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2304" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy5vx19ey0wo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>文体, 国际</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr">
+        <is>
+          <t>'Hero, legend, sweetheart': Tributes to Jurassic Park actor Sam Neill, who has died aged 78</t>
+        </is>
+      </c>
+      <c r="D2305" t="inlineStr">
+        <is>
+          <t>《侏罗纪公园》演员萨姆·尼尔去世，享年78岁，各界人士悼念。</t>
+        </is>
+      </c>
+      <c r="E2305" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2305" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy06e5e1lygo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2306" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr">
+        <is>
+          <t>A versatile actor whose roles went far beyond Jurassic Park - Sam Neill dies aged 78</t>
+        </is>
+      </c>
+      <c r="D2306" t="inlineStr">
+        <is>
+          <t>演员萨姆·尼尔去世，享年78岁，其五十年职业生涯塑造众多经典角色。</t>
+        </is>
+      </c>
+      <c r="E2306" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2306" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2wrvqq9rlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr">
+        <is>
+          <t>Most clinical? Least creative? BBC Sport compares the last four teams in the World Cup</t>
+        </is>
+      </c>
+      <c r="D2307" t="inlineStr">
+        <is>
+          <t>BBC对比世界杯四强法国、西班牙、阿根廷、英格兰数据，分析优劣。</t>
+        </is>
+      </c>
+      <c r="E2307" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2307" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cx2k9qj2nyvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr">
+        <is>
+          <t>Sam Neill, known for 'Jurassic Park' and 'The Piano,' dies at 78, his family says</t>
+        </is>
+      </c>
+      <c r="D2308" t="inlineStr">
+        <is>
+          <t>《侏罗纪公园》演员萨姆·尼尔因罕见淋巴瘤在悉尼去世，享年78岁。</t>
+        </is>
+      </c>
+      <c r="E2308" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2308" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/13/nx-s1-5891505/actor-sam-neill-dies</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-14
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2308"/>
+  <dimension ref="A1:F2344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74293,6 +74293,1158 @@
         </is>
       </c>
     </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260714 19:00</t>
+        </is>
+      </c>
+      <c r="D2309" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平人工智能开放共赢理念、王沪宁会见越南代表团及访朝等多项重要新闻。</t>
+        </is>
+      </c>
+      <c r="E2309" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2309" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEG9R1UFyTeQvba5tybD0K260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2310" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr">
+        <is>
+          <t>[视频]《习近平谈治国理政》第五卷吉尔吉斯斯坦推介会在比什凯克举行</t>
+        </is>
+      </c>
+      <c r="D2310" t="inlineStr">
+        <is>
+          <t>《习近平谈治国理政》第五卷吉尔吉斯斯坦推介会在比什凯克举行。</t>
+        </is>
+      </c>
+      <c r="E2310" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2310" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDETQ7oDuPGkledhEYronWA260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁会见越南共产党代表团</t>
+        </is>
+      </c>
+      <c r="D2311" t="inlineStr">
+        <is>
+          <t>王沪宁在京会见越南共产党代表团，双方愿推动中越命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E2311" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2311" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDE7hUQ7Zn0kqhWglIwqTrV260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2312" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁将访问朝鲜</t>
+        </is>
+      </c>
+      <c r="D2312" t="inlineStr">
+        <is>
+          <t>王沪宁将于7月15日至17日率团对朝鲜进行正式友好访问。</t>
+        </is>
+      </c>
+      <c r="E2312" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2312" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDExo7I2SGiBeIMe7ANlV8K260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr">
+        <is>
+          <t>[视频]中央党校（国家行政学院）举行2026年春季学期毕业典礼 蔡奇出席并为学员颁发毕业证书</t>
+        </is>
+      </c>
+      <c r="D2313" t="inlineStr">
+        <is>
+          <t>中央党校举行2026年春季学期毕业典礼，蔡奇出席并颁发证书。</t>
+        </is>
+      </c>
+      <c r="E2313" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2313" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEZEkBaT4nsZLvOm7IH2WZ260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2314" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr">
+        <is>
+          <t>[视频]中共中央决定给予马兴瑞开除党籍、开除公职处分</t>
+        </is>
+      </c>
+      <c r="D2314" t="inlineStr">
+        <is>
+          <t>中共中央决定给予马兴瑞开除党籍、开除公职处分。</t>
+        </is>
+      </c>
+      <c r="E2314" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2314" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDElUJ9x73ckQ23CB9qEPYe260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr">
+        <is>
+          <t>[视频]我国将不断完善自然资源资产监督考核</t>
+        </is>
+      </c>
+      <c r="D2315" t="inlineStr">
+        <is>
+          <t>我国将完善自然资源资产管理责任考核，探索损害赔偿机制，引导正确政绩观。</t>
+        </is>
+      </c>
+      <c r="E2315" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2315" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEaEHcbroTZ5O9TkgT7OP0260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2316" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr">
+        <is>
+          <t>Singapore court orders Bloomberg to pay $356,000 to ministers in defamation case</t>
+        </is>
+      </c>
+      <c r="D2316" t="inlineStr">
+        <is>
+          <t>新加坡法院判彭博社因报道部长豪华平房交易诽谤，需赔偿35.6万美元。</t>
+        </is>
+      </c>
+      <c r="E2316" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2316" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx232p85lp5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr">
+        <is>
+          <t>MPs expected to approve long-delayed 'Hillsborough Law'</t>
+        </is>
+      </c>
+      <c r="D2317" t="inlineStr">
+        <is>
+          <t>英国议会预计将批准长期拖延的“希尔斯堡法案”，首相斯塔默任内最后推动。</t>
+        </is>
+      </c>
+      <c r="E2317" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2317" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9q2qwnvd75o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2318" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr">
+        <is>
+          <t>Government failing Farage over security, says Jenrick</t>
+        </is>
+      </c>
+      <c r="D2318" t="inlineStr">
+        <is>
+          <t>詹里克称政府对法拉奇的安保不力，安·维德库姆之死引发政治人物安全讨论。</t>
+        </is>
+      </c>
+      <c r="E2318" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2318" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyg9452qlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr">
+        <is>
+          <t>[视频]今年上半年我国货物贸易进出口同比增长16.9%</t>
+        </is>
+      </c>
+      <c r="D2319" t="inlineStr">
+        <is>
+          <t>上半年我国货物贸易进出口25.47万亿元，同比增长16.9%。</t>
+        </is>
+      </c>
+      <c r="E2319" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2319" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEftty4i8DZlSlVRJMvYWo260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2320" t="inlineStr">
+        <is>
+          <t>经济, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2320" t="inlineStr">
+        <is>
+          <t>十五五规划促消费，新能源汽车注册占比近半，医保参保人数增加。</t>
+        </is>
+      </c>
+      <c r="E2320" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2320" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEaARM9uaeZa49sNuEmVIx260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr">
+        <is>
+          <t>Diamond giant De Beers halts work at flagship South African mine as demand plummets</t>
+        </is>
+      </c>
+      <c r="D2321" t="inlineStr">
+        <is>
+          <t>钻石巨头戴比尔斯因需求暴跌，暂停南非旗舰矿生产两年，影响超4000名员工。</t>
+        </is>
+      </c>
+      <c r="E2321" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2321" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjrgr7lr1ejo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2322" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】开放共赢 促进人工智能更好造福各国人民</t>
+        </is>
+      </c>
+      <c r="D2322" t="inlineStr">
+        <is>
+          <t>习近平指出人工智能应造福各国人民，中国以开放姿态促进全球AI协同与普惠发展。</t>
+        </is>
+      </c>
+      <c r="E2322" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2322" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEfeBuLeLMo0zbla4ysIdQ260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr">
+        <is>
+          <t>[视频]【活力中国调研行】“拔节生长”的未来之城</t>
+        </is>
+      </c>
+      <c r="D2323" t="inlineStr">
+        <is>
+          <t>雄安新区与北京形成创新共同体，协同推动技术落地与产业转化。</t>
+        </is>
+      </c>
+      <c r="E2323" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2323" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDE8y6QS0yLOjWqjMOG2SE5260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2324" t="inlineStr">
+        <is>
+          <t>军事, 国际, 经济</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr">
+        <is>
+          <t>[视频]美军称打击伊朗海岸防御系统 伊朗称打击巴林美军第五舰队基地</t>
+        </is>
+      </c>
+      <c r="D2324" t="inlineStr">
+        <is>
+          <t>美军打击伊朗海岸系统，伊朗回击美军基地，国际油价大涨。</t>
+        </is>
+      </c>
+      <c r="E2324" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2324" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDErYz0d70vCQ0rYRKD6GiF260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr">
+        <is>
+          <t>[视频]也门萨那机场遭袭 胡塞武装回击沙特一机场</t>
+        </is>
+      </c>
+      <c r="D2325" t="inlineStr">
+        <is>
+          <t>也门萨那机场遭沙特空袭，胡塞武装回击沙特机场，局势紧张。</t>
+        </is>
+      </c>
+      <c r="E2325" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2325" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEtemzjG69wQ7HkrdBOSMg260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2326" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr">
+        <is>
+          <t>Israeli strike on police post in north Gaza kills seven, officials say</t>
+        </is>
+      </c>
+      <c r="D2326" t="inlineStr">
+        <is>
+          <t>以军空袭加沙北部警察哨所，致7人死亡，包括一名哈马斯高级警官。</t>
+        </is>
+      </c>
+      <c r="E2326" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2326" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cqj1jqeyl5ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr">
+        <is>
+          <t>Yemen's Houthis launch missiles at Saudi Arabia after strikes on Sanaa airport</t>
+        </is>
+      </c>
+      <c r="D2327" t="inlineStr">
+        <is>
+          <t>也门胡塞武装向沙特发射导弹，报复其空袭萨那机场，威胁进一步行动。</t>
+        </is>
+      </c>
+      <c r="E2327" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2327" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp9ldle3d3xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2328" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr">
+        <is>
+          <t>[视频]各地各部门多措施应对台风“巴威”影响</t>
+        </is>
+      </c>
+      <c r="D2328" t="inlineStr">
+        <is>
+          <t>台风“巴威”致东北多地暴雨，辽宁、吉林受灾严重，各部门全力应对。</t>
+        </is>
+      </c>
+      <c r="E2328" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2328" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDEJb7PuinmnFrGv8ylczTk260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>民生, 经济</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr">
+        <is>
+          <t>UK wasted £10bn on PPE that left NHS staff poorly protected, Covid inquiry finds</t>
+        </is>
+      </c>
+      <c r="D2329" t="inlineStr">
+        <is>
+          <t>新冠调查发现英国浪费100亿英镑购买个人防护装备，导致医护人员保护不足。</t>
+        </is>
+      </c>
+      <c r="E2329" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2329" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czrxrlydyzzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2330" t="inlineStr">
+        <is>
+          <t>国际, 军事, 文体</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2330" t="inlineStr">
+        <is>
+          <t>涉乌多国部队将演习，古巴谴责美国制裁，国际乒联恢复俄运动员资格。</t>
+        </is>
+      </c>
+      <c r="E2330" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2330" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/14/VIDELp8U0ue2BbdBFkuWwxRb260714.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr">
+        <is>
+          <t>How US commerce secretary's Epstein links were uncovered by British whistleblower</t>
+        </is>
+      </c>
+      <c r="D2331" t="inlineStr">
+        <is>
+          <t>英国揭发者从公开的爱泼斯坦文件中发现美国商务部长与爱泼斯坦关联。</t>
+        </is>
+      </c>
+      <c r="E2331" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2331" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9q28dlyxrzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2332" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr">
+        <is>
+          <t>U.S. to reinstate Hormuz blockade. And, states sue over Paramount-Warner deal</t>
+        </is>
+      </c>
+      <c r="D2332" t="inlineStr">
+        <is>
+          <t>美国计划恢复霍尔木兹海峡封锁，多州起诉阻止派拉蒙-华纳合并。</t>
+        </is>
+      </c>
+      <c r="E2332" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2332" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/14/g-s1-133443/up-first-newsletter-iran-strait-hormuz-maine-ice-shooting-paramount-warner-bros-merger</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr">
+        <is>
+          <t>The U.S. is set to reinstate a blockade over the Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D2333" t="inlineStr">
+        <is>
+          <t>美方宣布周二恢复对伊朗船只的霍尔木兹海峡封锁，伊朗誓言维护控制权。</t>
+        </is>
+      </c>
+      <c r="E2333" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2333" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/14/nx-s1-5893257/us-iran-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2334" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr">
+        <is>
+          <t>'If we die, we die together': Wife of man nearly sucked out of Ryanair plane speaks of ordeal</t>
+        </is>
+      </c>
+      <c r="D2334" t="inlineStr">
+        <is>
+          <t>瑞安航空乘客险被吸出机舱，其妻称丈夫重伤休克，讲述惊魂经历。</t>
+        </is>
+      </c>
+      <c r="E2334" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2334" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly8yjnw822o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr">
+        <is>
+          <t>Bangkok fire investigation finds locked doors and flammable decor as deaths climb to 30</t>
+        </is>
+      </c>
+      <c r="D2335" t="inlineStr">
+        <is>
+          <t>曼谷火灾调查：门被锁、装饰易燃致30死，幸存者称缺少紧急出口标识。</t>
+        </is>
+      </c>
+      <c r="E2335" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2335" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyxyzlp9p2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2336" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr">
+        <is>
+          <t>Australian police reveal unseen photos 25 years after British backpacker murder</t>
+        </is>
+      </c>
+      <c r="D2336" t="inlineStr">
+        <is>
+          <t>澳洲警方在英背包客谋杀案25年后公布未公开照片，冀寻线索找遗体。</t>
+        </is>
+      </c>
+      <c r="E2336" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2336" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crlwln0gkzlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>社会, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr">
+        <is>
+          <t>Colombian national killed by ICE agent during operation in Maine</t>
+        </is>
+      </c>
+      <c r="D2337" t="inlineStr">
+        <is>
+          <t>一名哥伦比亚公民在缅因州被ICE探员在行动中击毙，一周内第二起类似事件。</t>
+        </is>
+      </c>
+      <c r="E2337" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2337" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2ly580kxnko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2338" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2338" t="inlineStr">
+        <is>
+          <t>Identity of Sydney daycare worker facing 329 child abuse offences revealed</t>
+        </is>
+      </c>
+      <c r="D2338" t="inlineStr">
+        <is>
+          <t>悉尼托儿所员工哈米什·泰特被指控在16年内虐待136名儿童，面临329项罪名。</t>
+        </is>
+      </c>
+      <c r="E2338" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2338" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yzy0lpello?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr">
+        <is>
+          <t>Wildfires burn in parts of UK as fire chiefs warn of extreme pressure</t>
+        </is>
+      </c>
+      <c r="D2339" t="inlineStr">
+        <is>
+          <t>英国多地发生野火，消防部门警告压力巨大，北威尔士等地宣布重大事件。</t>
+        </is>
+      </c>
+      <c r="E2339" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2339" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyey14r4wzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2340" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2340" t="inlineStr">
+        <is>
+          <t>Man who staged wife's suicide jailed for  murder</t>
+        </is>
+      </c>
+      <c r="D2340" t="inlineStr">
+        <is>
+          <t>男子伪造妻子自杀被判谋杀罪，女儿在法庭上称其为“善妒、狡猾、自恋的恶棍”。</t>
+        </is>
+      </c>
+      <c r="E2340" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2340" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8626147e6no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2341" t="inlineStr">
+        <is>
+          <t>社会, 军事</t>
+        </is>
+      </c>
+      <c r="C2341" t="inlineStr">
+        <is>
+          <t>Families of RAF Chinook crash victims ask court to allow case to proceed</t>
+        </is>
+      </c>
+      <c r="D2341" t="inlineStr">
+        <is>
+          <t>1994年苏格兰奇努克直升机坠毁，29人遇难，遇难者家属请求法院允许案件继续审理。</t>
+        </is>
+      </c>
+      <c r="E2341" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2341" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crm0mkgxn9eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2342" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2342" t="inlineStr">
+        <is>
+          <t>Death toll from a Bangkok music bar fire rises to 30, dozens remain in hospital</t>
+        </is>
+      </c>
+      <c r="D2342" t="inlineStr">
+        <is>
+          <t>曼谷音乐酒吧火灾死亡人数升至30人，数十人住院，其中24人危重。</t>
+        </is>
+      </c>
+      <c r="E2342" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2342" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/14/g-s1-133425/death-toll-bangkok-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2343" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2343" t="inlineStr">
+        <is>
+          <t>Scott Mills was highest-paid BBC star before sacking</t>
+        </is>
+      </c>
+      <c r="D2343" t="inlineStr">
+        <is>
+          <t>前BBC广播二台主持人斯科特·米尔斯在上个财年赚取约74.5万英镑，后被解雇。</t>
+        </is>
+      </c>
+      <c r="E2343" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2343" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gynyz4wqpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B2344" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2344" t="inlineStr">
+        <is>
+          <t>Who will win the World Cup? The view from the semi-finalists' countries</t>
+        </is>
+      </c>
+      <c r="D2344" t="inlineStr">
+        <is>
+          <t>BBC体育采访四强国家的记者和球迷，探讨谁将赢得世界杯。</t>
+        </is>
+      </c>
+      <c r="E2344" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2344" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cjrgew3wv4xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-15
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2344"/>
+  <dimension ref="A1:F2383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75445,6 +75445,1254 @@
         </is>
       </c>
     </row>
+    <row r="2345">
+      <c r="A2345" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2345" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2345" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260715 19:00</t>
+        </is>
+      </c>
+      <c r="D2345" t="inlineStr">
+        <is>
+          <t>今日新闻联播主要内容涵盖习总书记考察上海、经济数据发布、防汛抢险、国际交往等。</t>
+        </is>
+      </c>
+      <c r="E2345" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2345" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEKrHkAz5OMOZIdqiBAQqI260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2346" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2346" t="inlineStr">
+        <is>
+          <t>[视频]习近平在上海考察时强调 全面践行人民城市理念 高质量推进城市更新</t>
+        </is>
+      </c>
+      <c r="D2346" t="inlineStr">
+        <is>
+          <t>习近平在上海考察，强调全面践行人民城市理念，高质量推进城市更新。</t>
+        </is>
+      </c>
+      <c r="E2346" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2346" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEL58MxDoQQygMG2x4IlyF260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2347" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2347" t="inlineStr">
+        <is>
+          <t>[视频]韩正会见新西兰前总理</t>
+        </is>
+      </c>
+      <c r="D2347" t="inlineStr">
+        <is>
+          <t>国家副主席韩正会见新西兰前总理约翰·基，共促中新关系发展。</t>
+        </is>
+      </c>
+      <c r="E2347" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2347" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEwGurfLWAl06VXfqTOoh7260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2348" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2348" t="inlineStr">
+        <is>
+          <t>Italy's Meloni suffers surprise setback in close vote on electoral reform</t>
+        </is>
+      </c>
+      <c r="D2348" t="inlineStr">
+        <is>
+          <t>意大利总理梅洛尼在选举改革投票中意外受挫，反对派要求其辞职。</t>
+        </is>
+      </c>
+      <c r="E2348" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2348" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1kykx3vnyyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2349" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2349" t="inlineStr">
+        <is>
+          <t>Venezuela government to launch formal talks with opposition members</t>
+        </is>
+      </c>
+      <c r="D2349" t="inlineStr">
+        <is>
+          <t>委内瑞拉政府将启动与反对派的正式对话，旨在加强民主制度。</t>
+        </is>
+      </c>
+      <c r="E2349" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2349" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1eye5320g5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2350" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2350" t="inlineStr">
+        <is>
+          <t>Sierra Leone drops treason charge against ex-president over attempted coup</t>
+        </is>
+      </c>
+      <c r="D2350" t="inlineStr">
+        <is>
+          <t>塞拉利昂撤销对前总统科罗马的叛国罪指控，其曾涉未遂政变。</t>
+        </is>
+      </c>
+      <c r="E2350" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2350" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2w2k3vklgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2351" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2351" t="inlineStr">
+        <is>
+          <t>Starmer says it's the 'end of my political journey' at his final Prime Minister's Questions</t>
+        </is>
+      </c>
+      <c r="D2351" t="inlineStr">
+        <is>
+          <t>斯塔默在最后一次首相质询中称其“政治旅程结束”，议员纷纷致意。</t>
+        </is>
+      </c>
+      <c r="E2351" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2351" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5yzynxwk05o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2352" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2352" t="inlineStr">
+        <is>
+          <t>Watch Starmer sign off final PMQs to standing ovation</t>
+        </is>
+      </c>
+      <c r="D2352" t="inlineStr">
+        <is>
+          <t>首相斯塔默在最后一次首相问答中获得全场起立鼓掌致意。</t>
+        </is>
+      </c>
+      <c r="E2352" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2352" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c07y74d8y51o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2353" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2353" t="inlineStr">
+        <is>
+          <t>Acting AG Todd Blanche faces a key test. And, ICE pauses most traffic stops</t>
+        </is>
+      </c>
+      <c r="D2353" t="inlineStr">
+        <is>
+          <t>代理司法部长布兰奇面临参议院确认听证；ICE暂停多数交通拦截。</t>
+        </is>
+      </c>
+      <c r="E2353" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2353" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/g-s1-133652/up-first-newsletter-todd-blanche-iran-strait-of-hormuz-ice-traffic-stops</t>
+        </is>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2354" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2354" t="inlineStr">
+        <is>
+          <t>[视频]上半年GDP同比增长4.7% 中国经济持续向新向优</t>
+        </is>
+      </c>
+      <c r="D2354" t="inlineStr">
+        <is>
+          <t>上半年中国GDP同比增长4.7%，经济展现韧性和活力，向新向优。</t>
+        </is>
+      </c>
+      <c r="E2354" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2354" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDE8J9TYzFLiE5b1K2LRplB260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2355" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2355" t="inlineStr">
+        <is>
+          <t>[视频]上半年金融总量合理增长 信贷结构持续优化</t>
+        </is>
+      </c>
+      <c r="D2355" t="inlineStr">
+        <is>
+          <t>上半年金融总量合理增长，信贷结构优化，支持实体经济和科技创新。</t>
+        </is>
+      </c>
+      <c r="E2355" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2355" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEbl9MSW2SR3clyLeIrmgV260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2356" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2356" t="inlineStr">
+        <is>
+          <t>[视频]我国持续推进农村公路提质升级</t>
+        </is>
+      </c>
+      <c r="D2356" t="inlineStr">
+        <is>
+          <t>我国推进农村公路提质升级，上半年新改建3.4万公里，提升服务能力。</t>
+        </is>
+      </c>
+      <c r="E2356" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2356" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEkMaaOLIklaVRWa0Saofq260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2357" t="inlineStr">
+        <is>
+          <t>经济, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2357" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2357" t="inlineStr">
+        <is>
+          <t>我国将建200个“无废城市”；上半年用电量增5.3%；一线城市房价环比上涨；AI服务新规施行。</t>
+        </is>
+      </c>
+      <c r="E2357" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2357" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDE3MXgBsu7acTDnbo7Zt8j260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2358" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2358" t="inlineStr">
+        <is>
+          <t>China economic growth falls sharply, missing target</t>
+        </is>
+      </c>
+      <c r="D2358" t="inlineStr">
+        <is>
+          <t>中国经济增长大幅下滑，未达目标，受国内需求疲软和伊朗战争影响。</t>
+        </is>
+      </c>
+      <c r="E2358" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2358" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cd959x4edy8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2359" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2359" t="inlineStr">
+        <is>
+          <t>China's economy grows 4.3% in Q2, slowest since late 2022</t>
+        </is>
+      </c>
+      <c r="D2359" t="inlineStr">
+        <is>
+          <t>中国第二季度经济增长4.3%，为2022年底以来最慢。</t>
+        </is>
+      </c>
+      <c r="E2359" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2359" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/g-s1-133672/chinas-economy-grows-4-3-in-q2-slowest-since-late-2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2360" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2360" t="inlineStr">
+        <is>
+          <t>American AI is expensive. Some startups are turning to cheap Chinese models</t>
+        </is>
+      </c>
+      <c r="D2360" t="inlineStr">
+        <is>
+          <t>美国AI成本高昂，部分初创公司转向廉价中国AI模型。</t>
+        </is>
+      </c>
+      <c r="E2360" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2360" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/nx-s1-5886476/startups-cheap-chinese-ai-models</t>
+        </is>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2361" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2361" t="inlineStr">
+        <is>
+          <t>[视频]美国称对伊朗实施打击并恢复海上封锁 伊朗称打击地区内美军基地</t>
+        </is>
+      </c>
+      <c r="D2361" t="inlineStr">
+        <is>
+          <t>美伊冲突升级：美国打击伊朗沿海目标并恢复海上封锁，伊朗袭击多国美军基地。</t>
+        </is>
+      </c>
+      <c r="E2361" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2361" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDE3lZ2PTxNJNuPOH1RbDwg260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2362" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2362" t="inlineStr">
+        <is>
+          <t>Iran threatens to block more trade routes as US launches fresh strikes</t>
+        </is>
+      </c>
+      <c r="D2362" t="inlineStr">
+        <is>
+          <t>美国总统特朗普威胁称，若伊朗不重返谈判，下周将打击其桥梁和发电厂。</t>
+        </is>
+      </c>
+      <c r="E2362" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2362" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9323zgq6wvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2363" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2363" t="inlineStr">
+        <is>
+          <t>Russian attacks kill eight as Ukraine hits Black Sea oil tankers</t>
+        </is>
+      </c>
+      <c r="D2363" t="inlineStr">
+        <is>
+          <t>俄袭击乌克兰致8人死亡；乌克兰击中黑海20艘俄油轮。</t>
+        </is>
+      </c>
+      <c r="E2363" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2363" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8929jv8kdzo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2364" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2364" t="inlineStr">
+        <is>
+          <t>Retired vice admiral on whether the U.S. can control the Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D2364" t="inlineStr">
+        <is>
+          <t>退役中将谈美国控制霍尔木兹海峡的能力，曾指挥第五舰队。</t>
+        </is>
+      </c>
+      <c r="E2364" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2364" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/nx-s1-5893471/retired-vice-admiral-on-whether-the-u-s-can-control-the-strait-of-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2365" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2365" t="inlineStr">
+        <is>
+          <t>[视频]东北地区全力开展防汛抢险排涝工作</t>
+        </is>
+      </c>
+      <c r="D2365" t="inlineStr">
+        <is>
+          <t>东北地区持续强降雨，各地全力开展防汛抢险排涝和群众转移工作。</t>
+        </is>
+      </c>
+      <c r="E2365" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2365" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEL6DTeyu5BjrKXReD5WDg260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2366" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2366" t="inlineStr">
+        <is>
+          <t>Heatwave prompts Italy's delivery riders to strike for extra rights</t>
+        </is>
+      </c>
+      <c r="D2366" t="inlineStr">
+        <is>
+          <t>意大利热浪导致外卖骑手罢工，要求保障健康与工资权益。</t>
+        </is>
+      </c>
+      <c r="E2366" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2366" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c1dydw0r246o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2367" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C2367" t="inlineStr">
+        <is>
+          <t>Tourists warned of methanol poisoning risks in new campaign</t>
+        </is>
+      </c>
+      <c r="D2367" t="inlineStr">
+        <is>
+          <t>新活动提醒游客警惕甲醇中毒风险及症状。</t>
+        </is>
+      </c>
+      <c r="E2367" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2367" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9929dg5l5lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2368" t="inlineStr">
+        <is>
+          <t>国际</t>
+        </is>
+      </c>
+      <c r="C2368" t="inlineStr">
+        <is>
+          <t>[视频]2026上合组织国家文明对话在比什凯克举行</t>
+        </is>
+      </c>
+      <c r="D2368" t="inlineStr">
+        <is>
+          <t>2026上合组织国家文明对话在比什凯克举行，强调文明互鉴与务实合作。</t>
+        </is>
+      </c>
+      <c r="E2368" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2368" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEYbKj6DV7QwudgrFq9KvQ260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2369" t="inlineStr">
+        <is>
+          <t>国际, 经济</t>
+        </is>
+      </c>
+      <c r="C2369" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2369" t="inlineStr">
+        <is>
+          <t>黎以举行新一轮会谈；欧盟对俄液化天然气进口创纪录；美联储主席称高通胀是过度负担。</t>
+        </is>
+      </c>
+      <c r="E2369" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2369" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDERzBYh6qjnb9TE7P2B3Fr260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2370" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2370" t="inlineStr">
+        <is>
+          <t>Seven Britons among those killed in Spain wildfires</t>
+        </is>
+      </c>
+      <c r="D2370" t="inlineStr">
+        <is>
+          <t>西班牙野火致七名英国人遇难，13名死者中12人为外国公民。</t>
+        </is>
+      </c>
+      <c r="E2370" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2370" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp8l87784ngo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2371" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2371" t="inlineStr">
+        <is>
+          <t>The U.S. and Iran standoff over the Strait of Hormuz intensifies</t>
+        </is>
+      </c>
+      <c r="D2371" t="inlineStr">
+        <is>
+          <t>伊朗威胁封锁霍尔木兹海峡石油航线，回应美国海上封锁。</t>
+        </is>
+      </c>
+      <c r="E2371" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2371" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/nx-s1-5894582/us-iran-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2372" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2372" t="inlineStr">
+        <is>
+          <t>Ebola is spreading faster in eastern Congo than it can be tracked, as deaths pass 700</t>
+        </is>
+      </c>
+      <c r="D2372" t="inlineStr">
+        <is>
+          <t>刚果埃博拉疫情传播速度超追踪能力，死亡人数超700。</t>
+        </is>
+      </c>
+      <c r="E2372" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2372" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/g-s1-133630/ebola-congo-deaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2373" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2373" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】办好群众身边事 学习教育见实效</t>
+        </is>
+      </c>
+      <c r="D2373" t="inlineStr">
+        <is>
+          <t>河南新乡、西藏那曲践行正确政绩观，解决群众健身、洗澡等身边事。</t>
+        </is>
+      </c>
+      <c r="E2373" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2373" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEBtmxjmrJ7yVZNiRqGel0260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2374" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2374" t="inlineStr">
+        <is>
+          <t>[视频]【文化中国行】呵护古城肌理 赓续千年姑苏繁华</t>
+        </is>
+      </c>
+      <c r="D2374" t="inlineStr">
+        <is>
+          <t>苏州以“绣花功夫”保护古城，活化历史文化资源，实现城市更新与文脉赓续相融共生。</t>
+        </is>
+      </c>
+      <c r="E2374" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2374" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/15/VIDEZP1Uhfyb1pgWbiGt5JBR260715.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2375" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2375" t="inlineStr">
+        <is>
+          <t>Rastafarians in Kenya fail in bid to get cannabis legalised for religious purposes</t>
+        </is>
+      </c>
+      <c r="D2375" t="inlineStr">
+        <is>
+          <t>肯尼亚法院驳回拉斯特法里教徒为宗教目的合法化大麻的请求。</t>
+        </is>
+      </c>
+      <c r="E2375" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2375" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0lyl5ryyr4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2376" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2376" t="inlineStr">
+        <is>
+          <t>Air India crash report likely to be ready in October, say investigators</t>
+        </is>
+      </c>
+      <c r="D2376" t="inlineStr">
+        <is>
+          <t>印度航空坠机事故调查报告预计十月完成，事故致260人遇难。</t>
+        </is>
+      </c>
+      <c r="E2376" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2376" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjrgrgx2d9qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2377" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2377" t="inlineStr">
+        <is>
+          <t>Man arrested over threatening to shoot Farage in social media post</t>
+        </is>
+      </c>
+      <c r="D2377" t="inlineStr">
+        <is>
+          <t>一名男子因在社交媒体上威胁要枪击法拉奇被捕。</t>
+        </is>
+      </c>
+      <c r="E2377" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2377" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c8r2r76vnd1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2378" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2378" t="inlineStr">
+        <is>
+          <t>Three men who raped woman on Brighton beach jailed</t>
+        </is>
+      </c>
+      <c r="D2378" t="inlineStr">
+        <is>
+          <t>三名男子因在布莱顿海滩强奸女性被判入狱。</t>
+        </is>
+      </c>
+      <c r="E2378" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2378" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cyv0vqp04pgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2379" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2379" t="inlineStr">
+        <is>
+          <t>UK's extreme weather is the new normal, Met Office says</t>
+        </is>
+      </c>
+      <c r="D2379" t="inlineStr">
+        <is>
+          <t>英国气象局称极端天气已成新常态，寒冷山区也在消失。</t>
+        </is>
+      </c>
+      <c r="E2379" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2379" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c802041g4v8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2380" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2380" t="inlineStr">
+        <is>
+          <t>Midnight social media curfew proposed for UK teens aged 16 and 17 - but they can opt out</t>
+        </is>
+      </c>
+      <c r="D2380" t="inlineStr">
+        <is>
+          <t>英国拟对16-17岁青少年实施午夜社交媒体宵禁，但可选择退出。</t>
+        </is>
+      </c>
+      <c r="E2380" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2380" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c982857nlrlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2381" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2381" t="inlineStr">
+        <is>
+          <t>Greetings from Paris, where an art installation transformed the Pont Neuf into a rocky cave</t>
+        </is>
+      </c>
+      <c r="D2381" t="inlineStr">
+        <is>
+          <t>巴黎最老桥被艺术家JR用织物变成岩洞装置，但未缓解热浪。</t>
+        </is>
+      </c>
+      <c r="E2381" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2381" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/g-s1-132781/paris-heat-pont-neuf-jr-cave-caverne</t>
+        </is>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2382" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2382" t="inlineStr">
+        <is>
+          <t>England close in on immortality with biggest match since 1966</t>
+        </is>
+      </c>
+      <c r="D2382" t="inlineStr">
+        <is>
+          <t>英格兰队将在世界杯半决赛对阵阿根廷，称1966年以来最重要比赛。</t>
+        </is>
+      </c>
+      <c r="E2382" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2382" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c20y0zzdx9go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2383" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2383" t="inlineStr">
+        <is>
+          <t>Old rivals, new battle: Argentina and England clash in World Cup Semifinal</t>
+        </is>
+      </c>
+      <c r="D2383" t="inlineStr">
+        <is>
+          <t>阿根廷与英格兰将在世界杯半决赛中争夺决赛席位。</t>
+        </is>
+      </c>
+      <c r="E2383" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2383" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/15/nx-s1-5893686/old-rivals-new-battle-argentina-and-england-clash-in-world-cup-semifinal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-16
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2383"/>
+  <dimension ref="A1:F2422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76693,6 +76693,1254 @@
         </is>
       </c>
     </row>
+    <row r="2384">
+      <c r="A2384" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2384" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2384" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260716 19:00</t>
+        </is>
+      </c>
+      <c r="D2384" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平会见哈总统、发表文章、上海考察反响、李强会谈等多项国内外要闻。</t>
+        </is>
+      </c>
+      <c r="E2384" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2384" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEzcwJJbxOoVpSM9e5zTk2260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2385" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2385" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见哈萨克斯坦总统</t>
+        </is>
+      </c>
+      <c r="D2385" t="inlineStr">
+        <is>
+          <t>习近平会见哈萨克斯坦总统，强调中哈关系历久弥坚，加强全面合作与战略对接。</t>
+        </is>
+      </c>
+      <c r="E2385" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2385" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDENqqswxVEagbGNVZdPKhk260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2386" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2386" t="inlineStr">
+        <is>
+          <t>[视频]《求是》杂志发表习近平总书记重要文章《在庆祝中国共产党成立105周年大会上的讲话》</t>
+        </is>
+      </c>
+      <c r="D2386" t="inlineStr">
+        <is>
+          <t>《求是》发表习近平重要文章，阐述中共105年奋斗成就与优秀特质。</t>
+        </is>
+      </c>
+      <c r="E2386" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2386" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEityfpJKn8vaq4eYywf8L260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2387" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2387" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：全面践行人民城市理念</t>
+        </is>
+      </c>
+      <c r="D2387" t="inlineStr">
+        <is>
+          <t>央视快评号召全面践行人民城市理念。</t>
+        </is>
+      </c>
+      <c r="E2387" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2387" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEUwb8l7V6AdEJ8bDy4Xs2260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2388" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2388" t="inlineStr">
+        <is>
+          <t>[视频]《习近平谈治国理政》第五卷哈萨克斯坦推介会在阿斯塔纳举行</t>
+        </is>
+      </c>
+      <c r="D2388" t="inlineStr">
+        <is>
+          <t>《习近平谈治国理政》第五卷在哈萨克斯坦举行推介会。</t>
+        </is>
+      </c>
+      <c r="E2388" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2388" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEwTXlbaJU9RRCA4g1p78j260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2389" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2389" t="inlineStr">
+        <is>
+          <t>[视频]李强同柬埔寨首相会谈</t>
+        </is>
+      </c>
+      <c r="D2389" t="inlineStr">
+        <is>
+          <t>李强同柬埔寨首相会谈，谈深化基建、贸易、新能源合作及打击网赌电诈。</t>
+        </is>
+      </c>
+      <c r="E2389" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2389" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEH7f29KwgNwOvs7wAzw34260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2390" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2390" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁出席《中朝友好合作互助条约》签订65周年纪念招待会</t>
+        </is>
+      </c>
+      <c r="D2390" t="inlineStr">
+        <is>
+          <t>王沪宁出席《中朝友好合作互助条约》签订65周年纪念招待会。</t>
+        </is>
+      </c>
+      <c r="E2390" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2390" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDExXhBlWfAvEFLcOk6MuO7260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2391" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2391" t="inlineStr">
+        <is>
+          <t>[视频]“在高质量发展中保障和改善民生”形势政策系列报告会第四场报告会在京举行</t>
+        </is>
+      </c>
+      <c r="D2391" t="inlineStr">
+        <is>
+          <t>“在高质量发展中保障和改善民生”报告会在京举行，强调生态文明建设与全面绿色转型。</t>
+        </is>
+      </c>
+      <c r="E2391" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2391" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEUlRq9qOsA7xL2h6n4lyf260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2392" t="inlineStr">
+        <is>
+          <t>政治, 军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2392" t="inlineStr">
+        <is>
+          <t>Protests in Ukrainian cities against Zelensky's removal of defence minister</t>
+        </is>
+      </c>
+      <c r="D2392" t="inlineStr">
+        <is>
+          <t>乌克兰多地抗议泽连斯基解雇国防部长，引发民愤和军方不满。</t>
+        </is>
+      </c>
+      <c r="E2392" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2392" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdx76069n3do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2393" t="inlineStr">
+        <is>
+          <t>政治, 国际, 文体</t>
+        </is>
+      </c>
+      <c r="C2393" t="inlineStr">
+        <is>
+          <t>UK says Falkland Islands 'definitely ours' after Argentina banner</t>
+        </is>
+      </c>
+      <c r="D2393" t="inlineStr">
+        <is>
+          <t>英国首相称福克兰群岛“绝对属于英国”，此前阿根廷因世界杯庆祝行为可能被国际足联处罚。</t>
+        </is>
+      </c>
+      <c r="E2393" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2393" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyen1ned7no?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2394" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2394" t="inlineStr">
+        <is>
+          <t>MI5 court evidence based on lies, report says</t>
+        </is>
+      </c>
+      <c r="D2394" t="inlineStr">
+        <is>
+          <t>报告批评英国军情五处高级官员在法庭证据中撒谎。</t>
+        </is>
+      </c>
+      <c r="E2394" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2394" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/crmrwe84rp2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2395" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2395" t="inlineStr">
+        <is>
+          <t>Who is the frontrunner to be the UK's next chancellor?</t>
+        </is>
+      </c>
+      <c r="D2395" t="inlineStr">
+        <is>
+          <t>安迪·伯纳姆将入主唐宁街，谁将成为英国下一任财政大臣引关注。</t>
+        </is>
+      </c>
+      <c r="E2395" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2395" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c36yj4pn7jdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2396" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2396" t="inlineStr">
+        <is>
+          <t>Hong Kong official warns booksellers on security risks after raids</t>
+        </is>
+      </c>
+      <c r="D2396" t="inlineStr">
+        <is>
+          <t>香港警方四个月内第三次突击搜查独立书店，警告书商注意安全风险。</t>
+        </is>
+      </c>
+      <c r="E2396" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2396" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/g-s1-133931/hong-kong-official-warns-booksellers-on-security-risks-after-raids</t>
+        </is>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2397" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C2397" t="inlineStr">
+        <is>
+          <t>Zelenskyy fires Ukraine's tech-savvy defense minister in government reshuffle</t>
+        </is>
+      </c>
+      <c r="D2397" t="inlineStr">
+        <is>
+          <t>乌克兰总统泽连斯基解雇推动无人机创新的国防部长，进行政府改组。</t>
+        </is>
+      </c>
+      <c r="E2397" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2397" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/g-s1-133920/ukraine-defense-minister-fired</t>
+        </is>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2398" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2398" t="inlineStr">
+        <is>
+          <t>The political risks from war in Iran. And, ICE's use of force is rising, report finds</t>
+        </is>
+      </c>
+      <c r="D2398" t="inlineStr">
+        <is>
+          <t>伊朗战争影响共和党政治；报告称特朗普第二任期ICE武力使用增多。</t>
+        </is>
+      </c>
+      <c r="E2398" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2398" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/g-s1-133918/up-first-newsletter-iran-us-trump-jay-clayton-ice-use-of-force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2399" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C2399" t="inlineStr">
+        <is>
+          <t>Dismissal of Ukraine's popular defense minister draws intense criticism</t>
+        </is>
+      </c>
+      <c r="D2399" t="inlineStr">
+        <is>
+          <t>乌克兰解雇受欢迎的国防部长引强烈批评，其曾用无人机扭转战局。</t>
+        </is>
+      </c>
+      <c r="E2399" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2399" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/nx-s1-5894781/dismissal-of-ukraines-popular-defense-minister-draws-intense-criticism</t>
+        </is>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2400" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C2400" t="inlineStr">
+        <is>
+          <t>British Steel taken into public ownership to protect 'vital' UK supply</t>
+        </is>
+      </c>
+      <c r="D2400" t="inlineStr">
+        <is>
+          <t>英国钢铁公司被国有化，以保障国内关键供应。</t>
+        </is>
+      </c>
+      <c r="E2400" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2400" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5y680w62wno?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2401" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2401" t="inlineStr">
+        <is>
+          <t>[视频]2026世界人工智能大会暨人工智能全球治理高级别会议明天开幕</t>
+        </is>
+      </c>
+      <c r="D2401" t="inlineStr">
+        <is>
+          <t>2026世界人工智能大会明天在上海开幕，聚焦“智能伙伴，共创未来”，规模创历届新高。</t>
+        </is>
+      </c>
+      <c r="E2401" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2401" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDELUkhGr6tAXVEqcmZs2FZ260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2402" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2402" t="inlineStr">
+        <is>
+          <t>[视频]美称对伊朗发动多轮打击 伊朗称打击美进攻性基础设施</t>
+        </is>
+      </c>
+      <c r="D2402" t="inlineStr">
+        <is>
+          <t>美国对伊朗发动多轮打击，伊朗反击美军基地，双方冲突升级。</t>
+        </is>
+      </c>
+      <c r="E2402" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2402" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDE8kAcaW7L26mEEN6j9nck260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2403" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2403" t="inlineStr">
+        <is>
+          <t>Iran targets military bases as US launches wave of strikes</t>
+        </is>
+      </c>
+      <c r="D2403" t="inlineStr">
+        <is>
+          <t>伊朗军事基地遭袭，美国发动多波打击，海湾国家同步报告攻击。</t>
+        </is>
+      </c>
+      <c r="E2403" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2403" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2lq1ed28jxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2404" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2404" t="inlineStr">
+        <is>
+          <t>US strikes oil tanker with missiles as it enforces new Iran blockade</t>
+        </is>
+      </c>
+      <c r="D2404" t="inlineStr">
+        <is>
+          <t>美国用导弹袭击驶往伊朗哈格岛油轮，加强新封锁措施。</t>
+        </is>
+      </c>
+      <c r="E2404" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2404" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyqwkegqk0o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2405" t="inlineStr">
+        <is>
+          <t>民生, 政治</t>
+        </is>
+      </c>
+      <c r="C2405" t="inlineStr">
+        <is>
+          <t>[视频]用心用情为居民做好事 办实事 解难事——习近平总书记在上海考察时的重要讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2405" t="inlineStr">
+        <is>
+          <t>习近平上海考察强调城市更新，干部居民反响热烈，称要提升居民幸福感。</t>
+        </is>
+      </c>
+      <c r="E2405" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2405" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEpfNIh7lE3zNOyvWG7agZ260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2406" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C2406" t="inlineStr">
+        <is>
+          <t>More than 800 Canadian wildfires burning as air quality alerts extend to US</t>
+        </is>
+      </c>
+      <c r="D2406" t="inlineStr">
+        <is>
+          <t>加拿大超800起野火燃烧，美国多州空气质量被评为“危险”。</t>
+        </is>
+      </c>
+      <c r="E2406" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2406" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0m7n427xd8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2407" t="inlineStr">
+        <is>
+          <t>民生, 国际</t>
+        </is>
+      </c>
+      <c r="C2407" t="inlineStr">
+        <is>
+          <t>Free meningitis B vaccine should be offered to all teenagers over 15,  UK experts say</t>
+        </is>
+      </c>
+      <c r="D2407" t="inlineStr">
+        <is>
+          <t>英国专家建议向15岁以上青少年免费提供B型脑膜炎疫苗，此前肯特郡爆发疫情致两人死亡。</t>
+        </is>
+      </c>
+      <c r="E2407" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2407" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c74glj9zkzko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2408">
+      <c r="A2408" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2408" t="inlineStr">
+        <is>
+          <t>国际, 军事, 经济</t>
+        </is>
+      </c>
+      <c r="C2408" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2408" t="inlineStr">
+        <is>
+          <t>国际快讯：乌欧推进武器合作、黎以谈判进展、德国总理批美关税、加拿大林火。</t>
+        </is>
+      </c>
+      <c r="E2408" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2408" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDERDfqifYnY340YMdPRt6Z260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2409" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2409" t="inlineStr">
+        <is>
+          <t>Teenager accused of carrying out sabotage actions in Poland for Russia</t>
+        </is>
+      </c>
+      <c r="D2409" t="inlineStr">
+        <is>
+          <t>波兰指控一名青少年为俄罗斯从事破坏活动，旨在煽动波兰与乌克兰间的民族紧张关系。</t>
+        </is>
+      </c>
+      <c r="E2409" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2409" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp305dx493do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2410" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2410" t="inlineStr">
+        <is>
+          <t>'Moment of joy' as Uganda discharges last Ebola patient</t>
+        </is>
+      </c>
+      <c r="D2410" t="inlineStr">
+        <is>
+          <t>乌干达最后一名埃博拉患者出院，多数病例来自刚果（金）旅行者。</t>
+        </is>
+      </c>
+      <c r="E2410" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2410" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2myxjv172o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2411" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2411" t="inlineStr">
+        <is>
+          <t>Venezuela's earthquake recovery overshadows its push for democracy</t>
+        </is>
+      </c>
+      <c r="D2411" t="inlineStr">
+        <is>
+          <t>委内瑞拉双震灾后重建，暂缓了民众对恢复民主斗争的关注。</t>
+        </is>
+      </c>
+      <c r="E2411" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2411" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/14/nx-s1-5893438/venezuelas-democracy-delayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2412" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2412" t="inlineStr">
+        <is>
+          <t>[视频]强降雨将影响我国多地 各地各部门积极应对</t>
+        </is>
+      </c>
+      <c r="D2412" t="inlineStr">
+        <is>
+          <t>东北强降雨结束，抢险排涝持续；黑龙江、吉林等地积极应对洪涝，转移群众与抢修。</t>
+        </is>
+      </c>
+      <c r="E2412" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2412" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEXMrxhvLms9wLR3f8Fh6F260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2413" t="inlineStr">
+        <is>
+          <t>社会, 政治, 文体</t>
+        </is>
+      </c>
+      <c r="C2413" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2413" t="inlineStr">
+        <is>
+          <t>国内联播快讯：文明乡风大会举行、世界市长对话、海军招飞完成、三支一扶启动。</t>
+        </is>
+      </c>
+      <c r="E2413" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2413" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/16/VIDEBd9ipQD7iyRrcwZgLlYh260716.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2414" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2414" t="inlineStr">
+        <is>
+          <t>Italian officials handed jail terms for Genoa bridge disaster that killed 43</t>
+        </is>
+      </c>
+      <c r="D2414" t="inlineStr">
+        <is>
+          <t>意大利前高速公路高管因2018年热那亚大桥坍塌事故被判12年监禁。</t>
+        </is>
+      </c>
+      <c r="E2414" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2414" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c36dnz1zez5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2415" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2415" t="inlineStr">
+        <is>
+          <t>Volunteer firefighter suspected of starting devastating France forest fire</t>
+        </is>
+      </c>
+      <c r="D2415" t="inlineStr">
+        <is>
+          <t>法国一名志愿消防员涉嫌纵火引发森林大火，总统称绝不纵容。</t>
+        </is>
+      </c>
+      <c r="E2415" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2415" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ce97zd8yx1xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2416" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2416" t="inlineStr">
+        <is>
+          <t>Children among dead at Algeria foster care home blaze - president</t>
+        </is>
+      </c>
+      <c r="D2416" t="inlineStr">
+        <is>
+          <t>阿尔及利亚一家寄养院火灾致11人死亡，包括儿童，另有19人受伤。</t>
+        </is>
+      </c>
+      <c r="E2416" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2416" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvgwd4nz344o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2417" t="inlineStr">
+        <is>
+          <t>社会, 经济</t>
+        </is>
+      </c>
+      <c r="C2417" t="inlineStr">
+        <is>
+          <t>Fraud crackdown on Ghana ID cards makes digital checks compulsory - photocopies banned</t>
+        </is>
+      </c>
+      <c r="D2417" t="inlineStr">
+        <is>
+          <t>加纳为打击欺诈，强制企业电子验证身份，禁止使用复印件。</t>
+        </is>
+      </c>
+      <c r="E2417" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2417" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn4n9q538z2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2418" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2418" t="inlineStr">
+        <is>
+          <t>The band playing when a Bangkok bar caught fire mourns its members among the 33 dead</t>
+        </is>
+      </c>
+      <c r="D2418" t="inlineStr">
+        <is>
+          <t>曼谷酒吧火灾致33死，演出乐队四人丧生，其他成员哀悼。</t>
+        </is>
+      </c>
+      <c r="E2418" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2418" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/g-s1-133907/death-toll-bangkok-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2419" t="inlineStr">
+        <is>
+          <t>文体, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2419" t="inlineStr">
+        <is>
+          <t>Argentina face action over Falklands banner</t>
+        </is>
+      </c>
+      <c r="D2419" t="inlineStr">
+        <is>
+          <t>阿根廷球员因在马岛半决赛后展示主权横幅，面临国际足联纪律处罚。</t>
+        </is>
+      </c>
+      <c r="E2419" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2419" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c935pgr4dklo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2420" t="inlineStr">
+        <is>
+          <t>文体, 社会</t>
+        </is>
+      </c>
+      <c r="C2420" t="inlineStr">
+        <is>
+          <t>Feeling gutted? Five ways to cope with England's World Cup defeat</t>
+        </is>
+      </c>
+      <c r="D2420" t="inlineStr">
+        <is>
+          <t>英格兰队世界杯出局后，球迷和专家分享五种应对失望情绪的方法。</t>
+        </is>
+      </c>
+      <c r="E2420" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2420" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gy5jwjvz7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2421" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2421" t="inlineStr">
+        <is>
+          <t>Why you should care about the third-place play-off between England and France</t>
+        </is>
+      </c>
+      <c r="D2421" t="inlineStr">
+        <is>
+          <t>分析称英格兰与法国世界杯季军争夺战值得观看，尽管球迷情绪低落。</t>
+        </is>
+      </c>
+      <c r="E2421" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2421" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cly5we2lgq4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B2422" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2422" t="inlineStr">
+        <is>
+          <t>No Asian team managed to go far this World Cup (again). What's holding them back?</t>
+        </is>
+      </c>
+      <c r="D2422" t="inlineStr">
+        <is>
+          <t>世界杯上亚洲球队已连续六届未能突破首轮淘汰赛，表现欠佳。</t>
+        </is>
+      </c>
+      <c r="E2422" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2422" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/16/nx-s1-5884732/world-cup-asian-football-confederation-korea-japan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-17
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2422"/>
+  <dimension ref="A1:F2457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -77941,6 +77941,1126 @@
         </is>
       </c>
     </row>
+    <row r="2423">
+      <c r="A2423" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2423" t="inlineStr">
+        <is>
+          <t>政治, 科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2423" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260717 19:00</t>
+        </is>
+      </c>
+      <c r="D2423" t="inlineStr">
+        <is>
+          <t>习近平出席AI大会并发表主旨讲话，会见多国领导人；赵乐际在甘肃调研；王沪宁访朝；多国冲突持续。</t>
+        </is>
+      </c>
+      <c r="E2423" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2423" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEkqSU1p2BvLSWvYqhMsXk260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2424" t="inlineStr">
+        <is>
+          <t>政治, 科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2424" t="inlineStr">
+        <is>
+          <t>[视频]习近平出席2026世界人工智能大会暨人工智能全球治理高级别会议开幕式并发表主旨讲话</t>
+        </is>
+      </c>
+      <c r="D2424" t="inlineStr">
+        <is>
+          <t>习近平出席世界人工智能大会开幕式，提出构建公正合理的全球AI治理体系四点意见。</t>
+        </is>
+      </c>
+      <c r="E2424" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2424" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEZkhwT6Qzq4TddOb2tY0Q260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2425" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2425" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见泰国总理</t>
+        </is>
+      </c>
+      <c r="D2425" t="inlineStr">
+        <is>
+          <t>习近平会见泰国总理，强调推进中泰命运共同体建设，加强多领域合作。</t>
+        </is>
+      </c>
+      <c r="E2425" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2425" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEEYcQo4wQcXOHotopOvKC260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2426" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2426" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见柬埔寨首相</t>
+        </is>
+      </c>
+      <c r="D2426" t="inlineStr">
+        <is>
+          <t>习近平会见柬埔寨首相，强调深化铁杆友谊，推动中柬命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E2426" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2426" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEYw7OdQuDy7GjsC0IdfoA260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2427" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2427" t="inlineStr">
+        <is>
+          <t>[视频]习近平会见联合国秘书长</t>
+        </is>
+      </c>
+      <c r="D2427" t="inlineStr">
+        <is>
+          <t>习近平会见联合国秘书长，强调维护多边主义，支持联合国在全球治理中发挥作用。</t>
+        </is>
+      </c>
+      <c r="E2427" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2427" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEjvKc7E2ATNKQ24DLHjW5260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2428" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2428" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际在甘肃调研</t>
+        </is>
+      </c>
+      <c r="D2428" t="inlineStr">
+        <is>
+          <t>赵乐际在甘肃调研，强调坚持党对人大工作的全面领导，推动人大工作高质量发展。</t>
+        </is>
+      </c>
+      <c r="E2428" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2428" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEV5MkKzxBIcigC4jdoJ9x260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2429" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2429" t="inlineStr">
+        <is>
+          <t>[视频]王沪宁对朝鲜进行正式友好访问</t>
+        </is>
+      </c>
+      <c r="D2429" t="inlineStr">
+        <is>
+          <t>王沪宁访问朝鲜，会见金正恩，庆祝条约签订65周年，推动中朝关系发展。</t>
+        </is>
+      </c>
+      <c r="E2429" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2429" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEFmBmfj2fSl7ugiCk8cjR260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2430" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2430" t="inlineStr">
+        <is>
+          <t>Japan relaxes royal succession rules - but ban on female emperors remains</t>
+        </is>
+      </c>
+      <c r="D2430" t="inlineStr">
+        <is>
+          <t>日本放宽皇室继承规则，允许收养男性远亲，但女性天皇禁令未变。</t>
+        </is>
+      </c>
+      <c r="E2430" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2430" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy07rz79zg9o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2431" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2431" t="inlineStr">
+        <is>
+          <t>Zeffman: Burnham promises huge change - now to find out how he will deliver it</t>
+        </is>
+      </c>
+      <c r="D2431" t="inlineStr">
+        <is>
+          <t>英国工党领袖伯纳姆承诺40年来最大政治变革，但落实方式待观察。</t>
+        </is>
+      </c>
+      <c r="E2431" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2431" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cz7djw5dznpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2432" t="inlineStr">
+        <is>
+          <t>政治, 社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2432" t="inlineStr">
+        <is>
+          <t>German politician faces calls to resign over surrogacy child</t>
+        </is>
+      </c>
+      <c r="D2432" t="inlineStr">
+        <is>
+          <t>德国政客因代孕子女面临辞职呼声，与所属政党反代孕立场相悖。</t>
+        </is>
+      </c>
+      <c r="E2432" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2432" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cq56ed827peo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2433" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2433" t="inlineStr">
+        <is>
+          <t>First Reform UK police commissioner elected</t>
+        </is>
+      </c>
+      <c r="D2433" t="inlineStr">
+        <is>
+          <t>英国改革党首次当选警察与犯罪事务专员。</t>
+        </is>
+      </c>
+      <c r="E2433" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2433" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c934p5vze87o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2434" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2434" t="inlineStr">
+        <is>
+          <t>Rubio convenes countries on left-wing political violence</t>
+        </is>
+      </c>
+      <c r="D2434" t="inlineStr">
+        <is>
+          <t>鲁比奥召集60多国讨论打击左翼政治暴力。</t>
+        </is>
+      </c>
+      <c r="E2434" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2434" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/17/g-s1-134148/rubio-convene-countries-on-left-wing-political-violence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2435" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2435" t="inlineStr">
+        <is>
+          <t>Japan revises law on royals, keeps blocking women from throne</t>
+        </is>
+      </c>
+      <c r="D2435" t="inlineStr">
+        <is>
+          <t>日本修订皇室法律，仍禁止女性继承皇位。</t>
+        </is>
+      </c>
+      <c r="E2435" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2435" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/17/g-s1-133536/japan-law-male-heirs-imperial-throne</t>
+        </is>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2436" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2436" t="inlineStr">
+        <is>
+          <t>[视频]上半年我国涉外收支规模创新高 外汇市场交易量稳步增长</t>
+        </is>
+      </c>
+      <c r="D2436" t="inlineStr">
+        <is>
+          <t>上半年我国涉外收支规模创新高，跨境资金净流入2472亿美元，对外净资产全球第二。</t>
+        </is>
+      </c>
+      <c r="E2436" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2436" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEusfkC9AoXNOMzlPiezd4260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2437" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2437" t="inlineStr">
+        <is>
+          <t>Trump Media to sell instant access to 'market-moving' social posts</t>
+        </is>
+      </c>
+      <c r="D2437" t="inlineStr">
+        <is>
+          <t>特朗普媒体推出付费快速推送服务，向华尔街交易员提供其最具影响力的社交帖子。</t>
+        </is>
+      </c>
+      <c r="E2437" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2437" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c79gw4lj89eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2438" t="inlineStr">
+        <is>
+          <t>经济, 政治</t>
+        </is>
+      </c>
+      <c r="C2438" t="inlineStr">
+        <is>
+          <t>China hits out at British Steel nationalisation</t>
+        </is>
+      </c>
+      <c r="D2438" t="inlineStr">
+        <is>
+          <t>中国批评英国将英国钢铁公司国有化，英方称此举旨在保护关键国家能力。</t>
+        </is>
+      </c>
+      <c r="E2438" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2438" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjd4kvxpd3do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2439" t="inlineStr">
+        <is>
+          <t>经济, 文体</t>
+        </is>
+      </c>
+      <c r="C2439" t="inlineStr">
+        <is>
+          <t>The financial winners and losers from the World Cup</t>
+        </is>
+      </c>
+      <c r="D2439" t="inlineStr">
+        <is>
+          <t>分析2026年世界杯场外巨大收入与亏损的赢家和输家。</t>
+        </is>
+      </c>
+      <c r="E2439" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2439" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgrkek8lrzvo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2440" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2440" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：携手构建公正合理的全球人工智能治理体系</t>
+        </is>
+      </c>
+      <c r="D2440" t="inlineStr">
+        <is>
+          <t>央视快评呼吁携手构建公正合理的全球人工智能治理体系。</t>
+        </is>
+      </c>
+      <c r="E2440" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2440" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEWw4EEq1C1wSZR1Htg3jC260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2441" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2441" t="inlineStr">
+        <is>
+          <t>First atmosphere found on Earth-like planet in habitable zone of distant star</t>
+        </is>
+      </c>
+      <c r="D2441" t="inlineStr">
+        <is>
+          <t>首次在宜居带类地行星发现大气层，系重要科研突破。</t>
+        </is>
+      </c>
+      <c r="E2441" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2441" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy4kdd1e0ejo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2442" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2442" t="inlineStr">
+        <is>
+          <t>China's Xi calls for step up of global effort in AI, as US curbs squeeze China's tech access</t>
+        </is>
+      </c>
+      <c r="D2442" t="inlineStr">
+        <is>
+          <t>美国限制中国获取先进技术，中国加速自主研发，科技竞争加剧。</t>
+        </is>
+      </c>
+      <c r="E2442" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2442" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/17/nx-s1-5897285/chinas-xi-calls-for-step-up-of-global-effort-in-ai-as-us-curbs-squeeze-chinas-tech-access</t>
+        </is>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2443" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2443" t="inlineStr">
+        <is>
+          <t>Pakistani forces kill 24 militants in border raids near Afghanistan</t>
+        </is>
+      </c>
+      <c r="D2443" t="inlineStr">
+        <is>
+          <t>巴基斯坦军方在阿富汗边境打击武装分子，24名 militants 被击毙。</t>
+        </is>
+      </c>
+      <c r="E2443" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2443" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/17/g-s1-134175/pakistani-forces-kill-24-militants-in-border-raids-near-afghanistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2444" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2444" t="inlineStr">
+        <is>
+          <t>U.S. strikes bridges in Iran, Tehran targets U.S. bases in the Gulf</t>
+        </is>
+      </c>
+      <c r="D2444" t="inlineStr">
+        <is>
+          <t>美国空袭伊朗桥梁，伊朗打击美方基地，霍尔木兹海峡冲突引全面战争担忧。</t>
+        </is>
+      </c>
+      <c r="E2444" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2444" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/17/g-s1-134158/us-iran-war-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2445" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2445" t="inlineStr">
+        <is>
+          <t>Longest dry spell in 30 years for parts of England as heatwave hits two-week mark</t>
+        </is>
+      </c>
+      <c r="D2445" t="inlineStr">
+        <is>
+          <t>英格兰部分地区遭遇30年来最长干旱，热浪持续两周。</t>
+        </is>
+      </c>
+      <c r="E2445" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2445" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/weather/articles/ckg4gqlye02o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2446" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2446" t="inlineStr">
+        <is>
+          <t>[视频]美军连续第六晚对伊朗实施打击 伊朗袭击美军基地</t>
+        </is>
+      </c>
+      <c r="D2446" t="inlineStr">
+        <is>
+          <t>美军连续六晚打击伊朗，伊朗反击美军基地，霍尔木兹海峡持续受阻。</t>
+        </is>
+      </c>
+      <c r="E2446" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2446" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDE3bx5jQhCovhvUJuL0IWp260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2447" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2447" t="inlineStr">
+        <is>
+          <t>[视频]乌总统称军方与国防部存在分歧 已任命新代理防长</t>
+        </is>
+      </c>
+      <c r="D2447" t="inlineStr">
+        <is>
+          <t>乌克兰总统称军方与国防部有分歧，任命新代理防长并改组内阁。</t>
+        </is>
+      </c>
+      <c r="E2447" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2447" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEhkAT0fBVXtKH0Z1CCubE260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2448" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2448" t="inlineStr">
+        <is>
+          <t>Iran accuses US of hitting civilian infrastructure</t>
+        </is>
+      </c>
+      <c r="D2448" t="inlineStr">
+        <is>
+          <t>伊朗指责美国打击民用设施，美军称旨在削弱伊朗军事能力。</t>
+        </is>
+      </c>
+      <c r="E2448" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2448" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c151gdjwd10o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2449" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2449" t="inlineStr">
+        <is>
+          <t>Trump alleges China meddled in 2020 election and questions voting security ahead of midterms</t>
+        </is>
+      </c>
+      <c r="D2449" t="inlineStr">
+        <is>
+          <t>特朗普指控中国干预2020大选，中方驳斥，民主党指责其破坏选举。</t>
+        </is>
+      </c>
+      <c r="E2449" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2449" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2k9wvv5wyo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2450" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2450" t="inlineStr">
+        <is>
+          <t>More than 500 Rohingya vanished at sea - what happened?</t>
+        </is>
+      </c>
+      <c r="D2450" t="inlineStr">
+        <is>
+          <t>两艘载约530名罗兴亚人的船自6月29日离开缅甸后失踪。</t>
+        </is>
+      </c>
+      <c r="E2450" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2450" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cr59n096mrmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2451" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2451" t="inlineStr">
+        <is>
+          <t>Philippines condemns monkey video on Chinese media as racist</t>
+        </is>
+      </c>
+      <c r="D2451" t="inlineStr">
+        <is>
+          <t>菲律宾谴责《中国日报》AI视频展示猴子穿菲服装声称南海主权，称其种族歧视。</t>
+        </is>
+      </c>
+      <c r="E2451" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2451" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj632307934o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2452" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2452" t="inlineStr">
+        <is>
+          <t>Canada fires prompt US air quality alerts as smoke blankets major cities</t>
+        </is>
+      </c>
+      <c r="D2452" t="inlineStr">
+        <is>
+          <t>加拿大800多处火灾烟雾弥漫至多伦多、纽约等城市，美国发布空气质量警报。</t>
+        </is>
+      </c>
+      <c r="E2452" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2452" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0m7n427xd8o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2453" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2453" t="inlineStr">
+        <is>
+          <t>[视频]国务院新闻办举行“促进团结进步 昂扬奋斗力量”中外记者见面会</t>
+        </is>
+      </c>
+      <c r="D2453" t="inlineStr">
+        <is>
+          <t>国务院新闻办举行记者见面会，六位代表分享民族团结进步故事。</t>
+        </is>
+      </c>
+      <c r="E2453" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2453" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/17/VIDEwQfREV2F8kOUNhVhZwSa260717.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2454" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2454" t="inlineStr">
+        <is>
+          <t>Uganda suspends school trips after 20 pupils die in bus crash</t>
+        </is>
+      </c>
+      <c r="D2454" t="inlineStr">
+        <is>
+          <t>乌干达一辆巴士坠毁致20名学生死亡，政府暂停学校旅行活动。</t>
+        </is>
+      </c>
+      <c r="E2454" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2454" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c151gegwqv1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2455" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2455" t="inlineStr">
+        <is>
+          <t>Olympic cyclist admits to driving despite ban after crash that killed wife</t>
+        </is>
+      </c>
+      <c r="D2455" t="inlineStr">
+        <is>
+          <t>奥运自行车手罗汉·丹尼斯承认在驾照吊销后驾驶，此前车祸致妻子死亡。</t>
+        </is>
+      </c>
+      <c r="E2455" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2455" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c62q3ywep1ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2456" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2456" t="inlineStr">
+        <is>
+          <t>Boy attacked by zoo crocodile has had seven operations and is smiling again, say parents</t>
+        </is>
+      </c>
+      <c r="D2456" t="inlineStr">
+        <is>
+          <t>三岁男童遭动物园鳄鱼袭击，经七次手术后已能微笑，父母称其恢复良好。</t>
+        </is>
+      </c>
+      <c r="E2456" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2456" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c998v0g2v0vo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2457" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2457" t="inlineStr">
+        <is>
+          <t>My Left Foot and Home Alone 2 actress Brenda Fricker dies at 81</t>
+        </is>
+      </c>
+      <c r="D2457" t="inlineStr">
+        <is>
+          <t>《我的左脚》奥斯卡得主、演员布伦达·弗里克去世，享年81岁。</t>
+        </is>
+      </c>
+      <c r="E2457" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2457" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0m70zremezo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-18
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2457"/>
+  <dimension ref="A1:F2490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -79061,6 +79061,1062 @@
         </is>
       </c>
     </row>
+    <row r="2458">
+      <c r="A2458" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2458" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2458" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260718 19:00</t>
+        </is>
+      </c>
+      <c r="D2458" t="inlineStr">
+        <is>
+          <t>新闻联播报道习近平指示重庆山体崩塌救援，以及人工智能大会反响等多条新闻。</t>
+        </is>
+      </c>
+      <c r="E2458" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2458" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEuDgFjNWQSHo4JOxH3eti260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2459" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2459" t="inlineStr">
+        <is>
+          <t>[视频]习近平对重庆彭水县山体崩塌作出重要指示强调 科学组织搜救 加强监测预警和巡查排险 切实保障人民群众生命财产安全 李强作出批示</t>
+        </is>
+      </c>
+      <c r="D2459" t="inlineStr">
+        <is>
+          <t>习近平就重庆彭水山体崩塌作出指示，强调科学搜救、保障群众安全，李强作批示。</t>
+        </is>
+      </c>
+      <c r="E2459" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2459" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEMeYtV11dhO9KnoEGb4DI260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2460" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2460" t="inlineStr">
+        <is>
+          <t>[视频]张国清赶赴重庆彭水县指导山体崩塌灾害现场搜救和应急处置工作</t>
+        </is>
+      </c>
+      <c r="D2460" t="inlineStr">
+        <is>
+          <t>张国清赴重庆彭水指导山体崩塌救援，强调保障人民生命安全。</t>
+        </is>
+      </c>
+      <c r="E2460" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2460" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDECWm8BDMpvlGDTYaDi7HM260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2461" t="inlineStr">
+        <is>
+          <t>政治, 国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2461" t="inlineStr">
+        <is>
+          <t>Trump threatens new Canada tariffs over fires sending 'filthy' air into US cities</t>
+        </is>
+      </c>
+      <c r="D2461" t="inlineStr">
+        <is>
+          <t>特朗普威胁对加拿大加征新关税，因林火产生的污染空气进入美国城市。</t>
+        </is>
+      </c>
+      <c r="E2461" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2461" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyq93j34lgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2462" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2462" t="inlineStr">
+        <is>
+          <t>He made history in Congress - then the Supreme Court changed its mind</t>
+        </is>
+      </c>
+      <c r="D2462" t="inlineStr">
+        <is>
+          <t>最高法院改变裁决，居民担忧议员若失席将失去联邦资金。</t>
+        </is>
+      </c>
+      <c r="E2462" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2462" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cn949jvjxplo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2463" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2463" t="inlineStr">
+        <is>
+          <t>Burnham to announce plans for new North Sea oil and gas drilling</t>
+        </is>
+      </c>
+      <c r="D2463" t="inlineStr">
+        <is>
+          <t>英国工党宣布北海石油钻探新计划，此前承诺不再发放新许可证。</t>
+        </is>
+      </c>
+      <c r="E2463" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2463" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c935yx2z9d4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2464" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2464" t="inlineStr">
+        <is>
+          <t>Ruthless plotter or dad dancer? Insiders reveal the real Andy Burnham</t>
+        </is>
+      </c>
+      <c r="D2464" t="inlineStr">
+        <is>
+          <t>20多位知情者揭秘安迪·伯纳姆的真实面貌，探讨其政治形象。</t>
+        </is>
+      </c>
+      <c r="E2464" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2464" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3043vl2l7zo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2465" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2465" t="inlineStr">
+        <is>
+          <t>[视频]上半年我国邮政行业寄递业务量同比增长4.2%</t>
+        </is>
+      </c>
+      <c r="D2465" t="inlineStr">
+        <is>
+          <t>上半年邮政行业寄递业务量达1088.9亿件，同比增长4.2%。</t>
+        </is>
+      </c>
+      <c r="E2465" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2465" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEWB9xfSNGF9hxEaKgrLrD260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2466" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2466" t="inlineStr">
+        <is>
+          <t>[视频]上半年全国铁路完成固定资产投资3632亿元</t>
+        </is>
+      </c>
+      <c r="D2466" t="inlineStr">
+        <is>
+          <t>上半年全国铁路完成固定资产投资3632亿元，同比增长2.1%。</t>
+        </is>
+      </c>
+      <c r="E2466" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2466" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDE24yglpnW0QXslwvXsp7G260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2467" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2467" t="inlineStr">
+        <is>
+          <t>[视频]【活力中国调研行】开在制造业重镇里的“AI超市”</t>
+        </is>
+      </c>
+      <c r="D2467" t="inlineStr">
+        <is>
+          <t>广东东莞制造业中小企业通过国家AI中试基地的“AI超市”，实现智能化转型升级。</t>
+        </is>
+      </c>
+      <c r="E2467" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2467" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDERXV0l3FJiwpunVIj9c0F260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2468" t="inlineStr">
+        <is>
+          <t>经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2468" t="inlineStr">
+        <is>
+          <t>[视频]“废品”变“资源” 以旧换新激发循环经济新活力</t>
+        </is>
+      </c>
+      <c r="D2468" t="inlineStr">
+        <is>
+          <t>以旧换新政策推动消费增长，带动回收产业链壮大，促进循环经济规模化和高值化。</t>
+        </is>
+      </c>
+      <c r="E2468" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2468" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEf3CwHu967kBp9xSIoyaJ260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2469" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2469" t="inlineStr">
+        <is>
+          <t>[视频]让人工智能更好造福人类——习近平主席在2026世界人工智能大会暨人工智能全球治理高级别会议开幕式上的主旨讲话引发热烈反响</t>
+        </is>
+      </c>
+      <c r="D2469" t="inlineStr">
+        <is>
+          <t>习近平在人工智能大会发表主旨讲话，提出全球治理四点意见，引发热烈反响。</t>
+        </is>
+      </c>
+      <c r="E2469" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2469" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEtGwuPJnmJ2GW8wQKMVCI260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2470" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2470" t="inlineStr">
+        <is>
+          <t>[视频]央视快评：共同促进全球人工智能向上向善、造福人类</t>
+        </is>
+      </c>
+      <c r="D2470" t="inlineStr">
+        <is>
+          <t>央视播发快评，呼吁共同促进全球人工智能向上向善、造福人类。</t>
+        </is>
+      </c>
+      <c r="E2470" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2470" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEYXPkfGYEnVrAitrvDZjw260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2471" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2471" t="inlineStr">
+        <is>
+          <t>[视频]多项首发技术和创新成果亮相世界人工智能大会</t>
+        </is>
+      </c>
+      <c r="D2471" t="inlineStr">
+        <is>
+          <t>2026世界人工智能大会在上海举行，发布多项行动计划和前沿技术，聚焦AI全球治理与创新应用。</t>
+        </is>
+      </c>
+      <c r="E2471" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2471" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEgMG3OKUJViWykmN4MyGA260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2472" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2472" t="inlineStr">
+        <is>
+          <t>Space start-up launches India’s first commercial rocket designed for orbit</t>
+        </is>
+      </c>
+      <c r="D2472" t="inlineStr">
+        <is>
+          <t>印度太空初创公司Skyroot成功发射首枚商业轨道火箭维克拉姆-1。</t>
+        </is>
+      </c>
+      <c r="E2472" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2472" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyekv7rld3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2473" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2473" t="inlineStr">
+        <is>
+          <t>[视频]美媒称美或扩大对伊朗军事行动 伊朗称打击多处美军基地</t>
+        </is>
+      </c>
+      <c r="D2473" t="inlineStr">
+        <is>
+          <t>美伊冲突升级，美军打击伊朗目标，伊朗反击美军基地并威胁扩大报复，国际油价上涨。</t>
+        </is>
+      </c>
+      <c r="E2473" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2473" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDE1vIp7TP7VBnGyX0ubFz4260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2474" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2474" t="inlineStr">
+        <is>
+          <t>Russian online retail warehouses hit by deadly Ukrainian strikes</t>
+        </is>
+      </c>
+      <c r="D2474" t="inlineStr">
+        <is>
+          <t>乌克兰无人机袭击俄罗斯Wildberries仓库，乌称打击的为供应制裁部件的物流设施。</t>
+        </is>
+      </c>
+      <c r="E2474" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2474" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/clyxlm877p2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2475" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2475" t="inlineStr">
+        <is>
+          <t>US strikes hit Iran for seventh consecutive night</t>
+        </is>
+      </c>
+      <c r="D2475" t="inlineStr">
+        <is>
+          <t>美国连续第七夜打击伊朗，伊朗报复美国盟友，科威特一水电设施被击中。</t>
+        </is>
+      </c>
+      <c r="E2475" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2475" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cy748n8zx8ro?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2476" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2476" t="inlineStr">
+        <is>
+          <t>8 killed and more than 60 wounded in Ukrainian drone attack on Russian regions</t>
+        </is>
+      </c>
+      <c r="D2476" t="inlineStr">
+        <is>
+          <t>乌克兰无人机袭击俄罗斯地区，造成8死60多伤，针对能源和军事目标。</t>
+        </is>
+      </c>
+      <c r="E2476" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2476" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/18/nx-s1-5898963/8-killed-and-more-than-60-wounded-in-ukrainian-drone-attack-on-russian-regions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2477" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2477" t="inlineStr">
+        <is>
+          <t>[视频]重庆彭水山体崩塌救援安置工作加紧进行</t>
+        </is>
+      </c>
+      <c r="D2477" t="inlineStr">
+        <is>
+          <t>重庆彭水山体崩塌救援安置加紧进行，各方调拨物资资金支援。</t>
+        </is>
+      </c>
+      <c r="E2477" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2477" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDE1zk8TJAJlbUHHvOHEA1s260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2478" t="inlineStr">
+        <is>
+          <t>民生, 社会, 经济</t>
+        </is>
+      </c>
+      <c r="C2478" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2478" t="inlineStr">
+        <is>
+          <t>国内联播快讯：土壤环境安全规划出台、数据量增长、民航运输量提升、海水淡化产业部署。</t>
+        </is>
+      </c>
+      <c r="E2478" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2478" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEBYifrRRUIM6qY1dOcTkP260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2479" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2479" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2479" t="inlineStr">
+        <is>
+          <t>国际联播快讯：伊拉克击落无人机、俄乌互相打击、德国参法核演习、英国工党新党首。</t>
+        </is>
+      </c>
+      <c r="E2479" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2479" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/18/VIDEYqBGT0WX7U7ggDjuDlIa260718.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2480" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2480" t="inlineStr">
+        <is>
+          <t>Laos says it can't determine cause of  tourist deaths linked to methanol</t>
+        </is>
+      </c>
+      <c r="D2480" t="inlineStr">
+        <is>
+          <t>老挝称无法确定2024年游客甲醇中毒死亡原因，因未进行尸检。</t>
+        </is>
+      </c>
+      <c r="E2480" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2480" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cdx8rj99endo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2481" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2481" t="inlineStr">
+        <is>
+          <t>Helicopters dump water as huge Norway fire destroys homes</t>
+        </is>
+      </c>
+      <c r="D2481" t="inlineStr">
+        <is>
+          <t>挪威德拉门大火烧毁超百栋房屋，直升机洒水灭火。</t>
+        </is>
+      </c>
+      <c r="E2481" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2481" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c4gj5944n4ko?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2482">
+      <c r="A2482" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2482" t="inlineStr">
+        <is>
+          <t>国际, 文体</t>
+        </is>
+      </c>
+      <c r="C2482" t="inlineStr">
+        <is>
+          <t>World Cup winner Capdevila appeals to Trump after US travel permit denied</t>
+        </is>
+      </c>
+      <c r="D2482" t="inlineStr">
+        <is>
+          <t>世界杯冠军卡普德维拉因美方拒签，呼吁特朗普帮助。</t>
+        </is>
+      </c>
+      <c r="E2482" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2482" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cx2l5jn17yjo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2483">
+      <c r="A2483" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2483" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2483" t="inlineStr">
+        <is>
+          <t>Why is it so hard for the U.S. to win wars?</t>
+        </is>
+      </c>
+      <c r="D2483" t="inlineStr">
+        <is>
+          <t>美国在阿富汗、伊拉克等战争中难以取得胜利，政治目标未能达成。</t>
+        </is>
+      </c>
+      <c r="E2483" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2483" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/18/g-s1-134037/why-is-it-so-hard-for-the-u-s-to-win-wars</t>
+        </is>
+      </c>
+    </row>
+    <row r="2484">
+      <c r="A2484" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2484" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2484" t="inlineStr">
+        <is>
+          <t>The U.S. and Iran blow past red lines as they lurch back toward all-out war</t>
+        </is>
+      </c>
+      <c r="D2484" t="inlineStr">
+        <is>
+          <t>美伊互袭军事目标，霍尔木兹海峡冲突加剧，局势濒临全面战争。</t>
+        </is>
+      </c>
+      <c r="E2484" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2484" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/18/nx-s1-5898916/us-iran-escalate-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2485">
+      <c r="A2485" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2485" t="inlineStr">
+        <is>
+          <t>社会, 政治</t>
+        </is>
+      </c>
+      <c r="C2485" t="inlineStr">
+        <is>
+          <t>Indian activist on hunger strike for 20 days forcibly taken to hospital</t>
+        </is>
+      </c>
+      <c r="D2485" t="inlineStr">
+        <is>
+          <t>印度活动家绝食20天后被强行送医，现改为在他人处无限期绝食。</t>
+        </is>
+      </c>
+      <c r="E2485" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2485" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cjej3dxxg2do?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2486">
+      <c r="A2486" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2486" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2486" t="inlineStr">
+        <is>
+          <t>Control, threats, disfiguring surgery: My life inside Jeffrey Epstein's 'cult'</t>
+        </is>
+      </c>
+      <c r="D2486" t="inlineStr">
+        <is>
+          <t>受害者讲述金融家爱泼斯坦如何以控制、威胁和整形手术操纵“助理”。</t>
+        </is>
+      </c>
+      <c r="E2486" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2486" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/czek5wl6p2go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2487">
+      <c r="A2487" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2487" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2487" t="inlineStr">
+        <is>
+          <t>Brad Pitt's children are dropping their dad's surname - here's why I did the same</t>
+        </is>
+      </c>
+      <c r="D2487" t="inlineStr">
+        <is>
+          <t>布拉德·皮特的子女放弃父姓，改用母姓。</t>
+        </is>
+      </c>
+      <c r="E2487" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2487" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2ln9l60g5o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2488">
+      <c r="A2488" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2488" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2488" t="inlineStr">
+        <is>
+          <t>The Bronze Final - the unwanted tie or a match with a 'golden layer'?</t>
+        </is>
+      </c>
+      <c r="D2488" t="inlineStr">
+        <is>
+          <t>探讨国际足联世界杯季军赛为何依然存在，是鸡肋还是含金量十足。</t>
+        </is>
+      </c>
+      <c r="E2488" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2488" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c4gk5jq2lj1o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2489">
+      <c r="A2489" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2489" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2489" t="inlineStr">
+        <is>
+          <t>Messi and Tom Brady in disbelief over 'prophetic' Lamine Yamal photo</t>
+        </is>
+      </c>
+      <c r="D2489" t="inlineStr">
+        <is>
+          <t>梅西与汤姆·布雷迪震惊于幼年梅西与亚马尔合影照的“预言性”。</t>
+        </is>
+      </c>
+      <c r="E2489" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2489" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c5yejxqll3go?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2490">
+      <c r="A2490" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B2490" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2490" t="inlineStr">
+        <is>
+          <t>False nines or firing forwards - England's potential life after Kane</t>
+        </is>
+      </c>
+      <c r="D2490" t="inlineStr">
+        <is>
+          <t>分析凯恩退役后英格兰队可能面临锋线变革，或使用伪9号。</t>
+        </is>
+      </c>
+      <c r="E2490" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2490" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cp87llz7539o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-19
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2490"/>
+  <dimension ref="A1:F2521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80117,6 +80117,998 @@
         </is>
       </c>
     </row>
+    <row r="2491">
+      <c r="A2491" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2491" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2491" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260719 21:00</t>
+        </is>
+      </c>
+      <c r="D2491" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道多项国内要闻及国际动态，包括城市民生、领导调研、物流发展等。</t>
+        </is>
+      </c>
+      <c r="E2491" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2491" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEq0sjDnvsKATGapoyWbwz260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2492" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2492" t="inlineStr">
+        <is>
+          <t>[视频]李希在重庆调研</t>
+        </is>
+      </c>
+      <c r="D2492" t="inlineStr">
+        <is>
+          <t>李希在重庆调研纪检监察工作，强调从严治党、服务民生和高质量发展。</t>
+        </is>
+      </c>
+      <c r="E2492" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2492" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEB2T9YEhrUoRQZ6MbTCRB260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2493" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2493" t="inlineStr">
+        <is>
+          <t>Burnham will be bolder but stick to Labour manifesto, deputy leader says</t>
+        </is>
+      </c>
+      <c r="D2493" t="inlineStr">
+        <is>
+          <t>英国副领袖称伯纳姆将更果敢，保守党领袖指责其讨好民众。</t>
+        </is>
+      </c>
+      <c r="E2493" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2493" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2k76gydreo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2494" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2494" t="inlineStr">
+        <is>
+          <t>Digital ID plan to be scrapped in Burnham's first major policy pledge</t>
+        </is>
+      </c>
+      <c r="D2494" t="inlineStr">
+        <is>
+          <t>英国新任首相拟废除数字身份证计划，称将聚焦民众当前需求。</t>
+        </is>
+      </c>
+      <c r="E2494" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2494" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c5y08z25q8eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2495" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2495" t="inlineStr">
+        <is>
+          <t>[视频]我国国家物流枢纽发展取得明显成效</t>
+        </is>
+      </c>
+      <c r="D2495" t="inlineStr">
+        <is>
+          <t>我国国家物流枢纽增至181个，去年吞吐量增长5.5%，智能化绿色化提速。</t>
+        </is>
+      </c>
+      <c r="E2495" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2495" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEvwFVzpp69hXkSD5GZ8f2260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2496" t="inlineStr">
+        <is>
+          <t>科技</t>
+        </is>
+      </c>
+      <c r="C2496" t="inlineStr">
+        <is>
+          <t>[视频]神舟二十三号乘组在轨近两月 各项工作有序推进</t>
+        </is>
+      </c>
+      <c r="D2496" t="inlineStr">
+        <is>
+          <t>神舟二十三号乘组在轨近两月，开展多项科学实验，包括太空人体研究计划。</t>
+        </is>
+      </c>
+      <c r="E2496" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2496" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEBxxgTl89vOUIfz7bWJV3260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2497" t="inlineStr">
+        <is>
+          <t>科技, 国际</t>
+        </is>
+      </c>
+      <c r="C2497" t="inlineStr">
+        <is>
+          <t>[视频]【新闻特写】连接彼此 共创未来</t>
+        </is>
+      </c>
+      <c r="D2497" t="inlineStr">
+        <is>
+          <t>上海2026世界人工智能大会促进全球交流，中外企业洽谈合作，技术寻找场景。</t>
+        </is>
+      </c>
+      <c r="E2497" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2497" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDE5wcrT07x7kqxIlVXeWnW260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2498" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2498" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2498" t="inlineStr">
+        <is>
+          <t>《2026中国AI盛典》启动；上海人形机器人中试服务平台启用；深圳上半年进出口增长33%。</t>
+        </is>
+      </c>
+      <c r="E2498" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2498" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEgEPHe2HfKlfwgUUEKv5t260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2499" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2499" t="inlineStr">
+        <is>
+          <t>[视频]美伊持续相互打击对方目标 伊朗称美违反承诺伊方已停止履行谅解备忘录</t>
+        </is>
+      </c>
+      <c r="D2499" t="inlineStr">
+        <is>
+          <t>美伊持续相互打击，伊朗称美违反备忘录，已停止履行伊美谅解备忘录。</t>
+        </is>
+      </c>
+      <c r="E2499" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2499" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEio3TwwL5x9kWvuT223aV260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2500">
+      <c r="A2500" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2500" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2500" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2500" t="inlineStr">
+        <is>
+          <t>俄乌互相打击物流设施；以军袭击加沙致儿童死亡；伊拉克重修输油管道；西班牙林火蔓延。</t>
+        </is>
+      </c>
+      <c r="E2500" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2500" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEVdlXXf31RiGjNK1rbFCL260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2501" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2501" t="inlineStr">
+        <is>
+          <t>US and Iran trade fire after two US soldiers killed in Jordan</t>
+        </is>
+      </c>
+      <c r="D2501" t="inlineStr">
+        <is>
+          <t>美伊交火，科威特水电厂遭袭起火，伊朗称美军击中在建核电站。</t>
+        </is>
+      </c>
+      <c r="E2501" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2501" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cgk417jp83po?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2502" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2502" t="inlineStr">
+        <is>
+          <t>Russia launches major ballistic missile attack on Ukrainian cities</t>
+        </is>
+      </c>
+      <c r="D2502" t="inlineStr">
+        <is>
+          <t>俄罗斯对乌克兰城市发动大规模导弹袭击，致5死35伤。</t>
+        </is>
+      </c>
+      <c r="E2502" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2502" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c2el7xpnzrpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2503" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2503" t="inlineStr">
+        <is>
+          <t>Deadly overnight Russian attack on Ukraine targets the capital</t>
+        </is>
+      </c>
+      <c r="D2503" t="inlineStr">
+        <is>
+          <t>俄军夜间向乌克兰发射41枚导弹和125架无人机，袭击首都基辅。</t>
+        </is>
+      </c>
+      <c r="E2503" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2503" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/19/nx-s1-5899518/russia-attack-kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2504" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2504" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】以人民为中心 绘就现代化城市民生幸福新画卷</t>
+        </is>
+      </c>
+      <c r="D2504" t="inlineStr">
+        <is>
+          <t>各地践行人民城市理念，提升宜居性和民生幸福，如北京热线升级、成都生态改善等。</t>
+        </is>
+      </c>
+      <c r="E2504" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2504" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEKB0zDafkD32iZL4Q9KWp260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2505" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2505" t="inlineStr">
+        <is>
+          <t>[视频]【树立和践行正确政绩观】为民造福 真抓实干 推动学习教育见行见效</t>
+        </is>
+      </c>
+      <c r="D2505" t="inlineStr">
+        <is>
+          <t>江西吉安、青海西宁通过开门教育和整改，解决民生痛点，推进城市更新。</t>
+        </is>
+      </c>
+      <c r="E2505" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2505" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEciAF87NQRHDxomwXeYsA260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2506" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2506" t="inlineStr">
+        <is>
+          <t>[视频]国家四部门部署做好地质灾害风险隐患巡查排查工作</t>
+        </is>
+      </c>
+      <c r="D2506" t="inlineStr">
+        <is>
+          <t>国家四部门部署加强地质灾害隐患排查和预警，确保群众安全转移。</t>
+        </is>
+      </c>
+      <c r="E2506" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2506" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDExlLD2sBiFfgtqjlexDCU260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2507" t="inlineStr">
+        <is>
+          <t>国际, 民生</t>
+        </is>
+      </c>
+      <c r="C2507" t="inlineStr">
+        <is>
+          <t>New EU border system tripling time at passport control, airport boss says</t>
+        </is>
+      </c>
+      <c r="D2507" t="inlineStr">
+        <is>
+          <t>欧盟新边境系统将导致护照检查时间增加两倍，瑞安航空警告旅客。</t>
+        </is>
+      </c>
+      <c r="E2507" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2507" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/ckg5gg6n9x3o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2508" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2508" t="inlineStr">
+        <is>
+          <t>Cuban dissident Luis Manuel Otero Alcántara goes into exile in US</t>
+        </is>
+      </c>
+      <c r="D2508" t="inlineStr">
+        <is>
+          <t>古巴异见人士奥坎塔拉在2021年抗议中被捕，服刑五年后流亡美国。</t>
+        </is>
+      </c>
+      <c r="E2508" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2508" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2k77p2r1xo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2509" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2509" t="inlineStr">
+        <is>
+          <t>Ferry carrying 116 passengers sinks off Guyana coast, authorities say</t>
+        </is>
+      </c>
+      <c r="D2509" t="inlineStr">
+        <is>
+          <t>一艘载有116人的渡轮在圭亚那海岸沉没，已有53人获救。</t>
+        </is>
+      </c>
+      <c r="E2509" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2509" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cm2gm99nrm7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2510" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2510" t="inlineStr">
+        <is>
+          <t>Cuban artist and dissident exiled from country after 5 years in prison arrives in US</t>
+        </is>
+      </c>
+      <c r="D2510" t="inlineStr">
+        <is>
+          <t>古巴异议艺术家兼音乐家奥尔特加服刑五年后获释，抵达美国迈阿密。</t>
+        </is>
+      </c>
+      <c r="E2510" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2510" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/19/nx-s1-5899494/cuban-artist-exile-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2511" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2511" t="inlineStr">
+        <is>
+          <t>[视频]“七一勋章”获得者吾哈斯·苏来曼：马背上的健康卫士</t>
+        </is>
+      </c>
+      <c r="D2511" t="inlineStr">
+        <is>
+          <t>“七一勋章”获得者吾哈斯·苏来曼从医五十余年，骑马巡诊守护牧民健康。</t>
+        </is>
+      </c>
+      <c r="E2511" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2511" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/19/VIDEuAX12GHFS7ufrjRuh3Ah260719.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2512" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2512" t="inlineStr">
+        <is>
+          <t>Tate brothers arrested in US as further UK charges take total to 59</t>
+        </is>
+      </c>
+      <c r="D2512" t="inlineStr">
+        <is>
+          <t>网红兄弟Tate在美国被捕，英国指控总数增至59项，律师称其无罪。</t>
+        </is>
+      </c>
+      <c r="E2512" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2512" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwymly9yd33o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2513">
+      <c r="A2513" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2513" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2513" t="inlineStr">
+        <is>
+          <t>Record numbers of honours for working class heroes</t>
+        </is>
+      </c>
+      <c r="D2513" t="inlineStr">
+        <is>
+          <t>来自贫困背景的获奖者人数创下纪录。</t>
+        </is>
+      </c>
+      <c r="E2513" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2513" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpd3dd3vv65o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2514" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2514" t="inlineStr">
+        <is>
+          <t>An Israeli paraglider tries to save migrating swifts that nest in the Western Wall</t>
+        </is>
+      </c>
+      <c r="D2514" t="inlineStr">
+        <is>
+          <t>以色列滑翔伞爱好者试图拯救筑巢在耶路撒冷西墙的迁徙雨燕。</t>
+        </is>
+      </c>
+      <c r="E2514" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2514" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/19/nx-s1-5870684/israel-swift-birds-jerusalem</t>
+        </is>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2515" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2515" t="inlineStr">
+        <is>
+          <t>Andrew and Tristan Tate arrested in Florida on charges of rape and sex trafficking</t>
+        </is>
+      </c>
+      <c r="D2515" t="inlineStr">
+        <is>
+          <t>网红安德鲁·塔特兄弟因强奸和性贩卖指控在佛罗里达被捕，英国寻求引渡。</t>
+        </is>
+      </c>
+      <c r="E2515" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2515" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/18/g-s1-134475/tate-brothers-arrested-miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2516" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2516" t="inlineStr">
+        <is>
+          <t>Runners take on 'world's coolest marathon' on drifting North Pole ice</t>
+        </is>
+      </c>
+      <c r="D2516" t="inlineStr">
+        <is>
+          <t>23名跑者参加北极点马拉松，在漂移冰面上挑战“世界最酷马拉松”。</t>
+        </is>
+      </c>
+      <c r="E2516" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2516" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/c9q9lw5rql4o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2517" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2517" t="inlineStr">
+        <is>
+          <t>Messi on the brink of history - will it be his last World Cup game?</t>
+        </is>
+      </c>
+      <c r="D2517" t="inlineStr">
+        <is>
+          <t>梅西将迎来第34场世界杯比赛，决赛或为其最后一届世界杯。</t>
+        </is>
+      </c>
+      <c r="E2517" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2517" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cql1xxxpndlo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2518" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2518" t="inlineStr">
+        <is>
+          <t>Why the World Cup half-time show may be a taste of things to come</t>
+        </is>
+      </c>
+      <c r="D2518" t="inlineStr">
+        <is>
+          <t>2026世界杯中场秀引发音乐融入体育赛事争议。</t>
+        </is>
+      </c>
+      <c r="E2518" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2518" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cwyr498vqqpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2519" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2519" t="inlineStr">
+        <is>
+          <t>Bruno Mars has an unexpected opening before Wembley party starts</t>
+        </is>
+      </c>
+      <c r="D2519" t="inlineStr">
+        <is>
+          <t>时隔八年，布鲁诺·马尔斯重返英国舞台，在温布利体育场举办精彩演出。</t>
+        </is>
+      </c>
+      <c r="E2519" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2519" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cyv0vvg1pqdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2520" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2520" t="inlineStr">
+        <is>
+          <t>I've been a World Cup official - I promise you there is no favouritism</t>
+        </is>
+      </c>
+      <c r="D2520" t="inlineStr">
+        <is>
+          <t>前世界杯裁判达伦·坎恩回应裁判偏袒阴谋论，讲述裁判真实想法。</t>
+        </is>
+      </c>
+      <c r="E2520" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2520" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/cm2g9g3v5gmo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B2521" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2521" t="inlineStr">
+        <is>
+          <t>Watch: Highlights as England stun France 6-4 in third-place play-off</t>
+        </is>
+      </c>
+      <c r="D2521" t="inlineStr">
+        <is>
+          <t>英格兰男足世界杯季军战6-4胜法国，萨卡帽子戏法创1966年以来最佳战绩。</t>
+        </is>
+      </c>
+      <c r="E2521" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2521" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/videos/cm2gn7v4jljo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-20
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2521"/>
+  <dimension ref="A1:F2558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81109,6 +81109,1190 @@
         </is>
       </c>
     </row>
+    <row r="2522">
+      <c r="A2522" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2522" t="inlineStr">
+        <is>
+          <t>政治, 经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2522" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260720 19:00</t>
+        </is>
+      </c>
+      <c r="D2522" t="inlineStr">
+        <is>
+          <t>新闻联播报道东西部协作、国务院常务会议、泰国总理访华、工业增长、AI大会等要闻。</t>
+        </is>
+      </c>
+      <c r="E2522" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2522" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEl36QYsQDjJej2cbTNGjS260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2523" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2523" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】常态化做好东西部协作 推动共同富裕迈出坚实步伐</t>
+        </is>
+      </c>
+      <c r="D2523" t="inlineStr">
+        <is>
+          <t>东西部协作助力乡村振兴，浙江茶苗捐赠带动四川等地茶产业，推动共同富裕。</t>
+        </is>
+      </c>
+      <c r="E2523" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2523" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEXUT7Tkt7bXSMlS6j0cf4260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2524" t="inlineStr">
+        <is>
+          <t>政治, 经济</t>
+        </is>
+      </c>
+      <c r="C2524" t="inlineStr">
+        <is>
+          <t>[视频]李强主持召开国务院常务会议</t>
+        </is>
+      </c>
+      <c r="D2524" t="inlineStr">
+        <is>
+          <t>李强主持召开国务院常务会议，审议服务业、六张网规划及知识产权保护等议题。</t>
+        </is>
+      </c>
+      <c r="E2524" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2524" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEqj4hCj83pvlSxUosa9V3260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2525" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2525" t="inlineStr">
+        <is>
+          <t>[视频]李强举行仪式欢迎泰国总理访华</t>
+        </is>
+      </c>
+      <c r="D2525" t="inlineStr">
+        <is>
+          <t>李强在北京人民大会堂举行仪式，欢迎泰国总理阿努廷正式访华。</t>
+        </is>
+      </c>
+      <c r="E2525" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2525" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEi6PE57Tm4tMnlDpajrLP260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2526" t="inlineStr">
+        <is>
+          <t>政治, 国际, 科技</t>
+        </is>
+      </c>
+      <c r="C2526" t="inlineStr">
+        <is>
+          <t>[视频]李强同泰国总理会谈</t>
+        </is>
+      </c>
+      <c r="D2526" t="inlineStr">
+        <is>
+          <t>李强同泰国总理会谈，双方同意深化一带一路、人工智能等合作，打击跨境犯罪。</t>
+        </is>
+      </c>
+      <c r="E2526" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2526" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDET5saix8hXX6X7Su8ubKe260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2527" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2527" t="inlineStr">
+        <is>
+          <t>[视频]赵乐际会见泰国总理</t>
+        </is>
+      </c>
+      <c r="D2527" t="inlineStr">
+        <is>
+          <t>赵乐际会见泰国总理阿努廷，强调加强立法机构交往，推动中泰命运共同体建设。</t>
+        </is>
+      </c>
+      <c r="E2527" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2527" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEyDdSW7SWTLm2lGrKLhBy260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2528" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2528" t="inlineStr">
+        <is>
+          <t>Hamas names Khalil al-Hayya as new overall leader</t>
+        </is>
+      </c>
+      <c r="D2528" t="inlineStr">
+        <is>
+          <t>哈马斯任命驻卡塔尔首席谈判官哈利勒·哈亚为新领导人。</t>
+        </is>
+      </c>
+      <c r="E2528" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2528" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx25nzkyj50o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2529" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2529" t="inlineStr">
+        <is>
+          <t>JD Vance says wife Usha and son 'happy and healthy' after birth of fourth child</t>
+        </is>
+      </c>
+      <c r="D2529" t="inlineStr">
+        <is>
+          <t>美国副总统万斯宣布妻子乌莎顺利产下第四子。</t>
+        </is>
+      </c>
+      <c r="E2529" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2529" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cj63kngxpxpo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2530" t="inlineStr">
+        <is>
+          <t>政治, 民生</t>
+        </is>
+      </c>
+      <c r="C2530" t="inlineStr">
+        <is>
+          <t>Burnham promises help with your money. How could it affect you?</t>
+        </is>
+      </c>
+      <c r="D2530" t="inlineStr">
+        <is>
+          <t>英国新首相伯纳姆承诺改善民生，让生活更实惠。</t>
+        </is>
+      </c>
+      <c r="E2530" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2530" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cp9ezldrkkgo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2531" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2531" t="inlineStr">
+        <is>
+          <t>Burnham's policy choices reveal what kind of PM he wants to be</t>
+        </is>
+      </c>
+      <c r="D2531" t="inlineStr">
+        <is>
+          <t>伯纳姆通过政策选择展现其首相愿景，承诺终结露宿现象。</t>
+        </is>
+      </c>
+      <c r="E2531" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2531" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c3r0x5nzg0eo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2532" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2532" t="inlineStr">
+        <is>
+          <t>Key takeaways as Andy Burnham becomes PM</t>
+        </is>
+      </c>
+      <c r="D2532" t="inlineStr">
+        <is>
+          <t>英国新任首相伯纳姆正式就职，公布执政优先事项。</t>
+        </is>
+      </c>
+      <c r="E2532" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2532" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c80nln7zgp7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2533" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2533" t="inlineStr">
+        <is>
+          <t>Watch: Starmer resigns, Burnham becomes PM... the day so far</t>
+        </is>
+      </c>
+      <c r="D2533" t="inlineStr">
+        <is>
+          <t>斯塔默辞职，伯纳姆被国王任命为英国新首相。</t>
+        </is>
+      </c>
+      <c r="E2533" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2533" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/videos/cd0xgxgz135o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2534" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2534" t="inlineStr">
+        <is>
+          <t>Who is Andy Burnham's wife, Marie-France van Heel?</t>
+        </is>
+      </c>
+      <c r="D2534" t="inlineStr">
+        <is>
+          <t>英国新首相伯纳姆的妻子玛丽-弗朗斯·范·希尔是营销高管。</t>
+        </is>
+      </c>
+      <c r="E2534" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2534" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c75y4q61eevo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2535" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2535" t="inlineStr">
+        <is>
+          <t>Prisons minister Lord Timpson quits government</t>
+        </is>
+      </c>
+      <c r="D2535" t="inlineStr">
+        <is>
+          <t>英国监狱大臣蒂姆森勋爵辞职，称已实现该职位所有目标。</t>
+        </is>
+      </c>
+      <c r="E2535" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2535" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg0xlrvv4mo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2536" t="inlineStr">
+        <is>
+          <t>政治, 国际</t>
+        </is>
+      </c>
+      <c r="C2536" t="inlineStr">
+        <is>
+          <t>Andy Burnham becomes U.K. prime minister</t>
+        </is>
+      </c>
+      <c r="D2536" t="inlineStr">
+        <is>
+          <t>安迪·伯纳姆接替基尔·斯塔默成为英国首相。</t>
+        </is>
+      </c>
+      <c r="E2536" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2536" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/19/nx-s1-5895993/andy-burnham-prime-minister-keir-starmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2537" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2537" t="inlineStr">
+        <is>
+          <t>[视频]上半年我国规模以上工业增加值同比增长5.4%</t>
+        </is>
+      </c>
+      <c r="D2537" t="inlineStr">
+        <is>
+          <t>上半年我国规模以上工业增加值同比增长5.4%，创新成果涌现，产业结构优化。</t>
+        </is>
+      </c>
+      <c r="E2537" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2537" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEX81o7FI2LEkvusNNgDml260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2538" t="inlineStr">
+        <is>
+          <t>科技, 经济</t>
+        </is>
+      </c>
+      <c r="C2538" t="inlineStr">
+        <is>
+          <t>[视频]世界人工智能大会达成丰硕成果</t>
+        </is>
+      </c>
+      <c r="D2538" t="inlineStr">
+        <is>
+          <t>2026世界人工智能大会闭幕，发布多项成果，设立1.18万亿元创新企业信贷额度。</t>
+        </is>
+      </c>
+      <c r="E2538" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2538" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEcPKAfKcEOi0fJwrePdfs260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2539" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2539" t="inlineStr">
+        <is>
+          <t>[视频]美称打击伊朗导弹发射场 伊朗称摧毁美军雷达系统</t>
+        </is>
+      </c>
+      <c r="D2539" t="inlineStr">
+        <is>
+          <t>美军连续打击伊朗目标，伊朗摧毁美军雷达系统并用弹道导弹反击，美伊冲突持续升级。</t>
+        </is>
+      </c>
+      <c r="E2539" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2539" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEbsz2321sOZu0LTAdx0Xt260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2540" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2540" t="inlineStr">
+        <is>
+          <t>Ten killed as Russian attacks on merchant ships in Black Sea intensify</t>
+        </is>
+      </c>
+      <c r="D2540" t="inlineStr">
+        <is>
+          <t>俄罗斯袭击黑海商船，7月敖德萨地区已致28人死亡。</t>
+        </is>
+      </c>
+      <c r="E2540" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2540" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gvpv3ewv2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2541" t="inlineStr">
+        <is>
+          <t>军事, 国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2541" t="inlineStr">
+        <is>
+          <t>3 U.S. personnel killed in Iran conflict. And, Hunter Biden opens up to NPR</t>
+        </is>
+      </c>
+      <c r="D2541" t="inlineStr">
+        <is>
+          <t>三名美军在伊朗冲突中丧生；亨特·拜登接受专访。</t>
+        </is>
+      </c>
+      <c r="E2541" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2541" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/20/g-s1-134553/up-first-newsletter-iran-us-service-members-hunter-biden</t>
+        </is>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2542" t="inlineStr">
+        <is>
+          <t>军事, 国际</t>
+        </is>
+      </c>
+      <c r="C2542" t="inlineStr">
+        <is>
+          <t>U.S. and Iran launch new strikes after 3 U.S. service members are killed</t>
+        </is>
+      </c>
+      <c r="D2542" t="inlineStr">
+        <is>
+          <t>美伊互相发动新袭击，和谈因霍尔木兹海峡协议破裂。</t>
+        </is>
+      </c>
+      <c r="E2542" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2542" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/20/nx-s1-5900601/us-iran-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2543" t="inlineStr">
+        <is>
+          <t>民生</t>
+        </is>
+      </c>
+      <c r="C2543" t="inlineStr">
+        <is>
+          <t>[视频]各地加快推进住宅老旧电梯更新改造</t>
+        </is>
+      </c>
+      <c r="D2543" t="inlineStr">
+        <is>
+          <t>国家安排超长期特别国债约309亿元，支持各地更新住宅老旧电梯19.7万台，并加装电梯2.8万台。</t>
+        </is>
+      </c>
+      <c r="E2543" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2543" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEA4coNYG9FN7PPvbvBKgD260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2544" t="inlineStr">
+        <is>
+          <t>民生, 社会</t>
+        </is>
+      </c>
+      <c r="C2544" t="inlineStr">
+        <is>
+          <t>[视频]未来三天广西湖南江西江苏等地雨势较强</t>
+        </is>
+      </c>
+      <c r="D2544" t="inlineStr">
+        <is>
+          <t>未来三天华南、江南等地有较强降雨，山洪、内涝风险高，需加强防范。</t>
+        </is>
+      </c>
+      <c r="E2544" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2544" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEeCdklt9l2XHqe6fIvE9E260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2545" t="inlineStr">
+        <is>
+          <t>国际, 科技</t>
+        </is>
+      </c>
+      <c r="C2545" t="inlineStr">
+        <is>
+          <t>[视频]国际媒体积极评价中国推动人工智能发展与全球人工智能治理</t>
+        </is>
+      </c>
+      <c r="D2545" t="inlineStr">
+        <is>
+          <t>国际媒体积极评价中国推动人工智能发展与全球治理，称中国为全球AI向上向善注入动力。</t>
+        </is>
+      </c>
+      <c r="E2545" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2545" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDE3qinlnWwALoJuWayBBU9260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2546" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2546" t="inlineStr">
+        <is>
+          <t>[视频]日本民众集会反对高市政权修宪扩军等危险动向</t>
+        </is>
+      </c>
+      <c r="D2546" t="inlineStr">
+        <is>
+          <t>日本民众在国会前集会，反对高市政权推动修宪和试图拥核等危险动向。</t>
+        </is>
+      </c>
+      <c r="E2546" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2546" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEQwmqXjpCkl3qUKmkq1Hc260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2547" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2547" t="inlineStr">
+        <is>
+          <t>[视频]国际联播快讯</t>
+        </is>
+      </c>
+      <c r="D2547" t="inlineStr">
+        <is>
+          <t>俄乌互相打击油气设施；美媒披露美沙核项目合作草案；加拿大林火致美国要求赔偿。</t>
+        </is>
+      </c>
+      <c r="E2547" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2547" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEg1Tk3igSfqr1Oc1QpPkn260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2548" t="inlineStr">
+        <is>
+          <t>国际, 军事</t>
+        </is>
+      </c>
+      <c r="C2548" t="inlineStr">
+        <is>
+          <t>Trump says US strikes hit Iran in 'honour' of American soldiers killed</t>
+        </is>
+      </c>
+      <c r="D2548" t="inlineStr">
+        <is>
+          <t>特朗普称美军为阵亡士兵打击伊朗，伊朗在叙利亚和约旦反击，两艘油轮在霍尔木兹海峡爆炸。</t>
+        </is>
+      </c>
+      <c r="E2548" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2548" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cly52xzjd3qo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2549" t="inlineStr">
+        <is>
+          <t>国际, 社会</t>
+        </is>
+      </c>
+      <c r="C2549" t="inlineStr">
+        <is>
+          <t>Scores feared dead after passenger ferry capsizes off Guyana</t>
+        </is>
+      </c>
+      <c r="D2549" t="inlineStr">
+        <is>
+          <t>圭亚那海域渡轮倾覆，67人获救，预计超130人遇难。</t>
+        </is>
+      </c>
+      <c r="E2549" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2549" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cm2gm99nrm7o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2550" t="inlineStr">
+        <is>
+          <t>国际, 政治</t>
+        </is>
+      </c>
+      <c r="C2550" t="inlineStr">
+        <is>
+          <t>Putin meets North Korean foreign minister in diplomatic push</t>
+        </is>
+      </c>
+      <c r="D2550" t="inlineStr">
+        <is>
+          <t>朝鲜外相访俄，或为金正恩访俄做准备。</t>
+        </is>
+      </c>
+      <c r="E2550" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2550" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/20/g-s1-134555/putin-meets-north-korean-foreign-minister-in-diplomatic-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2551" t="inlineStr">
+        <is>
+          <t>社会, 民生, 科技</t>
+        </is>
+      </c>
+      <c r="C2551" t="inlineStr">
+        <is>
+          <t>[视频]国内联播快讯</t>
+        </is>
+      </c>
+      <c r="D2551" t="inlineStr">
+        <is>
+          <t>水利部启动水文现代化建设三年行动；国务院食安办部署暑期汛期食品安全；将开展村镇微能网试点和未成年人网络保护专项行动。</t>
+        </is>
+      </c>
+      <c r="E2551" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2551" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/20/VIDEacJarp0aBrD0os264Dec260720.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2552" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2552" t="inlineStr">
+        <is>
+          <t>Boy, 13, dies during World Cup celebrations in Spain</t>
+        </is>
+      </c>
+      <c r="D2552" t="inlineStr">
+        <is>
+          <t>西班牙世界杯庆祝活动中，一喷泉部分坍塌致13岁男孩死亡。</t>
+        </is>
+      </c>
+      <c r="E2552" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2552" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c0qvdy0jv05o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2553" t="inlineStr">
+        <is>
+          <t>社会, 民生</t>
+        </is>
+      </c>
+      <c r="C2553" t="inlineStr">
+        <is>
+          <t>Police block thousands of 'cockroach' protesters marching on India's parliament</t>
+        </is>
+      </c>
+      <c r="D2553" t="inlineStr">
+        <is>
+          <t>印度警方阻止数千名要求教育改革抗议者前往议会，发生冲突。</t>
+        </is>
+      </c>
+      <c r="E2553" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2553" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cvg9w9dxd7lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2554" t="inlineStr">
+        <is>
+          <t>社会</t>
+        </is>
+      </c>
+      <c r="C2554" t="inlineStr">
+        <is>
+          <t>Rare identical quadruplets born in Australia</t>
+        </is>
+      </c>
+      <c r="D2554" t="inlineStr">
+        <is>
+          <t>澳大利亚一对夫妇自然受孕诞下罕见四胞胎女婴。</t>
+        </is>
+      </c>
+      <c r="E2554" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2554" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cx2jnj3428lo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2555" t="inlineStr">
+        <is>
+          <t>社会, 文体</t>
+        </is>
+      </c>
+      <c r="C2555" t="inlineStr">
+        <is>
+          <t>Ofcom launches investigation into Married at First Sight UK</t>
+        </is>
+      </c>
+      <c r="D2555" t="inlineStr">
+        <is>
+          <t>英国通信管理局对《一见钟情结婚》节目启动调查，此前曝出强奸指控。</t>
+        </is>
+      </c>
+      <c r="E2555" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2555" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c4gyyx2zg59o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2556" t="inlineStr">
+        <is>
+          <t>社会, 国际</t>
+        </is>
+      </c>
+      <c r="C2556" t="inlineStr">
+        <is>
+          <t>At least 930 people have died in Congo's Ebola outbreak</t>
+        </is>
+      </c>
+      <c r="D2556" t="inlineStr">
+        <is>
+          <t>刚果埃博拉疫情已致至少930人死亡，新增37例。</t>
+        </is>
+      </c>
+      <c r="E2556" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2556" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/20/g-s1-134548/ebola-congo-deaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2557" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2557" t="inlineStr">
+        <is>
+          <t>Newcastle, Liverpool and England legend Keegan dies</t>
+        </is>
+      </c>
+      <c r="D2557" t="inlineStr">
+        <is>
+          <t>英格兰传奇球星凯文·基冈去世，享年75岁。</t>
+        </is>
+      </c>
+      <c r="E2557" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2557" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/football/articles/c2lyl82n2e2o?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2558" t="inlineStr">
+        <is>
+          <t>文体</t>
+        </is>
+      </c>
+      <c r="C2558" t="inlineStr">
+        <is>
+          <t>Lamine Yamal celebrates World Cup win with little brother who charmed fans</t>
+        </is>
+      </c>
+      <c r="D2558" t="inlineStr">
+        <is>
+          <t>亚马尔三岁弟弟因世界杯夺冠走红，被球迷赞为西班牙队新星。</t>
+        </is>
+      </c>
+      <c r="E2558" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2558" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c89nvnklkpdo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📰 Daily news update: 2026-07-21
</commit_message>
<xml_diff>
--- a/data/daily_news.xlsx
+++ b/data/daily_news.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2558"/>
+  <dimension ref="A1:F2595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82293,6 +82293,1190 @@
         </is>
       </c>
     </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2559" t="inlineStr">
+        <is>
+          <t>政治, 经济, 民生</t>
+        </is>
+      </c>
+      <c r="C2559" t="inlineStr">
+        <is>
+          <t>《新闻联播》 20260721 19:00</t>
+        </is>
+      </c>
+      <c r="D2559" t="inlineStr">
+        <is>
+          <t>《新闻联播》报道节能降碳、粮食生产、交通规划等多项国内国际新闻。</t>
+        </is>
+      </c>
+      <c r="E2559" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2559" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/21/VIDEE5isjDLlQsaBNYZPXfzR260721.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2560" t="inlineStr">
+        <is>
+          <t>政治, 军事</t>
+        </is>
+      </c>
+      <c r="C2560" t="inlineStr">
+        <is>
+          <t>Row escalates in Ukraine over army chief's future</t>
+        </is>
+      </c>
+      <c r="D2560" t="inlineStr">
+        <is>
+          <t>乌克兰围绕军队总司令的未来爆发争议，抗议者要求其下台。</t>
+        </is>
+      </c>
+      <c r="E2560" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2560" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c7vgel8374yo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2561" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2561" t="inlineStr">
+        <is>
+          <t>Shock and anger after top Ghanaian politician sentenced to 20 years for illegal mining</t>
+        </is>
+      </c>
+      <c r="D2561" t="inlineStr">
+        <is>
+          <t>加纳知名政客因非法采矿被判20年监禁及罚款，引发社会震惊与愤怒。</t>
+        </is>
+      </c>
+      <c r="E2561" t="inlineStr">
+        <is>
+          <t>BBC World</t>
+        </is>
+      </c>
+      <c r="F2561" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/cpvwnjllwvwo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2562" t="inlineStr">
+        <is>
+          <t>政治</t>
+        </is>
+      </c>
+      <c r="C2562" t="inlineStr">
+        <is>
+          <t>London-based civil servants offered move to No 10 North in Manchester</t>
+        </is>
+      </c>
+      <c r="D2562" t="inlineStr">
+        <is>
+          <t>伦敦公务员被通知可搬迁至曼彻斯特的“北方唐宁街10号”，并提供安置方案。</t>
+        </is>
+      </c>
+      <c r="E2562" t="inlineStr">
+        <is>
+          <t>BBC Top</t>
+        </is>
+      </c>
+      <c r="F2562" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/news/articles/c9d8p0l29pxo?at_medium=RSS&amp;at_campaign=rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2563" t="inlineStr">
+        <is>
+          <t>政治, 社会</t>
+        </is>
+      </c>
+      <c r="C2563" t="inlineStr">
+        <is>
+          <t>India's youth-led Cockroach movement vows to continue protest after police crackdown</t>
+        </is>
+      </c>
+      <c r="D2563" t="inlineStr">
+        <is>
+          <t>印度青年领导的“蟑螂运动”在警方镇压后誓言继续抗议，已演变为全国性挑战总理莫迪政府。</t>
+        </is>
+      </c>
+      <c r="E2563" t="inlineStr">
+        <is>
+          <t>NPR World</t>
+        </is>
+      </c>
+      <c r="F2563" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/07/21/g-s1-134722/indias-youth-led-cockroach-movement-vows-to-continue-protest-after-police-crackdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2564" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2564" t="inlineStr">
+        <is>
+          <t>[视频]【新思想引领新征程】加力推进节能降碳 书写绿色发展新答卷</t>
+        </is>
+      </c>
+      <c r="D2564" t="inlineStr">
+        <is>
+          <t>我国加力推进节能降碳，能源利用效率提升，绿色生产生活方式加快形成。</t>
+        </is>
+      </c>
+      <c r="E2564" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2564" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/21/VIDEdWaANn0x9nbjTWimAK0o260721.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2565" t="inlineStr">
+        <is>
+          <t>经济, 科技</t>
+        </is>
+      </c>
+      <c r="C2565" t="inlineStr">
+        <is>
+          <t>[视频]【“十五五”开好局起好步】2030年我国基本建成现代化综合交通运输体系</t>
+        </is>
+      </c>
+      <c r="D2565" t="inlineStr">
+        <is>
+          <t>我国2030年将基本建成现代化综合交通运输体系，推进大通道建设。</t>
+        </is>
+      </c>
+      <c r="E2565" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2565" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/21/VIDEel3NGnt8ds3J4SOIU0yj260721.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2566" t="inlineStr">
+        <is>
+          <t>经济</t>
+        </is>
+      </c>
+      <c r="C2566" t="inlineStr">
+        <is>
+          <t>[视频]万亿元民营企业再贷款落地 支持民营经济发展</t>
+        </is>
+      </c>
+      <c r="D2566" t="inlineStr">
+        <is>
+          <t>中国人民银行新设1万亿元民营企业再贷款，缓解民营中型企业融资难题。</t>
+        </is>
+      </c>
+      <c r="E2566" t="inlineStr">
+        <is>
+          <t>新闻联播</t>
+        </is>
+      </c>
+      <c r="F2566" t="inlineStr">
+        <is>
+          <t>https://tv.cctv.com/2026/07/21/VIDEfqnZx8HYikU8kPWiH4of260721.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B2567" t="inlineStr">
+        <is>
+          <t>经济, 国际</t>
+        </is>
+      </c>
+      <c r="C2567" t="inlineStr">
+        <is>
+          <t>[视频]免签政策持续发力 入境游市场热力攀升</t>
+        </is>
+      </c>
+      <c r="D2567" t=